<commit_message>
Atualiza Disponibilidade Diária com o relatório de 06/07/2026
Novo relatório do dia 06/07 (não havia relatórios entre 03 e 05/07),
reprocessado sem inconsistências.
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,6 +687,81 @@
       <c r="U3" t="inlineStr">
         <is>
           <t>Disponibilidade_02_07_2026.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L4" t="n">
+        <v>21</v>
+      </c>
+      <c r="M4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2703, 2708, 2709, 2741</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2721, 2723</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>10070:00</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>4317:55</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>42.88</v>
+      </c>
+      <c r="T4" t="n">
+        <v>24</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Disponibilidade_06_07_2026.txt</t>
         </is>
       </c>
     </row>
@@ -701,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2484,6 +2559,858 @@
         <v>46205</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2733</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2739</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Agd parecer do AT do PAMASP sobre FCU</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>07/07</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2727</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1º/15º GAV</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2702</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A / 500FH</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>14/07</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2703</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2729</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>31/07</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Realizando inspeções 4300 FH/HSI.</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2722</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>5º ETA</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2709</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Pane no sistema de flape</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>07/07</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2720</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2721</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Motor recolhido para reparo na geradora de gases</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>13/07</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2736</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2737</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2738</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2740</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2741</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>07/07</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2723</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Itens entregues. Agd AT de hélice para definição de recolhimento ou translado da aeronave para o Parque</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2742</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>DACTA II</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2704</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>75 APE</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2724</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ANV acidentada.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>91 AIFP. Serão atendidas pela Vee One e FAB</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Aguardando avaliação de sinistro</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>06/07</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2730</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 44 IPLR</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2732</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 13 IPLR</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2734</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 57 IPLR</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>46209</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corrige bug de BOM que quebrava a busca automática da Disponibilidade Diária
O GitHub Actions não disparou o agendamento das 10h de hoje (falha conhecida
do GitHub Actions com a 1ª execução de um schedule recém-criado) e, ao
buscar manualmente pra compensar, descobrimos que o parser quebrava de
verdade: o Google Docs exporta texto com BOM, que a busca manual (feita por
mim em conversas anteriores) nunca expunha, mas o caminho automático sim.
Corrigido lendo/decodificando com utf-8-sig em vez de utf-8.

Atualiza também o relatório de 07/07/2026 (11 D / 21 M).
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -762,6 +762,81 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>Disponibilidade_06_07_2026.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C5" t="n">
+        <v>21</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" t="n">
+        <v>21</v>
+      </c>
+      <c r="M5" t="n">
+        <v>19</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2702, 2709, 2719, 2721, 2733, 2736, 2741, 2743</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>22</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2721, 2723</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>10070:00</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>4374:25</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>43.44</v>
+      </c>
+      <c r="T5" t="n">
+        <v>24</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Disponibilidade_07_07_2026.txt</t>
         </is>
       </c>
     </row>
@@ -776,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3411,6 +3486,888 @@
         <v>46209</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2733</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>14/07</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2739</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Agd parecer do AT do PAMASP sobre FCU</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>07/07</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2727</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1º/15º GAV</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2702</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A / 500FH</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>14/07</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2703</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2729</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>31/07</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Realizando inspeções 4300 FH/HSI.</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2722</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>5º ETA</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2709</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Pane no sistema de flape</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2720</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2721</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Motor recolhido para reparo na geradora de gases</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>13/07</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2736</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2737</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2738</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2740</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2741</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2723</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Itens entregues. Agd AT de hélice para definição de recolhimento ou translado da aeronave para o Parque</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2742</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>DACTA II</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2704</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>75 APE</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2724</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>ANV acidentada.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>91 AIFP. Serão atendidas pela Vee One e FAB</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Aguardando avaliação de sinistro</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>06/07</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2730</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 44 IPLR</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2732</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 13 IPLR</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2734</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 57 IPLR</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corrige bug: Disponibilidade Diária podia nunca reprocessar
atualizar_do_drive() pulava o reprocessamento inteiro quando o .txt do dia
já existia localmente (early return antes de chamar main()) — isso deixou
a planilha tratada (e o site) desatualizada em relação aos dados de
08/07/2026, mesmo com o relatório certo já salvo. Agora sempre reprocessa
(main()), independente de ter baixado algo novo ou não; só o status
"atualizado" vs "sem_novidade" e o registro de fetch remoto dependem de
achar um relatório realmente novo.
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -837,6 +837,81 @@
       <c r="U5" t="inlineStr">
         <is>
           <t>Disponibilidade_07_07_2026.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L6" t="n">
+        <v>19</v>
+      </c>
+      <c r="M6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2709, 2719, 2736, 2741, 2743</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>22</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2709, 2721, 2723</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>10070:00</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>4406:50</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>43.76</v>
+      </c>
+      <c r="T6" t="n">
+        <v>24</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Disponibilidade_08_07_2026.txt</t>
         </is>
       </c>
     </row>
@@ -851,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4368,6 +4443,868 @@
         <v>46210</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2733</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>14/07</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2739</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2727</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1º/15º GAV</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2702</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2703</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2729</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>31/07</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Realizando inspeções 4300 FH/HSI.</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2722</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>5º ETA</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2709</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Pane no sistema de flape</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2720</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2721</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Motor recolhido para reparo na geradora de gases</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>13/07</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2736</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2737</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2738</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2740</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2741</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2723</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Itens entregues. Agd AT de hélice para definição de recolhimento ou translado da aeronave para o Parque</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2742</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>DACTA II</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2704</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>75 APE</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2724</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>ANV acidentada.</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>91 AIFP. Serão atendidas pela Vee One e FAB</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Aguardando avaliação de sinistro</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>06/07</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2730</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 44 IPLR</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2732</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 13 IPLR</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2734</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 57 IPLR</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="n">
+        <v>46211</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (09/07/2026 09:58)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,6 +912,81 @@
       <c r="U6" t="inlineStr">
         <is>
           <t>Disponibilidade_08_07_2026.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" t="n">
+        <v>18</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" t="n">
+        <v>13</v>
+      </c>
+      <c r="L7" t="n">
+        <v>18</v>
+      </c>
+      <c r="M7" t="n">
+        <v>19</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2709, 2719, 2721, 2733, 2736, 2741, 2743</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>21</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2709, 2721, 2723</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>10070:00</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>4463:45</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>44.33</v>
+      </c>
+      <c r="T7" t="n">
+        <v>24</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Disponibilidade_09_07_2026.txt</t>
         </is>
       </c>
     </row>
@@ -926,7 +1001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5305,6 +5380,878 @@
         <v>46211</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2733</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>14/07</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2739</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2727</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1º/15º GAV</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2702</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2703</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2729</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>31/07</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Realizando inspeções 4300 FH/HSI.</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2722</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>5º ETA</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2709</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Pane no sistema de flape</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2720</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>EM PESQUISA DE PANE DE FCU</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>09/07</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2721</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Motor recolhido para reparo na geradora de gases</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>13/07</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2736</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2737</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2738</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2740</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2741</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2723</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Itens entregues. Agd AT de hélice para definição de recolhimento ou translado da aeronave para o Parque</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2742</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>DACTA II</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2704</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>75 APE</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2724</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>ANV acidentada.</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>91 AIFP. Serão atendidas pela Vee One e FAB</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Aguardando avaliação de sinistro</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>06/07</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2730</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 44 IPLR</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2732</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 13 IPLR</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2734</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 57 IPLR</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="n">
+        <v>46212</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (09/07/2026 23:46)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,114 +422,114 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -616,7 +604,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -691,7 +679,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -766,7 +754,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -841,7 +829,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -916,7 +904,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -1005,42 +993,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1066,7 +1054,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1090,7 +1078,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1126,7 +1114,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1150,7 +1138,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1174,7 +1162,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1199,7 +1187,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1208,7 +1196,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1233,7 +1221,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1242,7 +1230,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1267,7 +1255,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1276,7 +1264,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1301,7 +1289,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1310,7 +1298,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1334,7 +1322,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1358,7 +1346,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1383,7 +1371,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1392,7 +1380,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1416,7 +1404,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1441,7 +1429,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1450,7 +1438,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1474,7 +1462,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1498,7 +1486,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1523,7 +1511,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1532,7 +1520,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1556,7 +1544,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1581,7 +1569,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1590,7 +1578,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1626,7 +1614,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1650,7 +1638,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1674,7 +1662,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1710,7 +1698,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1738,7 +1726,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1774,7 +1762,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1799,7 +1787,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1808,7 +1796,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1844,7 +1832,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1880,7 +1868,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1916,7 +1904,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1940,7 +1928,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -1964,7 +1952,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2000,7 +1988,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2024,7 +2012,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2048,7 +2036,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="2" t="n">
+      <c r="H35" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2073,7 +2061,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2082,7 +2070,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="H36" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2107,7 +2095,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2116,7 +2104,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2141,7 +2129,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2150,7 +2138,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2175,7 +2163,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E39" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2184,7 +2172,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2208,7 +2196,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="2" t="n">
+      <c r="H40" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2232,7 +2220,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="2" t="n">
+      <c r="H41" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2257,7 +2245,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E42" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2266,7 +2254,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="H42" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2290,7 +2278,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2315,7 +2303,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2324,7 +2312,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="H44" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2348,7 +2336,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="2" t="n">
+      <c r="H45" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2372,7 +2360,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2396,7 +2384,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="2" t="n">
+      <c r="H47" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2420,7 +2408,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="2" t="n">
+      <c r="H48" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2445,7 +2433,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E49" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2454,7 +2442,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="H49" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2490,7 +2478,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2514,7 +2502,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="2" t="n">
+      <c r="H51" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2538,7 +2526,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="2" t="n">
+      <c r="H52" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2574,7 +2562,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="H53" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2602,7 +2590,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2638,7 +2626,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="H55" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2663,7 +2651,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2672,7 +2660,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="H56" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2708,7 +2696,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="H57" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2744,7 +2732,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="n">
+      <c r="H58" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2780,7 +2768,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="H59" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2804,7 +2792,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="2" t="n">
+      <c r="H60" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2828,7 +2816,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="2" t="n">
+      <c r="H61" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2853,7 +2841,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2862,7 +2850,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="2" t="n">
+      <c r="H62" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2886,7 +2874,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="2" t="n">
+      <c r="H63" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2911,7 +2899,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n">
+      <c r="E64" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2920,7 +2908,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="H64" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2944,7 +2932,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="2" t="n">
+      <c r="H65" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2968,7 +2956,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="2" t="n">
+      <c r="H66" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2993,7 +2981,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n">
+      <c r="E67" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3002,7 +2990,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="2" t="n">
+      <c r="H67" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3027,7 +3015,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n">
+      <c r="E68" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3036,7 +3024,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="2" t="n">
+      <c r="H68" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3060,7 +3048,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="2" t="n">
+      <c r="H69" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3084,7 +3072,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="2" t="n">
+      <c r="H70" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3109,7 +3097,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="2" t="n">
+      <c r="E71" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3118,7 +3106,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="2" t="n">
+      <c r="H71" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3142,7 +3130,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="2" t="n">
+      <c r="H72" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3167,7 +3155,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n">
+      <c r="E73" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3176,7 +3164,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="2" t="n">
+      <c r="H73" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3200,7 +3188,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="2" t="n">
+      <c r="H74" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3224,7 +3212,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="2" t="n">
+      <c r="H75" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3248,7 +3236,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="2" t="n">
+      <c r="H76" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3272,7 +3260,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="2" t="n">
+      <c r="H77" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3297,7 +3285,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E78" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3306,7 +3294,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="2" t="n">
+      <c r="H78" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3342,7 +3330,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="2" t="n">
+      <c r="H79" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3366,7 +3354,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="2" t="n">
+      <c r="H80" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3390,7 +3378,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="2" t="n">
+      <c r="H81" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3426,7 +3414,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="2" t="n">
+      <c r="H82" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3454,7 +3442,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="2" t="n">
+      <c r="H83" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3490,7 +3478,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="2" t="n">
+      <c r="H84" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3515,7 +3503,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n">
+      <c r="E85" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3524,7 +3512,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="2" t="n">
+      <c r="H85" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3560,7 +3548,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="2" t="n">
+      <c r="H86" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3596,7 +3584,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="2" t="n">
+      <c r="H87" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3632,7 +3620,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="2" t="n">
+      <c r="H88" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3656,7 +3644,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="2" t="n">
+      <c r="H89" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3681,7 +3669,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3690,7 +3678,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="2" t="n">
+      <c r="H90" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3715,7 +3703,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n">
+      <c r="E91" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3724,7 +3712,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="2" t="n">
+      <c r="H91" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3748,7 +3736,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="2" t="n">
+      <c r="H92" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3773,7 +3761,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="2" t="n">
+      <c r="E93" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3782,7 +3770,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="2" t="n">
+      <c r="H93" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3806,7 +3794,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="2" t="n">
+      <c r="H94" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3830,7 +3818,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="2" t="n">
+      <c r="H95" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3855,7 +3843,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="2" t="n">
+      <c r="E96" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3864,7 +3852,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="2" t="n">
+      <c r="H96" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3889,7 +3877,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="2" t="n">
+      <c r="E97" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3898,7 +3886,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="2" t="n">
+      <c r="H97" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3922,7 +3910,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="2" t="n">
+      <c r="H98" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3947,7 +3935,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n">
+      <c r="E99" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -3956,7 +3944,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="2" t="n">
+      <c r="H99" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3981,7 +3969,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -3990,7 +3978,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="2" t="n">
+      <c r="H100" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4014,7 +4002,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="2" t="n">
+      <c r="H101" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4039,7 +4027,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="2" t="n">
+      <c r="E102" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4048,7 +4036,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="2" t="n">
+      <c r="H102" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4073,7 +4061,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n">
+      <c r="E103" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4082,7 +4070,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="2" t="n">
+      <c r="H103" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4106,7 +4094,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="2" t="n">
+      <c r="H104" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4130,7 +4118,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="2" t="n">
+      <c r="H105" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4154,7 +4142,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="2" t="n">
+      <c r="H106" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4179,7 +4167,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n">
+      <c r="E107" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4188,7 +4176,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="2" t="n">
+      <c r="H107" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4224,7 +4212,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="2" t="n">
+      <c r="H108" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4248,7 +4236,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="2" t="n">
+      <c r="H109" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4272,7 +4260,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="2" t="n">
+      <c r="H110" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4308,7 +4296,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="2" t="n">
+      <c r="H111" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4336,7 +4324,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="2" t="n">
+      <c r="H112" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4372,7 +4360,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="2" t="n">
+      <c r="H113" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4397,7 +4385,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n">
+      <c r="E114" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4406,7 +4394,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="2" t="n">
+      <c r="H114" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4442,7 +4430,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="2" t="n">
+      <c r="H115" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4478,7 +4466,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="2" t="n">
+      <c r="H116" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4514,7 +4502,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="2" t="n">
+      <c r="H117" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4538,7 +4526,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="2" t="n">
+      <c r="H118" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4563,7 +4551,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n">
+      <c r="E119" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4572,7 +4560,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="2" t="n">
+      <c r="H119" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4596,7 +4584,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="2" t="n">
+      <c r="H120" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4620,7 +4608,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="2" t="n">
+      <c r="H121" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4644,7 +4632,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="2" t="n">
+      <c r="H122" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4668,7 +4656,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="2" t="n">
+      <c r="H123" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4692,7 +4680,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="2" t="n">
+      <c r="H124" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4717,7 +4705,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n">
+      <c r="E125" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4726,7 +4714,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="2" t="n">
+      <c r="H125" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4751,7 +4739,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E126" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4760,7 +4748,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="2" t="n">
+      <c r="H126" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4784,7 +4772,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="2" t="n">
+      <c r="H127" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4809,7 +4797,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="2" t="n">
+      <c r="E128" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4818,7 +4806,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="2" t="n">
+      <c r="H128" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4843,7 +4831,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n">
+      <c r="E129" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4852,7 +4840,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="2" t="n">
+      <c r="H129" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4876,7 +4864,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="2" t="n">
+      <c r="H130" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4901,7 +4889,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="2" t="n">
+      <c r="E131" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4910,7 +4898,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="2" t="n">
+      <c r="H131" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4935,7 +4923,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n">
+      <c r="E132" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -4944,7 +4932,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="2" t="n">
+      <c r="H132" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4968,7 +4956,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="2" t="n">
+      <c r="H133" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4992,7 +4980,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="2" t="n">
+      <c r="H134" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5016,7 +5004,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="2" t="n">
+      <c r="H135" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5041,7 +5029,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n">
+      <c r="E136" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5050,7 +5038,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="2" t="n">
+      <c r="H136" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5086,7 +5074,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="2" t="n">
+      <c r="H137" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5110,7 +5098,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="2" t="n">
+      <c r="H138" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5134,7 +5122,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="2" t="n">
+      <c r="H139" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5170,7 +5158,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="2" t="n">
+      <c r="H140" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5198,7 +5186,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="2" t="n">
+      <c r="H141" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5234,7 +5222,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="2" t="n">
+      <c r="H142" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5259,7 +5247,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="2" t="n">
+      <c r="E143" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5268,7 +5256,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="2" t="n">
+      <c r="H143" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5304,7 +5292,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="2" t="n">
+      <c r="H144" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5340,7 +5328,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="2" t="n">
+      <c r="H145" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5376,7 +5364,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="2" t="n">
+      <c r="H146" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5400,7 +5388,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="2" t="n">
+      <c r="H147" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5425,7 +5413,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E148" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5434,7 +5422,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="2" t="n">
+      <c r="H148" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5458,7 +5446,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="2" t="n">
+      <c r="H149" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5482,7 +5470,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="2" t="n">
+      <c r="H150" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5506,7 +5494,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="2" t="n">
+      <c r="H151" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5530,7 +5518,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="2" t="n">
+      <c r="H152" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5554,7 +5542,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="2" t="n">
+      <c r="H153" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5579,7 +5567,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n">
+      <c r="E154" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5588,7 +5576,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="2" t="n">
+      <c r="H154" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5613,7 +5601,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="2" t="n">
+      <c r="E155" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5622,7 +5610,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="2" t="n">
+      <c r="H155" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5646,7 +5634,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="2" t="n">
+      <c r="H156" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5671,7 +5659,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="2" t="n">
+      <c r="E157" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5680,7 +5668,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="2" t="n">
+      <c r="H157" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5705,7 +5693,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n">
+      <c r="E158" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5714,7 +5702,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="2" t="n">
+      <c r="H158" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5739,7 +5727,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="2" t="n">
+      <c r="E159" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5748,7 +5736,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="2" t="n">
+      <c r="H159" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5773,7 +5761,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n">
+      <c r="E160" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5782,7 +5770,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="2" t="n">
+      <c r="H160" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5807,7 +5795,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="2" t="n">
+      <c r="E161" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5816,7 +5804,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="2" t="n">
+      <c r="H161" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5840,7 +5828,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="2" t="n">
+      <c r="H162" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5864,7 +5852,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="2" t="n">
+      <c r="H163" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5888,7 +5876,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="2" t="n">
+      <c r="H164" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5913,7 +5901,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="2" t="n">
+      <c r="E165" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5922,7 +5910,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="2" t="n">
+      <c r="H165" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5958,7 +5946,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n">
+      <c r="H166" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5982,7 +5970,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="2" t="n">
+      <c r="H167" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6006,7 +5994,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="2" t="n">
+      <c r="H168" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6042,7 +6030,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n">
+      <c r="H169" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6070,7 +6058,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="2" t="n">
+      <c r="H170" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6106,7 +6094,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="2" t="n">
+      <c r="H171" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6131,7 +6119,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="2" t="n">
+      <c r="E172" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6140,7 +6128,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="2" t="n">
+      <c r="H172" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6176,7 +6164,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="2" t="n">
+      <c r="H173" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6212,7 +6200,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="2" t="n">
+      <c r="H174" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6248,7 +6236,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="2" t="n">
+      <c r="H175" s="1" t="n">
         <v>46212</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (10/07/2026 10:10)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -418,118 +430,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -604,7 +616,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -679,7 +691,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -754,7 +766,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -829,7 +841,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -904,7 +916,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -975,6 +987,81 @@
       <c r="U7" t="inlineStr">
         <is>
           <t>Disponibilidade_09_07_2026.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" t="n">
+        <v>18</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>16</v>
+      </c>
+      <c r="L8" t="n">
+        <v>19</v>
+      </c>
+      <c r="M8" t="n">
+        <v>18</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2709, 2719, 2720, 2727, 2736, 2741, 2743</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>21</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2709, 2721, 2723</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>10070:00</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>4481:45</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>44.51</v>
+      </c>
+      <c r="T8" t="n">
+        <v>24</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Disponibilidade_10_07_2026.txt</t>
         </is>
       </c>
     </row>
@@ -989,46 +1076,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H175"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1054,7 +1141,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1078,7 +1165,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1114,7 +1201,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1138,7 +1225,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1162,7 +1249,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1187,7 +1274,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1196,7 +1283,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1221,7 +1308,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1230,7 +1317,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1255,7 +1342,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1264,7 +1351,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1289,7 +1376,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1298,7 +1385,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1322,7 +1409,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1346,7 +1433,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1371,7 +1458,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1380,7 +1467,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1404,7 +1491,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1429,7 +1516,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1438,7 +1525,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1462,7 +1549,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1486,7 +1573,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1511,7 +1598,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1520,7 +1607,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1544,7 +1631,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1569,7 +1656,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1578,7 +1665,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1614,7 +1701,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1638,7 +1725,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1662,7 +1749,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1698,7 +1785,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1726,7 +1813,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1762,7 +1849,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1787,7 +1874,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1796,7 +1883,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1832,7 +1919,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1868,7 +1955,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1904,7 +1991,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1928,7 +2015,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="1" t="n">
+      <c r="H31" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -1952,7 +2039,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -1988,7 +2075,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2012,7 +2099,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2036,7 +2123,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="1" t="n">
+      <c r="H35" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2061,7 +2148,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2070,7 +2157,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="1" t="n">
+      <c r="H36" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2095,7 +2182,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2104,7 +2191,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2129,7 +2216,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2138,7 +2225,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2163,7 +2250,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2172,7 +2259,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2196,7 +2283,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="1" t="n">
+      <c r="H40" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2220,7 +2307,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="1" t="n">
+      <c r="H41" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2245,7 +2332,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="E42" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2254,7 +2341,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2278,7 +2365,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2303,7 +2390,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="E44" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2312,7 +2399,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2336,7 +2423,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="1" t="n">
+      <c r="H45" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2360,7 +2447,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="1" t="n">
+      <c r="H46" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2384,7 +2471,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="1" t="n">
+      <c r="H47" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2408,7 +2495,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="1" t="n">
+      <c r="H48" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2433,7 +2520,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="E49" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2442,7 +2529,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="1" t="n">
+      <c r="H49" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2478,7 +2565,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2502,7 +2589,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2526,7 +2613,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="1" t="n">
+      <c r="H52" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2562,7 +2649,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="1" t="n">
+      <c r="H53" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2590,7 +2677,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="1" t="n">
+      <c r="H54" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2626,7 +2713,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="1" t="n">
+      <c r="H55" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2651,7 +2738,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="1" t="n">
+      <c r="E56" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2660,7 +2747,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="1" t="n">
+      <c r="H56" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2696,7 +2783,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="1" t="n">
+      <c r="H57" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2732,7 +2819,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2768,7 +2855,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="1" t="n">
+      <c r="H59" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2792,7 +2879,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="1" t="n">
+      <c r="H60" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2816,7 +2903,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="1" t="n">
+      <c r="H61" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2841,7 +2928,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="1" t="n">
+      <c r="E62" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2850,7 +2937,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="1" t="n">
+      <c r="H62" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2874,7 +2961,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="1" t="n">
+      <c r="H63" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2899,7 +2986,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="1" t="n">
+      <c r="E64" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2908,7 +2995,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="1" t="n">
+      <c r="H64" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2932,7 +3019,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2956,7 +3043,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2981,7 +3068,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="1" t="n">
+      <c r="E67" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -2990,7 +3077,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="1" t="n">
+      <c r="H67" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3015,7 +3102,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="1" t="n">
+      <c r="E68" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3024,7 +3111,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="1" t="n">
+      <c r="H68" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3048,7 +3135,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="1" t="n">
+      <c r="H69" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3072,7 +3159,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="1" t="n">
+      <c r="H70" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3097,7 +3184,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="1" t="n">
+      <c r="E71" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3106,7 +3193,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="1" t="n">
+      <c r="H71" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3130,7 +3217,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="1" t="n">
+      <c r="H72" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3155,7 +3242,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="1" t="n">
+      <c r="E73" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3164,7 +3251,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="1" t="n">
+      <c r="H73" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3188,7 +3275,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="1" t="n">
+      <c r="H74" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3212,7 +3299,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="1" t="n">
+      <c r="H75" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3236,7 +3323,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="1" t="n">
+      <c r="H76" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3260,7 +3347,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="1" t="n">
+      <c r="H77" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3285,7 +3372,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="1" t="n">
+      <c r="E78" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3294,7 +3381,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="1" t="n">
+      <c r="H78" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3330,7 +3417,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="1" t="n">
+      <c r="H79" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3354,7 +3441,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="1" t="n">
+      <c r="H80" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3378,7 +3465,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="1" t="n">
+      <c r="H81" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3414,7 +3501,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="1" t="n">
+      <c r="H82" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3442,7 +3529,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="1" t="n">
+      <c r="H83" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3478,7 +3565,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="1" t="n">
+      <c r="H84" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3503,7 +3590,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="1" t="n">
+      <c r="E85" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3512,7 +3599,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="1" t="n">
+      <c r="H85" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3548,7 +3635,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="1" t="n">
+      <c r="H86" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3584,7 +3671,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="1" t="n">
+      <c r="H87" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3620,7 +3707,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="1" t="n">
+      <c r="H88" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3644,7 +3731,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="1" t="n">
+      <c r="H89" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3669,7 +3756,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="1" t="n">
+      <c r="E90" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3678,7 +3765,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="1" t="n">
+      <c r="H90" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3703,7 +3790,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="1" t="n">
+      <c r="E91" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3712,7 +3799,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="1" t="n">
+      <c r="H91" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3736,7 +3823,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="1" t="n">
+      <c r="H92" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3761,7 +3848,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="1" t="n">
+      <c r="E93" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3770,7 +3857,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="1" t="n">
+      <c r="H93" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3794,7 +3881,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="1" t="n">
+      <c r="H94" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3818,7 +3905,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="1" t="n">
+      <c r="H95" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3843,7 +3930,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="1" t="n">
+      <c r="E96" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3852,7 +3939,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="1" t="n">
+      <c r="H96" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3877,7 +3964,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="1" t="n">
+      <c r="E97" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3886,7 +3973,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="1" t="n">
+      <c r="H97" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3910,7 +3997,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="1" t="n">
+      <c r="H98" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3935,7 +4022,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="1" t="n">
+      <c r="E99" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -3944,7 +4031,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="1" t="n">
+      <c r="H99" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3969,7 +4056,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="1" t="n">
+      <c r="E100" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -3978,7 +4065,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="1" t="n">
+      <c r="H100" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4002,7 +4089,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="1" t="n">
+      <c r="H101" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4027,7 +4114,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="1" t="n">
+      <c r="E102" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4036,7 +4123,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="1" t="n">
+      <c r="H102" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4061,7 +4148,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="1" t="n">
+      <c r="E103" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4070,7 +4157,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="1" t="n">
+      <c r="H103" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4094,7 +4181,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="1" t="n">
+      <c r="H104" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4118,7 +4205,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="1" t="n">
+      <c r="H105" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4142,7 +4229,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="1" t="n">
+      <c r="H106" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4167,7 +4254,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="1" t="n">
+      <c r="E107" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4176,7 +4263,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="1" t="n">
+      <c r="H107" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4212,7 +4299,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="1" t="n">
+      <c r="H108" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4236,7 +4323,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="1" t="n">
+      <c r="H109" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4260,7 +4347,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="1" t="n">
+      <c r="H110" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4296,7 +4383,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="1" t="n">
+      <c r="H111" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4324,7 +4411,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="1" t="n">
+      <c r="H112" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4360,7 +4447,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="1" t="n">
+      <c r="H113" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4385,7 +4472,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="1" t="n">
+      <c r="E114" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4394,7 +4481,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="1" t="n">
+      <c r="H114" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4430,7 +4517,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="1" t="n">
+      <c r="H115" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4466,7 +4553,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="1" t="n">
+      <c r="H116" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4502,7 +4589,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="1" t="n">
+      <c r="H117" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4526,7 +4613,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="1" t="n">
+      <c r="H118" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4551,7 +4638,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="1" t="n">
+      <c r="E119" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4560,7 +4647,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="1" t="n">
+      <c r="H119" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4584,7 +4671,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="1" t="n">
+      <c r="H120" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4608,7 +4695,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="1" t="n">
+      <c r="H121" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4632,7 +4719,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="1" t="n">
+      <c r="H122" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4656,7 +4743,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="1" t="n">
+      <c r="H123" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4680,7 +4767,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="1" t="n">
+      <c r="H124" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4705,7 +4792,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="1" t="n">
+      <c r="E125" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4714,7 +4801,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="1" t="n">
+      <c r="H125" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4739,7 +4826,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="1" t="n">
+      <c r="E126" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4748,7 +4835,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="1" t="n">
+      <c r="H126" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4772,7 +4859,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="1" t="n">
+      <c r="H127" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4797,7 +4884,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="1" t="n">
+      <c r="E128" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4806,7 +4893,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="1" t="n">
+      <c r="H128" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4831,7 +4918,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="1" t="n">
+      <c r="E129" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4840,7 +4927,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="1" t="n">
+      <c r="H129" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4864,7 +4951,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="1" t="n">
+      <c r="H130" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4889,7 +4976,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="1" t="n">
+      <c r="E131" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4898,7 +4985,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="1" t="n">
+      <c r="H131" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4923,7 +5010,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="1" t="n">
+      <c r="E132" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -4932,7 +5019,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="1" t="n">
+      <c r="H132" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4956,7 +5043,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="1" t="n">
+      <c r="H133" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4980,7 +5067,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="1" t="n">
+      <c r="H134" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5004,7 +5091,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="1" t="n">
+      <c r="H135" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5029,7 +5116,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="1" t="n">
+      <c r="E136" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5038,7 +5125,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="1" t="n">
+      <c r="H136" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5074,7 +5161,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="1" t="n">
+      <c r="H137" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5098,7 +5185,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="1" t="n">
+      <c r="H138" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5122,7 +5209,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="1" t="n">
+      <c r="H139" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5158,7 +5245,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="1" t="n">
+      <c r="H140" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5186,7 +5273,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="1" t="n">
+      <c r="H141" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5222,7 +5309,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="1" t="n">
+      <c r="H142" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5247,7 +5334,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="1" t="n">
+      <c r="E143" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5256,7 +5343,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="1" t="n">
+      <c r="H143" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5292,7 +5379,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="1" t="n">
+      <c r="H144" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5328,7 +5415,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="1" t="n">
+      <c r="H145" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5364,7 +5451,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="1" t="n">
+      <c r="H146" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5388,7 +5475,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="1" t="n">
+      <c r="H147" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5413,7 +5500,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="1" t="n">
+      <c r="E148" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5422,7 +5509,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="1" t="n">
+      <c r="H148" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5446,7 +5533,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="1" t="n">
+      <c r="H149" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5470,7 +5557,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="1" t="n">
+      <c r="H150" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5494,7 +5581,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="1" t="n">
+      <c r="H151" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5518,7 +5605,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="1" t="n">
+      <c r="H152" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5542,7 +5629,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="1" t="n">
+      <c r="H153" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5567,7 +5654,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="1" t="n">
+      <c r="E154" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5576,7 +5663,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="1" t="n">
+      <c r="H154" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5601,7 +5688,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="1" t="n">
+      <c r="E155" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5610,7 +5697,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="1" t="n">
+      <c r="H155" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5634,7 +5721,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="1" t="n">
+      <c r="H156" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5659,7 +5746,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="1" t="n">
+      <c r="E157" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5668,7 +5755,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="1" t="n">
+      <c r="H157" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5693,7 +5780,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="1" t="n">
+      <c r="E158" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5702,7 +5789,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="1" t="n">
+      <c r="H158" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5727,7 +5814,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="1" t="n">
+      <c r="E159" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5736,7 +5823,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="1" t="n">
+      <c r="H159" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5761,7 +5848,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="1" t="n">
+      <c r="E160" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5770,7 +5857,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="1" t="n">
+      <c r="H160" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5795,7 +5882,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="1" t="n">
+      <c r="E161" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5804,7 +5891,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="1" t="n">
+      <c r="H161" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5828,7 +5915,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="1" t="n">
+      <c r="H162" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5852,7 +5939,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="1" t="n">
+      <c r="H163" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5876,7 +5963,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="1" t="n">
+      <c r="H164" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5901,7 +5988,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="1" t="n">
+      <c r="E165" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5910,7 +5997,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="1" t="n">
+      <c r="H165" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5946,7 +6033,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="1" t="n">
+      <c r="H166" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5970,7 +6057,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="1" t="n">
+      <c r="H167" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5994,7 +6081,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="1" t="n">
+      <c r="H168" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6030,7 +6117,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="1" t="n">
+      <c r="H169" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6058,7 +6145,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="1" t="n">
+      <c r="H170" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6094,7 +6181,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="1" t="n">
+      <c r="H171" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6119,7 +6206,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="1" t="n">
+      <c r="E172" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6128,7 +6215,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="1" t="n">
+      <c r="H172" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6164,7 +6251,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="1" t="n">
+      <c r="H173" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6200,7 +6287,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="1" t="n">
+      <c r="H174" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6236,8 +6323,890 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="1" t="n">
+      <c r="H175" s="2" t="n">
         <v>46212</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2733</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M, 01 IPLR de FCU</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>14/07</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2739</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2727</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1º/15º GAV</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Pesquisa de pane no painel de alarmes.</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>13/07</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2702</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2703</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr"/>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2729</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>31/07</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Realizando inspeções 4300 FH/HSI.</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2722</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2º ETA</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>5º ETA</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2709</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>ITR</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Agd transmissão do atuador do flape</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2720</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Pesquisa de pane de FCU</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2721</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>6º ETA</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Motor recolhido para reparo na geradora de gases</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>13/07</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2736</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>10/07</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2737</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2738</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr"/>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2740</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2741</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>7º ETA</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>15/07</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2723</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Itens entregues. Agd AT de hélice para definição de recolhimento ou translado da aeronave para o Parque</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2742</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>DACTA II</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr"/>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2704</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr"/>
+      <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>75 APE</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>A ser definido.</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2724</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>ANV acidentada.</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>91 AIFP. Serão atendidas pela Vee One e FAB</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>A DET</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Aguardando avaliação de sinistro</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>06/07</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2730</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 44 IPLR</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2732</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 13 IPLR</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP.</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="n">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2734</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>PAMA-LS</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>SEM MOTOR - 57 IPLR</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Aguarda DPE do PAMASP e PAMALS.</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="n">
+        <v>46213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (10/07/2026 17:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,114 +422,114 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -616,7 +604,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -691,7 +679,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -766,7 +754,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -841,7 +829,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -916,7 +904,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -991,7 +979,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="B8" t="n">
@@ -1080,42 +1068,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1141,7 +1129,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1165,7 +1153,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1201,7 +1189,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1225,7 +1213,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1249,7 +1237,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1274,7 +1262,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1283,7 +1271,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1308,7 +1296,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1317,7 +1305,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1342,7 +1330,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1351,7 +1339,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1376,7 +1364,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1385,7 +1373,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1409,7 +1397,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1433,7 +1421,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1458,7 +1446,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1467,7 +1455,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1491,7 +1479,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1516,7 +1504,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1525,7 +1513,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1549,7 +1537,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1573,7 +1561,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1598,7 +1586,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1607,7 +1595,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1631,7 +1619,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1656,7 +1644,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1665,7 +1653,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1701,7 +1689,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1725,7 +1713,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1749,7 +1737,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1785,7 +1773,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1813,7 +1801,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1849,7 +1837,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1874,7 +1862,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1883,7 +1871,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1919,7 +1907,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1955,7 +1943,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1991,7 +1979,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -2015,7 +2003,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2039,7 +2027,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2075,7 +2063,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2099,7 +2087,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2123,7 +2111,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="2" t="n">
+      <c r="H35" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2148,7 +2136,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2157,7 +2145,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="H36" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2182,7 +2170,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2191,7 +2179,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2216,7 +2204,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2225,7 +2213,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2250,7 +2238,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E39" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2259,7 +2247,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2283,7 +2271,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="2" t="n">
+      <c r="H40" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2307,7 +2295,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="2" t="n">
+      <c r="H41" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2332,7 +2320,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E42" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2341,7 +2329,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="H42" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2365,7 +2353,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2390,7 +2378,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2399,7 +2387,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="H44" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2423,7 +2411,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="2" t="n">
+      <c r="H45" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2447,7 +2435,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2471,7 +2459,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="2" t="n">
+      <c r="H47" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2495,7 +2483,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="2" t="n">
+      <c r="H48" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2520,7 +2508,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E49" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2529,7 +2517,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="H49" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2565,7 +2553,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2589,7 +2577,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="2" t="n">
+      <c r="H51" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2613,7 +2601,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="2" t="n">
+      <c r="H52" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2649,7 +2637,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="H53" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2677,7 +2665,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2713,7 +2701,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="H55" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2738,7 +2726,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2747,7 +2735,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="H56" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2783,7 +2771,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="H57" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2819,7 +2807,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="n">
+      <c r="H58" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2855,7 +2843,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="H59" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2879,7 +2867,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="2" t="n">
+      <c r="H60" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2903,7 +2891,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="2" t="n">
+      <c r="H61" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2928,7 +2916,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2937,7 +2925,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="2" t="n">
+      <c r="H62" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2961,7 +2949,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="2" t="n">
+      <c r="H63" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2986,7 +2974,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n">
+      <c r="E64" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2995,7 +2983,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="H64" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3019,7 +3007,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="2" t="n">
+      <c r="H65" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3043,7 +3031,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="2" t="n">
+      <c r="H66" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3068,7 +3056,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n">
+      <c r="E67" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3077,7 +3065,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="2" t="n">
+      <c r="H67" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3102,7 +3090,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n">
+      <c r="E68" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3111,7 +3099,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="2" t="n">
+      <c r="H68" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3135,7 +3123,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="2" t="n">
+      <c r="H69" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3159,7 +3147,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="2" t="n">
+      <c r="H70" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3184,7 +3172,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="2" t="n">
+      <c r="E71" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3193,7 +3181,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="2" t="n">
+      <c r="H71" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3217,7 +3205,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="2" t="n">
+      <c r="H72" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3242,7 +3230,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n">
+      <c r="E73" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3251,7 +3239,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="2" t="n">
+      <c r="H73" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3275,7 +3263,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="2" t="n">
+      <c r="H74" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3299,7 +3287,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="2" t="n">
+      <c r="H75" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3323,7 +3311,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="2" t="n">
+      <c r="H76" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3347,7 +3335,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="2" t="n">
+      <c r="H77" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3372,7 +3360,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E78" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3381,7 +3369,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="2" t="n">
+      <c r="H78" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3417,7 +3405,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="2" t="n">
+      <c r="H79" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3441,7 +3429,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="2" t="n">
+      <c r="H80" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3465,7 +3453,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="2" t="n">
+      <c r="H81" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3501,7 +3489,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="2" t="n">
+      <c r="H82" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3529,7 +3517,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="2" t="n">
+      <c r="H83" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3565,7 +3553,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="2" t="n">
+      <c r="H84" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3590,7 +3578,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n">
+      <c r="E85" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3599,7 +3587,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="2" t="n">
+      <c r="H85" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3635,7 +3623,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="2" t="n">
+      <c r="H86" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3671,7 +3659,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="2" t="n">
+      <c r="H87" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3707,7 +3695,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="2" t="n">
+      <c r="H88" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3731,7 +3719,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="2" t="n">
+      <c r="H89" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3756,7 +3744,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3765,7 +3753,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="2" t="n">
+      <c r="H90" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3790,7 +3778,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n">
+      <c r="E91" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3799,7 +3787,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="2" t="n">
+      <c r="H91" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3823,7 +3811,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="2" t="n">
+      <c r="H92" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3848,7 +3836,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="2" t="n">
+      <c r="E93" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3857,7 +3845,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="2" t="n">
+      <c r="H93" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3881,7 +3869,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="2" t="n">
+      <c r="H94" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3905,7 +3893,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="2" t="n">
+      <c r="H95" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3930,7 +3918,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="2" t="n">
+      <c r="E96" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3939,7 +3927,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="2" t="n">
+      <c r="H96" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3964,7 +3952,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="2" t="n">
+      <c r="E97" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3973,7 +3961,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="2" t="n">
+      <c r="H97" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3997,7 +3985,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="2" t="n">
+      <c r="H98" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4022,7 +4010,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n">
+      <c r="E99" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4031,7 +4019,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="2" t="n">
+      <c r="H99" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4056,7 +4044,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4065,7 +4053,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="2" t="n">
+      <c r="H100" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4089,7 +4077,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="2" t="n">
+      <c r="H101" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4114,7 +4102,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="2" t="n">
+      <c r="E102" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4123,7 +4111,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="2" t="n">
+      <c r="H102" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4148,7 +4136,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n">
+      <c r="E103" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4157,7 +4145,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="2" t="n">
+      <c r="H103" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4181,7 +4169,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="2" t="n">
+      <c r="H104" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4205,7 +4193,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="2" t="n">
+      <c r="H105" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4229,7 +4217,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="2" t="n">
+      <c r="H106" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4254,7 +4242,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n">
+      <c r="E107" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4263,7 +4251,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="2" t="n">
+      <c r="H107" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4299,7 +4287,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="2" t="n">
+      <c r="H108" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4323,7 +4311,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="2" t="n">
+      <c r="H109" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4347,7 +4335,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="2" t="n">
+      <c r="H110" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4383,7 +4371,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="2" t="n">
+      <c r="H111" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4411,7 +4399,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="2" t="n">
+      <c r="H112" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4447,7 +4435,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="2" t="n">
+      <c r="H113" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4472,7 +4460,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n">
+      <c r="E114" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4481,7 +4469,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="2" t="n">
+      <c r="H114" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4517,7 +4505,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="2" t="n">
+      <c r="H115" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4553,7 +4541,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="2" t="n">
+      <c r="H116" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4589,7 +4577,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="2" t="n">
+      <c r="H117" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4613,7 +4601,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="2" t="n">
+      <c r="H118" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4638,7 +4626,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n">
+      <c r="E119" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4647,7 +4635,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="2" t="n">
+      <c r="H119" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4671,7 +4659,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="2" t="n">
+      <c r="H120" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4695,7 +4683,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="2" t="n">
+      <c r="H121" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4719,7 +4707,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="2" t="n">
+      <c r="H122" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4743,7 +4731,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="2" t="n">
+      <c r="H123" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4767,7 +4755,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="2" t="n">
+      <c r="H124" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4792,7 +4780,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n">
+      <c r="E125" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4801,7 +4789,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="2" t="n">
+      <c r="H125" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4826,7 +4814,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E126" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4835,7 +4823,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="2" t="n">
+      <c r="H126" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4859,7 +4847,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="2" t="n">
+      <c r="H127" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4884,7 +4872,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="2" t="n">
+      <c r="E128" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4893,7 +4881,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="2" t="n">
+      <c r="H128" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4918,7 +4906,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n">
+      <c r="E129" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4927,7 +4915,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="2" t="n">
+      <c r="H129" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4951,7 +4939,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="2" t="n">
+      <c r="H130" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4976,7 +4964,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="2" t="n">
+      <c r="E131" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4985,7 +4973,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="2" t="n">
+      <c r="H131" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5010,7 +4998,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n">
+      <c r="E132" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -5019,7 +5007,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="2" t="n">
+      <c r="H132" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5043,7 +5031,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="2" t="n">
+      <c r="H133" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5067,7 +5055,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="2" t="n">
+      <c r="H134" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5091,7 +5079,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="2" t="n">
+      <c r="H135" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5116,7 +5104,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n">
+      <c r="E136" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5125,7 +5113,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="2" t="n">
+      <c r="H136" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5161,7 +5149,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="2" t="n">
+      <c r="H137" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5185,7 +5173,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="2" t="n">
+      <c r="H138" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5209,7 +5197,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="2" t="n">
+      <c r="H139" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5245,7 +5233,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="2" t="n">
+      <c r="H140" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5273,7 +5261,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="2" t="n">
+      <c r="H141" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5309,7 +5297,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="2" t="n">
+      <c r="H142" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5334,7 +5322,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="2" t="n">
+      <c r="E143" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5343,7 +5331,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="2" t="n">
+      <c r="H143" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5379,7 +5367,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="2" t="n">
+      <c r="H144" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5415,7 +5403,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="2" t="n">
+      <c r="H145" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5451,7 +5439,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="2" t="n">
+      <c r="H146" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5475,7 +5463,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="2" t="n">
+      <c r="H147" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5500,7 +5488,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E148" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5509,7 +5497,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="2" t="n">
+      <c r="H148" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5533,7 +5521,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="2" t="n">
+      <c r="H149" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5557,7 +5545,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="2" t="n">
+      <c r="H150" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5581,7 +5569,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="2" t="n">
+      <c r="H151" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5605,7 +5593,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="2" t="n">
+      <c r="H152" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5629,7 +5617,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="2" t="n">
+      <c r="H153" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5654,7 +5642,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n">
+      <c r="E154" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5663,7 +5651,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="2" t="n">
+      <c r="H154" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5688,7 +5676,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="2" t="n">
+      <c r="E155" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5697,7 +5685,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="2" t="n">
+      <c r="H155" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5721,7 +5709,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="2" t="n">
+      <c r="H156" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5746,7 +5734,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="2" t="n">
+      <c r="E157" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5755,7 +5743,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="2" t="n">
+      <c r="H157" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5780,7 +5768,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n">
+      <c r="E158" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5789,7 +5777,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="2" t="n">
+      <c r="H158" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5814,7 +5802,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="2" t="n">
+      <c r="E159" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5823,7 +5811,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="2" t="n">
+      <c r="H159" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5848,7 +5836,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n">
+      <c r="E160" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5857,7 +5845,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="2" t="n">
+      <c r="H160" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5882,7 +5870,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="2" t="n">
+      <c r="E161" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5891,7 +5879,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="2" t="n">
+      <c r="H161" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5915,7 +5903,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="2" t="n">
+      <c r="H162" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5939,7 +5927,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="2" t="n">
+      <c r="H163" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5963,7 +5951,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="2" t="n">
+      <c r="H164" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5988,7 +5976,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="2" t="n">
+      <c r="E165" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5997,7 +5985,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="2" t="n">
+      <c r="H165" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6033,7 +6021,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n">
+      <c r="H166" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6057,7 +6045,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="2" t="n">
+      <c r="H167" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6081,7 +6069,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="2" t="n">
+      <c r="H168" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6117,7 +6105,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n">
+      <c r="H169" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6145,7 +6133,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="2" t="n">
+      <c r="H170" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6181,7 +6169,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="2" t="n">
+      <c r="H171" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6206,7 +6194,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="2" t="n">
+      <c r="E172" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6215,7 +6203,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="2" t="n">
+      <c r="H172" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6251,7 +6239,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="2" t="n">
+      <c r="H173" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6287,7 +6275,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="2" t="n">
+      <c r="H174" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6323,7 +6311,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="2" t="n">
+      <c r="H175" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6347,7 +6335,7 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr"/>
-      <c r="H176" s="2" t="n">
+      <c r="H176" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6372,7 +6360,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M, 01 IPLR de FCU</t>
         </is>
       </c>
-      <c r="E177" s="2" t="n">
+      <c r="E177" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -6381,7 +6369,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H177" s="2" t="n">
+      <c r="H177" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6405,7 +6393,7 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
-      <c r="H178" s="2" t="n">
+      <c r="H178" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6430,7 +6418,7 @@
           <t>Pesquisa de pane no painel de alarmes.</t>
         </is>
       </c>
-      <c r="E179" s="2" t="n">
+      <c r="E179" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -6439,7 +6427,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H179" s="2" t="n">
+      <c r="H179" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6463,7 +6451,7 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
-      <c r="H180" s="2" t="n">
+      <c r="H180" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6487,7 +6475,7 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr"/>
-      <c r="H181" s="2" t="n">
+      <c r="H181" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6511,7 +6499,7 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
-      <c r="H182" s="2" t="n">
+      <c r="H182" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6536,7 +6524,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E183" s="2" t="n">
+      <c r="E183" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -6545,7 +6533,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H183" s="2" t="n">
+      <c r="H183" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6570,7 +6558,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E184" s="2" t="n">
+      <c r="E184" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -6579,7 +6567,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H184" s="2" t="n">
+      <c r="H184" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6603,7 +6591,7 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr"/>
-      <c r="H185" s="2" t="n">
+      <c r="H185" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6628,7 +6616,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E186" s="2" t="n">
+      <c r="E186" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -6637,7 +6625,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H186" s="2" t="n">
+      <c r="H186" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6662,7 +6650,7 @@
           <t>Agd transmissão do atuador do flape</t>
         </is>
       </c>
-      <c r="E187" s="2" t="n">
+      <c r="E187" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -6671,7 +6659,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H187" s="2" t="n">
+      <c r="H187" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6696,7 +6684,7 @@
           <t>Pesquisa de pane de FCU</t>
         </is>
       </c>
-      <c r="E188" s="2" t="n">
+      <c r="E188" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -6705,7 +6693,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H188" s="2" t="n">
+      <c r="H188" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6730,7 +6718,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E189" s="2" t="n">
+      <c r="E189" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -6739,7 +6727,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H189" s="2" t="n">
+      <c r="H189" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6764,7 +6752,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E190" s="2" t="n">
+      <c r="E190" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -6773,7 +6761,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H190" s="2" t="n">
+      <c r="H190" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6797,7 +6785,7 @@
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
-      <c r="H191" s="2" t="n">
+      <c r="H191" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6821,7 +6809,7 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
-      <c r="H192" s="2" t="n">
+      <c r="H192" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6845,7 +6833,7 @@
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr"/>
-      <c r="H193" s="2" t="n">
+      <c r="H193" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6870,7 +6858,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E194" s="2" t="n">
+      <c r="E194" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -6879,7 +6867,7 @@
           <t>15/07</t>
         </is>
       </c>
-      <c r="H194" s="2" t="n">
+      <c r="H194" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6915,7 +6903,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H195" s="2" t="n">
+      <c r="H195" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6939,7 +6927,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr"/>
-      <c r="H196" s="2" t="n">
+      <c r="H196" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6963,7 +6951,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
-      <c r="H197" s="2" t="n">
+      <c r="H197" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6999,7 +6987,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H198" s="2" t="n">
+      <c r="H198" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7027,7 +7015,7 @@
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
-      <c r="H199" s="2" t="n">
+      <c r="H199" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7063,7 +7051,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H200" s="2" t="n">
+      <c r="H200" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7088,7 +7076,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E201" s="2" t="n">
+      <c r="E201" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -7097,7 +7085,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H201" s="2" t="n">
+      <c r="H201" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7133,7 +7121,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H202" s="2" t="n">
+      <c r="H202" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7169,7 +7157,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H203" s="2" t="n">
+      <c r="H203" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7205,7 +7193,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H204" s="2" t="n">
+      <c r="H204" s="1" t="n">
         <v>46213</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (10/07/2026 16:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -422,114 +434,114 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -604,7 +616,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -679,7 +691,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -754,7 +766,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -829,7 +841,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -904,7 +916,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -979,7 +991,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="B8" t="n">
@@ -1068,42 +1080,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1129,7 +1141,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1153,7 +1165,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1189,7 +1201,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1213,7 +1225,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1237,7 +1249,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1262,7 +1274,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1271,7 +1283,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1296,7 +1308,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1305,7 +1317,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1330,7 +1342,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1339,7 +1351,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1364,7 +1376,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1373,7 +1385,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1397,7 +1409,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1421,7 +1433,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1446,7 +1458,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1455,7 +1467,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1479,7 +1491,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1504,7 +1516,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1513,7 +1525,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1537,7 +1549,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1561,7 +1573,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1586,7 +1598,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1595,7 +1607,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1619,7 +1631,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1644,7 +1656,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1653,7 +1665,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1689,7 +1701,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1713,7 +1725,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1737,7 +1749,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1773,7 +1785,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1801,7 +1813,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1837,7 +1849,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1862,7 +1874,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1871,7 +1883,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1907,7 +1919,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1943,7 +1955,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1979,7 +1991,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -2003,7 +2015,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="1" t="n">
+      <c r="H31" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2027,7 +2039,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2063,7 +2075,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2087,7 +2099,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2111,7 +2123,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="1" t="n">
+      <c r="H35" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2136,7 +2148,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2145,7 +2157,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="1" t="n">
+      <c r="H36" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2170,7 +2182,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2179,7 +2191,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2204,7 +2216,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2213,7 +2225,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2238,7 +2250,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2247,7 +2259,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2271,7 +2283,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="1" t="n">
+      <c r="H40" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2295,7 +2307,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="1" t="n">
+      <c r="H41" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2320,7 +2332,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="E42" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2329,7 +2341,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2353,7 +2365,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2378,7 +2390,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="E44" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2387,7 +2399,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2411,7 +2423,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="1" t="n">
+      <c r="H45" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2435,7 +2447,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="1" t="n">
+      <c r="H46" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2459,7 +2471,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="1" t="n">
+      <c r="H47" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2483,7 +2495,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="1" t="n">
+      <c r="H48" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2508,7 +2520,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="E49" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2517,7 +2529,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="1" t="n">
+      <c r="H49" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2553,7 +2565,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2577,7 +2589,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2601,7 +2613,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="1" t="n">
+      <c r="H52" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2637,7 +2649,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="1" t="n">
+      <c r="H53" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2665,7 +2677,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="1" t="n">
+      <c r="H54" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2701,7 +2713,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="1" t="n">
+      <c r="H55" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2726,7 +2738,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="1" t="n">
+      <c r="E56" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2735,7 +2747,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="1" t="n">
+      <c r="H56" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2771,7 +2783,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="1" t="n">
+      <c r="H57" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2807,7 +2819,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2843,7 +2855,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="1" t="n">
+      <c r="H59" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2867,7 +2879,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="1" t="n">
+      <c r="H60" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2891,7 +2903,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="1" t="n">
+      <c r="H61" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2916,7 +2928,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="1" t="n">
+      <c r="E62" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2925,7 +2937,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="1" t="n">
+      <c r="H62" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2949,7 +2961,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="1" t="n">
+      <c r="H63" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2974,7 +2986,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="1" t="n">
+      <c r="E64" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2983,7 +2995,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="1" t="n">
+      <c r="H64" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3007,7 +3019,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3031,7 +3043,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3056,7 +3068,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="1" t="n">
+      <c r="E67" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3065,7 +3077,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="1" t="n">
+      <c r="H67" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3090,7 +3102,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="1" t="n">
+      <c r="E68" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3099,7 +3111,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="1" t="n">
+      <c r="H68" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3123,7 +3135,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="1" t="n">
+      <c r="H69" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3147,7 +3159,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="1" t="n">
+      <c r="H70" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3172,7 +3184,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="1" t="n">
+      <c r="E71" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3181,7 +3193,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="1" t="n">
+      <c r="H71" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3205,7 +3217,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="1" t="n">
+      <c r="H72" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3230,7 +3242,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="1" t="n">
+      <c r="E73" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3239,7 +3251,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="1" t="n">
+      <c r="H73" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3263,7 +3275,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="1" t="n">
+      <c r="H74" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3287,7 +3299,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="1" t="n">
+      <c r="H75" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3311,7 +3323,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="1" t="n">
+      <c r="H76" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3335,7 +3347,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="1" t="n">
+      <c r="H77" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3360,7 +3372,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="1" t="n">
+      <c r="E78" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3369,7 +3381,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="1" t="n">
+      <c r="H78" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3405,7 +3417,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="1" t="n">
+      <c r="H79" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3429,7 +3441,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="1" t="n">
+      <c r="H80" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3453,7 +3465,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="1" t="n">
+      <c r="H81" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3489,7 +3501,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="1" t="n">
+      <c r="H82" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3517,7 +3529,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="1" t="n">
+      <c r="H83" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3553,7 +3565,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="1" t="n">
+      <c r="H84" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3578,7 +3590,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="1" t="n">
+      <c r="E85" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3587,7 +3599,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="1" t="n">
+      <c r="H85" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3623,7 +3635,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="1" t="n">
+      <c r="H86" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3659,7 +3671,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="1" t="n">
+      <c r="H87" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3695,7 +3707,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="1" t="n">
+      <c r="H88" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3719,7 +3731,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="1" t="n">
+      <c r="H89" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3744,7 +3756,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="1" t="n">
+      <c r="E90" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3753,7 +3765,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="1" t="n">
+      <c r="H90" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3778,7 +3790,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="1" t="n">
+      <c r="E91" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3787,7 +3799,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="1" t="n">
+      <c r="H91" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3811,7 +3823,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="1" t="n">
+      <c r="H92" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3836,7 +3848,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="1" t="n">
+      <c r="E93" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3845,7 +3857,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="1" t="n">
+      <c r="H93" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3869,7 +3881,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="1" t="n">
+      <c r="H94" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3893,7 +3905,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="1" t="n">
+      <c r="H95" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3918,7 +3930,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="1" t="n">
+      <c r="E96" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3927,7 +3939,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="1" t="n">
+      <c r="H96" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3952,7 +3964,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="1" t="n">
+      <c r="E97" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3961,7 +3973,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="1" t="n">
+      <c r="H97" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3985,7 +3997,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="1" t="n">
+      <c r="H98" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4010,7 +4022,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="1" t="n">
+      <c r="E99" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4019,7 +4031,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="1" t="n">
+      <c r="H99" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4044,7 +4056,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="1" t="n">
+      <c r="E100" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4053,7 +4065,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="1" t="n">
+      <c r="H100" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4077,7 +4089,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="1" t="n">
+      <c r="H101" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4102,7 +4114,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="1" t="n">
+      <c r="E102" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4111,7 +4123,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="1" t="n">
+      <c r="H102" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4136,7 +4148,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="1" t="n">
+      <c r="E103" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4145,7 +4157,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="1" t="n">
+      <c r="H103" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4169,7 +4181,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="1" t="n">
+      <c r="H104" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4193,7 +4205,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="1" t="n">
+      <c r="H105" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4217,7 +4229,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="1" t="n">
+      <c r="H106" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4242,7 +4254,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="1" t="n">
+      <c r="E107" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4251,7 +4263,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="1" t="n">
+      <c r="H107" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4287,7 +4299,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="1" t="n">
+      <c r="H108" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4311,7 +4323,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="1" t="n">
+      <c r="H109" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4335,7 +4347,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="1" t="n">
+      <c r="H110" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4371,7 +4383,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="1" t="n">
+      <c r="H111" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4399,7 +4411,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="1" t="n">
+      <c r="H112" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4435,7 +4447,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="1" t="n">
+      <c r="H113" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4460,7 +4472,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="1" t="n">
+      <c r="E114" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4469,7 +4481,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="1" t="n">
+      <c r="H114" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4505,7 +4517,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="1" t="n">
+      <c r="H115" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4541,7 +4553,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="1" t="n">
+      <c r="H116" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4577,7 +4589,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="1" t="n">
+      <c r="H117" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4601,7 +4613,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="1" t="n">
+      <c r="H118" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4626,7 +4638,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="1" t="n">
+      <c r="E119" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4635,7 +4647,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="1" t="n">
+      <c r="H119" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4659,7 +4671,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="1" t="n">
+      <c r="H120" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4683,7 +4695,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="1" t="n">
+      <c r="H121" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4707,7 +4719,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="1" t="n">
+      <c r="H122" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4731,7 +4743,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="1" t="n">
+      <c r="H123" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4755,7 +4767,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="1" t="n">
+      <c r="H124" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4780,7 +4792,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="1" t="n">
+      <c r="E125" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4789,7 +4801,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="1" t="n">
+      <c r="H125" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4814,7 +4826,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="1" t="n">
+      <c r="E126" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4823,7 +4835,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="1" t="n">
+      <c r="H126" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4847,7 +4859,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="1" t="n">
+      <c r="H127" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4872,7 +4884,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="1" t="n">
+      <c r="E128" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4881,7 +4893,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="1" t="n">
+      <c r="H128" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4906,7 +4918,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="1" t="n">
+      <c r="E129" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4915,7 +4927,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="1" t="n">
+      <c r="H129" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4939,7 +4951,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="1" t="n">
+      <c r="H130" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4964,7 +4976,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="1" t="n">
+      <c r="E131" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4973,7 +4985,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="1" t="n">
+      <c r="H131" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4998,7 +5010,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="1" t="n">
+      <c r="E132" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -5007,7 +5019,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="1" t="n">
+      <c r="H132" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5031,7 +5043,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="1" t="n">
+      <c r="H133" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5055,7 +5067,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="1" t="n">
+      <c r="H134" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5079,7 +5091,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="1" t="n">
+      <c r="H135" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5104,7 +5116,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="1" t="n">
+      <c r="E136" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5113,7 +5125,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="1" t="n">
+      <c r="H136" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5149,7 +5161,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="1" t="n">
+      <c r="H137" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5173,7 +5185,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="1" t="n">
+      <c r="H138" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5197,7 +5209,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="1" t="n">
+      <c r="H139" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5233,7 +5245,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="1" t="n">
+      <c r="H140" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5261,7 +5273,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="1" t="n">
+      <c r="H141" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5297,7 +5309,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="1" t="n">
+      <c r="H142" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5322,7 +5334,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="1" t="n">
+      <c r="E143" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5331,7 +5343,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="1" t="n">
+      <c r="H143" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5367,7 +5379,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="1" t="n">
+      <c r="H144" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5403,7 +5415,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="1" t="n">
+      <c r="H145" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5439,7 +5451,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="1" t="n">
+      <c r="H146" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5463,7 +5475,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="1" t="n">
+      <c r="H147" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5488,7 +5500,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="1" t="n">
+      <c r="E148" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5497,7 +5509,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="1" t="n">
+      <c r="H148" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5521,7 +5533,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="1" t="n">
+      <c r="H149" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5545,7 +5557,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="1" t="n">
+      <c r="H150" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5569,7 +5581,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="1" t="n">
+      <c r="H151" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5593,7 +5605,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="1" t="n">
+      <c r="H152" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5617,7 +5629,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="1" t="n">
+      <c r="H153" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5642,7 +5654,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="1" t="n">
+      <c r="E154" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5651,7 +5663,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="1" t="n">
+      <c r="H154" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5676,7 +5688,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="1" t="n">
+      <c r="E155" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5685,7 +5697,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="1" t="n">
+      <c r="H155" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5709,7 +5721,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="1" t="n">
+      <c r="H156" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5734,7 +5746,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="1" t="n">
+      <c r="E157" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5743,7 +5755,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="1" t="n">
+      <c r="H157" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5768,7 +5780,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="1" t="n">
+      <c r="E158" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5777,7 +5789,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="1" t="n">
+      <c r="H158" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5802,7 +5814,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="1" t="n">
+      <c r="E159" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5811,7 +5823,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="1" t="n">
+      <c r="H159" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5836,7 +5848,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="1" t="n">
+      <c r="E160" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5845,7 +5857,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="1" t="n">
+      <c r="H160" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5870,7 +5882,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="1" t="n">
+      <c r="E161" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5879,7 +5891,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="1" t="n">
+      <c r="H161" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5903,7 +5915,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="1" t="n">
+      <c r="H162" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5927,7 +5939,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="1" t="n">
+      <c r="H163" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5951,7 +5963,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="1" t="n">
+      <c r="H164" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5976,7 +5988,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="1" t="n">
+      <c r="E165" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5985,7 +5997,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="1" t="n">
+      <c r="H165" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6021,7 +6033,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="1" t="n">
+      <c r="H166" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6045,7 +6057,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="1" t="n">
+      <c r="H167" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6069,7 +6081,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="1" t="n">
+      <c r="H168" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6105,7 +6117,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="1" t="n">
+      <c r="H169" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6133,7 +6145,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="1" t="n">
+      <c r="H170" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6169,7 +6181,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="1" t="n">
+      <c r="H171" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6194,7 +6206,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="1" t="n">
+      <c r="E172" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6203,7 +6215,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="1" t="n">
+      <c r="H172" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6239,7 +6251,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="1" t="n">
+      <c r="H173" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6275,7 +6287,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="1" t="n">
+      <c r="H174" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6311,7 +6323,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="1" t="n">
+      <c r="H175" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6335,7 +6347,7 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr"/>
-      <c r="H176" s="1" t="n">
+      <c r="H176" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6360,7 +6372,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M, 01 IPLR de FCU</t>
         </is>
       </c>
-      <c r="E177" s="1" t="n">
+      <c r="E177" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -6369,7 +6381,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H177" s="1" t="n">
+      <c r="H177" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6393,7 +6405,7 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
-      <c r="H178" s="1" t="n">
+      <c r="H178" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6418,7 +6430,7 @@
           <t>Pesquisa de pane no painel de alarmes.</t>
         </is>
       </c>
-      <c r="E179" s="1" t="n">
+      <c r="E179" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -6427,7 +6439,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H179" s="1" t="n">
+      <c r="H179" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6451,7 +6463,7 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
-      <c r="H180" s="1" t="n">
+      <c r="H180" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6475,7 +6487,7 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr"/>
-      <c r="H181" s="1" t="n">
+      <c r="H181" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6499,7 +6511,7 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
-      <c r="H182" s="1" t="n">
+      <c r="H182" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6524,7 +6536,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E183" s="1" t="n">
+      <c r="E183" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -6533,7 +6545,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H183" s="1" t="n">
+      <c r="H183" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6558,7 +6570,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E184" s="1" t="n">
+      <c r="E184" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -6567,7 +6579,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H184" s="1" t="n">
+      <c r="H184" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6591,7 +6603,7 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr"/>
-      <c r="H185" s="1" t="n">
+      <c r="H185" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6616,7 +6628,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E186" s="1" t="n">
+      <c r="E186" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -6625,7 +6637,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H186" s="1" t="n">
+      <c r="H186" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6650,7 +6662,7 @@
           <t>Agd transmissão do atuador do flape</t>
         </is>
       </c>
-      <c r="E187" s="1" t="n">
+      <c r="E187" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -6659,7 +6671,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H187" s="1" t="n">
+      <c r="H187" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6684,7 +6696,7 @@
           <t>Pesquisa de pane de FCU</t>
         </is>
       </c>
-      <c r="E188" s="1" t="n">
+      <c r="E188" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -6693,7 +6705,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H188" s="1" t="n">
+      <c r="H188" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6718,7 +6730,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E189" s="1" t="n">
+      <c r="E189" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -6727,7 +6739,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H189" s="1" t="n">
+      <c r="H189" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6752,7 +6764,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E190" s="1" t="n">
+      <c r="E190" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -6761,7 +6773,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H190" s="1" t="n">
+      <c r="H190" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6785,7 +6797,7 @@
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
-      <c r="H191" s="1" t="n">
+      <c r="H191" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6809,7 +6821,7 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
-      <c r="H192" s="1" t="n">
+      <c r="H192" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6833,7 +6845,7 @@
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr"/>
-      <c r="H193" s="1" t="n">
+      <c r="H193" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6858,7 +6870,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E194" s="1" t="n">
+      <c r="E194" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -6867,7 +6879,7 @@
           <t>15/07</t>
         </is>
       </c>
-      <c r="H194" s="1" t="n">
+      <c r="H194" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6903,7 +6915,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H195" s="1" t="n">
+      <c r="H195" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6927,7 +6939,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr"/>
-      <c r="H196" s="1" t="n">
+      <c r="H196" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6951,7 +6963,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
-      <c r="H197" s="1" t="n">
+      <c r="H197" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6987,7 +6999,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H198" s="1" t="n">
+      <c r="H198" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7015,7 +7027,7 @@
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
-      <c r="H199" s="1" t="n">
+      <c r="H199" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7051,7 +7063,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H200" s="1" t="n">
+      <c r="H200" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7076,7 +7088,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E201" s="1" t="n">
+      <c r="E201" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -7085,7 +7097,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H201" s="1" t="n">
+      <c r="H201" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7121,7 +7133,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H202" s="1" t="n">
+      <c r="H202" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7157,7 +7169,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H203" s="1" t="n">
+      <c r="H203" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7193,7 +7205,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H204" s="1" t="n">
+      <c r="H204" s="2" t="n">
         <v>46213</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (10/07/2026 22:38)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,114 +422,114 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -616,7 +604,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -691,7 +679,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -766,7 +754,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -841,7 +829,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -916,7 +904,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -991,7 +979,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="B8" t="n">
@@ -1080,42 +1068,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1141,7 +1129,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1165,7 +1153,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1201,7 +1189,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1225,7 +1213,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1249,7 +1237,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1274,7 +1262,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1283,7 +1271,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1308,7 +1296,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1317,7 +1305,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1342,7 +1330,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1351,7 +1339,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1376,7 +1364,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1385,7 +1373,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1409,7 +1397,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1433,7 +1421,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1458,7 +1446,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1467,7 +1455,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1491,7 +1479,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1516,7 +1504,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1525,7 +1513,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1549,7 +1537,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1573,7 +1561,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1598,7 +1586,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1607,7 +1595,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1631,7 +1619,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1656,7 +1644,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1665,7 +1653,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1701,7 +1689,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1725,7 +1713,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1749,7 +1737,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1785,7 +1773,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1813,7 +1801,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1849,7 +1837,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1874,7 +1862,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1883,7 +1871,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1919,7 +1907,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1955,7 +1943,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1991,7 +1979,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -2015,7 +2003,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2039,7 +2027,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2075,7 +2063,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2099,7 +2087,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2123,7 +2111,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="2" t="n">
+      <c r="H35" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2148,7 +2136,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2157,7 +2145,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="H36" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2182,7 +2170,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2191,7 +2179,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2216,7 +2204,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2225,7 +2213,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2250,7 +2238,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E39" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2259,7 +2247,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2283,7 +2271,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="2" t="n">
+      <c r="H40" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2307,7 +2295,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="2" t="n">
+      <c r="H41" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2332,7 +2320,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E42" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2341,7 +2329,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="H42" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2365,7 +2353,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2390,7 +2378,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2399,7 +2387,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="H44" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2423,7 +2411,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="2" t="n">
+      <c r="H45" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2447,7 +2435,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2471,7 +2459,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="2" t="n">
+      <c r="H47" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2495,7 +2483,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="2" t="n">
+      <c r="H48" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2520,7 +2508,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E49" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2529,7 +2517,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="H49" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2565,7 +2553,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2589,7 +2577,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="2" t="n">
+      <c r="H51" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2613,7 +2601,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="2" t="n">
+      <c r="H52" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2649,7 +2637,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="H53" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2677,7 +2665,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2713,7 +2701,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="H55" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2738,7 +2726,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2747,7 +2735,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="H56" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2783,7 +2771,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="H57" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2819,7 +2807,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="n">
+      <c r="H58" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2855,7 +2843,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="H59" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2879,7 +2867,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="2" t="n">
+      <c r="H60" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2903,7 +2891,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="2" t="n">
+      <c r="H61" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2928,7 +2916,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2937,7 +2925,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="2" t="n">
+      <c r="H62" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2961,7 +2949,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="2" t="n">
+      <c r="H63" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2986,7 +2974,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n">
+      <c r="E64" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2995,7 +2983,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="H64" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3019,7 +3007,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="2" t="n">
+      <c r="H65" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3043,7 +3031,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="2" t="n">
+      <c r="H66" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3068,7 +3056,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n">
+      <c r="E67" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3077,7 +3065,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="2" t="n">
+      <c r="H67" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3102,7 +3090,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n">
+      <c r="E68" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3111,7 +3099,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="2" t="n">
+      <c r="H68" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3135,7 +3123,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="2" t="n">
+      <c r="H69" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3159,7 +3147,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="2" t="n">
+      <c r="H70" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3184,7 +3172,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="2" t="n">
+      <c r="E71" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3193,7 +3181,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="2" t="n">
+      <c r="H71" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3217,7 +3205,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="2" t="n">
+      <c r="H72" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3242,7 +3230,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n">
+      <c r="E73" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3251,7 +3239,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="2" t="n">
+      <c r="H73" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3275,7 +3263,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="2" t="n">
+      <c r="H74" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3299,7 +3287,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="2" t="n">
+      <c r="H75" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3323,7 +3311,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="2" t="n">
+      <c r="H76" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3347,7 +3335,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="2" t="n">
+      <c r="H77" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3372,7 +3360,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E78" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3381,7 +3369,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="2" t="n">
+      <c r="H78" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3417,7 +3405,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="2" t="n">
+      <c r="H79" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3441,7 +3429,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="2" t="n">
+      <c r="H80" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3465,7 +3453,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="2" t="n">
+      <c r="H81" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3501,7 +3489,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="2" t="n">
+      <c r="H82" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3529,7 +3517,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="2" t="n">
+      <c r="H83" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3565,7 +3553,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="2" t="n">
+      <c r="H84" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3590,7 +3578,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n">
+      <c r="E85" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3599,7 +3587,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="2" t="n">
+      <c r="H85" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3635,7 +3623,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="2" t="n">
+      <c r="H86" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3671,7 +3659,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="2" t="n">
+      <c r="H87" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3707,7 +3695,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="2" t="n">
+      <c r="H88" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3731,7 +3719,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="2" t="n">
+      <c r="H89" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3756,7 +3744,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3765,7 +3753,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="2" t="n">
+      <c r="H90" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3790,7 +3778,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n">
+      <c r="E91" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3799,7 +3787,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="2" t="n">
+      <c r="H91" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3823,7 +3811,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="2" t="n">
+      <c r="H92" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3848,7 +3836,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="2" t="n">
+      <c r="E93" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3857,7 +3845,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="2" t="n">
+      <c r="H93" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3881,7 +3869,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="2" t="n">
+      <c r="H94" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3905,7 +3893,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="2" t="n">
+      <c r="H95" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3930,7 +3918,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="2" t="n">
+      <c r="E96" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3939,7 +3927,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="2" t="n">
+      <c r="H96" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3964,7 +3952,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="2" t="n">
+      <c r="E97" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3973,7 +3961,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="2" t="n">
+      <c r="H97" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3997,7 +3985,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="2" t="n">
+      <c r="H98" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4022,7 +4010,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n">
+      <c r="E99" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4031,7 +4019,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="2" t="n">
+      <c r="H99" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4056,7 +4044,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4065,7 +4053,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="2" t="n">
+      <c r="H100" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4089,7 +4077,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="2" t="n">
+      <c r="H101" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4114,7 +4102,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="2" t="n">
+      <c r="E102" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4123,7 +4111,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="2" t="n">
+      <c r="H102" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4148,7 +4136,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n">
+      <c r="E103" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4157,7 +4145,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="2" t="n">
+      <c r="H103" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4181,7 +4169,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="2" t="n">
+      <c r="H104" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4205,7 +4193,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="2" t="n">
+      <c r="H105" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4229,7 +4217,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="2" t="n">
+      <c r="H106" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4254,7 +4242,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n">
+      <c r="E107" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4263,7 +4251,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="2" t="n">
+      <c r="H107" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4299,7 +4287,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="2" t="n">
+      <c r="H108" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4323,7 +4311,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="2" t="n">
+      <c r="H109" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4347,7 +4335,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="2" t="n">
+      <c r="H110" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4383,7 +4371,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="2" t="n">
+      <c r="H111" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4411,7 +4399,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="2" t="n">
+      <c r="H112" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4447,7 +4435,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="2" t="n">
+      <c r="H113" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4472,7 +4460,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n">
+      <c r="E114" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4481,7 +4469,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="2" t="n">
+      <c r="H114" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4517,7 +4505,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="2" t="n">
+      <c r="H115" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4553,7 +4541,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="2" t="n">
+      <c r="H116" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4589,7 +4577,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="2" t="n">
+      <c r="H117" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4613,7 +4601,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="2" t="n">
+      <c r="H118" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4638,7 +4626,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n">
+      <c r="E119" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4647,7 +4635,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="2" t="n">
+      <c r="H119" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4671,7 +4659,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="2" t="n">
+      <c r="H120" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4695,7 +4683,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="2" t="n">
+      <c r="H121" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4719,7 +4707,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="2" t="n">
+      <c r="H122" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4743,7 +4731,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="2" t="n">
+      <c r="H123" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4767,7 +4755,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="2" t="n">
+      <c r="H124" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4792,7 +4780,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n">
+      <c r="E125" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4801,7 +4789,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="2" t="n">
+      <c r="H125" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4826,7 +4814,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E126" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4835,7 +4823,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="2" t="n">
+      <c r="H126" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4859,7 +4847,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="2" t="n">
+      <c r="H127" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4884,7 +4872,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="2" t="n">
+      <c r="E128" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4893,7 +4881,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="2" t="n">
+      <c r="H128" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4918,7 +4906,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n">
+      <c r="E129" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4927,7 +4915,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="2" t="n">
+      <c r="H129" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4951,7 +4939,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="2" t="n">
+      <c r="H130" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4976,7 +4964,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="2" t="n">
+      <c r="E131" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4985,7 +4973,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="2" t="n">
+      <c r="H131" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5010,7 +4998,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n">
+      <c r="E132" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -5019,7 +5007,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="2" t="n">
+      <c r="H132" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5043,7 +5031,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="2" t="n">
+      <c r="H133" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5067,7 +5055,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="2" t="n">
+      <c r="H134" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5091,7 +5079,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="2" t="n">
+      <c r="H135" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5116,7 +5104,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n">
+      <c r="E136" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5125,7 +5113,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="2" t="n">
+      <c r="H136" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5161,7 +5149,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="2" t="n">
+      <c r="H137" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5185,7 +5173,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="2" t="n">
+      <c r="H138" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5209,7 +5197,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="2" t="n">
+      <c r="H139" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5245,7 +5233,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="2" t="n">
+      <c r="H140" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5273,7 +5261,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="2" t="n">
+      <c r="H141" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5309,7 +5297,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="2" t="n">
+      <c r="H142" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5334,7 +5322,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="2" t="n">
+      <c r="E143" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5343,7 +5331,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="2" t="n">
+      <c r="H143" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5379,7 +5367,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="2" t="n">
+      <c r="H144" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5415,7 +5403,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="2" t="n">
+      <c r="H145" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5451,7 +5439,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="2" t="n">
+      <c r="H146" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5475,7 +5463,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="2" t="n">
+      <c r="H147" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5500,7 +5488,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E148" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5509,7 +5497,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="2" t="n">
+      <c r="H148" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5533,7 +5521,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="2" t="n">
+      <c r="H149" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5557,7 +5545,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="2" t="n">
+      <c r="H150" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5581,7 +5569,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="2" t="n">
+      <c r="H151" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5605,7 +5593,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="2" t="n">
+      <c r="H152" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5629,7 +5617,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="2" t="n">
+      <c r="H153" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5654,7 +5642,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n">
+      <c r="E154" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5663,7 +5651,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="2" t="n">
+      <c r="H154" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5688,7 +5676,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="2" t="n">
+      <c r="E155" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5697,7 +5685,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="2" t="n">
+      <c r="H155" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5721,7 +5709,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="2" t="n">
+      <c r="H156" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5746,7 +5734,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="2" t="n">
+      <c r="E157" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5755,7 +5743,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="2" t="n">
+      <c r="H157" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5780,7 +5768,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n">
+      <c r="E158" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5789,7 +5777,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="2" t="n">
+      <c r="H158" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5814,7 +5802,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="2" t="n">
+      <c r="E159" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5823,7 +5811,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="2" t="n">
+      <c r="H159" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5848,7 +5836,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n">
+      <c r="E160" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5857,7 +5845,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="2" t="n">
+      <c r="H160" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5882,7 +5870,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="2" t="n">
+      <c r="E161" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5891,7 +5879,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="2" t="n">
+      <c r="H161" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5915,7 +5903,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="2" t="n">
+      <c r="H162" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5939,7 +5927,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="2" t="n">
+      <c r="H163" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5963,7 +5951,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="2" t="n">
+      <c r="H164" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5988,7 +5976,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="2" t="n">
+      <c r="E165" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5997,7 +5985,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="2" t="n">
+      <c r="H165" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6033,7 +6021,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n">
+      <c r="H166" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6057,7 +6045,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="2" t="n">
+      <c r="H167" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6081,7 +6069,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="2" t="n">
+      <c r="H168" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6117,7 +6105,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n">
+      <c r="H169" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6145,7 +6133,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="2" t="n">
+      <c r="H170" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6181,7 +6169,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="2" t="n">
+      <c r="H171" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6206,7 +6194,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="2" t="n">
+      <c r="E172" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6215,7 +6203,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="2" t="n">
+      <c r="H172" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6251,7 +6239,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="2" t="n">
+      <c r="H173" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6287,7 +6275,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="2" t="n">
+      <c r="H174" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6323,7 +6311,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="2" t="n">
+      <c r="H175" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6347,7 +6335,7 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr"/>
-      <c r="H176" s="2" t="n">
+      <c r="H176" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6372,7 +6360,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M, 01 IPLR de FCU</t>
         </is>
       </c>
-      <c r="E177" s="2" t="n">
+      <c r="E177" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -6381,7 +6369,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H177" s="2" t="n">
+      <c r="H177" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6405,7 +6393,7 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
-      <c r="H178" s="2" t="n">
+      <c r="H178" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6430,7 +6418,7 @@
           <t>Pesquisa de pane no painel de alarmes.</t>
         </is>
       </c>
-      <c r="E179" s="2" t="n">
+      <c r="E179" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -6439,7 +6427,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H179" s="2" t="n">
+      <c r="H179" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6463,7 +6451,7 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
-      <c r="H180" s="2" t="n">
+      <c r="H180" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6487,7 +6475,7 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr"/>
-      <c r="H181" s="2" t="n">
+      <c r="H181" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6511,7 +6499,7 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
-      <c r="H182" s="2" t="n">
+      <c r="H182" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6536,7 +6524,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E183" s="2" t="n">
+      <c r="E183" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -6545,7 +6533,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H183" s="2" t="n">
+      <c r="H183" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6570,7 +6558,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E184" s="2" t="n">
+      <c r="E184" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -6579,7 +6567,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H184" s="2" t="n">
+      <c r="H184" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6603,7 +6591,7 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr"/>
-      <c r="H185" s="2" t="n">
+      <c r="H185" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6628,7 +6616,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E186" s="2" t="n">
+      <c r="E186" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -6637,7 +6625,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H186" s="2" t="n">
+      <c r="H186" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6662,7 +6650,7 @@
           <t>Agd transmissão do atuador do flape</t>
         </is>
       </c>
-      <c r="E187" s="2" t="n">
+      <c r="E187" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -6671,7 +6659,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H187" s="2" t="n">
+      <c r="H187" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6696,7 +6684,7 @@
           <t>Pesquisa de pane de FCU</t>
         </is>
       </c>
-      <c r="E188" s="2" t="n">
+      <c r="E188" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -6705,7 +6693,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H188" s="2" t="n">
+      <c r="H188" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6730,7 +6718,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E189" s="2" t="n">
+      <c r="E189" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -6739,7 +6727,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H189" s="2" t="n">
+      <c r="H189" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6764,7 +6752,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E190" s="2" t="n">
+      <c r="E190" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -6773,7 +6761,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H190" s="2" t="n">
+      <c r="H190" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6797,7 +6785,7 @@
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
-      <c r="H191" s="2" t="n">
+      <c r="H191" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6821,7 +6809,7 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
-      <c r="H192" s="2" t="n">
+      <c r="H192" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6845,7 +6833,7 @@
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr"/>
-      <c r="H193" s="2" t="n">
+      <c r="H193" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6870,7 +6858,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E194" s="2" t="n">
+      <c r="E194" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -6879,7 +6867,7 @@
           <t>15/07</t>
         </is>
       </c>
-      <c r="H194" s="2" t="n">
+      <c r="H194" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6915,7 +6903,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H195" s="2" t="n">
+      <c r="H195" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6939,7 +6927,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr"/>
-      <c r="H196" s="2" t="n">
+      <c r="H196" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6963,7 +6951,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
-      <c r="H197" s="2" t="n">
+      <c r="H197" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6999,7 +6987,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H198" s="2" t="n">
+      <c r="H198" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7027,7 +7015,7 @@
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
-      <c r="H199" s="2" t="n">
+      <c r="H199" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7063,7 +7051,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H200" s="2" t="n">
+      <c r="H200" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7088,7 +7076,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E201" s="2" t="n">
+      <c r="E201" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -7097,7 +7085,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H201" s="2" t="n">
+      <c r="H201" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7133,7 +7121,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H202" s="2" t="n">
+      <c r="H202" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7169,7 +7157,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H203" s="2" t="n">
+      <c r="H203" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7205,7 +7193,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H204" s="2" t="n">
+      <c r="H204" s="1" t="n">
         <v>46213</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (10/07/2026 20:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -422,114 +434,114 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -604,7 +616,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -679,7 +691,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -754,7 +766,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -829,7 +841,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -904,7 +916,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -979,7 +991,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="B8" t="n">
@@ -1068,42 +1080,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1129,7 +1141,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1153,7 +1165,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1189,7 +1201,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1213,7 +1225,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1237,7 +1249,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1262,7 +1274,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1271,7 +1283,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1296,7 +1308,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1305,7 +1317,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1330,7 +1342,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1339,7 +1351,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1364,7 +1376,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1373,7 +1385,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1397,7 +1409,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1421,7 +1433,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1446,7 +1458,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1455,7 +1467,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1479,7 +1491,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1504,7 +1516,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1513,7 +1525,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1537,7 +1549,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1561,7 +1573,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1586,7 +1598,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1595,7 +1607,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1619,7 +1631,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1644,7 +1656,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1653,7 +1665,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1689,7 +1701,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1713,7 +1725,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1737,7 +1749,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1773,7 +1785,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1801,7 +1813,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1837,7 +1849,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1862,7 +1874,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1871,7 +1883,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1907,7 +1919,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1943,7 +1955,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1979,7 +1991,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -2003,7 +2015,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="1" t="n">
+      <c r="H31" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2027,7 +2039,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2063,7 +2075,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2087,7 +2099,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2111,7 +2123,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="1" t="n">
+      <c r="H35" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2136,7 +2148,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2145,7 +2157,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="1" t="n">
+      <c r="H36" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2170,7 +2182,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2179,7 +2191,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2204,7 +2216,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2213,7 +2225,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2238,7 +2250,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2247,7 +2259,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2271,7 +2283,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="1" t="n">
+      <c r="H40" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2295,7 +2307,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="1" t="n">
+      <c r="H41" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2320,7 +2332,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="E42" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2329,7 +2341,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2353,7 +2365,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2378,7 +2390,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="E44" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2387,7 +2399,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2411,7 +2423,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="1" t="n">
+      <c r="H45" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2435,7 +2447,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="1" t="n">
+      <c r="H46" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2459,7 +2471,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="1" t="n">
+      <c r="H47" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2483,7 +2495,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="1" t="n">
+      <c r="H48" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2508,7 +2520,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="E49" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2517,7 +2529,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="1" t="n">
+      <c r="H49" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2553,7 +2565,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2577,7 +2589,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2601,7 +2613,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="1" t="n">
+      <c r="H52" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2637,7 +2649,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="1" t="n">
+      <c r="H53" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2665,7 +2677,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="1" t="n">
+      <c r="H54" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2701,7 +2713,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="1" t="n">
+      <c r="H55" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2726,7 +2738,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="1" t="n">
+      <c r="E56" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2735,7 +2747,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="1" t="n">
+      <c r="H56" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2771,7 +2783,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="1" t="n">
+      <c r="H57" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2807,7 +2819,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2843,7 +2855,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="1" t="n">
+      <c r="H59" s="2" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2867,7 +2879,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="1" t="n">
+      <c r="H60" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2891,7 +2903,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="1" t="n">
+      <c r="H61" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2916,7 +2928,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="1" t="n">
+      <c r="E62" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2925,7 +2937,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="1" t="n">
+      <c r="H62" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2949,7 +2961,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="1" t="n">
+      <c r="H63" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2974,7 +2986,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="1" t="n">
+      <c r="E64" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2983,7 +2995,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="1" t="n">
+      <c r="H64" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3007,7 +3019,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3031,7 +3043,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3056,7 +3068,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="1" t="n">
+      <c r="E67" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3065,7 +3077,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="1" t="n">
+      <c r="H67" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3090,7 +3102,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="1" t="n">
+      <c r="E68" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3099,7 +3111,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="1" t="n">
+      <c r="H68" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3123,7 +3135,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="1" t="n">
+      <c r="H69" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3147,7 +3159,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="1" t="n">
+      <c r="H70" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3172,7 +3184,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="1" t="n">
+      <c r="E71" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3181,7 +3193,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="1" t="n">
+      <c r="H71" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3205,7 +3217,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="1" t="n">
+      <c r="H72" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3230,7 +3242,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="1" t="n">
+      <c r="E73" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3239,7 +3251,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="1" t="n">
+      <c r="H73" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3263,7 +3275,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="1" t="n">
+      <c r="H74" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3287,7 +3299,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="1" t="n">
+      <c r="H75" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3311,7 +3323,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="1" t="n">
+      <c r="H76" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3335,7 +3347,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="1" t="n">
+      <c r="H77" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3360,7 +3372,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="1" t="n">
+      <c r="E78" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3369,7 +3381,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="1" t="n">
+      <c r="H78" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3405,7 +3417,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="1" t="n">
+      <c r="H79" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3429,7 +3441,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="1" t="n">
+      <c r="H80" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3453,7 +3465,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="1" t="n">
+      <c r="H81" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3489,7 +3501,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="1" t="n">
+      <c r="H82" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3517,7 +3529,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="1" t="n">
+      <c r="H83" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3553,7 +3565,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="1" t="n">
+      <c r="H84" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3578,7 +3590,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="1" t="n">
+      <c r="E85" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3587,7 +3599,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="1" t="n">
+      <c r="H85" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3623,7 +3635,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="1" t="n">
+      <c r="H86" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3659,7 +3671,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="1" t="n">
+      <c r="H87" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3695,7 +3707,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="1" t="n">
+      <c r="H88" s="2" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3719,7 +3731,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="1" t="n">
+      <c r="H89" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3744,7 +3756,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="1" t="n">
+      <c r="E90" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3753,7 +3765,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="1" t="n">
+      <c r="H90" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3778,7 +3790,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="1" t="n">
+      <c r="E91" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3787,7 +3799,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="1" t="n">
+      <c r="H91" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3811,7 +3823,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="1" t="n">
+      <c r="H92" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3836,7 +3848,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="1" t="n">
+      <c r="E93" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3845,7 +3857,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="1" t="n">
+      <c r="H93" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3869,7 +3881,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="1" t="n">
+      <c r="H94" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3893,7 +3905,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="1" t="n">
+      <c r="H95" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3918,7 +3930,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="1" t="n">
+      <c r="E96" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3927,7 +3939,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="1" t="n">
+      <c r="H96" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3952,7 +3964,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="1" t="n">
+      <c r="E97" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3961,7 +3973,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="1" t="n">
+      <c r="H97" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3985,7 +3997,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="1" t="n">
+      <c r="H98" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4010,7 +4022,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="1" t="n">
+      <c r="E99" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4019,7 +4031,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="1" t="n">
+      <c r="H99" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4044,7 +4056,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="1" t="n">
+      <c r="E100" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4053,7 +4065,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="1" t="n">
+      <c r="H100" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4077,7 +4089,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="1" t="n">
+      <c r="H101" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4102,7 +4114,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="1" t="n">
+      <c r="E102" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4111,7 +4123,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="1" t="n">
+      <c r="H102" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4136,7 +4148,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="1" t="n">
+      <c r="E103" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4145,7 +4157,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="1" t="n">
+      <c r="H103" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4169,7 +4181,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="1" t="n">
+      <c r="H104" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4193,7 +4205,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="1" t="n">
+      <c r="H105" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4217,7 +4229,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="1" t="n">
+      <c r="H106" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4242,7 +4254,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="1" t="n">
+      <c r="E107" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4251,7 +4263,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="1" t="n">
+      <c r="H107" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4287,7 +4299,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="1" t="n">
+      <c r="H108" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4311,7 +4323,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="1" t="n">
+      <c r="H109" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4335,7 +4347,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="1" t="n">
+      <c r="H110" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4371,7 +4383,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="1" t="n">
+      <c r="H111" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4399,7 +4411,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="1" t="n">
+      <c r="H112" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4435,7 +4447,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="1" t="n">
+      <c r="H113" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4460,7 +4472,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="1" t="n">
+      <c r="E114" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4469,7 +4481,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="1" t="n">
+      <c r="H114" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4505,7 +4517,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="1" t="n">
+      <c r="H115" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4541,7 +4553,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="1" t="n">
+      <c r="H116" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4577,7 +4589,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="1" t="n">
+      <c r="H117" s="2" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4601,7 +4613,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="1" t="n">
+      <c r="H118" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4626,7 +4638,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="1" t="n">
+      <c r="E119" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4635,7 +4647,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="1" t="n">
+      <c r="H119" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4659,7 +4671,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="1" t="n">
+      <c r="H120" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4683,7 +4695,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="1" t="n">
+      <c r="H121" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4707,7 +4719,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="1" t="n">
+      <c r="H122" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4731,7 +4743,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="1" t="n">
+      <c r="H123" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4755,7 +4767,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="1" t="n">
+      <c r="H124" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4780,7 +4792,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="1" t="n">
+      <c r="E125" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4789,7 +4801,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="1" t="n">
+      <c r="H125" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4814,7 +4826,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="1" t="n">
+      <c r="E126" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4823,7 +4835,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="1" t="n">
+      <c r="H126" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4847,7 +4859,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="1" t="n">
+      <c r="H127" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4872,7 +4884,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="1" t="n">
+      <c r="E128" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4881,7 +4893,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="1" t="n">
+      <c r="H128" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4906,7 +4918,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="1" t="n">
+      <c r="E129" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4915,7 +4927,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="1" t="n">
+      <c r="H129" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4939,7 +4951,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="1" t="n">
+      <c r="H130" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4964,7 +4976,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="1" t="n">
+      <c r="E131" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4973,7 +4985,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="1" t="n">
+      <c r="H131" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4998,7 +5010,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="1" t="n">
+      <c r="E132" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -5007,7 +5019,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="1" t="n">
+      <c r="H132" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5031,7 +5043,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="1" t="n">
+      <c r="H133" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5055,7 +5067,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="1" t="n">
+      <c r="H134" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5079,7 +5091,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="1" t="n">
+      <c r="H135" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5104,7 +5116,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="1" t="n">
+      <c r="E136" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5113,7 +5125,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="1" t="n">
+      <c r="H136" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5149,7 +5161,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="1" t="n">
+      <c r="H137" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5173,7 +5185,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="1" t="n">
+      <c r="H138" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5197,7 +5209,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="1" t="n">
+      <c r="H139" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5233,7 +5245,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="1" t="n">
+      <c r="H140" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5261,7 +5273,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="1" t="n">
+      <c r="H141" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5297,7 +5309,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="1" t="n">
+      <c r="H142" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5322,7 +5334,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="1" t="n">
+      <c r="E143" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5331,7 +5343,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="1" t="n">
+      <c r="H143" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5367,7 +5379,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="1" t="n">
+      <c r="H144" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5403,7 +5415,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="1" t="n">
+      <c r="H145" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5439,7 +5451,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="1" t="n">
+      <c r="H146" s="2" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5463,7 +5475,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="1" t="n">
+      <c r="H147" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5488,7 +5500,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="1" t="n">
+      <c r="E148" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5497,7 +5509,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="1" t="n">
+      <c r="H148" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5521,7 +5533,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="1" t="n">
+      <c r="H149" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5545,7 +5557,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="1" t="n">
+      <c r="H150" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5569,7 +5581,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="1" t="n">
+      <c r="H151" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5593,7 +5605,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="1" t="n">
+      <c r="H152" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5617,7 +5629,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="1" t="n">
+      <c r="H153" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5642,7 +5654,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="1" t="n">
+      <c r="E154" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5651,7 +5663,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="1" t="n">
+      <c r="H154" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5676,7 +5688,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="1" t="n">
+      <c r="E155" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5685,7 +5697,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="1" t="n">
+      <c r="H155" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5709,7 +5721,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="1" t="n">
+      <c r="H156" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5734,7 +5746,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="1" t="n">
+      <c r="E157" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5743,7 +5755,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="1" t="n">
+      <c r="H157" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5768,7 +5780,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="1" t="n">
+      <c r="E158" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5777,7 +5789,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="1" t="n">
+      <c r="H158" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5802,7 +5814,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="1" t="n">
+      <c r="E159" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5811,7 +5823,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="1" t="n">
+      <c r="H159" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5836,7 +5848,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="1" t="n">
+      <c r="E160" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5845,7 +5857,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="1" t="n">
+      <c r="H160" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5870,7 +5882,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="1" t="n">
+      <c r="E161" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5879,7 +5891,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="1" t="n">
+      <c r="H161" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5903,7 +5915,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="1" t="n">
+      <c r="H162" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5927,7 +5939,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="1" t="n">
+      <c r="H163" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5951,7 +5963,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="1" t="n">
+      <c r="H164" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5976,7 +5988,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="1" t="n">
+      <c r="E165" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5985,7 +5997,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="1" t="n">
+      <c r="H165" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6021,7 +6033,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="1" t="n">
+      <c r="H166" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6045,7 +6057,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="1" t="n">
+      <c r="H167" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6069,7 +6081,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="1" t="n">
+      <c r="H168" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6105,7 +6117,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="1" t="n">
+      <c r="H169" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6133,7 +6145,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="1" t="n">
+      <c r="H170" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6169,7 +6181,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="1" t="n">
+      <c r="H171" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6194,7 +6206,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="1" t="n">
+      <c r="E172" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6203,7 +6215,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="1" t="n">
+      <c r="H172" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6239,7 +6251,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="1" t="n">
+      <c r="H173" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6275,7 +6287,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="1" t="n">
+      <c r="H174" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6311,7 +6323,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="1" t="n">
+      <c r="H175" s="2" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6335,7 +6347,7 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr"/>
-      <c r="H176" s="1" t="n">
+      <c r="H176" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6360,7 +6372,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M, 01 IPLR de FCU</t>
         </is>
       </c>
-      <c r="E177" s="1" t="n">
+      <c r="E177" s="2" t="n">
         <v>46217</v>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -6369,7 +6381,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H177" s="1" t="n">
+      <c r="H177" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6393,7 +6405,7 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
-      <c r="H178" s="1" t="n">
+      <c r="H178" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6418,7 +6430,7 @@
           <t>Pesquisa de pane no painel de alarmes.</t>
         </is>
       </c>
-      <c r="E179" s="1" t="n">
+      <c r="E179" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -6427,7 +6439,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H179" s="1" t="n">
+      <c r="H179" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6451,7 +6463,7 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
-      <c r="H180" s="1" t="n">
+      <c r="H180" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6475,7 +6487,7 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr"/>
-      <c r="H181" s="1" t="n">
+      <c r="H181" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6499,7 +6511,7 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
-      <c r="H182" s="1" t="n">
+      <c r="H182" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6524,7 +6536,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E183" s="1" t="n">
+      <c r="E183" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -6533,7 +6545,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H183" s="1" t="n">
+      <c r="H183" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6558,7 +6570,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E184" s="1" t="n">
+      <c r="E184" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -6567,7 +6579,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H184" s="1" t="n">
+      <c r="H184" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6591,7 +6603,7 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr"/>
-      <c r="H185" s="1" t="n">
+      <c r="H185" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6616,7 +6628,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E186" s="1" t="n">
+      <c r="E186" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -6625,7 +6637,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H186" s="1" t="n">
+      <c r="H186" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6650,7 +6662,7 @@
           <t>Agd transmissão do atuador do flape</t>
         </is>
       </c>
-      <c r="E187" s="1" t="n">
+      <c r="E187" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -6659,7 +6671,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H187" s="1" t="n">
+      <c r="H187" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6684,7 +6696,7 @@
           <t>Pesquisa de pane de FCU</t>
         </is>
       </c>
-      <c r="E188" s="1" t="n">
+      <c r="E188" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -6693,7 +6705,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H188" s="1" t="n">
+      <c r="H188" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6718,7 +6730,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E189" s="1" t="n">
+      <c r="E189" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -6727,7 +6739,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H189" s="1" t="n">
+      <c r="H189" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6752,7 +6764,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E190" s="1" t="n">
+      <c r="E190" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -6761,7 +6773,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H190" s="1" t="n">
+      <c r="H190" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6785,7 +6797,7 @@
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
-      <c r="H191" s="1" t="n">
+      <c r="H191" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6809,7 +6821,7 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
-      <c r="H192" s="1" t="n">
+      <c r="H192" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6833,7 +6845,7 @@
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr"/>
-      <c r="H193" s="1" t="n">
+      <c r="H193" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6858,7 +6870,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E194" s="1" t="n">
+      <c r="E194" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -6867,7 +6879,7 @@
           <t>15/07</t>
         </is>
       </c>
-      <c r="H194" s="1" t="n">
+      <c r="H194" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6903,7 +6915,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H195" s="1" t="n">
+      <c r="H195" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6927,7 +6939,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr"/>
-      <c r="H196" s="1" t="n">
+      <c r="H196" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6951,7 +6963,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
-      <c r="H197" s="1" t="n">
+      <c r="H197" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6987,7 +6999,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H198" s="1" t="n">
+      <c r="H198" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7015,7 +7027,7 @@
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
-      <c r="H199" s="1" t="n">
+      <c r="H199" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7051,7 +7063,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H200" s="1" t="n">
+      <c r="H200" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7076,7 +7088,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E201" s="1" t="n">
+      <c r="E201" s="2" t="n">
         <v>46209</v>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -7085,7 +7097,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H201" s="1" t="n">
+      <c r="H201" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7121,7 +7133,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H202" s="1" t="n">
+      <c r="H202" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7157,7 +7169,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H203" s="1" t="n">
+      <c r="H203" s="2" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7193,7 +7205,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H204" s="1" t="n">
+      <c r="H204" s="2" t="n">
         <v>46213</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (11/07/2026 07:19)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,114 +422,114 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>disponiveis_hoje</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>montadas_hoje</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>di</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>do_</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ii</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>in_</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>itr</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>is_</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ip</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_disponiveis</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>previsao_fim_dia_montadas</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_qtd</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>previsao_semana_disponiveis_novas</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_qtd</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>previsao_semana_montadas_novas</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>esforco_anual_previsto</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>esforco_anual_realizado</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>esforco_percentual</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>motores_disponiveis</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>arquivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B2" t="n">
@@ -616,7 +604,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46205</v>
       </c>
       <c r="B3" t="n">
@@ -691,7 +679,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="B4" t="n">
@@ -766,7 +754,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="B5" t="n">
@@ -841,7 +829,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="B6" t="n">
@@ -916,7 +904,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="B7" t="n">
@@ -991,7 +979,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="B8" t="n">
@@ -1080,42 +1068,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ocorrencia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>dpe_data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>dpe_condicao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>dpe_texto_original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>data_referencia</t>
         </is>
@@ -1141,7 +1129,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1165,7 +1153,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1201,7 +1189,7 @@
           <t>01 DIA após chegada do item.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1225,7 +1213,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1249,7 +1237,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1274,7 +1262,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1283,7 +1271,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1308,7 +1296,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1317,7 +1305,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1342,7 +1330,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1351,7 +1339,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1376,7 +1364,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1385,7 +1373,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1409,7 +1397,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1433,7 +1421,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1458,7 +1446,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1467,7 +1455,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1491,7 +1479,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1516,7 +1504,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1525,7 +1513,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1549,7 +1537,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1573,7 +1561,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1598,7 +1586,7 @@
           <t>Realizando inspeções programadas.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1607,7 +1595,7 @@
           <t>01/07</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1631,7 +1619,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1656,7 +1644,7 @@
           <t>Pesquisa de pane de vazamento de óleo do motor.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1665,7 +1653,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1701,7 +1689,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1725,7 +1713,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1749,7 +1737,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1785,7 +1773,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1813,7 +1801,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1849,7 +1837,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1874,7 +1862,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1883,7 +1871,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1919,7 +1907,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1955,7 +1943,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -1991,7 +1979,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46204</v>
       </c>
     </row>
@@ -2015,7 +2003,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2039,7 +2027,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2075,7 +2063,7 @@
           <t>01 DIA após resposta do AT.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2099,7 +2087,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2123,7 +2111,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="2" t="n">
+      <c r="H35" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2148,7 +2136,7 @@
           <t>Realizando inspeções ID 0A,20,21,22 / 4100FH</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2157,7 +2145,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="H36" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2182,7 +2170,7 @@
           <t>Pesquisa no sistema de indicação de flape.</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2191,7 +2179,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2216,7 +2204,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2225,7 +2213,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2250,7 +2238,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E39" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2259,7 +2247,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2283,7 +2271,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="2" t="n">
+      <c r="H40" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2307,7 +2295,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="2" t="n">
+      <c r="H41" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2332,7 +2320,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E42" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2341,7 +2329,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="H42" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2365,7 +2353,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2390,7 +2378,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2399,7 +2387,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="H44" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2423,7 +2411,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="2" t="n">
+      <c r="H45" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2447,7 +2435,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2471,7 +2459,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="2" t="n">
+      <c r="H47" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2495,7 +2483,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="2" t="n">
+      <c r="H48" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2520,7 +2508,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E49" s="1" t="n">
         <v>46206</v>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2529,7 +2517,7 @@
           <t>03/07</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="H49" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2565,7 +2553,7 @@
           <t>02 DIAS após chegada do item.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2589,7 +2577,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="2" t="n">
+      <c r="H51" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2613,7 +2601,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="2" t="n">
+      <c r="H52" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2649,7 +2637,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="H53" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2677,7 +2665,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2713,7 +2701,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="H55" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2738,7 +2726,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n">
+      <c r="E56" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2747,7 +2735,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="H56" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2783,7 +2771,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="H57" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2819,7 +2807,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="n">
+      <c r="H58" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2855,7 +2843,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="H59" s="1" t="n">
         <v>46205</v>
       </c>
     </row>
@@ -2879,7 +2867,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="2" t="n">
+      <c r="H60" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2903,7 +2891,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="2" t="n">
+      <c r="H61" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2928,7 +2916,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2937,7 +2925,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H62" s="2" t="n">
+      <c r="H62" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2961,7 +2949,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="2" t="n">
+      <c r="H63" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -2986,7 +2974,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n">
+      <c r="E64" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -2995,7 +2983,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="H64" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3019,7 +3007,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="2" t="n">
+      <c r="H65" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3043,7 +3031,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="2" t="n">
+      <c r="H66" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3068,7 +3056,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n">
+      <c r="E67" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3077,7 +3065,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H67" s="2" t="n">
+      <c r="H67" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3102,7 +3090,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n">
+      <c r="E68" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3111,7 +3099,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H68" s="2" t="n">
+      <c r="H68" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3135,7 +3123,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="2" t="n">
+      <c r="H69" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3159,7 +3147,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="2" t="n">
+      <c r="H70" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3184,7 +3172,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E71" s="2" t="n">
+      <c r="E71" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3193,7 +3181,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H71" s="2" t="n">
+      <c r="H71" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3217,7 +3205,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="2" t="n">
+      <c r="H72" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3242,7 +3230,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n">
+      <c r="E73" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3251,7 +3239,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H73" s="2" t="n">
+      <c r="H73" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3275,7 +3263,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="2" t="n">
+      <c r="H74" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3299,7 +3287,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="2" t="n">
+      <c r="H75" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3323,7 +3311,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="2" t="n">
+      <c r="H76" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3347,7 +3335,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="2" t="n">
+      <c r="H77" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3372,7 +3360,7 @@
           <t>Motor apresentando T5 limítrofe, em pesquisa de pane e substituição do terminal T5</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n">
+      <c r="E78" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3381,7 +3369,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H78" s="2" t="n">
+      <c r="H78" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3417,7 +3405,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H79" s="2" t="n">
+      <c r="H79" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3441,7 +3429,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="2" t="n">
+      <c r="H80" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3465,7 +3453,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="2" t="n">
+      <c r="H81" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3501,7 +3489,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H82" s="2" t="n">
+      <c r="H82" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3529,7 +3517,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="2" t="n">
+      <c r="H83" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3565,7 +3553,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H84" s="2" t="n">
+      <c r="H84" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3590,7 +3578,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n">
+      <c r="E85" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3599,7 +3587,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H85" s="2" t="n">
+      <c r="H85" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3635,7 +3623,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H86" s="2" t="n">
+      <c r="H86" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3671,7 +3659,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H87" s="2" t="n">
+      <c r="H87" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3707,7 +3695,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H88" s="2" t="n">
+      <c r="H88" s="1" t="n">
         <v>46209</v>
       </c>
     </row>
@@ -3731,7 +3719,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="2" t="n">
+      <c r="H89" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3756,7 +3744,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n">
+      <c r="E90" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3765,7 +3753,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H90" s="2" t="n">
+      <c r="H90" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3790,7 +3778,7 @@
           <t>Agd parecer do AT do PAMASP sobre FCU</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n">
+      <c r="E91" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3799,7 +3787,7 @@
           <t>07/07</t>
         </is>
       </c>
-      <c r="H91" s="2" t="n">
+      <c r="H91" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3823,7 +3811,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="2" t="n">
+      <c r="H92" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3848,7 +3836,7 @@
           <t>Realizando inspeções ID 0A / 500FH</t>
         </is>
       </c>
-      <c r="E93" s="2" t="n">
+      <c r="E93" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -3857,7 +3845,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H93" s="2" t="n">
+      <c r="H93" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3881,7 +3869,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="2" t="n">
+      <c r="H94" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3905,7 +3893,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="2" t="n">
+      <c r="H95" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3930,7 +3918,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E96" s="2" t="n">
+      <c r="E96" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -3939,7 +3927,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H96" s="2" t="n">
+      <c r="H96" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3964,7 +3952,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E97" s="2" t="n">
+      <c r="E97" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3973,7 +3961,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H97" s="2" t="n">
+      <c r="H97" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -3997,7 +3985,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="2" t="n">
+      <c r="H98" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4022,7 +4010,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n">
+      <c r="E99" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4031,7 +4019,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H99" s="2" t="n">
+      <c r="H99" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4056,7 +4044,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n">
+      <c r="E100" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4065,7 +4053,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H100" s="2" t="n">
+      <c r="H100" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4089,7 +4077,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="2" t="n">
+      <c r="H101" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4114,7 +4102,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E102" s="2" t="n">
+      <c r="E102" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4123,7 +4111,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H102" s="2" t="n">
+      <c r="H102" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4148,7 +4136,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n">
+      <c r="E103" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4157,7 +4145,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H103" s="2" t="n">
+      <c r="H103" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4181,7 +4169,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="2" t="n">
+      <c r="H104" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4205,7 +4193,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="2" t="n">
+      <c r="H105" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4229,7 +4217,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="2" t="n">
+      <c r="H106" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4254,7 +4242,7 @@
           <t>MOTOR NÃO COMPLETANDO O CICLO DE PARTIDA, ESTABILIZANDO COM 40% DE NG</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n">
+      <c r="E107" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4263,7 +4251,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H107" s="2" t="n">
+      <c r="H107" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4299,7 +4287,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H108" s="2" t="n">
+      <c r="H108" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4323,7 +4311,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="2" t="n">
+      <c r="H109" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4347,7 +4335,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="2" t="n">
+      <c r="H110" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4383,7 +4371,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H111" s="2" t="n">
+      <c r="H111" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4411,7 +4399,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="2" t="n">
+      <c r="H112" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4447,7 +4435,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H113" s="2" t="n">
+      <c r="H113" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4472,7 +4460,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n">
+      <c r="E114" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -4481,7 +4469,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H114" s="2" t="n">
+      <c r="H114" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4517,7 +4505,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H115" s="2" t="n">
+      <c r="H115" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4553,7 +4541,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H116" s="2" t="n">
+      <c r="H116" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4589,7 +4577,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H117" s="2" t="n">
+      <c r="H117" s="1" t="n">
         <v>46210</v>
       </c>
     </row>
@@ -4613,7 +4601,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="2" t="n">
+      <c r="H118" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4638,7 +4626,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n">
+      <c r="E119" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -4647,7 +4635,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H119" s="2" t="n">
+      <c r="H119" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4671,7 +4659,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="2" t="n">
+      <c r="H120" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4695,7 +4683,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="2" t="n">
+      <c r="H121" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4719,7 +4707,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="2" t="n">
+      <c r="H122" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4743,7 +4731,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="2" t="n">
+      <c r="H123" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4767,7 +4755,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="2" t="n">
+      <c r="H124" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4792,7 +4780,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n">
+      <c r="E125" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -4801,7 +4789,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H125" s="2" t="n">
+      <c r="H125" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4826,7 +4814,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E126" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4835,7 +4823,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H126" s="2" t="n">
+      <c r="H126" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4859,7 +4847,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="2" t="n">
+      <c r="H127" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4884,7 +4872,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E128" s="2" t="n">
+      <c r="E128" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -4893,7 +4881,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H128" s="2" t="n">
+      <c r="H128" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4918,7 +4906,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n">
+      <c r="E129" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -4927,7 +4915,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H129" s="2" t="n">
+      <c r="H129" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4951,7 +4939,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="2" t="n">
+      <c r="H130" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -4976,7 +4964,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E131" s="2" t="n">
+      <c r="E131" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -4985,7 +4973,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H131" s="2" t="n">
+      <c r="H131" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5010,7 +4998,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n">
+      <c r="E132" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -5019,7 +5007,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H132" s="2" t="n">
+      <c r="H132" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5043,7 +5031,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="2" t="n">
+      <c r="H133" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5067,7 +5055,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="2" t="n">
+      <c r="H134" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5091,7 +5079,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="2" t="n">
+      <c r="H135" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5116,7 +5104,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n">
+      <c r="E136" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -5125,7 +5113,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H136" s="2" t="n">
+      <c r="H136" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5161,7 +5149,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H137" s="2" t="n">
+      <c r="H137" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5185,7 +5173,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="2" t="n">
+      <c r="H138" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5209,7 +5197,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="2" t="n">
+      <c r="H139" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5245,7 +5233,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H140" s="2" t="n">
+      <c r="H140" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5273,7 +5261,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="2" t="n">
+      <c r="H141" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5309,7 +5297,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H142" s="2" t="n">
+      <c r="H142" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5334,7 +5322,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E143" s="2" t="n">
+      <c r="E143" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -5343,7 +5331,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H143" s="2" t="n">
+      <c r="H143" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5379,7 +5367,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H144" s="2" t="n">
+      <c r="H144" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5415,7 +5403,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H145" s="2" t="n">
+      <c r="H145" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5451,7 +5439,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H146" s="2" t="n">
+      <c r="H146" s="1" t="n">
         <v>46211</v>
       </c>
     </row>
@@ -5475,7 +5463,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" s="2" t="n">
+      <c r="H147" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5500,7 +5488,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E148" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -5509,7 +5497,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H148" s="2" t="n">
+      <c r="H148" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5533,7 +5521,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
-      <c r="H149" s="2" t="n">
+      <c r="H149" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5557,7 +5545,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
-      <c r="H150" s="2" t="n">
+      <c r="H150" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5581,7 +5569,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
-      <c r="H151" s="2" t="n">
+      <c r="H151" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5605,7 +5593,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
-      <c r="H152" s="2" t="n">
+      <c r="H152" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5629,7 +5617,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
-      <c r="H153" s="2" t="n">
+      <c r="H153" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5654,7 +5642,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n">
+      <c r="E154" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -5663,7 +5651,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H154" s="2" t="n">
+      <c r="H154" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5688,7 +5676,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E155" s="2" t="n">
+      <c r="E155" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -5697,7 +5685,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H155" s="2" t="n">
+      <c r="H155" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5721,7 +5709,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
-      <c r="H156" s="2" t="n">
+      <c r="H156" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5746,7 +5734,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E157" s="2" t="n">
+      <c r="E157" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5755,7 +5743,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H157" s="2" t="n">
+      <c r="H157" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5780,7 +5768,7 @@
           <t>Pane no sistema de flape</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n">
+      <c r="E158" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5789,7 +5777,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H158" s="2" t="n">
+      <c r="H158" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5814,7 +5802,7 @@
           <t>EM PESQUISA DE PANE DE FCU</t>
         </is>
       </c>
-      <c r="E159" s="2" t="n">
+      <c r="E159" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5823,7 +5811,7 @@
           <t>09/07</t>
         </is>
       </c>
-      <c r="H159" s="2" t="n">
+      <c r="H159" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5848,7 +5836,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n">
+      <c r="E160" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5857,7 +5845,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H160" s="2" t="n">
+      <c r="H160" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5882,7 +5870,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E161" s="2" t="n">
+      <c r="E161" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5891,7 +5879,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H161" s="2" t="n">
+      <c r="H161" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5915,7 +5903,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr"/>
-      <c r="H162" s="2" t="n">
+      <c r="H162" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5939,7 +5927,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
-      <c r="H163" s="2" t="n">
+      <c r="H163" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5963,7 +5951,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
-      <c r="H164" s="2" t="n">
+      <c r="H164" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -5988,7 +5976,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E165" s="2" t="n">
+      <c r="E165" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5997,7 +5985,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H165" s="2" t="n">
+      <c r="H165" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6033,7 +6021,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n">
+      <c r="H166" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6057,7 +6045,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" s="2" t="n">
+      <c r="H167" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6081,7 +6069,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr"/>
-      <c r="H168" s="2" t="n">
+      <c r="H168" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6117,7 +6105,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n">
+      <c r="H169" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6145,7 +6133,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr"/>
-      <c r="H170" s="2" t="n">
+      <c r="H170" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6181,7 +6169,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H171" s="2" t="n">
+      <c r="H171" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6206,7 +6194,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E172" s="2" t="n">
+      <c r="E172" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -6215,7 +6203,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H172" s="2" t="n">
+      <c r="H172" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6251,7 +6239,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H173" s="2" t="n">
+      <c r="H173" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6287,7 +6275,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H174" s="2" t="n">
+      <c r="H174" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6323,7 +6311,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H175" s="2" t="n">
+      <c r="H175" s="1" t="n">
         <v>46212</v>
       </c>
     </row>
@@ -6347,7 +6335,7 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr"/>
-      <c r="H176" s="2" t="n">
+      <c r="H176" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6372,7 +6360,7 @@
           <t>ANV REALIZANDO INSPEÇÃO PROGRAMADA ID5-15-06/+4200FH DO MOTOR/48M, 01 IPLR de FCU</t>
         </is>
       </c>
-      <c r="E177" s="2" t="n">
+      <c r="E177" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -6381,7 +6369,7 @@
           <t>14/07</t>
         </is>
       </c>
-      <c r="H177" s="2" t="n">
+      <c r="H177" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6405,7 +6393,7 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
-      <c r="H178" s="2" t="n">
+      <c r="H178" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6430,7 +6418,7 @@
           <t>Pesquisa de pane no painel de alarmes.</t>
         </is>
       </c>
-      <c r="E179" s="2" t="n">
+      <c r="E179" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -6439,7 +6427,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H179" s="2" t="n">
+      <c r="H179" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6463,7 +6451,7 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
-      <c r="H180" s="2" t="n">
+      <c r="H180" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6487,7 +6475,7 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr"/>
-      <c r="H181" s="2" t="n">
+      <c r="H181" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6511,7 +6499,7 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
-      <c r="H182" s="2" t="n">
+      <c r="H182" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6536,7 +6524,7 @@
           <t>Realizando inspeções ID 0A,02,07,10,11,12,21,22 / 2900FH/HSI</t>
         </is>
       </c>
-      <c r="E183" s="2" t="n">
+      <c r="E183" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -6545,7 +6533,7 @@
           <t>31/07</t>
         </is>
       </c>
-      <c r="H183" s="2" t="n">
+      <c r="H183" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6570,7 +6558,7 @@
           <t>Realizando inspeções 4300 FH/HSI.</t>
         </is>
       </c>
-      <c r="E184" s="2" t="n">
+      <c r="E184" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -6579,7 +6567,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H184" s="2" t="n">
+      <c r="H184" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6603,7 +6591,7 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr"/>
-      <c r="H185" s="2" t="n">
+      <c r="H185" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6628,7 +6616,7 @@
           <t>ANV REALIZANDO INSPEÇÕES ID5-15-0A/07 E 4400FH</t>
         </is>
       </c>
-      <c r="E186" s="2" t="n">
+      <c r="E186" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -6637,7 +6625,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H186" s="2" t="n">
+      <c r="H186" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6662,7 +6650,7 @@
           <t>Agd transmissão do atuador do flape</t>
         </is>
       </c>
-      <c r="E187" s="2" t="n">
+      <c r="E187" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -6671,7 +6659,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H187" s="2" t="n">
+      <c r="H187" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6696,7 +6684,7 @@
           <t>Pesquisa de pane de FCU</t>
         </is>
       </c>
-      <c r="E188" s="2" t="n">
+      <c r="E188" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -6705,7 +6693,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H188" s="2" t="n">
+      <c r="H188" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6730,7 +6718,7 @@
           <t>Motor recolhido para reparo na geradora de gases</t>
         </is>
       </c>
-      <c r="E189" s="2" t="n">
+      <c r="E189" s="1" t="n">
         <v>46216</v>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -6739,7 +6727,7 @@
           <t>13/07</t>
         </is>
       </c>
-      <c r="H189" s="2" t="n">
+      <c r="H189" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6764,7 +6752,7 @@
           <t>REALIZANDO INSPEÇÃO ID5-15-0A (3130021644), 3900H (MOT) (3130021645) ,MOT2M6 (MOT)( 3130021646)</t>
         </is>
       </c>
-      <c r="E190" s="2" t="n">
+      <c r="E190" s="1" t="n">
         <v>46213</v>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -6773,7 +6761,7 @@
           <t>10/07</t>
         </is>
       </c>
-      <c r="H190" s="2" t="n">
+      <c r="H190" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6797,7 +6785,7 @@
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr"/>
-      <c r="H191" s="2" t="n">
+      <c r="H191" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6821,7 +6809,7 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
-      <c r="H192" s="2" t="n">
+      <c r="H192" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6845,7 +6833,7 @@
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr"/>
-      <c r="H193" s="2" t="n">
+      <c r="H193" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6870,7 +6858,7 @@
           <t>Motor não completando ciclo de partida, estabilizando com 40% de NG</t>
         </is>
       </c>
-      <c r="E194" s="2" t="n">
+      <c r="E194" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -6879,7 +6867,7 @@
           <t>15/07</t>
         </is>
       </c>
-      <c r="H194" s="2" t="n">
+      <c r="H194" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6915,7 +6903,7 @@
           <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
         </is>
       </c>
-      <c r="H195" s="2" t="n">
+      <c r="H195" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6939,7 +6927,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr"/>
-      <c r="H196" s="2" t="n">
+      <c r="H196" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6963,7 +6951,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
-      <c r="H197" s="2" t="n">
+      <c r="H197" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -6999,7 +6987,7 @@
           <t>A ser definido.</t>
         </is>
       </c>
-      <c r="H198" s="2" t="n">
+      <c r="H198" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7027,7 +7015,7 @@
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
-      <c r="H199" s="2" t="n">
+      <c r="H199" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7063,7 +7051,7 @@
           <t>A DET</t>
         </is>
       </c>
-      <c r="H200" s="2" t="n">
+      <c r="H200" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7088,7 +7076,7 @@
           <t>Aguardando avaliação de sinistro</t>
         </is>
       </c>
-      <c r="E201" s="2" t="n">
+      <c r="E201" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -7097,7 +7085,7 @@
           <t>06/07</t>
         </is>
       </c>
-      <c r="H201" s="2" t="n">
+      <c r="H201" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7133,7 +7121,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H202" s="2" t="n">
+      <c r="H202" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7169,7 +7157,7 @@
           <t>Aguarda DPE do PAMASP.</t>
         </is>
       </c>
-      <c r="H203" s="2" t="n">
+      <c r="H203" s="1" t="n">
         <v>46213</v>
       </c>
     </row>
@@ -7205,7 +7193,7 @@
           <t>Aguarda DPE do PAMASP e PAMALS.</t>
         </is>
       </c>
-      <c r="H204" s="2" t="n">
+      <c r="H204" s="1" t="n">
         <v>46213</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (15/07/2026 16:10)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -540,16 +540,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -565,7 +557,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -573,30 +565,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -896,72 +870,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1026,7 +1000,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1091,7 +1065,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1156,7 +1130,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1221,7 +1195,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1286,7 +1260,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1351,7 +1325,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1416,7 +1390,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1481,7 +1455,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1546,7 +1520,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1621,28 +1595,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>61</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1656,7 +1630,7 @@
       <c r="C2" t="s">
         <v>100</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1670,7 +1644,7 @@
       <c r="C3" t="s">
         <v>100</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1693,7 +1667,7 @@
       <c r="G4" t="s">
         <v>147</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1707,7 +1681,7 @@
       <c r="C5" t="s">
         <v>100</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1721,7 +1695,7 @@
       <c r="C6" t="s">
         <v>100</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1738,13 +1712,13 @@
       <c r="D7" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>155</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1761,13 +1735,13 @@
       <c r="D8" t="s">
         <v>109</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>155</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="D9" t="s">
         <v>110</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>156</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1807,13 +1781,13 @@
       <c r="D10" t="s">
         <v>111</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>157</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1827,7 +1801,7 @@
       <c r="C11" t="s">
         <v>100</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1841,7 +1815,7 @@
       <c r="C12" t="s">
         <v>100</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1858,13 +1832,13 @@
       <c r="D13" t="s">
         <v>112</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>155</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1878,7 +1852,7 @@
       <c r="C14" t="s">
         <v>104</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1895,13 +1869,13 @@
       <c r="D15" t="s">
         <v>113</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>158</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1915,7 +1889,7 @@
       <c r="C16" t="s">
         <v>100</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1929,7 +1903,7 @@
       <c r="C17" t="s">
         <v>100</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1946,13 +1920,13 @@
       <c r="D18" t="s">
         <v>114</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1966,7 +1940,7 @@
       <c r="C19" t="s">
         <v>100</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1983,13 +1957,13 @@
       <c r="D20" t="s">
         <v>115</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>155</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2012,7 +1986,7 @@
       <c r="G21" t="s">
         <v>148</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2026,7 +2000,7 @@
       <c r="C22" t="s">
         <v>104</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2040,7 +2014,7 @@
       <c r="C23" t="s">
         <v>100</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2063,7 +2037,7 @@
       <c r="G24" t="s">
         <v>149</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2080,7 +2054,7 @@
       <c r="D25" t="s">
         <v>117</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2103,7 +2077,7 @@
       <c r="G26" t="s">
         <v>150</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2120,13 +2094,13 @@
       <c r="D27" t="s">
         <v>119</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>160</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2149,7 +2123,7 @@
       <c r="G28" t="s">
         <v>151</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2172,7 +2146,7 @@
       <c r="G29" t="s">
         <v>151</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2195,7 +2169,7 @@
       <c r="G30" t="s">
         <v>152</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2209,7 +2183,7 @@
       <c r="C31" t="s">
         <v>100</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2223,7 +2197,7 @@
       <c r="C32" t="s">
         <v>100</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2246,7 +2220,7 @@
       <c r="G33" t="s">
         <v>153</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2260,7 +2234,7 @@
       <c r="C34" t="s">
         <v>100</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2274,7 +2248,7 @@
       <c r="C35" t="s">
         <v>100</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2291,13 +2265,13 @@
       <c r="D36" t="s">
         <v>108</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>155</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2314,13 +2288,13 @@
       <c r="D37" t="s">
         <v>109</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>155</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2337,13 +2311,13 @@
       <c r="D38" t="s">
         <v>110</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>156</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2360,13 +2334,13 @@
       <c r="D39" t="s">
         <v>111</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>157</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2380,7 +2354,7 @@
       <c r="C40" t="s">
         <v>100</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2394,7 +2368,7 @@
       <c r="C41" t="s">
         <v>100</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2411,13 +2385,13 @@
       <c r="D42" t="s">
         <v>112</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>155</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2431,7 +2405,7 @@
       <c r="C43" t="s">
         <v>100</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2448,13 +2422,13 @@
       <c r="D44" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>158</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2468,7 +2442,7 @@
       <c r="C45" t="s">
         <v>100</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2482,7 +2456,7 @@
       <c r="C46" t="s">
         <v>100</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2496,7 +2470,7 @@
       <c r="C47" t="s">
         <v>104</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2510,7 +2484,7 @@
       <c r="C48" t="s">
         <v>100</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2527,13 +2501,13 @@
       <c r="D49" t="s">
         <v>124</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>155</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2556,7 +2530,7 @@
       <c r="G50" t="s">
         <v>148</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2570,7 +2544,7 @@
       <c r="C51" t="s">
         <v>104</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2584,7 +2558,7 @@
       <c r="C52" t="s">
         <v>100</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2607,7 +2581,7 @@
       <c r="G53" t="s">
         <v>149</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2624,7 +2598,7 @@
       <c r="D54" t="s">
         <v>117</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2647,7 +2621,7 @@
       <c r="G55" t="s">
         <v>150</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2664,13 +2638,13 @@
       <c r="D56" t="s">
         <v>119</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>160</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2693,7 +2667,7 @@
       <c r="G57" t="s">
         <v>151</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2716,7 +2690,7 @@
       <c r="G58" t="s">
         <v>151</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2739,7 +2713,7 @@
       <c r="G59" t="s">
         <v>152</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2753,7 +2727,7 @@
       <c r="C60" t="s">
         <v>100</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2767,7 +2741,7 @@
       <c r="C61" t="s">
         <v>100</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2784,13 +2758,13 @@
       <c r="D62" t="s">
         <v>123</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>161</v>
       </c>
-      <c r="H62" s="2">
+      <c r="H62" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2804,7 +2778,7 @@
       <c r="C63" t="s">
         <v>100</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2821,13 +2795,13 @@
       <c r="D64" t="s">
         <v>125</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>162</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2841,7 +2815,7 @@
       <c r="C65" t="s">
         <v>100</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2855,7 +2829,7 @@
       <c r="C66" t="s">
         <v>104</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2872,13 +2846,13 @@
       <c r="D67" t="s">
         <v>110</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>156</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2895,13 +2869,13 @@
       <c r="D68" t="s">
         <v>111</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>157</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2915,7 +2889,7 @@
       <c r="C69" t="s">
         <v>100</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2929,7 +2903,7 @@
       <c r="C70" t="s">
         <v>100</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2946,13 +2920,13 @@
       <c r="D71" t="s">
         <v>112</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>161</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2966,7 +2940,7 @@
       <c r="C72" t="s">
         <v>100</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2983,13 +2957,13 @@
       <c r="D73" t="s">
         <v>113</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>158</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3003,7 +2977,7 @@
       <c r="C74" t="s">
         <v>100</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3017,7 +2991,7 @@
       <c r="C75" t="s">
         <v>100</v>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3031,7 +3005,7 @@
       <c r="C76" t="s">
         <v>100</v>
       </c>
-      <c r="H76" s="2">
+      <c r="H76" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3045,7 +3019,7 @@
       <c r="C77" t="s">
         <v>100</v>
       </c>
-      <c r="H77" s="2">
+      <c r="H77" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3062,13 +3036,13 @@
       <c r="D78" t="s">
         <v>124</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="1">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>161</v>
       </c>
-      <c r="H78" s="2">
+      <c r="H78" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3091,7 +3065,7 @@
       <c r="G79" t="s">
         <v>154</v>
       </c>
-      <c r="H79" s="2">
+      <c r="H79" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3105,7 +3079,7 @@
       <c r="C80" t="s">
         <v>104</v>
       </c>
-      <c r="H80" s="2">
+      <c r="H80" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3119,7 +3093,7 @@
       <c r="C81" t="s">
         <v>100</v>
       </c>
-      <c r="H81" s="2">
+      <c r="H81" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3142,7 +3116,7 @@
       <c r="G82" t="s">
         <v>149</v>
       </c>
-      <c r="H82" s="2">
+      <c r="H82" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3159,7 +3133,7 @@
       <c r="D83" t="s">
         <v>117</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3182,7 +3156,7 @@
       <c r="G84" t="s">
         <v>150</v>
       </c>
-      <c r="H84" s="2">
+      <c r="H84" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3199,13 +3173,13 @@
       <c r="D85" t="s">
         <v>119</v>
       </c>
-      <c r="E85" s="2">
+      <c r="E85" s="1">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>160</v>
       </c>
-      <c r="H85" s="2">
+      <c r="H85" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3228,7 +3202,7 @@
       <c r="G86" t="s">
         <v>151</v>
       </c>
-      <c r="H86" s="2">
+      <c r="H86" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3251,7 +3225,7 @@
       <c r="G87" t="s">
         <v>151</v>
       </c>
-      <c r="H87" s="2">
+      <c r="H87" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3274,7 +3248,7 @@
       <c r="G88" t="s">
         <v>152</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3288,7 +3262,7 @@
       <c r="C89" t="s">
         <v>100</v>
       </c>
-      <c r="H89" s="2">
+      <c r="H89" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3305,13 +3279,13 @@
       <c r="D90" t="s">
         <v>127</v>
       </c>
-      <c r="E90" s="2">
+      <c r="E90" s="1">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>162</v>
       </c>
-      <c r="H90" s="2">
+      <c r="H90" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3328,13 +3302,13 @@
       <c r="D91" t="s">
         <v>123</v>
       </c>
-      <c r="E91" s="2">
+      <c r="E91" s="1">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>161</v>
       </c>
-      <c r="H91" s="2">
+      <c r="H91" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="C92" t="s">
         <v>100</v>
       </c>
-      <c r="H92" s="2">
+      <c r="H92" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3365,13 +3339,13 @@
       <c r="D93" t="s">
         <v>125</v>
       </c>
-      <c r="E93" s="2">
+      <c r="E93" s="1">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>162</v>
       </c>
-      <c r="H93" s="2">
+      <c r="H93" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3385,7 +3359,7 @@
       <c r="C94" t="s">
         <v>100</v>
       </c>
-      <c r="H94" s="2">
+      <c r="H94" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3399,7 +3373,7 @@
       <c r="C95" t="s">
         <v>104</v>
       </c>
-      <c r="H95" s="2">
+      <c r="H95" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3416,13 +3390,13 @@
       <c r="D96" t="s">
         <v>110</v>
       </c>
-      <c r="E96" s="2">
+      <c r="E96" s="1">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>156</v>
       </c>
-      <c r="H96" s="2">
+      <c r="H96" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3439,13 +3413,13 @@
       <c r="D97" t="s">
         <v>111</v>
       </c>
-      <c r="E97" s="2">
+      <c r="E97" s="1">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>157</v>
       </c>
-      <c r="H97" s="2">
+      <c r="H97" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3459,7 +3433,7 @@
       <c r="C98" t="s">
         <v>100</v>
       </c>
-      <c r="H98" s="2">
+      <c r="H98" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3476,13 +3450,13 @@
       <c r="D99" t="s">
         <v>128</v>
       </c>
-      <c r="E99" s="2">
+      <c r="E99" s="1">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>157</v>
       </c>
-      <c r="H99" s="2">
+      <c r="H99" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3499,13 +3473,13 @@
       <c r="D100" t="s">
         <v>112</v>
       </c>
-      <c r="E100" s="2">
+      <c r="E100" s="1">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>157</v>
       </c>
-      <c r="H100" s="2">
+      <c r="H100" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3519,7 +3493,7 @@
       <c r="C101" t="s">
         <v>100</v>
       </c>
-      <c r="H101" s="2">
+      <c r="H101" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3536,13 +3510,13 @@
       <c r="D102" t="s">
         <v>113</v>
       </c>
-      <c r="E102" s="2">
+      <c r="E102" s="1">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>158</v>
       </c>
-      <c r="H102" s="2">
+      <c r="H102" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3559,13 +3533,13 @@
       <c r="D103" t="s">
         <v>129</v>
       </c>
-      <c r="E103" s="2">
+      <c r="E103" s="1">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>157</v>
       </c>
-      <c r="H103" s="2">
+      <c r="H103" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3579,7 +3553,7 @@
       <c r="C104" t="s">
         <v>100</v>
       </c>
-      <c r="H104" s="2">
+      <c r="H104" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3593,7 +3567,7 @@
       <c r="C105" t="s">
         <v>100</v>
       </c>
-      <c r="H105" s="2">
+      <c r="H105" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3607,7 +3581,7 @@
       <c r="C106" t="s">
         <v>100</v>
       </c>
-      <c r="H106" s="2">
+      <c r="H106" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3624,13 +3598,13 @@
       <c r="D107" t="s">
         <v>130</v>
       </c>
-      <c r="E107" s="2">
+      <c r="E107" s="1">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>157</v>
       </c>
-      <c r="H107" s="2">
+      <c r="H107" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3653,7 +3627,7 @@
       <c r="G108" t="s">
         <v>154</v>
       </c>
-      <c r="H108" s="2">
+      <c r="H108" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3667,7 +3641,7 @@
       <c r="C109" t="s">
         <v>104</v>
       </c>
-      <c r="H109" s="2">
+      <c r="H109" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3681,7 +3655,7 @@
       <c r="C110" t="s">
         <v>100</v>
       </c>
-      <c r="H110" s="2">
+      <c r="H110" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3704,7 +3678,7 @@
       <c r="G111" t="s">
         <v>149</v>
       </c>
-      <c r="H111" s="2">
+      <c r="H111" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3721,7 +3695,7 @@
       <c r="D112" t="s">
         <v>117</v>
       </c>
-      <c r="H112" s="2">
+      <c r="H112" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3744,7 +3718,7 @@
       <c r="G113" t="s">
         <v>150</v>
       </c>
-      <c r="H113" s="2">
+      <c r="H113" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3761,13 +3735,13 @@
       <c r="D114" t="s">
         <v>119</v>
       </c>
-      <c r="E114" s="2">
+      <c r="E114" s="1">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>160</v>
       </c>
-      <c r="H114" s="2">
+      <c r="H114" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3790,7 +3764,7 @@
       <c r="G115" t="s">
         <v>151</v>
       </c>
-      <c r="H115" s="2">
+      <c r="H115" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3813,7 +3787,7 @@
       <c r="G116" t="s">
         <v>151</v>
       </c>
-      <c r="H116" s="2">
+      <c r="H116" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3836,7 +3810,7 @@
       <c r="G117" t="s">
         <v>152</v>
       </c>
-      <c r="H117" s="2">
+      <c r="H117" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3850,7 +3824,7 @@
       <c r="C118" t="s">
         <v>100</v>
       </c>
-      <c r="H118" s="2">
+      <c r="H118" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3867,13 +3841,13 @@
       <c r="D119" t="s">
         <v>127</v>
       </c>
-      <c r="E119" s="2">
+      <c r="E119" s="1">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>162</v>
       </c>
-      <c r="H119" s="2">
+      <c r="H119" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3887,7 +3861,7 @@
       <c r="C120" t="s">
         <v>104</v>
       </c>
-      <c r="H120" s="2">
+      <c r="H120" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3901,7 +3875,7 @@
       <c r="C121" t="s">
         <v>100</v>
       </c>
-      <c r="H121" s="2">
+      <c r="H121" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3915,7 +3889,7 @@
       <c r="C122" t="s">
         <v>104</v>
       </c>
-      <c r="H122" s="2">
+      <c r="H122" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3929,7 +3903,7 @@
       <c r="C123" t="s">
         <v>104</v>
       </c>
-      <c r="H123" s="2">
+      <c r="H123" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3943,7 +3917,7 @@
       <c r="C124" t="s">
         <v>104</v>
       </c>
-      <c r="H124" s="2">
+      <c r="H124" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3960,13 +3934,13 @@
       <c r="D125" t="s">
         <v>110</v>
       </c>
-      <c r="E125" s="2">
+      <c r="E125" s="1">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>156</v>
       </c>
-      <c r="H125" s="2">
+      <c r="H125" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -3983,13 +3957,13 @@
       <c r="D126" t="s">
         <v>111</v>
       </c>
-      <c r="E126" s="2">
+      <c r="E126" s="1">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>157</v>
       </c>
-      <c r="H126" s="2">
+      <c r="H126" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4003,7 +3977,7 @@
       <c r="C127" t="s">
         <v>100</v>
       </c>
-      <c r="H127" s="2">
+      <c r="H127" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4020,13 +3994,13 @@
       <c r="D128" t="s">
         <v>128</v>
       </c>
-      <c r="E128" s="2">
+      <c r="E128" s="1">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>157</v>
       </c>
-      <c r="H128" s="2">
+      <c r="H128" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4043,13 +4017,13 @@
       <c r="D129" t="s">
         <v>112</v>
       </c>
-      <c r="E129" s="2">
+      <c r="E129" s="1">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>157</v>
       </c>
-      <c r="H129" s="2">
+      <c r="H129" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4063,7 +4037,7 @@
       <c r="C130" t="s">
         <v>100</v>
       </c>
-      <c r="H130" s="2">
+      <c r="H130" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4080,13 +4054,13 @@
       <c r="D131" t="s">
         <v>113</v>
       </c>
-      <c r="E131" s="2">
+      <c r="E131" s="1">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>158</v>
       </c>
-      <c r="H131" s="2">
+      <c r="H131" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4103,13 +4077,13 @@
       <c r="D132" t="s">
         <v>129</v>
       </c>
-      <c r="E132" s="2">
+      <c r="E132" s="1">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>157</v>
       </c>
-      <c r="H132" s="2">
+      <c r="H132" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4123,7 +4097,7 @@
       <c r="C133" t="s">
         <v>100</v>
       </c>
-      <c r="H133" s="2">
+      <c r="H133" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4137,7 +4111,7 @@
       <c r="C134" t="s">
         <v>100</v>
       </c>
-      <c r="H134" s="2">
+      <c r="H134" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4151,7 +4125,7 @@
       <c r="C135" t="s">
         <v>100</v>
       </c>
-      <c r="H135" s="2">
+      <c r="H135" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4168,13 +4142,13 @@
       <c r="D136" t="s">
         <v>131</v>
       </c>
-      <c r="E136" s="2">
+      <c r="E136" s="1">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>157</v>
       </c>
-      <c r="H136" s="2">
+      <c r="H136" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4197,7 +4171,7 @@
       <c r="G137" t="s">
         <v>154</v>
       </c>
-      <c r="H137" s="2">
+      <c r="H137" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4211,7 +4185,7 @@
       <c r="C138" t="s">
         <v>104</v>
       </c>
-      <c r="H138" s="2">
+      <c r="H138" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4225,7 +4199,7 @@
       <c r="C139" t="s">
         <v>100</v>
       </c>
-      <c r="H139" s="2">
+      <c r="H139" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4248,7 +4222,7 @@
       <c r="G140" t="s">
         <v>149</v>
       </c>
-      <c r="H140" s="2">
+      <c r="H140" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4265,7 +4239,7 @@
       <c r="D141" t="s">
         <v>117</v>
       </c>
-      <c r="H141" s="2">
+      <c r="H141" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4288,7 +4262,7 @@
       <c r="G142" t="s">
         <v>150</v>
       </c>
-      <c r="H142" s="2">
+      <c r="H142" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4305,13 +4279,13 @@
       <c r="D143" t="s">
         <v>119</v>
       </c>
-      <c r="E143" s="2">
+      <c r="E143" s="1">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>160</v>
       </c>
-      <c r="H143" s="2">
+      <c r="H143" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4334,7 +4308,7 @@
       <c r="G144" t="s">
         <v>151</v>
       </c>
-      <c r="H144" s="2">
+      <c r="H144" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4357,7 +4331,7 @@
       <c r="G145" t="s">
         <v>151</v>
       </c>
-      <c r="H145" s="2">
+      <c r="H145" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4380,7 +4354,7 @@
       <c r="G146" t="s">
         <v>152</v>
       </c>
-      <c r="H146" s="2">
+      <c r="H146" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4394,7 +4368,7 @@
       <c r="C147" t="s">
         <v>100</v>
       </c>
-      <c r="H147" s="2">
+      <c r="H147" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4411,13 +4385,13 @@
       <c r="D148" t="s">
         <v>127</v>
       </c>
-      <c r="E148" s="2">
+      <c r="E148" s="1">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>162</v>
       </c>
-      <c r="H148" s="2">
+      <c r="H148" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4431,7 +4405,7 @@
       <c r="C149" t="s">
         <v>104</v>
       </c>
-      <c r="H149" s="2">
+      <c r="H149" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4445,7 +4419,7 @@
       <c r="C150" t="s">
         <v>100</v>
       </c>
-      <c r="H150" s="2">
+      <c r="H150" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4459,7 +4433,7 @@
       <c r="C151" t="s">
         <v>100</v>
       </c>
-      <c r="H151" s="2">
+      <c r="H151" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4473,7 +4447,7 @@
       <c r="C152" t="s">
         <v>104</v>
       </c>
-      <c r="H152" s="2">
+      <c r="H152" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4487,7 +4461,7 @@
       <c r="C153" t="s">
         <v>104</v>
       </c>
-      <c r="H153" s="2">
+      <c r="H153" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4504,13 +4478,13 @@
       <c r="D154" t="s">
         <v>110</v>
       </c>
-      <c r="E154" s="2">
+      <c r="E154" s="1">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>156</v>
       </c>
-      <c r="H154" s="2">
+      <c r="H154" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4527,13 +4501,13 @@
       <c r="D155" t="s">
         <v>111</v>
       </c>
-      <c r="E155" s="2">
+      <c r="E155" s="1">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>157</v>
       </c>
-      <c r="H155" s="2">
+      <c r="H155" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4547,7 +4521,7 @@
       <c r="C156" t="s">
         <v>100</v>
       </c>
-      <c r="H156" s="2">
+      <c r="H156" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4564,13 +4538,13 @@
       <c r="D157" t="s">
         <v>128</v>
       </c>
-      <c r="E157" s="2">
+      <c r="E157" s="1">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>157</v>
       </c>
-      <c r="H157" s="2">
+      <c r="H157" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4587,13 +4561,13 @@
       <c r="D158" t="s">
         <v>112</v>
       </c>
-      <c r="E158" s="2">
+      <c r="E158" s="1">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>157</v>
       </c>
-      <c r="H158" s="2">
+      <c r="H158" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4610,13 +4584,13 @@
       <c r="D159" t="s">
         <v>132</v>
       </c>
-      <c r="E159" s="2">
+      <c r="E159" s="1">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>163</v>
       </c>
-      <c r="H159" s="2">
+      <c r="H159" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4633,13 +4607,13 @@
       <c r="D160" t="s">
         <v>113</v>
       </c>
-      <c r="E160" s="2">
+      <c r="E160" s="1">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>158</v>
       </c>
-      <c r="H160" s="2">
+      <c r="H160" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4656,13 +4630,13 @@
       <c r="D161" t="s">
         <v>129</v>
       </c>
-      <c r="E161" s="2">
+      <c r="E161" s="1">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>157</v>
       </c>
-      <c r="H161" s="2">
+      <c r="H161" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4676,7 +4650,7 @@
       <c r="C162" t="s">
         <v>100</v>
       </c>
-      <c r="H162" s="2">
+      <c r="H162" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4690,7 +4664,7 @@
       <c r="C163" t="s">
         <v>100</v>
       </c>
-      <c r="H163" s="2">
+      <c r="H163" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4704,7 +4678,7 @@
       <c r="C164" t="s">
         <v>100</v>
       </c>
-      <c r="H164" s="2">
+      <c r="H164" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4721,13 +4695,13 @@
       <c r="D165" t="s">
         <v>131</v>
       </c>
-      <c r="E165" s="2">
+      <c r="E165" s="1">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>157</v>
       </c>
-      <c r="H165" s="2">
+      <c r="H165" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4750,7 +4724,7 @@
       <c r="G166" t="s">
         <v>154</v>
       </c>
-      <c r="H166" s="2">
+      <c r="H166" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4764,7 +4738,7 @@
       <c r="C167" t="s">
         <v>104</v>
       </c>
-      <c r="H167" s="2">
+      <c r="H167" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4778,7 +4752,7 @@
       <c r="C168" t="s">
         <v>100</v>
       </c>
-      <c r="H168" s="2">
+      <c r="H168" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4801,7 +4775,7 @@
       <c r="G169" t="s">
         <v>149</v>
       </c>
-      <c r="H169" s="2">
+      <c r="H169" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4818,7 +4792,7 @@
       <c r="D170" t="s">
         <v>117</v>
       </c>
-      <c r="H170" s="2">
+      <c r="H170" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4841,7 +4815,7 @@
       <c r="G171" t="s">
         <v>150</v>
       </c>
-      <c r="H171" s="2">
+      <c r="H171" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4858,13 +4832,13 @@
       <c r="D172" t="s">
         <v>119</v>
       </c>
-      <c r="E172" s="2">
+      <c r="E172" s="1">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>160</v>
       </c>
-      <c r="H172" s="2">
+      <c r="H172" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4887,7 +4861,7 @@
       <c r="G173" t="s">
         <v>151</v>
       </c>
-      <c r="H173" s="2">
+      <c r="H173" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4910,7 +4884,7 @@
       <c r="G174" t="s">
         <v>151</v>
       </c>
-      <c r="H174" s="2">
+      <c r="H174" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4933,7 +4907,7 @@
       <c r="G175" t="s">
         <v>152</v>
       </c>
-      <c r="H175" s="2">
+      <c r="H175" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4947,7 +4921,7 @@
       <c r="C176" t="s">
         <v>100</v>
       </c>
-      <c r="H176" s="2">
+      <c r="H176" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -4964,13 +4938,13 @@
       <c r="D177" t="s">
         <v>133</v>
       </c>
-      <c r="E177" s="2">
+      <c r="E177" s="1">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>162</v>
       </c>
-      <c r="H177" s="2">
+      <c r="H177" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -4984,7 +4958,7 @@
       <c r="C178" t="s">
         <v>100</v>
       </c>
-      <c r="H178" s="2">
+      <c r="H178" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5001,13 +4975,13 @@
       <c r="D179" t="s">
         <v>134</v>
       </c>
-      <c r="E179" s="2">
+      <c r="E179" s="1">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>158</v>
       </c>
-      <c r="H179" s="2">
+      <c r="H179" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5021,7 +4995,7 @@
       <c r="C180" t="s">
         <v>100</v>
       </c>
-      <c r="H180" s="2">
+      <c r="H180" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5035,7 +5009,7 @@
       <c r="C181" t="s">
         <v>104</v>
       </c>
-      <c r="H181" s="2">
+      <c r="H181" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5049,7 +5023,7 @@
       <c r="C182" t="s">
         <v>104</v>
       </c>
-      <c r="H182" s="2">
+      <c r="H182" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5066,13 +5040,13 @@
       <c r="D183" t="s">
         <v>110</v>
       </c>
-      <c r="E183" s="2">
+      <c r="E183" s="1">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>156</v>
       </c>
-      <c r="H183" s="2">
+      <c r="H183" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5089,13 +5063,13 @@
       <c r="D184" t="s">
         <v>111</v>
       </c>
-      <c r="E184" s="2">
+      <c r="E184" s="1">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>157</v>
       </c>
-      <c r="H184" s="2">
+      <c r="H184" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5109,7 +5083,7 @@
       <c r="C185" t="s">
         <v>100</v>
       </c>
-      <c r="H185" s="2">
+      <c r="H185" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5126,13 +5100,13 @@
       <c r="D186" t="s">
         <v>128</v>
       </c>
-      <c r="E186" s="2">
+      <c r="E186" s="1">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>157</v>
       </c>
-      <c r="H186" s="2">
+      <c r="H186" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5149,13 +5123,13 @@
       <c r="D187" t="s">
         <v>135</v>
       </c>
-      <c r="E187" s="2">
+      <c r="E187" s="1">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>157</v>
       </c>
-      <c r="H187" s="2">
+      <c r="H187" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5172,13 +5146,13 @@
       <c r="D188" t="s">
         <v>136</v>
       </c>
-      <c r="E188" s="2">
+      <c r="E188" s="1">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>157</v>
       </c>
-      <c r="H188" s="2">
+      <c r="H188" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5195,13 +5169,13 @@
       <c r="D189" t="s">
         <v>113</v>
       </c>
-      <c r="E189" s="2">
+      <c r="E189" s="1">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>158</v>
       </c>
-      <c r="H189" s="2">
+      <c r="H189" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5218,13 +5192,13 @@
       <c r="D190" t="s">
         <v>129</v>
       </c>
-      <c r="E190" s="2">
+      <c r="E190" s="1">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>157</v>
       </c>
-      <c r="H190" s="2">
+      <c r="H190" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5238,7 +5212,7 @@
       <c r="C191" t="s">
         <v>100</v>
       </c>
-      <c r="H191" s="2">
+      <c r="H191" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5252,7 +5226,7 @@
       <c r="C192" t="s">
         <v>100</v>
       </c>
-      <c r="H192" s="2">
+      <c r="H192" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5266,7 +5240,7 @@
       <c r="C193" t="s">
         <v>100</v>
       </c>
-      <c r="H193" s="2">
+      <c r="H193" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5283,13 +5257,13 @@
       <c r="D194" t="s">
         <v>131</v>
       </c>
-      <c r="E194" s="2">
+      <c r="E194" s="1">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>164</v>
       </c>
-      <c r="H194" s="2">
+      <c r="H194" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5312,7 +5286,7 @@
       <c r="G195" t="s">
         <v>154</v>
       </c>
-      <c r="H195" s="2">
+      <c r="H195" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5326,7 +5300,7 @@
       <c r="C196" t="s">
         <v>104</v>
       </c>
-      <c r="H196" s="2">
+      <c r="H196" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5340,7 +5314,7 @@
       <c r="C197" t="s">
         <v>100</v>
       </c>
-      <c r="H197" s="2">
+      <c r="H197" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5363,7 +5337,7 @@
       <c r="G198" t="s">
         <v>149</v>
       </c>
-      <c r="H198" s="2">
+      <c r="H198" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5380,7 +5354,7 @@
       <c r="D199" t="s">
         <v>117</v>
       </c>
-      <c r="H199" s="2">
+      <c r="H199" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5403,7 +5377,7 @@
       <c r="G200" t="s">
         <v>150</v>
       </c>
-      <c r="H200" s="2">
+      <c r="H200" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5420,13 +5394,13 @@
       <c r="D201" t="s">
         <v>119</v>
       </c>
-      <c r="E201" s="2">
+      <c r="E201" s="1">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>160</v>
       </c>
-      <c r="H201" s="2">
+      <c r="H201" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5449,7 +5423,7 @@
       <c r="G202" t="s">
         <v>151</v>
       </c>
-      <c r="H202" s="2">
+      <c r="H202" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5472,7 +5446,7 @@
       <c r="G203" t="s">
         <v>151</v>
       </c>
-      <c r="H203" s="2">
+      <c r="H203" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5495,7 +5469,7 @@
       <c r="G204" t="s">
         <v>152</v>
       </c>
-      <c r="H204" s="2">
+      <c r="H204" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5509,7 +5483,7 @@
       <c r="C205" t="s">
         <v>100</v>
       </c>
-      <c r="H205" s="2">
+      <c r="H205" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5526,13 +5500,13 @@
       <c r="D206" t="s">
         <v>133</v>
       </c>
-      <c r="E206" s="2">
+      <c r="E206" s="1">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>162</v>
       </c>
-      <c r="H206" s="2">
+      <c r="H206" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5546,7 +5520,7 @@
       <c r="C207" t="s">
         <v>100</v>
       </c>
-      <c r="H207" s="2">
+      <c r="H207" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5560,7 +5534,7 @@
       <c r="C208" t="s">
         <v>104</v>
       </c>
-      <c r="H208" s="2">
+      <c r="H208" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5574,7 +5548,7 @@
       <c r="C209" t="s">
         <v>100</v>
       </c>
-      <c r="H209" s="2">
+      <c r="H209" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5588,7 +5562,7 @@
       <c r="C210" t="s">
         <v>104</v>
       </c>
-      <c r="H210" s="2">
+      <c r="H210" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5602,7 +5576,7 @@
       <c r="C211" t="s">
         <v>104</v>
       </c>
-      <c r="H211" s="2">
+      <c r="H211" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5619,13 +5593,13 @@
       <c r="D212" t="s">
         <v>110</v>
       </c>
-      <c r="E212" s="2">
+      <c r="E212" s="1">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>156</v>
       </c>
-      <c r="H212" s="2">
+      <c r="H212" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5639,7 +5613,7 @@
       <c r="C213" t="s">
         <v>104</v>
       </c>
-      <c r="H213" s="2">
+      <c r="H213" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5653,7 +5627,7 @@
       <c r="C214" t="s">
         <v>100</v>
       </c>
-      <c r="H214" s="2">
+      <c r="H214" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5670,13 +5644,13 @@
       <c r="D215" t="s">
         <v>128</v>
       </c>
-      <c r="E215" s="2">
+      <c r="E215" s="1">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>165</v>
       </c>
-      <c r="H215" s="2">
+      <c r="H215" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5693,13 +5667,13 @@
       <c r="D216" t="s">
         <v>135</v>
       </c>
-      <c r="E216" s="2">
+      <c r="E216" s="1">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>158</v>
       </c>
-      <c r="H216" s="2">
+      <c r="H216" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5713,7 +5687,7 @@
       <c r="C217" t="s">
         <v>100</v>
       </c>
-      <c r="H217" s="2">
+      <c r="H217" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5730,13 +5704,13 @@
       <c r="D218" t="s">
         <v>113</v>
       </c>
-      <c r="E218" s="2">
+      <c r="E218" s="1">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>158</v>
       </c>
-      <c r="H218" s="2">
+      <c r="H218" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5750,7 +5724,7 @@
       <c r="C219" t="s">
         <v>100</v>
       </c>
-      <c r="H219" s="2">
+      <c r="H219" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5764,7 +5738,7 @@
       <c r="C220" t="s">
         <v>100</v>
       </c>
-      <c r="H220" s="2">
+      <c r="H220" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5781,13 +5755,13 @@
       <c r="D221" t="s">
         <v>137</v>
       </c>
-      <c r="E221" s="2">
+      <c r="E221" s="1">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>162</v>
       </c>
-      <c r="H221" s="2">
+      <c r="H221" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5801,7 +5775,7 @@
       <c r="C222" t="s">
         <v>100</v>
       </c>
-      <c r="H222" s="2">
+      <c r="H222" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5818,13 +5792,13 @@
       <c r="D223" t="s">
         <v>138</v>
       </c>
-      <c r="E223" s="2">
+      <c r="E223" s="1">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>166</v>
       </c>
-      <c r="H223" s="2">
+      <c r="H223" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5847,7 +5821,7 @@
       <c r="G224" t="s">
         <v>154</v>
       </c>
-      <c r="H224" s="2">
+      <c r="H224" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5861,7 +5835,7 @@
       <c r="C225" t="s">
         <v>104</v>
       </c>
-      <c r="H225" s="2">
+      <c r="H225" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5875,7 +5849,7 @@
       <c r="C226" t="s">
         <v>100</v>
       </c>
-      <c r="H226" s="2">
+      <c r="H226" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5898,7 +5872,7 @@
       <c r="G227" t="s">
         <v>149</v>
       </c>
-      <c r="H227" s="2">
+      <c r="H227" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5915,7 +5889,7 @@
       <c r="D228" t="s">
         <v>117</v>
       </c>
-      <c r="H228" s="2">
+      <c r="H228" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5938,7 +5912,7 @@
       <c r="G229" t="s">
         <v>150</v>
       </c>
-      <c r="H229" s="2">
+      <c r="H229" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5955,13 +5929,13 @@
       <c r="D230" t="s">
         <v>139</v>
       </c>
-      <c r="E230" s="2">
+      <c r="E230" s="1">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>167</v>
       </c>
-      <c r="H230" s="2">
+      <c r="H230" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5984,7 +5958,7 @@
       <c r="G231" t="s">
         <v>151</v>
       </c>
-      <c r="H231" s="2">
+      <c r="H231" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6007,7 +5981,7 @@
       <c r="G232" t="s">
         <v>151</v>
       </c>
-      <c r="H232" s="2">
+      <c r="H232" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6030,7 +6004,7 @@
       <c r="G233" t="s">
         <v>152</v>
       </c>
-      <c r="H233" s="2">
+      <c r="H233" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6044,7 +6018,7 @@
       <c r="C234" t="s">
         <v>100</v>
       </c>
-      <c r="H234" s="2">
+      <c r="H234" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6061,13 +6035,13 @@
       <c r="D235" t="s">
         <v>140</v>
       </c>
-      <c r="E235" s="2">
+      <c r="E235" s="1">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>162</v>
       </c>
-      <c r="H235" s="2">
+      <c r="H235" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6081,7 +6055,7 @@
       <c r="C236" t="s">
         <v>100</v>
       </c>
-      <c r="H236" s="2">
+      <c r="H236" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6095,7 +6069,7 @@
       <c r="C237" t="s">
         <v>104</v>
       </c>
-      <c r="H237" s="2">
+      <c r="H237" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6109,7 +6083,7 @@
       <c r="C238" t="s">
         <v>100</v>
       </c>
-      <c r="H238" s="2">
+      <c r="H238" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6123,7 +6097,7 @@
       <c r="C239" t="s">
         <v>104</v>
       </c>
-      <c r="H239" s="2">
+      <c r="H239" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6137,7 +6111,7 @@
       <c r="C240" t="s">
         <v>104</v>
       </c>
-      <c r="H240" s="2">
+      <c r="H240" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6154,13 +6128,13 @@
       <c r="D241" t="s">
         <v>110</v>
       </c>
-      <c r="E241" s="2">
+      <c r="E241" s="1">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>156</v>
       </c>
-      <c r="H241" s="2">
+      <c r="H241" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6174,7 +6148,7 @@
       <c r="C242" t="s">
         <v>104</v>
       </c>
-      <c r="H242" s="2">
+      <c r="H242" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6191,13 +6165,13 @@
       <c r="D243" t="s">
         <v>141</v>
       </c>
-      <c r="E243" s="2">
+      <c r="E243" s="1">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>168</v>
       </c>
-      <c r="H243" s="2">
+      <c r="H243" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6214,13 +6188,13 @@
       <c r="D244" t="s">
         <v>142</v>
       </c>
-      <c r="E244" s="2">
+      <c r="E244" s="1">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>165</v>
       </c>
-      <c r="H244" s="2">
+      <c r="H244" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6234,7 +6208,7 @@
       <c r="C245" t="s">
         <v>104</v>
       </c>
-      <c r="H245" s="2">
+      <c r="H245" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6248,7 +6222,7 @@
       <c r="C246" t="s">
         <v>100</v>
       </c>
-      <c r="H246" s="2">
+      <c r="H246" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6265,13 +6239,13 @@
       <c r="D247" t="s">
         <v>113</v>
       </c>
-      <c r="E247" s="2">
+      <c r="E247" s="1">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>169</v>
       </c>
-      <c r="H247" s="2">
+      <c r="H247" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6285,7 +6259,7 @@
       <c r="C248" t="s">
         <v>100</v>
       </c>
-      <c r="H248" s="2">
+      <c r="H248" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6299,7 +6273,7 @@
       <c r="C249" t="s">
         <v>100</v>
       </c>
-      <c r="H249" s="2">
+      <c r="H249" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6316,13 +6290,13 @@
       <c r="D250" t="s">
         <v>143</v>
       </c>
-      <c r="E250" s="2">
+      <c r="E250" s="1">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>164</v>
       </c>
-      <c r="H250" s="2">
+      <c r="H250" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6336,7 +6310,7 @@
       <c r="C251" t="s">
         <v>100</v>
       </c>
-      <c r="H251" s="2">
+      <c r="H251" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6353,13 +6327,13 @@
       <c r="D252" t="s">
         <v>144</v>
       </c>
-      <c r="E252" s="2">
+      <c r="E252" s="1">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>166</v>
       </c>
-      <c r="H252" s="2">
+      <c r="H252" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6382,7 +6356,7 @@
       <c r="G253" t="s">
         <v>154</v>
       </c>
-      <c r="H253" s="2">
+      <c r="H253" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6396,7 +6370,7 @@
       <c r="C254" t="s">
         <v>104</v>
       </c>
-      <c r="H254" s="2">
+      <c r="H254" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6410,7 +6384,7 @@
       <c r="C255" t="s">
         <v>100</v>
       </c>
-      <c r="H255" s="2">
+      <c r="H255" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6433,7 +6407,7 @@
       <c r="G256" t="s">
         <v>149</v>
       </c>
-      <c r="H256" s="2">
+      <c r="H256" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6450,7 +6424,7 @@
       <c r="D257" t="s">
         <v>117</v>
       </c>
-      <c r="H257" s="2">
+      <c r="H257" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6473,7 +6447,7 @@
       <c r="G258" t="s">
         <v>150</v>
       </c>
-      <c r="H258" s="2">
+      <c r="H258" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6490,13 +6464,13 @@
       <c r="D259" t="s">
         <v>139</v>
       </c>
-      <c r="E259" s="2">
+      <c r="E259" s="1">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>167</v>
       </c>
-      <c r="H259" s="2">
+      <c r="H259" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6519,7 +6493,7 @@
       <c r="G260" t="s">
         <v>151</v>
       </c>
-      <c r="H260" s="2">
+      <c r="H260" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6542,7 +6516,7 @@
       <c r="G261" t="s">
         <v>151</v>
       </c>
-      <c r="H261" s="2">
+      <c r="H261" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6565,7 +6539,7 @@
       <c r="G262" t="s">
         <v>152</v>
       </c>
-      <c r="H262" s="2">
+      <c r="H262" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6579,7 +6553,7 @@
       <c r="C263" t="s">
         <v>100</v>
       </c>
-      <c r="H263" s="2">
+      <c r="H263" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6596,13 +6570,13 @@
       <c r="D264" t="s">
         <v>140</v>
       </c>
-      <c r="E264" s="2">
+      <c r="E264" s="1">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>162</v>
       </c>
-      <c r="H264" s="2">
+      <c r="H264" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6616,7 +6590,7 @@
       <c r="C265" t="s">
         <v>100</v>
       </c>
-      <c r="H265" s="2">
+      <c r="H265" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6630,7 +6604,7 @@
       <c r="C266" t="s">
         <v>104</v>
       </c>
-      <c r="H266" s="2">
+      <c r="H266" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6644,7 +6618,7 @@
       <c r="C267" t="s">
         <v>100</v>
       </c>
-      <c r="H267" s="2">
+      <c r="H267" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6658,7 +6632,7 @@
       <c r="C268" t="s">
         <v>104</v>
       </c>
-      <c r="H268" s="2">
+      <c r="H268" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6672,7 +6646,7 @@
       <c r="C269" t="s">
         <v>104</v>
       </c>
-      <c r="H269" s="2">
+      <c r="H269" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6689,13 +6663,13 @@
       <c r="D270" t="s">
         <v>110</v>
       </c>
-      <c r="E270" s="2">
+      <c r="E270" s="1">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>156</v>
       </c>
-      <c r="H270" s="2">
+      <c r="H270" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6709,7 +6683,7 @@
       <c r="C271" t="s">
         <v>104</v>
       </c>
-      <c r="H271" s="2">
+      <c r="H271" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6726,13 +6700,13 @@
       <c r="D272" t="s">
         <v>141</v>
       </c>
-      <c r="E272" s="2">
+      <c r="E272" s="1">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>168</v>
       </c>
-      <c r="H272" s="2">
+      <c r="H272" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6749,13 +6723,13 @@
       <c r="D273" t="s">
         <v>142</v>
       </c>
-      <c r="E273" s="2">
+      <c r="E273" s="1">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>170</v>
       </c>
-      <c r="H273" s="2">
+      <c r="H273" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6769,7 +6743,7 @@
       <c r="C274" t="s">
         <v>100</v>
       </c>
-      <c r="H274" s="2">
+      <c r="H274" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6783,7 +6757,7 @@
       <c r="C275" t="s">
         <v>100</v>
       </c>
-      <c r="H275" s="2">
+      <c r="H275" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6800,13 +6774,13 @@
       <c r="D276" t="s">
         <v>113</v>
       </c>
-      <c r="E276" s="2">
+      <c r="E276" s="1">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>169</v>
       </c>
-      <c r="H276" s="2">
+      <c r="H276" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6820,7 +6794,7 @@
       <c r="C277" t="s">
         <v>100</v>
       </c>
-      <c r="H277" s="2">
+      <c r="H277" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6837,13 +6811,13 @@
       <c r="D278" t="s">
         <v>145</v>
       </c>
-      <c r="E278" s="2">
+      <c r="E278" s="1">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>171</v>
       </c>
-      <c r="H278" s="2">
+      <c r="H278" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6860,13 +6834,13 @@
       <c r="D279" t="s">
         <v>143</v>
       </c>
-      <c r="E279" s="2">
+      <c r="E279" s="1">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>170</v>
       </c>
-      <c r="H279" s="2">
+      <c r="H279" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6880,7 +6854,7 @@
       <c r="C280" t="s">
         <v>100</v>
       </c>
-      <c r="H280" s="2">
+      <c r="H280" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6897,13 +6871,13 @@
       <c r="D281" t="s">
         <v>146</v>
       </c>
-      <c r="E281" s="2">
+      <c r="E281" s="1">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>166</v>
       </c>
-      <c r="H281" s="2">
+      <c r="H281" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6926,7 +6900,7 @@
       <c r="G282" t="s">
         <v>154</v>
       </c>
-      <c r="H282" s="2">
+      <c r="H282" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6940,7 +6914,7 @@
       <c r="C283" t="s">
         <v>104</v>
       </c>
-      <c r="H283" s="2">
+      <c r="H283" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6954,7 +6928,7 @@
       <c r="C284" t="s">
         <v>100</v>
       </c>
-      <c r="H284" s="2">
+      <c r="H284" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6977,7 +6951,7 @@
       <c r="G285" t="s">
         <v>149</v>
       </c>
-      <c r="H285" s="2">
+      <c r="H285" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6994,7 +6968,7 @@
       <c r="D286" t="s">
         <v>117</v>
       </c>
-      <c r="H286" s="2">
+      <c r="H286" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7017,7 +6991,7 @@
       <c r="G287" t="s">
         <v>150</v>
       </c>
-      <c r="H287" s="2">
+      <c r="H287" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7034,13 +7008,13 @@
       <c r="D288" t="s">
         <v>139</v>
       </c>
-      <c r="E288" s="2">
+      <c r="E288" s="1">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>167</v>
       </c>
-      <c r="H288" s="2">
+      <c r="H288" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7063,7 +7037,7 @@
       <c r="G289" t="s">
         <v>151</v>
       </c>
-      <c r="H289" s="2">
+      <c r="H289" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7086,7 +7060,7 @@
       <c r="G290" t="s">
         <v>151</v>
       </c>
-      <c r="H290" s="2">
+      <c r="H290" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7109,7 +7083,7 @@
       <c r="G291" t="s">
         <v>152</v>
       </c>
-      <c r="H291" s="2">
+      <c r="H291" s="1">
         <v>46218</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (21/07/2026 16:07)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -612,16 +612,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -637,7 +629,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -645,30 +637,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -968,72 +942,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1098,7 +1072,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1163,7 +1137,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1228,7 +1202,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1293,7 +1267,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1358,7 +1332,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1423,7 +1397,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1488,7 +1462,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1553,7 +1527,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1618,7 +1592,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1683,7 +1657,7 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>46220</v>
       </c>
       <c r="B12">
@@ -1748,7 +1722,7 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46224</v>
       </c>
       <c r="B13">
@@ -1823,28 +1797,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1858,7 +1832,7 @@
       <c r="C2" t="s">
         <v>107</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1872,7 +1846,7 @@
       <c r="C3" t="s">
         <v>107</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1895,7 +1869,7 @@
       <c r="G4" t="s">
         <v>164</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1909,7 +1883,7 @@
       <c r="C5" t="s">
         <v>107</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1923,7 +1897,7 @@
       <c r="C6" t="s">
         <v>107</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1940,13 +1914,13 @@
       <c r="D7" t="s">
         <v>115</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>179</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1963,13 +1937,13 @@
       <c r="D8" t="s">
         <v>116</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>179</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1986,13 +1960,13 @@
       <c r="D9" t="s">
         <v>117</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>180</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2009,13 +1983,13 @@
       <c r="D10" t="s">
         <v>118</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>181</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2029,7 +2003,7 @@
       <c r="C11" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2043,7 +2017,7 @@
       <c r="C12" t="s">
         <v>107</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2060,13 +2034,13 @@
       <c r="D13" t="s">
         <v>119</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>179</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2080,7 +2054,7 @@
       <c r="C14" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2097,13 +2071,13 @@
       <c r="D15" t="s">
         <v>120</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>182</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2117,7 +2091,7 @@
       <c r="C16" t="s">
         <v>107</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2131,7 +2105,7 @@
       <c r="C17" t="s">
         <v>107</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2148,13 +2122,13 @@
       <c r="D18" t="s">
         <v>121</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>183</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2168,7 +2142,7 @@
       <c r="C19" t="s">
         <v>107</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2185,13 +2159,13 @@
       <c r="D20" t="s">
         <v>122</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>179</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2214,7 +2188,7 @@
       <c r="G21" t="s">
         <v>165</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2228,7 +2202,7 @@
       <c r="C22" t="s">
         <v>111</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2242,7 +2216,7 @@
       <c r="C23" t="s">
         <v>107</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2265,7 +2239,7 @@
       <c r="G24" t="s">
         <v>166</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2282,7 +2256,7 @@
       <c r="D25" t="s">
         <v>124</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2305,7 +2279,7 @@
       <c r="G26" t="s">
         <v>167</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2322,13 +2296,13 @@
       <c r="D27" t="s">
         <v>126</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>184</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2351,7 +2325,7 @@
       <c r="G28" t="s">
         <v>168</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2374,7 +2348,7 @@
       <c r="G29" t="s">
         <v>168</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2397,7 +2371,7 @@
       <c r="G30" t="s">
         <v>169</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2411,7 +2385,7 @@
       <c r="C31" t="s">
         <v>107</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2425,7 +2399,7 @@
       <c r="C32" t="s">
         <v>107</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2448,7 +2422,7 @@
       <c r="G33" t="s">
         <v>170</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2462,7 +2436,7 @@
       <c r="C34" t="s">
         <v>107</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2476,7 +2450,7 @@
       <c r="C35" t="s">
         <v>107</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2493,13 +2467,13 @@
       <c r="D36" t="s">
         <v>115</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>179</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2516,13 +2490,13 @@
       <c r="D37" t="s">
         <v>116</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>179</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2539,13 +2513,13 @@
       <c r="D38" t="s">
         <v>117</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>180</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2562,13 +2536,13 @@
       <c r="D39" t="s">
         <v>118</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2582,7 +2556,7 @@
       <c r="C40" t="s">
         <v>107</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2596,7 +2570,7 @@
       <c r="C41" t="s">
         <v>107</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2613,13 +2587,13 @@
       <c r="D42" t="s">
         <v>119</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>179</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2633,7 +2607,7 @@
       <c r="C43" t="s">
         <v>107</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2650,13 +2624,13 @@
       <c r="D44" t="s">
         <v>120</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>182</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2670,7 +2644,7 @@
       <c r="C45" t="s">
         <v>107</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2684,7 +2658,7 @@
       <c r="C46" t="s">
         <v>107</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2698,7 +2672,7 @@
       <c r="C47" t="s">
         <v>111</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2712,7 +2686,7 @@
       <c r="C48" t="s">
         <v>107</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2729,13 +2703,13 @@
       <c r="D49" t="s">
         <v>131</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>179</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2758,7 +2732,7 @@
       <c r="G50" t="s">
         <v>165</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2772,7 +2746,7 @@
       <c r="C51" t="s">
         <v>111</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2786,7 +2760,7 @@
       <c r="C52" t="s">
         <v>107</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2809,7 +2783,7 @@
       <c r="G53" t="s">
         <v>166</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2826,7 +2800,7 @@
       <c r="D54" t="s">
         <v>124</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2849,7 +2823,7 @@
       <c r="G55" t="s">
         <v>167</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2866,13 +2840,13 @@
       <c r="D56" t="s">
         <v>126</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>184</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2895,7 +2869,7 @@
       <c r="G57" t="s">
         <v>168</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2918,7 +2892,7 @@
       <c r="G58" t="s">
         <v>168</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2941,7 +2915,7 @@
       <c r="G59" t="s">
         <v>169</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2955,7 +2929,7 @@
       <c r="C60" t="s">
         <v>107</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2969,7 +2943,7 @@
       <c r="C61" t="s">
         <v>107</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2986,13 +2960,13 @@
       <c r="D62" t="s">
         <v>130</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>185</v>
       </c>
-      <c r="H62" s="2">
+      <c r="H62" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3006,7 +2980,7 @@
       <c r="C63" t="s">
         <v>107</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3023,13 +2997,13 @@
       <c r="D64" t="s">
         <v>132</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>186</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3043,7 +3017,7 @@
       <c r="C65" t="s">
         <v>107</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3057,7 +3031,7 @@
       <c r="C66" t="s">
         <v>111</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3074,13 +3048,13 @@
       <c r="D67" t="s">
         <v>117</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>180</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3097,13 +3071,13 @@
       <c r="D68" t="s">
         <v>118</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>181</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3117,7 +3091,7 @@
       <c r="C69" t="s">
         <v>107</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3131,7 +3105,7 @@
       <c r="C70" t="s">
         <v>107</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3148,13 +3122,13 @@
       <c r="D71" t="s">
         <v>119</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>185</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3168,7 +3142,7 @@
       <c r="C72" t="s">
         <v>107</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3185,13 +3159,13 @@
       <c r="D73" t="s">
         <v>120</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>182</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3205,7 +3179,7 @@
       <c r="C74" t="s">
         <v>107</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3219,7 +3193,7 @@
       <c r="C75" t="s">
         <v>107</v>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3233,7 +3207,7 @@
       <c r="C76" t="s">
         <v>107</v>
       </c>
-      <c r="H76" s="2">
+      <c r="H76" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3247,7 +3221,7 @@
       <c r="C77" t="s">
         <v>107</v>
       </c>
-      <c r="H77" s="2">
+      <c r="H77" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3264,13 +3238,13 @@
       <c r="D78" t="s">
         <v>131</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="1">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>185</v>
       </c>
-      <c r="H78" s="2">
+      <c r="H78" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3293,7 +3267,7 @@
       <c r="G79" t="s">
         <v>171</v>
       </c>
-      <c r="H79" s="2">
+      <c r="H79" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3307,7 +3281,7 @@
       <c r="C80" t="s">
         <v>111</v>
       </c>
-      <c r="H80" s="2">
+      <c r="H80" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3321,7 +3295,7 @@
       <c r="C81" t="s">
         <v>107</v>
       </c>
-      <c r="H81" s="2">
+      <c r="H81" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3344,7 +3318,7 @@
       <c r="G82" t="s">
         <v>166</v>
       </c>
-      <c r="H82" s="2">
+      <c r="H82" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3361,7 +3335,7 @@
       <c r="D83" t="s">
         <v>124</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3384,7 +3358,7 @@
       <c r="G84" t="s">
         <v>167</v>
       </c>
-      <c r="H84" s="2">
+      <c r="H84" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3401,13 +3375,13 @@
       <c r="D85" t="s">
         <v>126</v>
       </c>
-      <c r="E85" s="2">
+      <c r="E85" s="1">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>184</v>
       </c>
-      <c r="H85" s="2">
+      <c r="H85" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3430,7 +3404,7 @@
       <c r="G86" t="s">
         <v>168</v>
       </c>
-      <c r="H86" s="2">
+      <c r="H86" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3453,7 +3427,7 @@
       <c r="G87" t="s">
         <v>168</v>
       </c>
-      <c r="H87" s="2">
+      <c r="H87" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3476,7 +3450,7 @@
       <c r="G88" t="s">
         <v>169</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3490,7 +3464,7 @@
       <c r="C89" t="s">
         <v>107</v>
       </c>
-      <c r="H89" s="2">
+      <c r="H89" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3507,13 +3481,13 @@
       <c r="D90" t="s">
         <v>134</v>
       </c>
-      <c r="E90" s="2">
+      <c r="E90" s="1">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>186</v>
       </c>
-      <c r="H90" s="2">
+      <c r="H90" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3530,13 +3504,13 @@
       <c r="D91" t="s">
         <v>130</v>
       </c>
-      <c r="E91" s="2">
+      <c r="E91" s="1">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>185</v>
       </c>
-      <c r="H91" s="2">
+      <c r="H91" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3550,7 +3524,7 @@
       <c r="C92" t="s">
         <v>107</v>
       </c>
-      <c r="H92" s="2">
+      <c r="H92" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3567,13 +3541,13 @@
       <c r="D93" t="s">
         <v>132</v>
       </c>
-      <c r="E93" s="2">
+      <c r="E93" s="1">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>186</v>
       </c>
-      <c r="H93" s="2">
+      <c r="H93" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3587,7 +3561,7 @@
       <c r="C94" t="s">
         <v>107</v>
       </c>
-      <c r="H94" s="2">
+      <c r="H94" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3601,7 +3575,7 @@
       <c r="C95" t="s">
         <v>111</v>
       </c>
-      <c r="H95" s="2">
+      <c r="H95" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3618,13 +3592,13 @@
       <c r="D96" t="s">
         <v>117</v>
       </c>
-      <c r="E96" s="2">
+      <c r="E96" s="1">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>180</v>
       </c>
-      <c r="H96" s="2">
+      <c r="H96" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3641,13 +3615,13 @@
       <c r="D97" t="s">
         <v>118</v>
       </c>
-      <c r="E97" s="2">
+      <c r="E97" s="1">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>181</v>
       </c>
-      <c r="H97" s="2">
+      <c r="H97" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3661,7 +3635,7 @@
       <c r="C98" t="s">
         <v>107</v>
       </c>
-      <c r="H98" s="2">
+      <c r="H98" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3678,13 +3652,13 @@
       <c r="D99" t="s">
         <v>135</v>
       </c>
-      <c r="E99" s="2">
+      <c r="E99" s="1">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>181</v>
       </c>
-      <c r="H99" s="2">
+      <c r="H99" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3701,13 +3675,13 @@
       <c r="D100" t="s">
         <v>119</v>
       </c>
-      <c r="E100" s="2">
+      <c r="E100" s="1">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>181</v>
       </c>
-      <c r="H100" s="2">
+      <c r="H100" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3721,7 +3695,7 @@
       <c r="C101" t="s">
         <v>107</v>
       </c>
-      <c r="H101" s="2">
+      <c r="H101" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3738,13 +3712,13 @@
       <c r="D102" t="s">
         <v>120</v>
       </c>
-      <c r="E102" s="2">
+      <c r="E102" s="1">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>182</v>
       </c>
-      <c r="H102" s="2">
+      <c r="H102" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3761,13 +3735,13 @@
       <c r="D103" t="s">
         <v>136</v>
       </c>
-      <c r="E103" s="2">
+      <c r="E103" s="1">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>181</v>
       </c>
-      <c r="H103" s="2">
+      <c r="H103" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3781,7 +3755,7 @@
       <c r="C104" t="s">
         <v>107</v>
       </c>
-      <c r="H104" s="2">
+      <c r="H104" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3795,7 +3769,7 @@
       <c r="C105" t="s">
         <v>107</v>
       </c>
-      <c r="H105" s="2">
+      <c r="H105" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3809,7 +3783,7 @@
       <c r="C106" t="s">
         <v>107</v>
       </c>
-      <c r="H106" s="2">
+      <c r="H106" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3826,13 +3800,13 @@
       <c r="D107" t="s">
         <v>137</v>
       </c>
-      <c r="E107" s="2">
+      <c r="E107" s="1">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>181</v>
       </c>
-      <c r="H107" s="2">
+      <c r="H107" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3855,7 +3829,7 @@
       <c r="G108" t="s">
         <v>171</v>
       </c>
-      <c r="H108" s="2">
+      <c r="H108" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3869,7 +3843,7 @@
       <c r="C109" t="s">
         <v>111</v>
       </c>
-      <c r="H109" s="2">
+      <c r="H109" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3883,7 +3857,7 @@
       <c r="C110" t="s">
         <v>107</v>
       </c>
-      <c r="H110" s="2">
+      <c r="H110" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3906,7 +3880,7 @@
       <c r="G111" t="s">
         <v>166</v>
       </c>
-      <c r="H111" s="2">
+      <c r="H111" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3923,7 +3897,7 @@
       <c r="D112" t="s">
         <v>124</v>
       </c>
-      <c r="H112" s="2">
+      <c r="H112" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3946,7 +3920,7 @@
       <c r="G113" t="s">
         <v>167</v>
       </c>
-      <c r="H113" s="2">
+      <c r="H113" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3963,13 +3937,13 @@
       <c r="D114" t="s">
         <v>126</v>
       </c>
-      <c r="E114" s="2">
+      <c r="E114" s="1">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>184</v>
       </c>
-      <c r="H114" s="2">
+      <c r="H114" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3992,7 +3966,7 @@
       <c r="G115" t="s">
         <v>168</v>
       </c>
-      <c r="H115" s="2">
+      <c r="H115" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4015,7 +3989,7 @@
       <c r="G116" t="s">
         <v>168</v>
       </c>
-      <c r="H116" s="2">
+      <c r="H116" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4038,7 +4012,7 @@
       <c r="G117" t="s">
         <v>169</v>
       </c>
-      <c r="H117" s="2">
+      <c r="H117" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4052,7 +4026,7 @@
       <c r="C118" t="s">
         <v>107</v>
       </c>
-      <c r="H118" s="2">
+      <c r="H118" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4069,13 +4043,13 @@
       <c r="D119" t="s">
         <v>134</v>
       </c>
-      <c r="E119" s="2">
+      <c r="E119" s="1">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>186</v>
       </c>
-      <c r="H119" s="2">
+      <c r="H119" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4089,7 +4063,7 @@
       <c r="C120" t="s">
         <v>111</v>
       </c>
-      <c r="H120" s="2">
+      <c r="H120" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4103,7 +4077,7 @@
       <c r="C121" t="s">
         <v>107</v>
       </c>
-      <c r="H121" s="2">
+      <c r="H121" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4117,7 +4091,7 @@
       <c r="C122" t="s">
         <v>111</v>
       </c>
-      <c r="H122" s="2">
+      <c r="H122" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4131,7 +4105,7 @@
       <c r="C123" t="s">
         <v>111</v>
       </c>
-      <c r="H123" s="2">
+      <c r="H123" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4145,7 +4119,7 @@
       <c r="C124" t="s">
         <v>111</v>
       </c>
-      <c r="H124" s="2">
+      <c r="H124" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4162,13 +4136,13 @@
       <c r="D125" t="s">
         <v>117</v>
       </c>
-      <c r="E125" s="2">
+      <c r="E125" s="1">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>180</v>
       </c>
-      <c r="H125" s="2">
+      <c r="H125" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4185,13 +4159,13 @@
       <c r="D126" t="s">
         <v>118</v>
       </c>
-      <c r="E126" s="2">
+      <c r="E126" s="1">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>181</v>
       </c>
-      <c r="H126" s="2">
+      <c r="H126" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4205,7 +4179,7 @@
       <c r="C127" t="s">
         <v>107</v>
       </c>
-      <c r="H127" s="2">
+      <c r="H127" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4222,13 +4196,13 @@
       <c r="D128" t="s">
         <v>135</v>
       </c>
-      <c r="E128" s="2">
+      <c r="E128" s="1">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>181</v>
       </c>
-      <c r="H128" s="2">
+      <c r="H128" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4245,13 +4219,13 @@
       <c r="D129" t="s">
         <v>119</v>
       </c>
-      <c r="E129" s="2">
+      <c r="E129" s="1">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>181</v>
       </c>
-      <c r="H129" s="2">
+      <c r="H129" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4265,7 +4239,7 @@
       <c r="C130" t="s">
         <v>107</v>
       </c>
-      <c r="H130" s="2">
+      <c r="H130" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4282,13 +4256,13 @@
       <c r="D131" t="s">
         <v>120</v>
       </c>
-      <c r="E131" s="2">
+      <c r="E131" s="1">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>182</v>
       </c>
-      <c r="H131" s="2">
+      <c r="H131" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4305,13 +4279,13 @@
       <c r="D132" t="s">
         <v>136</v>
       </c>
-      <c r="E132" s="2">
+      <c r="E132" s="1">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>181</v>
       </c>
-      <c r="H132" s="2">
+      <c r="H132" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4325,7 +4299,7 @@
       <c r="C133" t="s">
         <v>107</v>
       </c>
-      <c r="H133" s="2">
+      <c r="H133" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4339,7 +4313,7 @@
       <c r="C134" t="s">
         <v>107</v>
       </c>
-      <c r="H134" s="2">
+      <c r="H134" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4353,7 +4327,7 @@
       <c r="C135" t="s">
         <v>107</v>
       </c>
-      <c r="H135" s="2">
+      <c r="H135" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4370,13 +4344,13 @@
       <c r="D136" t="s">
         <v>138</v>
       </c>
-      <c r="E136" s="2">
+      <c r="E136" s="1">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>181</v>
       </c>
-      <c r="H136" s="2">
+      <c r="H136" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4399,7 +4373,7 @@
       <c r="G137" t="s">
         <v>171</v>
       </c>
-      <c r="H137" s="2">
+      <c r="H137" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4413,7 +4387,7 @@
       <c r="C138" t="s">
         <v>111</v>
       </c>
-      <c r="H138" s="2">
+      <c r="H138" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4427,7 +4401,7 @@
       <c r="C139" t="s">
         <v>107</v>
       </c>
-      <c r="H139" s="2">
+      <c r="H139" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4450,7 +4424,7 @@
       <c r="G140" t="s">
         <v>166</v>
       </c>
-      <c r="H140" s="2">
+      <c r="H140" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4467,7 +4441,7 @@
       <c r="D141" t="s">
         <v>124</v>
       </c>
-      <c r="H141" s="2">
+      <c r="H141" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="G142" t="s">
         <v>167</v>
       </c>
-      <c r="H142" s="2">
+      <c r="H142" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4507,13 +4481,13 @@
       <c r="D143" t="s">
         <v>126</v>
       </c>
-      <c r="E143" s="2">
+      <c r="E143" s="1">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>184</v>
       </c>
-      <c r="H143" s="2">
+      <c r="H143" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4536,7 +4510,7 @@
       <c r="G144" t="s">
         <v>168</v>
       </c>
-      <c r="H144" s="2">
+      <c r="H144" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4559,7 +4533,7 @@
       <c r="G145" t="s">
         <v>168</v>
       </c>
-      <c r="H145" s="2">
+      <c r="H145" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4582,7 +4556,7 @@
       <c r="G146" t="s">
         <v>169</v>
       </c>
-      <c r="H146" s="2">
+      <c r="H146" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4596,7 +4570,7 @@
       <c r="C147" t="s">
         <v>107</v>
       </c>
-      <c r="H147" s="2">
+      <c r="H147" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4613,13 +4587,13 @@
       <c r="D148" t="s">
         <v>134</v>
       </c>
-      <c r="E148" s="2">
+      <c r="E148" s="1">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>186</v>
       </c>
-      <c r="H148" s="2">
+      <c r="H148" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4633,7 +4607,7 @@
       <c r="C149" t="s">
         <v>111</v>
       </c>
-      <c r="H149" s="2">
+      <c r="H149" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4647,7 +4621,7 @@
       <c r="C150" t="s">
         <v>107</v>
       </c>
-      <c r="H150" s="2">
+      <c r="H150" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4661,7 +4635,7 @@
       <c r="C151" t="s">
         <v>107</v>
       </c>
-      <c r="H151" s="2">
+      <c r="H151" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4675,7 +4649,7 @@
       <c r="C152" t="s">
         <v>111</v>
       </c>
-      <c r="H152" s="2">
+      <c r="H152" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4689,7 +4663,7 @@
       <c r="C153" t="s">
         <v>111</v>
       </c>
-      <c r="H153" s="2">
+      <c r="H153" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4706,13 +4680,13 @@
       <c r="D154" t="s">
         <v>117</v>
       </c>
-      <c r="E154" s="2">
+      <c r="E154" s="1">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>180</v>
       </c>
-      <c r="H154" s="2">
+      <c r="H154" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4729,13 +4703,13 @@
       <c r="D155" t="s">
         <v>118</v>
       </c>
-      <c r="E155" s="2">
+      <c r="E155" s="1">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>181</v>
       </c>
-      <c r="H155" s="2">
+      <c r="H155" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4749,7 +4723,7 @@
       <c r="C156" t="s">
         <v>107</v>
       </c>
-      <c r="H156" s="2">
+      <c r="H156" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4766,13 +4740,13 @@
       <c r="D157" t="s">
         <v>135</v>
       </c>
-      <c r="E157" s="2">
+      <c r="E157" s="1">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>181</v>
       </c>
-      <c r="H157" s="2">
+      <c r="H157" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4789,13 +4763,13 @@
       <c r="D158" t="s">
         <v>119</v>
       </c>
-      <c r="E158" s="2">
+      <c r="E158" s="1">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>181</v>
       </c>
-      <c r="H158" s="2">
+      <c r="H158" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4812,13 +4786,13 @@
       <c r="D159" t="s">
         <v>139</v>
       </c>
-      <c r="E159" s="2">
+      <c r="E159" s="1">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>187</v>
       </c>
-      <c r="H159" s="2">
+      <c r="H159" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4835,13 +4809,13 @@
       <c r="D160" t="s">
         <v>120</v>
       </c>
-      <c r="E160" s="2">
+      <c r="E160" s="1">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>182</v>
       </c>
-      <c r="H160" s="2">
+      <c r="H160" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4858,13 +4832,13 @@
       <c r="D161" t="s">
         <v>136</v>
       </c>
-      <c r="E161" s="2">
+      <c r="E161" s="1">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>181</v>
       </c>
-      <c r="H161" s="2">
+      <c r="H161" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4878,7 +4852,7 @@
       <c r="C162" t="s">
         <v>107</v>
       </c>
-      <c r="H162" s="2">
+      <c r="H162" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4892,7 +4866,7 @@
       <c r="C163" t="s">
         <v>107</v>
       </c>
-      <c r="H163" s="2">
+      <c r="H163" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4906,7 +4880,7 @@
       <c r="C164" t="s">
         <v>107</v>
       </c>
-      <c r="H164" s="2">
+      <c r="H164" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4923,13 +4897,13 @@
       <c r="D165" t="s">
         <v>138</v>
       </c>
-      <c r="E165" s="2">
+      <c r="E165" s="1">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>181</v>
       </c>
-      <c r="H165" s="2">
+      <c r="H165" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4952,7 +4926,7 @@
       <c r="G166" t="s">
         <v>171</v>
       </c>
-      <c r="H166" s="2">
+      <c r="H166" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4966,7 +4940,7 @@
       <c r="C167" t="s">
         <v>111</v>
       </c>
-      <c r="H167" s="2">
+      <c r="H167" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4980,7 +4954,7 @@
       <c r="C168" t="s">
         <v>107</v>
       </c>
-      <c r="H168" s="2">
+      <c r="H168" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5003,7 +4977,7 @@
       <c r="G169" t="s">
         <v>166</v>
       </c>
-      <c r="H169" s="2">
+      <c r="H169" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5020,7 +4994,7 @@
       <c r="D170" t="s">
         <v>124</v>
       </c>
-      <c r="H170" s="2">
+      <c r="H170" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5043,7 +5017,7 @@
       <c r="G171" t="s">
         <v>167</v>
       </c>
-      <c r="H171" s="2">
+      <c r="H171" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5060,13 +5034,13 @@
       <c r="D172" t="s">
         <v>126</v>
       </c>
-      <c r="E172" s="2">
+      <c r="E172" s="1">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>184</v>
       </c>
-      <c r="H172" s="2">
+      <c r="H172" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5089,7 +5063,7 @@
       <c r="G173" t="s">
         <v>168</v>
       </c>
-      <c r="H173" s="2">
+      <c r="H173" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5112,7 +5086,7 @@
       <c r="G174" t="s">
         <v>168</v>
       </c>
-      <c r="H174" s="2">
+      <c r="H174" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5135,7 +5109,7 @@
       <c r="G175" t="s">
         <v>169</v>
       </c>
-      <c r="H175" s="2">
+      <c r="H175" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5149,7 +5123,7 @@
       <c r="C176" t="s">
         <v>107</v>
       </c>
-      <c r="H176" s="2">
+      <c r="H176" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5166,13 +5140,13 @@
       <c r="D177" t="s">
         <v>140</v>
       </c>
-      <c r="E177" s="2">
+      <c r="E177" s="1">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>186</v>
       </c>
-      <c r="H177" s="2">
+      <c r="H177" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5186,7 +5160,7 @@
       <c r="C178" t="s">
         <v>107</v>
       </c>
-      <c r="H178" s="2">
+      <c r="H178" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5203,13 +5177,13 @@
       <c r="D179" t="s">
         <v>141</v>
       </c>
-      <c r="E179" s="2">
+      <c r="E179" s="1">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>182</v>
       </c>
-      <c r="H179" s="2">
+      <c r="H179" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5223,7 +5197,7 @@
       <c r="C180" t="s">
         <v>107</v>
       </c>
-      <c r="H180" s="2">
+      <c r="H180" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5237,7 +5211,7 @@
       <c r="C181" t="s">
         <v>111</v>
       </c>
-      <c r="H181" s="2">
+      <c r="H181" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5251,7 +5225,7 @@
       <c r="C182" t="s">
         <v>111</v>
       </c>
-      <c r="H182" s="2">
+      <c r="H182" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5268,13 +5242,13 @@
       <c r="D183" t="s">
         <v>117</v>
       </c>
-      <c r="E183" s="2">
+      <c r="E183" s="1">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>180</v>
       </c>
-      <c r="H183" s="2">
+      <c r="H183" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5291,13 +5265,13 @@
       <c r="D184" t="s">
         <v>118</v>
       </c>
-      <c r="E184" s="2">
+      <c r="E184" s="1">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>181</v>
       </c>
-      <c r="H184" s="2">
+      <c r="H184" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5311,7 +5285,7 @@
       <c r="C185" t="s">
         <v>107</v>
       </c>
-      <c r="H185" s="2">
+      <c r="H185" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5328,13 +5302,13 @@
       <c r="D186" t="s">
         <v>135</v>
       </c>
-      <c r="E186" s="2">
+      <c r="E186" s="1">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>181</v>
       </c>
-      <c r="H186" s="2">
+      <c r="H186" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5351,13 +5325,13 @@
       <c r="D187" t="s">
         <v>142</v>
       </c>
-      <c r="E187" s="2">
+      <c r="E187" s="1">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>181</v>
       </c>
-      <c r="H187" s="2">
+      <c r="H187" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5374,13 +5348,13 @@
       <c r="D188" t="s">
         <v>143</v>
       </c>
-      <c r="E188" s="2">
+      <c r="E188" s="1">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>181</v>
       </c>
-      <c r="H188" s="2">
+      <c r="H188" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5397,13 +5371,13 @@
       <c r="D189" t="s">
         <v>120</v>
       </c>
-      <c r="E189" s="2">
+      <c r="E189" s="1">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>182</v>
       </c>
-      <c r="H189" s="2">
+      <c r="H189" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5420,13 +5394,13 @@
       <c r="D190" t="s">
         <v>136</v>
       </c>
-      <c r="E190" s="2">
+      <c r="E190" s="1">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>181</v>
       </c>
-      <c r="H190" s="2">
+      <c r="H190" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5440,7 +5414,7 @@
       <c r="C191" t="s">
         <v>107</v>
       </c>
-      <c r="H191" s="2">
+      <c r="H191" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5454,7 +5428,7 @@
       <c r="C192" t="s">
         <v>107</v>
       </c>
-      <c r="H192" s="2">
+      <c r="H192" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5468,7 +5442,7 @@
       <c r="C193" t="s">
         <v>107</v>
       </c>
-      <c r="H193" s="2">
+      <c r="H193" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5485,13 +5459,13 @@
       <c r="D194" t="s">
         <v>138</v>
       </c>
-      <c r="E194" s="2">
+      <c r="E194" s="1">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>188</v>
       </c>
-      <c r="H194" s="2">
+      <c r="H194" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5514,7 +5488,7 @@
       <c r="G195" t="s">
         <v>171</v>
       </c>
-      <c r="H195" s="2">
+      <c r="H195" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5528,7 +5502,7 @@
       <c r="C196" t="s">
         <v>111</v>
       </c>
-      <c r="H196" s="2">
+      <c r="H196" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5542,7 +5516,7 @@
       <c r="C197" t="s">
         <v>107</v>
       </c>
-      <c r="H197" s="2">
+      <c r="H197" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5565,7 +5539,7 @@
       <c r="G198" t="s">
         <v>166</v>
       </c>
-      <c r="H198" s="2">
+      <c r="H198" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5582,7 +5556,7 @@
       <c r="D199" t="s">
         <v>124</v>
       </c>
-      <c r="H199" s="2">
+      <c r="H199" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5605,7 +5579,7 @@
       <c r="G200" t="s">
         <v>167</v>
       </c>
-      <c r="H200" s="2">
+      <c r="H200" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5622,13 +5596,13 @@
       <c r="D201" t="s">
         <v>126</v>
       </c>
-      <c r="E201" s="2">
+      <c r="E201" s="1">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>184</v>
       </c>
-      <c r="H201" s="2">
+      <c r="H201" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5651,7 +5625,7 @@
       <c r="G202" t="s">
         <v>168</v>
       </c>
-      <c r="H202" s="2">
+      <c r="H202" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5674,7 +5648,7 @@
       <c r="G203" t="s">
         <v>168</v>
       </c>
-      <c r="H203" s="2">
+      <c r="H203" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5697,7 +5671,7 @@
       <c r="G204" t="s">
         <v>169</v>
       </c>
-      <c r="H204" s="2">
+      <c r="H204" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5711,7 +5685,7 @@
       <c r="C205" t="s">
         <v>107</v>
       </c>
-      <c r="H205" s="2">
+      <c r="H205" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5728,13 +5702,13 @@
       <c r="D206" t="s">
         <v>140</v>
       </c>
-      <c r="E206" s="2">
+      <c r="E206" s="1">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>186</v>
       </c>
-      <c r="H206" s="2">
+      <c r="H206" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5748,7 +5722,7 @@
       <c r="C207" t="s">
         <v>107</v>
       </c>
-      <c r="H207" s="2">
+      <c r="H207" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5762,7 +5736,7 @@
       <c r="C208" t="s">
         <v>111</v>
       </c>
-      <c r="H208" s="2">
+      <c r="H208" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5776,7 +5750,7 @@
       <c r="C209" t="s">
         <v>107</v>
       </c>
-      <c r="H209" s="2">
+      <c r="H209" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5790,7 +5764,7 @@
       <c r="C210" t="s">
         <v>111</v>
       </c>
-      <c r="H210" s="2">
+      <c r="H210" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5804,7 +5778,7 @@
       <c r="C211" t="s">
         <v>111</v>
       </c>
-      <c r="H211" s="2">
+      <c r="H211" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5821,13 +5795,13 @@
       <c r="D212" t="s">
         <v>117</v>
       </c>
-      <c r="E212" s="2">
+      <c r="E212" s="1">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>180</v>
       </c>
-      <c r="H212" s="2">
+      <c r="H212" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5841,7 +5815,7 @@
       <c r="C213" t="s">
         <v>111</v>
       </c>
-      <c r="H213" s="2">
+      <c r="H213" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5855,7 +5829,7 @@
       <c r="C214" t="s">
         <v>107</v>
       </c>
-      <c r="H214" s="2">
+      <c r="H214" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5872,13 +5846,13 @@
       <c r="D215" t="s">
         <v>135</v>
       </c>
-      <c r="E215" s="2">
+      <c r="E215" s="1">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>189</v>
       </c>
-      <c r="H215" s="2">
+      <c r="H215" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5895,13 +5869,13 @@
       <c r="D216" t="s">
         <v>142</v>
       </c>
-      <c r="E216" s="2">
+      <c r="E216" s="1">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>182</v>
       </c>
-      <c r="H216" s="2">
+      <c r="H216" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5915,7 +5889,7 @@
       <c r="C217" t="s">
         <v>107</v>
       </c>
-      <c r="H217" s="2">
+      <c r="H217" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5932,13 +5906,13 @@
       <c r="D218" t="s">
         <v>120</v>
       </c>
-      <c r="E218" s="2">
+      <c r="E218" s="1">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>182</v>
       </c>
-      <c r="H218" s="2">
+      <c r="H218" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5952,7 +5926,7 @@
       <c r="C219" t="s">
         <v>107</v>
       </c>
-      <c r="H219" s="2">
+      <c r="H219" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5966,7 +5940,7 @@
       <c r="C220" t="s">
         <v>107</v>
       </c>
-      <c r="H220" s="2">
+      <c r="H220" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5983,13 +5957,13 @@
       <c r="D221" t="s">
         <v>144</v>
       </c>
-      <c r="E221" s="2">
+      <c r="E221" s="1">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>186</v>
       </c>
-      <c r="H221" s="2">
+      <c r="H221" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6003,7 +5977,7 @@
       <c r="C222" t="s">
         <v>107</v>
       </c>
-      <c r="H222" s="2">
+      <c r="H222" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6020,13 +5994,13 @@
       <c r="D223" t="s">
         <v>145</v>
       </c>
-      <c r="E223" s="2">
+      <c r="E223" s="1">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>190</v>
       </c>
-      <c r="H223" s="2">
+      <c r="H223" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6049,7 +6023,7 @@
       <c r="G224" t="s">
         <v>171</v>
       </c>
-      <c r="H224" s="2">
+      <c r="H224" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6063,7 +6037,7 @@
       <c r="C225" t="s">
         <v>111</v>
       </c>
-      <c r="H225" s="2">
+      <c r="H225" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6077,7 +6051,7 @@
       <c r="C226" t="s">
         <v>107</v>
       </c>
-      <c r="H226" s="2">
+      <c r="H226" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6100,7 +6074,7 @@
       <c r="G227" t="s">
         <v>166</v>
       </c>
-      <c r="H227" s="2">
+      <c r="H227" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6117,7 +6091,7 @@
       <c r="D228" t="s">
         <v>124</v>
       </c>
-      <c r="H228" s="2">
+      <c r="H228" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6140,7 +6114,7 @@
       <c r="G229" t="s">
         <v>167</v>
       </c>
-      <c r="H229" s="2">
+      <c r="H229" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6157,13 +6131,13 @@
       <c r="D230" t="s">
         <v>146</v>
       </c>
-      <c r="E230" s="2">
+      <c r="E230" s="1">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>191</v>
       </c>
-      <c r="H230" s="2">
+      <c r="H230" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6186,7 +6160,7 @@
       <c r="G231" t="s">
         <v>168</v>
       </c>
-      <c r="H231" s="2">
+      <c r="H231" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6209,7 +6183,7 @@
       <c r="G232" t="s">
         <v>168</v>
       </c>
-      <c r="H232" s="2">
+      <c r="H232" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6232,7 +6206,7 @@
       <c r="G233" t="s">
         <v>169</v>
       </c>
-      <c r="H233" s="2">
+      <c r="H233" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="C234" t="s">
         <v>107</v>
       </c>
-      <c r="H234" s="2">
+      <c r="H234" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6263,13 +6237,13 @@
       <c r="D235" t="s">
         <v>147</v>
       </c>
-      <c r="E235" s="2">
+      <c r="E235" s="1">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>186</v>
       </c>
-      <c r="H235" s="2">
+      <c r="H235" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6283,7 +6257,7 @@
       <c r="C236" t="s">
         <v>107</v>
       </c>
-      <c r="H236" s="2">
+      <c r="H236" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6297,7 +6271,7 @@
       <c r="C237" t="s">
         <v>111</v>
       </c>
-      <c r="H237" s="2">
+      <c r="H237" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6311,7 +6285,7 @@
       <c r="C238" t="s">
         <v>107</v>
       </c>
-      <c r="H238" s="2">
+      <c r="H238" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6325,7 +6299,7 @@
       <c r="C239" t="s">
         <v>111</v>
       </c>
-      <c r="H239" s="2">
+      <c r="H239" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6339,7 +6313,7 @@
       <c r="C240" t="s">
         <v>111</v>
       </c>
-      <c r="H240" s="2">
+      <c r="H240" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6356,13 +6330,13 @@
       <c r="D241" t="s">
         <v>117</v>
       </c>
-      <c r="E241" s="2">
+      <c r="E241" s="1">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>180</v>
       </c>
-      <c r="H241" s="2">
+      <c r="H241" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6376,7 +6350,7 @@
       <c r="C242" t="s">
         <v>111</v>
       </c>
-      <c r="H242" s="2">
+      <c r="H242" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6393,13 +6367,13 @@
       <c r="D243" t="s">
         <v>148</v>
       </c>
-      <c r="E243" s="2">
+      <c r="E243" s="1">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>192</v>
       </c>
-      <c r="H243" s="2">
+      <c r="H243" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6416,13 +6390,13 @@
       <c r="D244" t="s">
         <v>149</v>
       </c>
-      <c r="E244" s="2">
+      <c r="E244" s="1">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>189</v>
       </c>
-      <c r="H244" s="2">
+      <c r="H244" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6436,7 +6410,7 @@
       <c r="C245" t="s">
         <v>111</v>
       </c>
-      <c r="H245" s="2">
+      <c r="H245" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6450,7 +6424,7 @@
       <c r="C246" t="s">
         <v>107</v>
       </c>
-      <c r="H246" s="2">
+      <c r="H246" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6467,13 +6441,13 @@
       <c r="D247" t="s">
         <v>120</v>
       </c>
-      <c r="E247" s="2">
+      <c r="E247" s="1">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>193</v>
       </c>
-      <c r="H247" s="2">
+      <c r="H247" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6487,7 +6461,7 @@
       <c r="C248" t="s">
         <v>107</v>
       </c>
-      <c r="H248" s="2">
+      <c r="H248" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6501,7 +6475,7 @@
       <c r="C249" t="s">
         <v>107</v>
       </c>
-      <c r="H249" s="2">
+      <c r="H249" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6518,13 +6492,13 @@
       <c r="D250" t="s">
         <v>150</v>
       </c>
-      <c r="E250" s="2">
+      <c r="E250" s="1">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>188</v>
       </c>
-      <c r="H250" s="2">
+      <c r="H250" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6538,7 +6512,7 @@
       <c r="C251" t="s">
         <v>107</v>
       </c>
-      <c r="H251" s="2">
+      <c r="H251" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6555,13 +6529,13 @@
       <c r="D252" t="s">
         <v>151</v>
       </c>
-      <c r="E252" s="2">
+      <c r="E252" s="1">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>190</v>
       </c>
-      <c r="H252" s="2">
+      <c r="H252" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6584,7 +6558,7 @@
       <c r="G253" t="s">
         <v>171</v>
       </c>
-      <c r="H253" s="2">
+      <c r="H253" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6598,7 +6572,7 @@
       <c r="C254" t="s">
         <v>111</v>
       </c>
-      <c r="H254" s="2">
+      <c r="H254" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6612,7 +6586,7 @@
       <c r="C255" t="s">
         <v>107</v>
       </c>
-      <c r="H255" s="2">
+      <c r="H255" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6635,7 +6609,7 @@
       <c r="G256" t="s">
         <v>166</v>
       </c>
-      <c r="H256" s="2">
+      <c r="H256" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6652,7 +6626,7 @@
       <c r="D257" t="s">
         <v>124</v>
       </c>
-      <c r="H257" s="2">
+      <c r="H257" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6675,7 +6649,7 @@
       <c r="G258" t="s">
         <v>167</v>
       </c>
-      <c r="H258" s="2">
+      <c r="H258" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6692,13 +6666,13 @@
       <c r="D259" t="s">
         <v>146</v>
       </c>
-      <c r="E259" s="2">
+      <c r="E259" s="1">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>191</v>
       </c>
-      <c r="H259" s="2">
+      <c r="H259" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6721,7 +6695,7 @@
       <c r="G260" t="s">
         <v>168</v>
       </c>
-      <c r="H260" s="2">
+      <c r="H260" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6744,7 +6718,7 @@
       <c r="G261" t="s">
         <v>168</v>
       </c>
-      <c r="H261" s="2">
+      <c r="H261" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6767,7 +6741,7 @@
       <c r="G262" t="s">
         <v>169</v>
       </c>
-      <c r="H262" s="2">
+      <c r="H262" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6781,7 +6755,7 @@
       <c r="C263" t="s">
         <v>107</v>
       </c>
-      <c r="H263" s="2">
+      <c r="H263" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6798,13 +6772,13 @@
       <c r="D264" t="s">
         <v>147</v>
       </c>
-      <c r="E264" s="2">
+      <c r="E264" s="1">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>186</v>
       </c>
-      <c r="H264" s="2">
+      <c r="H264" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6818,7 +6792,7 @@
       <c r="C265" t="s">
         <v>107</v>
       </c>
-      <c r="H265" s="2">
+      <c r="H265" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6832,7 +6806,7 @@
       <c r="C266" t="s">
         <v>111</v>
       </c>
-      <c r="H266" s="2">
+      <c r="H266" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6846,7 +6820,7 @@
       <c r="C267" t="s">
         <v>107</v>
       </c>
-      <c r="H267" s="2">
+      <c r="H267" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6860,7 +6834,7 @@
       <c r="C268" t="s">
         <v>111</v>
       </c>
-      <c r="H268" s="2">
+      <c r="H268" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6874,7 +6848,7 @@
       <c r="C269" t="s">
         <v>111</v>
       </c>
-      <c r="H269" s="2">
+      <c r="H269" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6891,13 +6865,13 @@
       <c r="D270" t="s">
         <v>117</v>
       </c>
-      <c r="E270" s="2">
+      <c r="E270" s="1">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>180</v>
       </c>
-      <c r="H270" s="2">
+      <c r="H270" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6911,7 +6885,7 @@
       <c r="C271" t="s">
         <v>111</v>
       </c>
-      <c r="H271" s="2">
+      <c r="H271" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6928,13 +6902,13 @@
       <c r="D272" t="s">
         <v>148</v>
       </c>
-      <c r="E272" s="2">
+      <c r="E272" s="1">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>192</v>
       </c>
-      <c r="H272" s="2">
+      <c r="H272" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6951,13 +6925,13 @@
       <c r="D273" t="s">
         <v>149</v>
       </c>
-      <c r="E273" s="2">
+      <c r="E273" s="1">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>194</v>
       </c>
-      <c r="H273" s="2">
+      <c r="H273" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6971,7 +6945,7 @@
       <c r="C274" t="s">
         <v>107</v>
       </c>
-      <c r="H274" s="2">
+      <c r="H274" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6985,7 +6959,7 @@
       <c r="C275" t="s">
         <v>107</v>
       </c>
-      <c r="H275" s="2">
+      <c r="H275" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7002,13 +6976,13 @@
       <c r="D276" t="s">
         <v>120</v>
       </c>
-      <c r="E276" s="2">
+      <c r="E276" s="1">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>193</v>
       </c>
-      <c r="H276" s="2">
+      <c r="H276" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7022,7 +6996,7 @@
       <c r="C277" t="s">
         <v>107</v>
       </c>
-      <c r="H277" s="2">
+      <c r="H277" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7039,13 +7013,13 @@
       <c r="D278" t="s">
         <v>152</v>
       </c>
-      <c r="E278" s="2">
+      <c r="E278" s="1">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>195</v>
       </c>
-      <c r="H278" s="2">
+      <c r="H278" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7062,13 +7036,13 @@
       <c r="D279" t="s">
         <v>150</v>
       </c>
-      <c r="E279" s="2">
+      <c r="E279" s="1">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>194</v>
       </c>
-      <c r="H279" s="2">
+      <c r="H279" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7082,7 +7056,7 @@
       <c r="C280" t="s">
         <v>107</v>
       </c>
-      <c r="H280" s="2">
+      <c r="H280" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7099,13 +7073,13 @@
       <c r="D281" t="s">
         <v>153</v>
       </c>
-      <c r="E281" s="2">
+      <c r="E281" s="1">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>190</v>
       </c>
-      <c r="H281" s="2">
+      <c r="H281" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7128,7 +7102,7 @@
       <c r="G282" t="s">
         <v>171</v>
       </c>
-      <c r="H282" s="2">
+      <c r="H282" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7142,7 +7116,7 @@
       <c r="C283" t="s">
         <v>111</v>
       </c>
-      <c r="H283" s="2">
+      <c r="H283" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7156,7 +7130,7 @@
       <c r="C284" t="s">
         <v>107</v>
       </c>
-      <c r="H284" s="2">
+      <c r="H284" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7179,7 +7153,7 @@
       <c r="G285" t="s">
         <v>166</v>
       </c>
-      <c r="H285" s="2">
+      <c r="H285" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="D286" t="s">
         <v>124</v>
       </c>
-      <c r="H286" s="2">
+      <c r="H286" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7219,7 +7193,7 @@
       <c r="G287" t="s">
         <v>167</v>
       </c>
-      <c r="H287" s="2">
+      <c r="H287" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7236,13 +7210,13 @@
       <c r="D288" t="s">
         <v>146</v>
       </c>
-      <c r="E288" s="2">
+      <c r="E288" s="1">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>191</v>
       </c>
-      <c r="H288" s="2">
+      <c r="H288" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7265,7 +7239,7 @@
       <c r="G289" t="s">
         <v>168</v>
       </c>
-      <c r="H289" s="2">
+      <c r="H289" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7288,7 +7262,7 @@
       <c r="G290" t="s">
         <v>168</v>
       </c>
-      <c r="H290" s="2">
+      <c r="H290" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7311,7 +7285,7 @@
       <c r="G291" t="s">
         <v>169</v>
       </c>
-      <c r="H291" s="2">
+      <c r="H291" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7325,7 +7299,7 @@
       <c r="C292" t="s">
         <v>107</v>
       </c>
-      <c r="H292" s="2">
+      <c r="H292" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7348,7 +7322,7 @@
       <c r="G293" t="s">
         <v>172</v>
       </c>
-      <c r="H293" s="2">
+      <c r="H293" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7362,7 +7336,7 @@
       <c r="C294" t="s">
         <v>107</v>
       </c>
-      <c r="H294" s="2">
+      <c r="H294" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7385,7 +7359,7 @@
       <c r="G295" t="s">
         <v>173</v>
       </c>
-      <c r="H295" s="2">
+      <c r="H295" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7399,7 +7373,7 @@
       <c r="C296" t="s">
         <v>107</v>
       </c>
-      <c r="H296" s="2">
+      <c r="H296" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7413,7 +7387,7 @@
       <c r="C297" t="s">
         <v>111</v>
       </c>
-      <c r="H297" s="2">
+      <c r="H297" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7436,7 +7410,7 @@
       <c r="G298" t="s">
         <v>174</v>
       </c>
-      <c r="H298" s="2">
+      <c r="H298" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7453,13 +7427,13 @@
       <c r="D299" t="s">
         <v>117</v>
       </c>
-      <c r="E299" s="2">
+      <c r="E299" s="1">
         <v>46234</v>
       </c>
       <c r="G299" t="s">
         <v>180</v>
       </c>
-      <c r="H299" s="2">
+      <c r="H299" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7473,7 +7447,7 @@
       <c r="C300" t="s">
         <v>107</v>
       </c>
-      <c r="H300" s="2">
+      <c r="H300" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7490,13 +7464,13 @@
       <c r="D301" t="s">
         <v>148</v>
       </c>
-      <c r="E301" s="2">
+      <c r="E301" s="1">
         <v>46224</v>
       </c>
       <c r="G301" t="s">
         <v>192</v>
       </c>
-      <c r="H301" s="2">
+      <c r="H301" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7513,13 +7487,13 @@
       <c r="D302" t="s">
         <v>149</v>
       </c>
-      <c r="E302" s="2">
+      <c r="E302" s="1">
         <v>46220</v>
       </c>
       <c r="G302" t="s">
         <v>189</v>
       </c>
-      <c r="H302" s="2">
+      <c r="H302" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7533,7 +7507,7 @@
       <c r="C303" t="s">
         <v>107</v>
       </c>
-      <c r="H303" s="2">
+      <c r="H303" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7547,7 +7521,7 @@
       <c r="C304" t="s">
         <v>107</v>
       </c>
-      <c r="H304" s="2">
+      <c r="H304" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7564,13 +7538,13 @@
       <c r="D305" t="s">
         <v>120</v>
       </c>
-      <c r="E305" s="2">
+      <c r="E305" s="1">
         <v>46237</v>
       </c>
       <c r="G305" t="s">
         <v>193</v>
       </c>
-      <c r="H305" s="2">
+      <c r="H305" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7584,7 +7558,7 @@
       <c r="C306" t="s">
         <v>107</v>
       </c>
-      <c r="H306" s="2">
+      <c r="H306" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7601,13 +7575,13 @@
       <c r="D307" t="s">
         <v>152</v>
       </c>
-      <c r="E307" s="2">
+      <c r="E307" s="1">
         <v>46227</v>
       </c>
       <c r="G307" t="s">
         <v>195</v>
       </c>
-      <c r="H307" s="2">
+      <c r="H307" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7621,7 +7595,7 @@
       <c r="C308" t="s">
         <v>111</v>
       </c>
-      <c r="H308" s="2">
+      <c r="H308" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7644,7 +7618,7 @@
       <c r="G309" t="s">
         <v>172</v>
       </c>
-      <c r="H309" s="2">
+      <c r="H309" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7667,7 +7641,7 @@
       <c r="G310" t="s">
         <v>175</v>
       </c>
-      <c r="H310" s="2">
+      <c r="H310" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7684,7 +7658,7 @@
       <c r="D311" t="s">
         <v>158</v>
       </c>
-      <c r="H311" s="2">
+      <c r="H311" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7698,7 +7672,7 @@
       <c r="C312" t="s">
         <v>111</v>
       </c>
-      <c r="H312" s="2">
+      <c r="H312" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="C313" t="s">
         <v>107</v>
       </c>
-      <c r="H313" s="2">
+      <c r="H313" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7735,7 +7709,7 @@
       <c r="G314" t="s">
         <v>166</v>
       </c>
-      <c r="H314" s="2">
+      <c r="H314" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7752,7 +7726,7 @@
       <c r="D315" t="s">
         <v>124</v>
       </c>
-      <c r="H315" s="2">
+      <c r="H315" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7775,7 +7749,7 @@
       <c r="G316" t="s">
         <v>167</v>
       </c>
-      <c r="H316" s="2">
+      <c r="H316" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7798,7 +7772,7 @@
       <c r="G317" t="s">
         <v>176</v>
       </c>
-      <c r="H317" s="2">
+      <c r="H317" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7821,7 +7795,7 @@
       <c r="G318" t="s">
         <v>168</v>
       </c>
-      <c r="H318" s="2">
+      <c r="H318" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="G319" t="s">
         <v>168</v>
       </c>
-      <c r="H319" s="2">
+      <c r="H319" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7867,7 +7841,7 @@
       <c r="G320" t="s">
         <v>169</v>
       </c>
-      <c r="H320" s="2">
+      <c r="H320" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7881,7 +7855,7 @@
       <c r="C321" t="s">
         <v>107</v>
       </c>
-      <c r="H321" s="2">
+      <c r="H321" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="G322" t="s">
         <v>177</v>
       </c>
-      <c r="H322" s="2">
+      <c r="H322" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7918,7 +7892,7 @@
       <c r="C323" t="s">
         <v>107</v>
       </c>
-      <c r="H323" s="2">
+      <c r="H323" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7941,7 +7915,7 @@
       <c r="G324" t="s">
         <v>178</v>
       </c>
-      <c r="H324" s="2">
+      <c r="H324" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7955,7 +7929,7 @@
       <c r="C325" t="s">
         <v>107</v>
       </c>
-      <c r="H325" s="2">
+      <c r="H325" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7969,7 +7943,7 @@
       <c r="C326" t="s">
         <v>111</v>
       </c>
-      <c r="H326" s="2">
+      <c r="H326" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7983,7 +7957,7 @@
       <c r="C327" t="s">
         <v>111</v>
       </c>
-      <c r="H327" s="2">
+      <c r="H327" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8000,13 +7974,13 @@
       <c r="D328" t="s">
         <v>117</v>
       </c>
-      <c r="E328" s="2">
+      <c r="E328" s="1">
         <v>46234</v>
       </c>
       <c r="G328" t="s">
         <v>180</v>
       </c>
-      <c r="H328" s="2">
+      <c r="H328" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8029,7 +8003,7 @@
       <c r="G329" t="s">
         <v>178</v>
       </c>
-      <c r="H329" s="2">
+      <c r="H329" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8052,7 +8026,7 @@
       <c r="G330" t="s">
         <v>178</v>
       </c>
-      <c r="H330" s="2">
+      <c r="H330" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8066,7 +8040,7 @@
       <c r="C331" t="s">
         <v>107</v>
       </c>
-      <c r="H331" s="2">
+      <c r="H331" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8089,7 +8063,7 @@
       <c r="G332" t="s">
         <v>178</v>
       </c>
-      <c r="H332" s="2">
+      <c r="H332" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8112,7 +8086,7 @@
       <c r="G333" t="s">
         <v>177</v>
       </c>
-      <c r="H333" s="2">
+      <c r="H333" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8129,13 +8103,13 @@
       <c r="D334" t="s">
         <v>120</v>
       </c>
-      <c r="E334" s="2">
+      <c r="E334" s="1">
         <v>46237</v>
       </c>
       <c r="G334" t="s">
         <v>193</v>
       </c>
-      <c r="H334" s="2">
+      <c r="H334" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8149,7 +8123,7 @@
       <c r="C335" t="s">
         <v>107</v>
       </c>
-      <c r="H335" s="2">
+      <c r="H335" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8166,13 +8140,13 @@
       <c r="D336" t="s">
         <v>152</v>
       </c>
-      <c r="E336" s="2">
+      <c r="E336" s="1">
         <v>46227</v>
       </c>
       <c r="G336" t="s">
         <v>195</v>
       </c>
-      <c r="H336" s="2">
+      <c r="H336" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8186,7 +8160,7 @@
       <c r="C337" t="s">
         <v>107</v>
       </c>
-      <c r="H337" s="2">
+      <c r="H337" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8200,7 +8174,7 @@
       <c r="C338" t="s">
         <v>107</v>
       </c>
-      <c r="H338" s="2">
+      <c r="H338" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8223,7 +8197,7 @@
       <c r="G339" t="s">
         <v>175</v>
       </c>
-      <c r="H339" s="2">
+      <c r="H339" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8240,7 +8214,7 @@
       <c r="D340" t="s">
         <v>163</v>
       </c>
-      <c r="H340" s="2">
+      <c r="H340" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8254,7 +8228,7 @@
       <c r="C341" t="s">
         <v>111</v>
       </c>
-      <c r="H341" s="2">
+      <c r="H341" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8268,7 +8242,7 @@
       <c r="C342" t="s">
         <v>107</v>
       </c>
-      <c r="H342" s="2">
+      <c r="H342" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8291,7 +8265,7 @@
       <c r="G343" t="s">
         <v>166</v>
       </c>
-      <c r="H343" s="2">
+      <c r="H343" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8308,7 +8282,7 @@
       <c r="D344" t="s">
         <v>124</v>
       </c>
-      <c r="H344" s="2">
+      <c r="H344" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8331,7 +8305,7 @@
       <c r="G345" t="s">
         <v>167</v>
       </c>
-      <c r="H345" s="2">
+      <c r="H345" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8354,7 +8328,7 @@
       <c r="G346" t="s">
         <v>176</v>
       </c>
-      <c r="H346" s="2">
+      <c r="H346" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8377,7 +8351,7 @@
       <c r="G347" t="s">
         <v>168</v>
       </c>
-      <c r="H347" s="2">
+      <c r="H347" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8400,7 +8374,7 @@
       <c r="G348" t="s">
         <v>168</v>
       </c>
-      <c r="H348" s="2">
+      <c r="H348" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8423,7 +8397,7 @@
       <c r="G349" t="s">
         <v>169</v>
       </c>
-      <c r="H349" s="2">
+      <c r="H349" s="1">
         <v>46224</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (22/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -639,16 +639,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -664,7 +656,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -672,30 +664,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -995,72 +969,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1125,7 +1099,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1190,7 +1164,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1255,7 +1229,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1320,7 +1294,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1385,7 +1359,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1450,7 +1424,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1515,7 +1489,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1580,7 +1554,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1645,7 +1619,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1710,7 +1684,7 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>46220</v>
       </c>
       <c r="B12">
@@ -1775,7 +1749,7 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46224</v>
       </c>
       <c r="B13">
@@ -1840,7 +1814,7 @@
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46225</v>
       </c>
       <c r="B14">
@@ -1915,28 +1889,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>71</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1950,7 +1924,7 @@
       <c r="C2" t="s">
         <v>112</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1964,7 +1938,7 @@
       <c r="C3" t="s">
         <v>112</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -1987,7 +1961,7 @@
       <c r="G4" t="s">
         <v>170</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2001,7 +1975,7 @@
       <c r="C5" t="s">
         <v>112</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2015,7 +1989,7 @@
       <c r="C6" t="s">
         <v>112</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2032,13 +2006,13 @@
       <c r="D7" t="s">
         <v>120</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>188</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2055,13 +2029,13 @@
       <c r="D8" t="s">
         <v>121</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>188</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2078,13 +2052,13 @@
       <c r="D9" t="s">
         <v>122</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>189</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2101,13 +2075,13 @@
       <c r="D10" t="s">
         <v>123</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>190</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2121,7 +2095,7 @@
       <c r="C11" t="s">
         <v>112</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2135,7 +2109,7 @@
       <c r="C12" t="s">
         <v>112</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2152,13 +2126,13 @@
       <c r="D13" t="s">
         <v>124</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>188</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2172,7 +2146,7 @@
       <c r="C14" t="s">
         <v>116</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2189,13 +2163,13 @@
       <c r="D15" t="s">
         <v>125</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>191</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2209,7 +2183,7 @@
       <c r="C16" t="s">
         <v>112</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2223,7 +2197,7 @@
       <c r="C17" t="s">
         <v>112</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2240,13 +2214,13 @@
       <c r="D18" t="s">
         <v>126</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>192</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2260,7 +2234,7 @@
       <c r="C19" t="s">
         <v>112</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2277,13 +2251,13 @@
       <c r="D20" t="s">
         <v>127</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>188</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2306,7 +2280,7 @@
       <c r="G21" t="s">
         <v>171</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2320,7 +2294,7 @@
       <c r="C22" t="s">
         <v>116</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2334,7 +2308,7 @@
       <c r="C23" t="s">
         <v>112</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2357,7 +2331,7 @@
       <c r="G24" t="s">
         <v>172</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2374,7 +2348,7 @@
       <c r="D25" t="s">
         <v>129</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2397,7 +2371,7 @@
       <c r="G26" t="s">
         <v>173</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2414,13 +2388,13 @@
       <c r="D27" t="s">
         <v>131</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>193</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2443,7 +2417,7 @@
       <c r="G28" t="s">
         <v>174</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2466,7 +2440,7 @@
       <c r="G29" t="s">
         <v>174</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2489,7 +2463,7 @@
       <c r="G30" t="s">
         <v>175</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2503,7 +2477,7 @@
       <c r="C31" t="s">
         <v>112</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2517,7 +2491,7 @@
       <c r="C32" t="s">
         <v>112</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2540,7 +2514,7 @@
       <c r="G33" t="s">
         <v>176</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2554,7 +2528,7 @@
       <c r="C34" t="s">
         <v>112</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2568,7 +2542,7 @@
       <c r="C35" t="s">
         <v>112</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2585,13 +2559,13 @@
       <c r="D36" t="s">
         <v>120</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>188</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2608,13 +2582,13 @@
       <c r="D37" t="s">
         <v>121</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>188</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2631,13 +2605,13 @@
       <c r="D38" t="s">
         <v>122</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>189</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2654,13 +2628,13 @@
       <c r="D39" t="s">
         <v>123</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>190</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2674,7 +2648,7 @@
       <c r="C40" t="s">
         <v>112</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2688,7 +2662,7 @@
       <c r="C41" t="s">
         <v>112</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2705,13 +2679,13 @@
       <c r="D42" t="s">
         <v>124</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>188</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2725,7 +2699,7 @@
       <c r="C43" t="s">
         <v>112</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2742,13 +2716,13 @@
       <c r="D44" t="s">
         <v>125</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>191</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2762,7 +2736,7 @@
       <c r="C45" t="s">
         <v>112</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2776,7 +2750,7 @@
       <c r="C46" t="s">
         <v>112</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2790,7 +2764,7 @@
       <c r="C47" t="s">
         <v>116</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2804,7 +2778,7 @@
       <c r="C48" t="s">
         <v>112</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2821,13 +2795,13 @@
       <c r="D49" t="s">
         <v>136</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>188</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2850,7 +2824,7 @@
       <c r="G50" t="s">
         <v>171</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2864,7 +2838,7 @@
       <c r="C51" t="s">
         <v>116</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2878,7 +2852,7 @@
       <c r="C52" t="s">
         <v>112</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2901,7 +2875,7 @@
       <c r="G53" t="s">
         <v>172</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2918,7 +2892,7 @@
       <c r="D54" t="s">
         <v>129</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2941,7 +2915,7 @@
       <c r="G55" t="s">
         <v>173</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2958,13 +2932,13 @@
       <c r="D56" t="s">
         <v>131</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>193</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2987,7 +2961,7 @@
       <c r="G57" t="s">
         <v>174</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3010,7 +2984,7 @@
       <c r="G58" t="s">
         <v>174</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3033,7 +3007,7 @@
       <c r="G59" t="s">
         <v>175</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3047,7 +3021,7 @@
       <c r="C60" t="s">
         <v>112</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3061,7 +3035,7 @@
       <c r="C61" t="s">
         <v>112</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3078,13 +3052,13 @@
       <c r="D62" t="s">
         <v>135</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>194</v>
       </c>
-      <c r="H62" s="2">
+      <c r="H62" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3098,7 +3072,7 @@
       <c r="C63" t="s">
         <v>112</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3115,13 +3089,13 @@
       <c r="D64" t="s">
         <v>137</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>195</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3135,7 +3109,7 @@
       <c r="C65" t="s">
         <v>112</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3149,7 +3123,7 @@
       <c r="C66" t="s">
         <v>116</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3166,13 +3140,13 @@
       <c r="D67" t="s">
         <v>122</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>189</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3189,13 +3163,13 @@
       <c r="D68" t="s">
         <v>123</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>190</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3209,7 +3183,7 @@
       <c r="C69" t="s">
         <v>112</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3223,7 +3197,7 @@
       <c r="C70" t="s">
         <v>112</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3240,13 +3214,13 @@
       <c r="D71" t="s">
         <v>124</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>194</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3260,7 +3234,7 @@
       <c r="C72" t="s">
         <v>112</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3277,13 +3251,13 @@
       <c r="D73" t="s">
         <v>125</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>191</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3297,7 +3271,7 @@
       <c r="C74" t="s">
         <v>112</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3311,7 +3285,7 @@
       <c r="C75" t="s">
         <v>112</v>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3325,7 +3299,7 @@
       <c r="C76" t="s">
         <v>112</v>
       </c>
-      <c r="H76" s="2">
+      <c r="H76" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3339,7 +3313,7 @@
       <c r="C77" t="s">
         <v>112</v>
       </c>
-      <c r="H77" s="2">
+      <c r="H77" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3356,13 +3330,13 @@
       <c r="D78" t="s">
         <v>136</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="1">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>194</v>
       </c>
-      <c r="H78" s="2">
+      <c r="H78" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3385,7 +3359,7 @@
       <c r="G79" t="s">
         <v>177</v>
       </c>
-      <c r="H79" s="2">
+      <c r="H79" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3399,7 +3373,7 @@
       <c r="C80" t="s">
         <v>116</v>
       </c>
-      <c r="H80" s="2">
+      <c r="H80" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3413,7 +3387,7 @@
       <c r="C81" t="s">
         <v>112</v>
       </c>
-      <c r="H81" s="2">
+      <c r="H81" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3436,7 +3410,7 @@
       <c r="G82" t="s">
         <v>172</v>
       </c>
-      <c r="H82" s="2">
+      <c r="H82" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3453,7 +3427,7 @@
       <c r="D83" t="s">
         <v>129</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3476,7 +3450,7 @@
       <c r="G84" t="s">
         <v>173</v>
       </c>
-      <c r="H84" s="2">
+      <c r="H84" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3493,13 +3467,13 @@
       <c r="D85" t="s">
         <v>131</v>
       </c>
-      <c r="E85" s="2">
+      <c r="E85" s="1">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>193</v>
       </c>
-      <c r="H85" s="2">
+      <c r="H85" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3522,7 +3496,7 @@
       <c r="G86" t="s">
         <v>174</v>
       </c>
-      <c r="H86" s="2">
+      <c r="H86" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3545,7 +3519,7 @@
       <c r="G87" t="s">
         <v>174</v>
       </c>
-      <c r="H87" s="2">
+      <c r="H87" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3568,7 +3542,7 @@
       <c r="G88" t="s">
         <v>175</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3582,7 +3556,7 @@
       <c r="C89" t="s">
         <v>112</v>
       </c>
-      <c r="H89" s="2">
+      <c r="H89" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3599,13 +3573,13 @@
       <c r="D90" t="s">
         <v>139</v>
       </c>
-      <c r="E90" s="2">
+      <c r="E90" s="1">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>195</v>
       </c>
-      <c r="H90" s="2">
+      <c r="H90" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3622,13 +3596,13 @@
       <c r="D91" t="s">
         <v>135</v>
       </c>
-      <c r="E91" s="2">
+      <c r="E91" s="1">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>194</v>
       </c>
-      <c r="H91" s="2">
+      <c r="H91" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3642,7 +3616,7 @@
       <c r="C92" t="s">
         <v>112</v>
       </c>
-      <c r="H92" s="2">
+      <c r="H92" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3659,13 +3633,13 @@
       <c r="D93" t="s">
         <v>137</v>
       </c>
-      <c r="E93" s="2">
+      <c r="E93" s="1">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>195</v>
       </c>
-      <c r="H93" s="2">
+      <c r="H93" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3679,7 +3653,7 @@
       <c r="C94" t="s">
         <v>112</v>
       </c>
-      <c r="H94" s="2">
+      <c r="H94" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3693,7 +3667,7 @@
       <c r="C95" t="s">
         <v>116</v>
       </c>
-      <c r="H95" s="2">
+      <c r="H95" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3710,13 +3684,13 @@
       <c r="D96" t="s">
         <v>122</v>
       </c>
-      <c r="E96" s="2">
+      <c r="E96" s="1">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>189</v>
       </c>
-      <c r="H96" s="2">
+      <c r="H96" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3733,13 +3707,13 @@
       <c r="D97" t="s">
         <v>123</v>
       </c>
-      <c r="E97" s="2">
+      <c r="E97" s="1">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>190</v>
       </c>
-      <c r="H97" s="2">
+      <c r="H97" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3753,7 +3727,7 @@
       <c r="C98" t="s">
         <v>112</v>
       </c>
-      <c r="H98" s="2">
+      <c r="H98" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3770,13 +3744,13 @@
       <c r="D99" t="s">
         <v>140</v>
       </c>
-      <c r="E99" s="2">
+      <c r="E99" s="1">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>190</v>
       </c>
-      <c r="H99" s="2">
+      <c r="H99" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3793,13 +3767,13 @@
       <c r="D100" t="s">
         <v>124</v>
       </c>
-      <c r="E100" s="2">
+      <c r="E100" s="1">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>190</v>
       </c>
-      <c r="H100" s="2">
+      <c r="H100" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3813,7 +3787,7 @@
       <c r="C101" t="s">
         <v>112</v>
       </c>
-      <c r="H101" s="2">
+      <c r="H101" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3830,13 +3804,13 @@
       <c r="D102" t="s">
         <v>125</v>
       </c>
-      <c r="E102" s="2">
+      <c r="E102" s="1">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>191</v>
       </c>
-      <c r="H102" s="2">
+      <c r="H102" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3853,13 +3827,13 @@
       <c r="D103" t="s">
         <v>141</v>
       </c>
-      <c r="E103" s="2">
+      <c r="E103" s="1">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>190</v>
       </c>
-      <c r="H103" s="2">
+      <c r="H103" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3873,7 +3847,7 @@
       <c r="C104" t="s">
         <v>112</v>
       </c>
-      <c r="H104" s="2">
+      <c r="H104" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3887,7 +3861,7 @@
       <c r="C105" t="s">
         <v>112</v>
       </c>
-      <c r="H105" s="2">
+      <c r="H105" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3901,7 +3875,7 @@
       <c r="C106" t="s">
         <v>112</v>
       </c>
-      <c r="H106" s="2">
+      <c r="H106" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3918,13 +3892,13 @@
       <c r="D107" t="s">
         <v>142</v>
       </c>
-      <c r="E107" s="2">
+      <c r="E107" s="1">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>190</v>
       </c>
-      <c r="H107" s="2">
+      <c r="H107" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3947,7 +3921,7 @@
       <c r="G108" t="s">
         <v>177</v>
       </c>
-      <c r="H108" s="2">
+      <c r="H108" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3961,7 +3935,7 @@
       <c r="C109" t="s">
         <v>116</v>
       </c>
-      <c r="H109" s="2">
+      <c r="H109" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3975,7 +3949,7 @@
       <c r="C110" t="s">
         <v>112</v>
       </c>
-      <c r="H110" s="2">
+      <c r="H110" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3998,7 +3972,7 @@
       <c r="G111" t="s">
         <v>172</v>
       </c>
-      <c r="H111" s="2">
+      <c r="H111" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4015,7 +3989,7 @@
       <c r="D112" t="s">
         <v>129</v>
       </c>
-      <c r="H112" s="2">
+      <c r="H112" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4038,7 +4012,7 @@
       <c r="G113" t="s">
         <v>173</v>
       </c>
-      <c r="H113" s="2">
+      <c r="H113" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4055,13 +4029,13 @@
       <c r="D114" t="s">
         <v>131</v>
       </c>
-      <c r="E114" s="2">
+      <c r="E114" s="1">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>193</v>
       </c>
-      <c r="H114" s="2">
+      <c r="H114" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4084,7 +4058,7 @@
       <c r="G115" t="s">
         <v>174</v>
       </c>
-      <c r="H115" s="2">
+      <c r="H115" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4107,7 +4081,7 @@
       <c r="G116" t="s">
         <v>174</v>
       </c>
-      <c r="H116" s="2">
+      <c r="H116" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4130,7 +4104,7 @@
       <c r="G117" t="s">
         <v>175</v>
       </c>
-      <c r="H117" s="2">
+      <c r="H117" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4144,7 +4118,7 @@
       <c r="C118" t="s">
         <v>112</v>
       </c>
-      <c r="H118" s="2">
+      <c r="H118" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4161,13 +4135,13 @@
       <c r="D119" t="s">
         <v>139</v>
       </c>
-      <c r="E119" s="2">
+      <c r="E119" s="1">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>195</v>
       </c>
-      <c r="H119" s="2">
+      <c r="H119" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4181,7 +4155,7 @@
       <c r="C120" t="s">
         <v>116</v>
       </c>
-      <c r="H120" s="2">
+      <c r="H120" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4195,7 +4169,7 @@
       <c r="C121" t="s">
         <v>112</v>
       </c>
-      <c r="H121" s="2">
+      <c r="H121" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4209,7 +4183,7 @@
       <c r="C122" t="s">
         <v>116</v>
       </c>
-      <c r="H122" s="2">
+      <c r="H122" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4223,7 +4197,7 @@
       <c r="C123" t="s">
         <v>116</v>
       </c>
-      <c r="H123" s="2">
+      <c r="H123" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4237,7 +4211,7 @@
       <c r="C124" t="s">
         <v>116</v>
       </c>
-      <c r="H124" s="2">
+      <c r="H124" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4254,13 +4228,13 @@
       <c r="D125" t="s">
         <v>122</v>
       </c>
-      <c r="E125" s="2">
+      <c r="E125" s="1">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>189</v>
       </c>
-      <c r="H125" s="2">
+      <c r="H125" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4277,13 +4251,13 @@
       <c r="D126" t="s">
         <v>123</v>
       </c>
-      <c r="E126" s="2">
+      <c r="E126" s="1">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>190</v>
       </c>
-      <c r="H126" s="2">
+      <c r="H126" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4297,7 +4271,7 @@
       <c r="C127" t="s">
         <v>112</v>
       </c>
-      <c r="H127" s="2">
+      <c r="H127" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4314,13 +4288,13 @@
       <c r="D128" t="s">
         <v>140</v>
       </c>
-      <c r="E128" s="2">
+      <c r="E128" s="1">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>190</v>
       </c>
-      <c r="H128" s="2">
+      <c r="H128" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4337,13 +4311,13 @@
       <c r="D129" t="s">
         <v>124</v>
       </c>
-      <c r="E129" s="2">
+      <c r="E129" s="1">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>190</v>
       </c>
-      <c r="H129" s="2">
+      <c r="H129" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4357,7 +4331,7 @@
       <c r="C130" t="s">
         <v>112</v>
       </c>
-      <c r="H130" s="2">
+      <c r="H130" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4374,13 +4348,13 @@
       <c r="D131" t="s">
         <v>125</v>
       </c>
-      <c r="E131" s="2">
+      <c r="E131" s="1">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>191</v>
       </c>
-      <c r="H131" s="2">
+      <c r="H131" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4397,13 +4371,13 @@
       <c r="D132" t="s">
         <v>141</v>
       </c>
-      <c r="E132" s="2">
+      <c r="E132" s="1">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>190</v>
       </c>
-      <c r="H132" s="2">
+      <c r="H132" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4417,7 +4391,7 @@
       <c r="C133" t="s">
         <v>112</v>
       </c>
-      <c r="H133" s="2">
+      <c r="H133" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4431,7 +4405,7 @@
       <c r="C134" t="s">
         <v>112</v>
       </c>
-      <c r="H134" s="2">
+      <c r="H134" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4445,7 +4419,7 @@
       <c r="C135" t="s">
         <v>112</v>
       </c>
-      <c r="H135" s="2">
+      <c r="H135" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4462,13 +4436,13 @@
       <c r="D136" t="s">
         <v>143</v>
       </c>
-      <c r="E136" s="2">
+      <c r="E136" s="1">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>190</v>
       </c>
-      <c r="H136" s="2">
+      <c r="H136" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4491,7 +4465,7 @@
       <c r="G137" t="s">
         <v>177</v>
       </c>
-      <c r="H137" s="2">
+      <c r="H137" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4505,7 +4479,7 @@
       <c r="C138" t="s">
         <v>116</v>
       </c>
-      <c r="H138" s="2">
+      <c r="H138" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4519,7 +4493,7 @@
       <c r="C139" t="s">
         <v>112</v>
       </c>
-      <c r="H139" s="2">
+      <c r="H139" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4542,7 +4516,7 @@
       <c r="G140" t="s">
         <v>172</v>
       </c>
-      <c r="H140" s="2">
+      <c r="H140" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4559,7 +4533,7 @@
       <c r="D141" t="s">
         <v>129</v>
       </c>
-      <c r="H141" s="2">
+      <c r="H141" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4582,7 +4556,7 @@
       <c r="G142" t="s">
         <v>173</v>
       </c>
-      <c r="H142" s="2">
+      <c r="H142" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4599,13 +4573,13 @@
       <c r="D143" t="s">
         <v>131</v>
       </c>
-      <c r="E143" s="2">
+      <c r="E143" s="1">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>193</v>
       </c>
-      <c r="H143" s="2">
+      <c r="H143" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4628,7 +4602,7 @@
       <c r="G144" t="s">
         <v>174</v>
       </c>
-      <c r="H144" s="2">
+      <c r="H144" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4651,7 +4625,7 @@
       <c r="G145" t="s">
         <v>174</v>
       </c>
-      <c r="H145" s="2">
+      <c r="H145" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4674,7 +4648,7 @@
       <c r="G146" t="s">
         <v>175</v>
       </c>
-      <c r="H146" s="2">
+      <c r="H146" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4688,7 +4662,7 @@
       <c r="C147" t="s">
         <v>112</v>
       </c>
-      <c r="H147" s="2">
+      <c r="H147" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4705,13 +4679,13 @@
       <c r="D148" t="s">
         <v>139</v>
       </c>
-      <c r="E148" s="2">
+      <c r="E148" s="1">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>195</v>
       </c>
-      <c r="H148" s="2">
+      <c r="H148" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4725,7 +4699,7 @@
       <c r="C149" t="s">
         <v>116</v>
       </c>
-      <c r="H149" s="2">
+      <c r="H149" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4739,7 +4713,7 @@
       <c r="C150" t="s">
         <v>112</v>
       </c>
-      <c r="H150" s="2">
+      <c r="H150" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4753,7 +4727,7 @@
       <c r="C151" t="s">
         <v>112</v>
       </c>
-      <c r="H151" s="2">
+      <c r="H151" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4767,7 +4741,7 @@
       <c r="C152" t="s">
         <v>116</v>
       </c>
-      <c r="H152" s="2">
+      <c r="H152" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4781,7 +4755,7 @@
       <c r="C153" t="s">
         <v>116</v>
       </c>
-      <c r="H153" s="2">
+      <c r="H153" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4798,13 +4772,13 @@
       <c r="D154" t="s">
         <v>122</v>
       </c>
-      <c r="E154" s="2">
+      <c r="E154" s="1">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>189</v>
       </c>
-      <c r="H154" s="2">
+      <c r="H154" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4821,13 +4795,13 @@
       <c r="D155" t="s">
         <v>123</v>
       </c>
-      <c r="E155" s="2">
+      <c r="E155" s="1">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>190</v>
       </c>
-      <c r="H155" s="2">
+      <c r="H155" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4841,7 +4815,7 @@
       <c r="C156" t="s">
         <v>112</v>
       </c>
-      <c r="H156" s="2">
+      <c r="H156" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4858,13 +4832,13 @@
       <c r="D157" t="s">
         <v>140</v>
       </c>
-      <c r="E157" s="2">
+      <c r="E157" s="1">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>190</v>
       </c>
-      <c r="H157" s="2">
+      <c r="H157" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4881,13 +4855,13 @@
       <c r="D158" t="s">
         <v>124</v>
       </c>
-      <c r="E158" s="2">
+      <c r="E158" s="1">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>190</v>
       </c>
-      <c r="H158" s="2">
+      <c r="H158" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4904,13 +4878,13 @@
       <c r="D159" t="s">
         <v>144</v>
       </c>
-      <c r="E159" s="2">
+      <c r="E159" s="1">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>196</v>
       </c>
-      <c r="H159" s="2">
+      <c r="H159" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4927,13 +4901,13 @@
       <c r="D160" t="s">
         <v>125</v>
       </c>
-      <c r="E160" s="2">
+      <c r="E160" s="1">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>191</v>
       </c>
-      <c r="H160" s="2">
+      <c r="H160" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4950,13 +4924,13 @@
       <c r="D161" t="s">
         <v>141</v>
       </c>
-      <c r="E161" s="2">
+      <c r="E161" s="1">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>190</v>
       </c>
-      <c r="H161" s="2">
+      <c r="H161" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4970,7 +4944,7 @@
       <c r="C162" t="s">
         <v>112</v>
       </c>
-      <c r="H162" s="2">
+      <c r="H162" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4984,7 +4958,7 @@
       <c r="C163" t="s">
         <v>112</v>
       </c>
-      <c r="H163" s="2">
+      <c r="H163" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4998,7 +4972,7 @@
       <c r="C164" t="s">
         <v>112</v>
       </c>
-      <c r="H164" s="2">
+      <c r="H164" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5015,13 +4989,13 @@
       <c r="D165" t="s">
         <v>143</v>
       </c>
-      <c r="E165" s="2">
+      <c r="E165" s="1">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>190</v>
       </c>
-      <c r="H165" s="2">
+      <c r="H165" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5044,7 +5018,7 @@
       <c r="G166" t="s">
         <v>177</v>
       </c>
-      <c r="H166" s="2">
+      <c r="H166" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5058,7 +5032,7 @@
       <c r="C167" t="s">
         <v>116</v>
       </c>
-      <c r="H167" s="2">
+      <c r="H167" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5072,7 +5046,7 @@
       <c r="C168" t="s">
         <v>112</v>
       </c>
-      <c r="H168" s="2">
+      <c r="H168" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5095,7 +5069,7 @@
       <c r="G169" t="s">
         <v>172</v>
       </c>
-      <c r="H169" s="2">
+      <c r="H169" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5112,7 +5086,7 @@
       <c r="D170" t="s">
         <v>129</v>
       </c>
-      <c r="H170" s="2">
+      <c r="H170" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5135,7 +5109,7 @@
       <c r="G171" t="s">
         <v>173</v>
       </c>
-      <c r="H171" s="2">
+      <c r="H171" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5152,13 +5126,13 @@
       <c r="D172" t="s">
         <v>131</v>
       </c>
-      <c r="E172" s="2">
+      <c r="E172" s="1">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>193</v>
       </c>
-      <c r="H172" s="2">
+      <c r="H172" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5181,7 +5155,7 @@
       <c r="G173" t="s">
         <v>174</v>
       </c>
-      <c r="H173" s="2">
+      <c r="H173" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5204,7 +5178,7 @@
       <c r="G174" t="s">
         <v>174</v>
       </c>
-      <c r="H174" s="2">
+      <c r="H174" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5227,7 +5201,7 @@
       <c r="G175" t="s">
         <v>175</v>
       </c>
-      <c r="H175" s="2">
+      <c r="H175" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5241,7 +5215,7 @@
       <c r="C176" t="s">
         <v>112</v>
       </c>
-      <c r="H176" s="2">
+      <c r="H176" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5258,13 +5232,13 @@
       <c r="D177" t="s">
         <v>145</v>
       </c>
-      <c r="E177" s="2">
+      <c r="E177" s="1">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>195</v>
       </c>
-      <c r="H177" s="2">
+      <c r="H177" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5278,7 +5252,7 @@
       <c r="C178" t="s">
         <v>112</v>
       </c>
-      <c r="H178" s="2">
+      <c r="H178" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5295,13 +5269,13 @@
       <c r="D179" t="s">
         <v>146</v>
       </c>
-      <c r="E179" s="2">
+      <c r="E179" s="1">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>191</v>
       </c>
-      <c r="H179" s="2">
+      <c r="H179" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5315,7 +5289,7 @@
       <c r="C180" t="s">
         <v>112</v>
       </c>
-      <c r="H180" s="2">
+      <c r="H180" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5329,7 +5303,7 @@
       <c r="C181" t="s">
         <v>116</v>
       </c>
-      <c r="H181" s="2">
+      <c r="H181" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5343,7 +5317,7 @@
       <c r="C182" t="s">
         <v>116</v>
       </c>
-      <c r="H182" s="2">
+      <c r="H182" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5360,13 +5334,13 @@
       <c r="D183" t="s">
         <v>122</v>
       </c>
-      <c r="E183" s="2">
+      <c r="E183" s="1">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>189</v>
       </c>
-      <c r="H183" s="2">
+      <c r="H183" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5383,13 +5357,13 @@
       <c r="D184" t="s">
         <v>123</v>
       </c>
-      <c r="E184" s="2">
+      <c r="E184" s="1">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>190</v>
       </c>
-      <c r="H184" s="2">
+      <c r="H184" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5403,7 +5377,7 @@
       <c r="C185" t="s">
         <v>112</v>
       </c>
-      <c r="H185" s="2">
+      <c r="H185" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5420,13 +5394,13 @@
       <c r="D186" t="s">
         <v>140</v>
       </c>
-      <c r="E186" s="2">
+      <c r="E186" s="1">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>190</v>
       </c>
-      <c r="H186" s="2">
+      <c r="H186" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5443,13 +5417,13 @@
       <c r="D187" t="s">
         <v>147</v>
       </c>
-      <c r="E187" s="2">
+      <c r="E187" s="1">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>190</v>
       </c>
-      <c r="H187" s="2">
+      <c r="H187" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5466,13 +5440,13 @@
       <c r="D188" t="s">
         <v>148</v>
       </c>
-      <c r="E188" s="2">
+      <c r="E188" s="1">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>190</v>
       </c>
-      <c r="H188" s="2">
+      <c r="H188" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5489,13 +5463,13 @@
       <c r="D189" t="s">
         <v>125</v>
       </c>
-      <c r="E189" s="2">
+      <c r="E189" s="1">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>191</v>
       </c>
-      <c r="H189" s="2">
+      <c r="H189" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5512,13 +5486,13 @@
       <c r="D190" t="s">
         <v>141</v>
       </c>
-      <c r="E190" s="2">
+      <c r="E190" s="1">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>190</v>
       </c>
-      <c r="H190" s="2">
+      <c r="H190" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5532,7 +5506,7 @@
       <c r="C191" t="s">
         <v>112</v>
       </c>
-      <c r="H191" s="2">
+      <c r="H191" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5546,7 +5520,7 @@
       <c r="C192" t="s">
         <v>112</v>
       </c>
-      <c r="H192" s="2">
+      <c r="H192" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5560,7 +5534,7 @@
       <c r="C193" t="s">
         <v>112</v>
       </c>
-      <c r="H193" s="2">
+      <c r="H193" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5577,13 +5551,13 @@
       <c r="D194" t="s">
         <v>143</v>
       </c>
-      <c r="E194" s="2">
+      <c r="E194" s="1">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>197</v>
       </c>
-      <c r="H194" s="2">
+      <c r="H194" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5606,7 +5580,7 @@
       <c r="G195" t="s">
         <v>177</v>
       </c>
-      <c r="H195" s="2">
+      <c r="H195" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5620,7 +5594,7 @@
       <c r="C196" t="s">
         <v>116</v>
       </c>
-      <c r="H196" s="2">
+      <c r="H196" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5634,7 +5608,7 @@
       <c r="C197" t="s">
         <v>112</v>
       </c>
-      <c r="H197" s="2">
+      <c r="H197" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5657,7 +5631,7 @@
       <c r="G198" t="s">
         <v>172</v>
       </c>
-      <c r="H198" s="2">
+      <c r="H198" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5674,7 +5648,7 @@
       <c r="D199" t="s">
         <v>129</v>
       </c>
-      <c r="H199" s="2">
+      <c r="H199" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5697,7 +5671,7 @@
       <c r="G200" t="s">
         <v>173</v>
       </c>
-      <c r="H200" s="2">
+      <c r="H200" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5714,13 +5688,13 @@
       <c r="D201" t="s">
         <v>131</v>
       </c>
-      <c r="E201" s="2">
+      <c r="E201" s="1">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>193</v>
       </c>
-      <c r="H201" s="2">
+      <c r="H201" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5743,7 +5717,7 @@
       <c r="G202" t="s">
         <v>174</v>
       </c>
-      <c r="H202" s="2">
+      <c r="H202" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5766,7 +5740,7 @@
       <c r="G203" t="s">
         <v>174</v>
       </c>
-      <c r="H203" s="2">
+      <c r="H203" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5789,7 +5763,7 @@
       <c r="G204" t="s">
         <v>175</v>
       </c>
-      <c r="H204" s="2">
+      <c r="H204" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5803,7 +5777,7 @@
       <c r="C205" t="s">
         <v>112</v>
       </c>
-      <c r="H205" s="2">
+      <c r="H205" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5820,13 +5794,13 @@
       <c r="D206" t="s">
         <v>145</v>
       </c>
-      <c r="E206" s="2">
+      <c r="E206" s="1">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>195</v>
       </c>
-      <c r="H206" s="2">
+      <c r="H206" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5840,7 +5814,7 @@
       <c r="C207" t="s">
         <v>112</v>
       </c>
-      <c r="H207" s="2">
+      <c r="H207" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5854,7 +5828,7 @@
       <c r="C208" t="s">
         <v>116</v>
       </c>
-      <c r="H208" s="2">
+      <c r="H208" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5868,7 +5842,7 @@
       <c r="C209" t="s">
         <v>112</v>
       </c>
-      <c r="H209" s="2">
+      <c r="H209" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5882,7 +5856,7 @@
       <c r="C210" t="s">
         <v>116</v>
       </c>
-      <c r="H210" s="2">
+      <c r="H210" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5896,7 +5870,7 @@
       <c r="C211" t="s">
         <v>116</v>
       </c>
-      <c r="H211" s="2">
+      <c r="H211" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5913,13 +5887,13 @@
       <c r="D212" t="s">
         <v>122</v>
       </c>
-      <c r="E212" s="2">
+      <c r="E212" s="1">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>189</v>
       </c>
-      <c r="H212" s="2">
+      <c r="H212" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5933,7 +5907,7 @@
       <c r="C213" t="s">
         <v>116</v>
       </c>
-      <c r="H213" s="2">
+      <c r="H213" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5947,7 +5921,7 @@
       <c r="C214" t="s">
         <v>112</v>
       </c>
-      <c r="H214" s="2">
+      <c r="H214" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5964,13 +5938,13 @@
       <c r="D215" t="s">
         <v>140</v>
       </c>
-      <c r="E215" s="2">
+      <c r="E215" s="1">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>198</v>
       </c>
-      <c r="H215" s="2">
+      <c r="H215" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5987,13 +5961,13 @@
       <c r="D216" t="s">
         <v>147</v>
       </c>
-      <c r="E216" s="2">
+      <c r="E216" s="1">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>191</v>
       </c>
-      <c r="H216" s="2">
+      <c r="H216" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6007,7 +5981,7 @@
       <c r="C217" t="s">
         <v>112</v>
       </c>
-      <c r="H217" s="2">
+      <c r="H217" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6024,13 +5998,13 @@
       <c r="D218" t="s">
         <v>125</v>
       </c>
-      <c r="E218" s="2">
+      <c r="E218" s="1">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>191</v>
       </c>
-      <c r="H218" s="2">
+      <c r="H218" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6044,7 +6018,7 @@
       <c r="C219" t="s">
         <v>112</v>
       </c>
-      <c r="H219" s="2">
+      <c r="H219" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6058,7 +6032,7 @@
       <c r="C220" t="s">
         <v>112</v>
       </c>
-      <c r="H220" s="2">
+      <c r="H220" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6075,13 +6049,13 @@
       <c r="D221" t="s">
         <v>149</v>
       </c>
-      <c r="E221" s="2">
+      <c r="E221" s="1">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>195</v>
       </c>
-      <c r="H221" s="2">
+      <c r="H221" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6095,7 +6069,7 @@
       <c r="C222" t="s">
         <v>112</v>
       </c>
-      <c r="H222" s="2">
+      <c r="H222" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6112,13 +6086,13 @@
       <c r="D223" t="s">
         <v>150</v>
       </c>
-      <c r="E223" s="2">
+      <c r="E223" s="1">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>199</v>
       </c>
-      <c r="H223" s="2">
+      <c r="H223" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6141,7 +6115,7 @@
       <c r="G224" t="s">
         <v>177</v>
       </c>
-      <c r="H224" s="2">
+      <c r="H224" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6155,7 +6129,7 @@
       <c r="C225" t="s">
         <v>116</v>
       </c>
-      <c r="H225" s="2">
+      <c r="H225" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6169,7 +6143,7 @@
       <c r="C226" t="s">
         <v>112</v>
       </c>
-      <c r="H226" s="2">
+      <c r="H226" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6192,7 +6166,7 @@
       <c r="G227" t="s">
         <v>172</v>
       </c>
-      <c r="H227" s="2">
+      <c r="H227" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6209,7 +6183,7 @@
       <c r="D228" t="s">
         <v>129</v>
       </c>
-      <c r="H228" s="2">
+      <c r="H228" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6232,7 +6206,7 @@
       <c r="G229" t="s">
         <v>173</v>
       </c>
-      <c r="H229" s="2">
+      <c r="H229" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6249,13 +6223,13 @@
       <c r="D230" t="s">
         <v>151</v>
       </c>
-      <c r="E230" s="2">
+      <c r="E230" s="1">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>200</v>
       </c>
-      <c r="H230" s="2">
+      <c r="H230" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6278,7 +6252,7 @@
       <c r="G231" t="s">
         <v>174</v>
       </c>
-      <c r="H231" s="2">
+      <c r="H231" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6301,7 +6275,7 @@
       <c r="G232" t="s">
         <v>174</v>
       </c>
-      <c r="H232" s="2">
+      <c r="H232" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6324,7 +6298,7 @@
       <c r="G233" t="s">
         <v>175</v>
       </c>
-      <c r="H233" s="2">
+      <c r="H233" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6338,7 +6312,7 @@
       <c r="C234" t="s">
         <v>112</v>
       </c>
-      <c r="H234" s="2">
+      <c r="H234" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6355,13 +6329,13 @@
       <c r="D235" t="s">
         <v>152</v>
       </c>
-      <c r="E235" s="2">
+      <c r="E235" s="1">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>195</v>
       </c>
-      <c r="H235" s="2">
+      <c r="H235" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6375,7 +6349,7 @@
       <c r="C236" t="s">
         <v>112</v>
       </c>
-      <c r="H236" s="2">
+      <c r="H236" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6389,7 +6363,7 @@
       <c r="C237" t="s">
         <v>116</v>
       </c>
-      <c r="H237" s="2">
+      <c r="H237" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6403,7 +6377,7 @@
       <c r="C238" t="s">
         <v>112</v>
       </c>
-      <c r="H238" s="2">
+      <c r="H238" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6417,7 +6391,7 @@
       <c r="C239" t="s">
         <v>116</v>
       </c>
-      <c r="H239" s="2">
+      <c r="H239" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6431,7 +6405,7 @@
       <c r="C240" t="s">
         <v>116</v>
       </c>
-      <c r="H240" s="2">
+      <c r="H240" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6448,13 +6422,13 @@
       <c r="D241" t="s">
         <v>122</v>
       </c>
-      <c r="E241" s="2">
+      <c r="E241" s="1">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>189</v>
       </c>
-      <c r="H241" s="2">
+      <c r="H241" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6468,7 +6442,7 @@
       <c r="C242" t="s">
         <v>116</v>
       </c>
-      <c r="H242" s="2">
+      <c r="H242" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6485,13 +6459,13 @@
       <c r="D243" t="s">
         <v>153</v>
       </c>
-      <c r="E243" s="2">
+      <c r="E243" s="1">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>201</v>
       </c>
-      <c r="H243" s="2">
+      <c r="H243" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6508,13 +6482,13 @@
       <c r="D244" t="s">
         <v>154</v>
       </c>
-      <c r="E244" s="2">
+      <c r="E244" s="1">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>198</v>
       </c>
-      <c r="H244" s="2">
+      <c r="H244" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6528,7 +6502,7 @@
       <c r="C245" t="s">
         <v>116</v>
       </c>
-      <c r="H245" s="2">
+      <c r="H245" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6542,7 +6516,7 @@
       <c r="C246" t="s">
         <v>112</v>
       </c>
-      <c r="H246" s="2">
+      <c r="H246" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6559,13 +6533,13 @@
       <c r="D247" t="s">
         <v>125</v>
       </c>
-      <c r="E247" s="2">
+      <c r="E247" s="1">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>202</v>
       </c>
-      <c r="H247" s="2">
+      <c r="H247" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6579,7 +6553,7 @@
       <c r="C248" t="s">
         <v>112</v>
       </c>
-      <c r="H248" s="2">
+      <c r="H248" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6593,7 +6567,7 @@
       <c r="C249" t="s">
         <v>112</v>
       </c>
-      <c r="H249" s="2">
+      <c r="H249" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6610,13 +6584,13 @@
       <c r="D250" t="s">
         <v>155</v>
       </c>
-      <c r="E250" s="2">
+      <c r="E250" s="1">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>197</v>
       </c>
-      <c r="H250" s="2">
+      <c r="H250" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6630,7 +6604,7 @@
       <c r="C251" t="s">
         <v>112</v>
       </c>
-      <c r="H251" s="2">
+      <c r="H251" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6647,13 +6621,13 @@
       <c r="D252" t="s">
         <v>156</v>
       </c>
-      <c r="E252" s="2">
+      <c r="E252" s="1">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>199</v>
       </c>
-      <c r="H252" s="2">
+      <c r="H252" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6676,7 +6650,7 @@
       <c r="G253" t="s">
         <v>177</v>
       </c>
-      <c r="H253" s="2">
+      <c r="H253" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6690,7 +6664,7 @@
       <c r="C254" t="s">
         <v>116</v>
       </c>
-      <c r="H254" s="2">
+      <c r="H254" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6704,7 +6678,7 @@
       <c r="C255" t="s">
         <v>112</v>
       </c>
-      <c r="H255" s="2">
+      <c r="H255" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6727,7 +6701,7 @@
       <c r="G256" t="s">
         <v>172</v>
       </c>
-      <c r="H256" s="2">
+      <c r="H256" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6744,7 +6718,7 @@
       <c r="D257" t="s">
         <v>129</v>
       </c>
-      <c r="H257" s="2">
+      <c r="H257" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6767,7 +6741,7 @@
       <c r="G258" t="s">
         <v>173</v>
       </c>
-      <c r="H258" s="2">
+      <c r="H258" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6784,13 +6758,13 @@
       <c r="D259" t="s">
         <v>151</v>
       </c>
-      <c r="E259" s="2">
+      <c r="E259" s="1">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>200</v>
       </c>
-      <c r="H259" s="2">
+      <c r="H259" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6813,7 +6787,7 @@
       <c r="G260" t="s">
         <v>174</v>
       </c>
-      <c r="H260" s="2">
+      <c r="H260" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6836,7 +6810,7 @@
       <c r="G261" t="s">
         <v>174</v>
       </c>
-      <c r="H261" s="2">
+      <c r="H261" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6859,7 +6833,7 @@
       <c r="G262" t="s">
         <v>175</v>
       </c>
-      <c r="H262" s="2">
+      <c r="H262" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6873,7 +6847,7 @@
       <c r="C263" t="s">
         <v>112</v>
       </c>
-      <c r="H263" s="2">
+      <c r="H263" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6890,13 +6864,13 @@
       <c r="D264" t="s">
         <v>152</v>
       </c>
-      <c r="E264" s="2">
+      <c r="E264" s="1">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>195</v>
       </c>
-      <c r="H264" s="2">
+      <c r="H264" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6910,7 +6884,7 @@
       <c r="C265" t="s">
         <v>112</v>
       </c>
-      <c r="H265" s="2">
+      <c r="H265" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6924,7 +6898,7 @@
       <c r="C266" t="s">
         <v>116</v>
       </c>
-      <c r="H266" s="2">
+      <c r="H266" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6938,7 +6912,7 @@
       <c r="C267" t="s">
         <v>112</v>
       </c>
-      <c r="H267" s="2">
+      <c r="H267" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6952,7 +6926,7 @@
       <c r="C268" t="s">
         <v>116</v>
       </c>
-      <c r="H268" s="2">
+      <c r="H268" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6966,7 +6940,7 @@
       <c r="C269" t="s">
         <v>116</v>
       </c>
-      <c r="H269" s="2">
+      <c r="H269" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6983,13 +6957,13 @@
       <c r="D270" t="s">
         <v>122</v>
       </c>
-      <c r="E270" s="2">
+      <c r="E270" s="1">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>189</v>
       </c>
-      <c r="H270" s="2">
+      <c r="H270" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7003,7 +6977,7 @@
       <c r="C271" t="s">
         <v>116</v>
       </c>
-      <c r="H271" s="2">
+      <c r="H271" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7020,13 +6994,13 @@
       <c r="D272" t="s">
         <v>153</v>
       </c>
-      <c r="E272" s="2">
+      <c r="E272" s="1">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>201</v>
       </c>
-      <c r="H272" s="2">
+      <c r="H272" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7043,13 +7017,13 @@
       <c r="D273" t="s">
         <v>154</v>
       </c>
-      <c r="E273" s="2">
+      <c r="E273" s="1">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>203</v>
       </c>
-      <c r="H273" s="2">
+      <c r="H273" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7063,7 +7037,7 @@
       <c r="C274" t="s">
         <v>112</v>
       </c>
-      <c r="H274" s="2">
+      <c r="H274" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7077,7 +7051,7 @@
       <c r="C275" t="s">
         <v>112</v>
       </c>
-      <c r="H275" s="2">
+      <c r="H275" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7094,13 +7068,13 @@
       <c r="D276" t="s">
         <v>125</v>
       </c>
-      <c r="E276" s="2">
+      <c r="E276" s="1">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>202</v>
       </c>
-      <c r="H276" s="2">
+      <c r="H276" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7114,7 +7088,7 @@
       <c r="C277" t="s">
         <v>112</v>
       </c>
-      <c r="H277" s="2">
+      <c r="H277" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7131,13 +7105,13 @@
       <c r="D278" t="s">
         <v>157</v>
       </c>
-      <c r="E278" s="2">
+      <c r="E278" s="1">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>204</v>
       </c>
-      <c r="H278" s="2">
+      <c r="H278" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7154,13 +7128,13 @@
       <c r="D279" t="s">
         <v>155</v>
       </c>
-      <c r="E279" s="2">
+      <c r="E279" s="1">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>203</v>
       </c>
-      <c r="H279" s="2">
+      <c r="H279" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7174,7 +7148,7 @@
       <c r="C280" t="s">
         <v>112</v>
       </c>
-      <c r="H280" s="2">
+      <c r="H280" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7191,13 +7165,13 @@
       <c r="D281" t="s">
         <v>158</v>
       </c>
-      <c r="E281" s="2">
+      <c r="E281" s="1">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>199</v>
       </c>
-      <c r="H281" s="2">
+      <c r="H281" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7220,7 +7194,7 @@
       <c r="G282" t="s">
         <v>177</v>
       </c>
-      <c r="H282" s="2">
+      <c r="H282" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7234,7 +7208,7 @@
       <c r="C283" t="s">
         <v>116</v>
       </c>
-      <c r="H283" s="2">
+      <c r="H283" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7248,7 +7222,7 @@
       <c r="C284" t="s">
         <v>112</v>
       </c>
-      <c r="H284" s="2">
+      <c r="H284" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7271,7 +7245,7 @@
       <c r="G285" t="s">
         <v>172</v>
       </c>
-      <c r="H285" s="2">
+      <c r="H285" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7288,7 +7262,7 @@
       <c r="D286" t="s">
         <v>129</v>
       </c>
-      <c r="H286" s="2">
+      <c r="H286" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7311,7 +7285,7 @@
       <c r="G287" t="s">
         <v>173</v>
       </c>
-      <c r="H287" s="2">
+      <c r="H287" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7328,13 +7302,13 @@
       <c r="D288" t="s">
         <v>151</v>
       </c>
-      <c r="E288" s="2">
+      <c r="E288" s="1">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>200</v>
       </c>
-      <c r="H288" s="2">
+      <c r="H288" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7357,7 +7331,7 @@
       <c r="G289" t="s">
         <v>174</v>
       </c>
-      <c r="H289" s="2">
+      <c r="H289" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7380,7 +7354,7 @@
       <c r="G290" t="s">
         <v>174</v>
       </c>
-      <c r="H290" s="2">
+      <c r="H290" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7403,7 +7377,7 @@
       <c r="G291" t="s">
         <v>175</v>
       </c>
-      <c r="H291" s="2">
+      <c r="H291" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7417,7 +7391,7 @@
       <c r="C292" t="s">
         <v>112</v>
       </c>
-      <c r="H292" s="2">
+      <c r="H292" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7440,7 +7414,7 @@
       <c r="G293" t="s">
         <v>178</v>
       </c>
-      <c r="H293" s="2">
+      <c r="H293" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7454,7 +7428,7 @@
       <c r="C294" t="s">
         <v>112</v>
       </c>
-      <c r="H294" s="2">
+      <c r="H294" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7477,7 +7451,7 @@
       <c r="G295" t="s">
         <v>179</v>
       </c>
-      <c r="H295" s="2">
+      <c r="H295" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7491,7 +7465,7 @@
       <c r="C296" t="s">
         <v>112</v>
       </c>
-      <c r="H296" s="2">
+      <c r="H296" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7505,7 +7479,7 @@
       <c r="C297" t="s">
         <v>116</v>
       </c>
-      <c r="H297" s="2">
+      <c r="H297" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7528,7 +7502,7 @@
       <c r="G298" t="s">
         <v>180</v>
       </c>
-      <c r="H298" s="2">
+      <c r="H298" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7545,13 +7519,13 @@
       <c r="D299" t="s">
         <v>122</v>
       </c>
-      <c r="E299" s="2">
+      <c r="E299" s="1">
         <v>46234</v>
       </c>
       <c r="G299" t="s">
         <v>189</v>
       </c>
-      <c r="H299" s="2">
+      <c r="H299" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7565,7 +7539,7 @@
       <c r="C300" t="s">
         <v>112</v>
       </c>
-      <c r="H300" s="2">
+      <c r="H300" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7582,13 +7556,13 @@
       <c r="D301" t="s">
         <v>153</v>
       </c>
-      <c r="E301" s="2">
+      <c r="E301" s="1">
         <v>46224</v>
       </c>
       <c r="G301" t="s">
         <v>201</v>
       </c>
-      <c r="H301" s="2">
+      <c r="H301" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7605,13 +7579,13 @@
       <c r="D302" t="s">
         <v>154</v>
       </c>
-      <c r="E302" s="2">
+      <c r="E302" s="1">
         <v>46220</v>
       </c>
       <c r="G302" t="s">
         <v>198</v>
       </c>
-      <c r="H302" s="2">
+      <c r="H302" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7625,7 +7599,7 @@
       <c r="C303" t="s">
         <v>112</v>
       </c>
-      <c r="H303" s="2">
+      <c r="H303" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7639,7 +7613,7 @@
       <c r="C304" t="s">
         <v>112</v>
       </c>
-      <c r="H304" s="2">
+      <c r="H304" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7656,13 +7630,13 @@
       <c r="D305" t="s">
         <v>125</v>
       </c>
-      <c r="E305" s="2">
+      <c r="E305" s="1">
         <v>46237</v>
       </c>
       <c r="G305" t="s">
         <v>202</v>
       </c>
-      <c r="H305" s="2">
+      <c r="H305" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7676,7 +7650,7 @@
       <c r="C306" t="s">
         <v>112</v>
       </c>
-      <c r="H306" s="2">
+      <c r="H306" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7693,13 +7667,13 @@
       <c r="D307" t="s">
         <v>157</v>
       </c>
-      <c r="E307" s="2">
+      <c r="E307" s="1">
         <v>46227</v>
       </c>
       <c r="G307" t="s">
         <v>204</v>
       </c>
-      <c r="H307" s="2">
+      <c r="H307" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7713,7 +7687,7 @@
       <c r="C308" t="s">
         <v>116</v>
       </c>
-      <c r="H308" s="2">
+      <c r="H308" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7736,7 +7710,7 @@
       <c r="G309" t="s">
         <v>178</v>
       </c>
-      <c r="H309" s="2">
+      <c r="H309" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7759,7 +7733,7 @@
       <c r="G310" t="s">
         <v>181</v>
       </c>
-      <c r="H310" s="2">
+      <c r="H310" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7776,7 +7750,7 @@
       <c r="D311" t="s">
         <v>163</v>
       </c>
-      <c r="H311" s="2">
+      <c r="H311" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7790,7 +7764,7 @@
       <c r="C312" t="s">
         <v>116</v>
       </c>
-      <c r="H312" s="2">
+      <c r="H312" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7804,7 +7778,7 @@
       <c r="C313" t="s">
         <v>112</v>
       </c>
-      <c r="H313" s="2">
+      <c r="H313" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7827,7 +7801,7 @@
       <c r="G314" t="s">
         <v>172</v>
       </c>
-      <c r="H314" s="2">
+      <c r="H314" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="D315" t="s">
         <v>129</v>
       </c>
-      <c r="H315" s="2">
+      <c r="H315" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7867,7 +7841,7 @@
       <c r="G316" t="s">
         <v>173</v>
       </c>
-      <c r="H316" s="2">
+      <c r="H316" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7890,7 +7864,7 @@
       <c r="G317" t="s">
         <v>182</v>
       </c>
-      <c r="H317" s="2">
+      <c r="H317" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7913,7 +7887,7 @@
       <c r="G318" t="s">
         <v>174</v>
       </c>
-      <c r="H318" s="2">
+      <c r="H318" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7936,7 +7910,7 @@
       <c r="G319" t="s">
         <v>174</v>
       </c>
-      <c r="H319" s="2">
+      <c r="H319" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7959,7 +7933,7 @@
       <c r="G320" t="s">
         <v>175</v>
       </c>
-      <c r="H320" s="2">
+      <c r="H320" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7973,7 +7947,7 @@
       <c r="C321" t="s">
         <v>112</v>
       </c>
-      <c r="H321" s="2">
+      <c r="H321" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -7996,7 +7970,7 @@
       <c r="G322" t="s">
         <v>183</v>
       </c>
-      <c r="H322" s="2">
+      <c r="H322" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8010,7 +7984,7 @@
       <c r="C323" t="s">
         <v>112</v>
       </c>
-      <c r="H323" s="2">
+      <c r="H323" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8033,7 +8007,7 @@
       <c r="G324" t="s">
         <v>184</v>
       </c>
-      <c r="H324" s="2">
+      <c r="H324" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8047,7 +8021,7 @@
       <c r="C325" t="s">
         <v>112</v>
       </c>
-      <c r="H325" s="2">
+      <c r="H325" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8061,7 +8035,7 @@
       <c r="C326" t="s">
         <v>116</v>
       </c>
-      <c r="H326" s="2">
+      <c r="H326" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8075,7 +8049,7 @@
       <c r="C327" t="s">
         <v>116</v>
       </c>
-      <c r="H327" s="2">
+      <c r="H327" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8092,13 +8066,13 @@
       <c r="D328" t="s">
         <v>122</v>
       </c>
-      <c r="E328" s="2">
+      <c r="E328" s="1">
         <v>46234</v>
       </c>
       <c r="G328" t="s">
         <v>189</v>
       </c>
-      <c r="H328" s="2">
+      <c r="H328" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8121,7 +8095,7 @@
       <c r="G329" t="s">
         <v>184</v>
       </c>
-      <c r="H329" s="2">
+      <c r="H329" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8144,7 +8118,7 @@
       <c r="G330" t="s">
         <v>184</v>
       </c>
-      <c r="H330" s="2">
+      <c r="H330" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8158,7 +8132,7 @@
       <c r="C331" t="s">
         <v>112</v>
       </c>
-      <c r="H331" s="2">
+      <c r="H331" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8181,7 +8155,7 @@
       <c r="G332" t="s">
         <v>184</v>
       </c>
-      <c r="H332" s="2">
+      <c r="H332" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8204,7 +8178,7 @@
       <c r="G333" t="s">
         <v>183</v>
       </c>
-      <c r="H333" s="2">
+      <c r="H333" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8221,13 +8195,13 @@
       <c r="D334" t="s">
         <v>125</v>
       </c>
-      <c r="E334" s="2">
+      <c r="E334" s="1">
         <v>46237</v>
       </c>
       <c r="G334" t="s">
         <v>202</v>
       </c>
-      <c r="H334" s="2">
+      <c r="H334" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8241,7 +8215,7 @@
       <c r="C335" t="s">
         <v>112</v>
       </c>
-      <c r="H335" s="2">
+      <c r="H335" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8258,13 +8232,13 @@
       <c r="D336" t="s">
         <v>157</v>
       </c>
-      <c r="E336" s="2">
+      <c r="E336" s="1">
         <v>46227</v>
       </c>
       <c r="G336" t="s">
         <v>204</v>
       </c>
-      <c r="H336" s="2">
+      <c r="H336" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8278,7 +8252,7 @@
       <c r="C337" t="s">
         <v>112</v>
       </c>
-      <c r="H337" s="2">
+      <c r="H337" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8292,7 +8266,7 @@
       <c r="C338" t="s">
         <v>112</v>
       </c>
-      <c r="H338" s="2">
+      <c r="H338" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8315,7 +8289,7 @@
       <c r="G339" t="s">
         <v>181</v>
       </c>
-      <c r="H339" s="2">
+      <c r="H339" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8332,7 +8306,7 @@
       <c r="D340" t="s">
         <v>168</v>
       </c>
-      <c r="H340" s="2">
+      <c r="H340" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8346,7 +8320,7 @@
       <c r="C341" t="s">
         <v>116</v>
       </c>
-      <c r="H341" s="2">
+      <c r="H341" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8360,7 +8334,7 @@
       <c r="C342" t="s">
         <v>112</v>
       </c>
-      <c r="H342" s="2">
+      <c r="H342" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8383,7 +8357,7 @@
       <c r="G343" t="s">
         <v>172</v>
       </c>
-      <c r="H343" s="2">
+      <c r="H343" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8400,7 +8374,7 @@
       <c r="D344" t="s">
         <v>129</v>
       </c>
-      <c r="H344" s="2">
+      <c r="H344" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8423,7 +8397,7 @@
       <c r="G345" t="s">
         <v>173</v>
       </c>
-      <c r="H345" s="2">
+      <c r="H345" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8446,7 +8420,7 @@
       <c r="G346" t="s">
         <v>182</v>
       </c>
-      <c r="H346" s="2">
+      <c r="H346" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8469,7 +8443,7 @@
       <c r="G347" t="s">
         <v>174</v>
       </c>
-      <c r="H347" s="2">
+      <c r="H347" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8492,7 +8466,7 @@
       <c r="G348" t="s">
         <v>174</v>
       </c>
-      <c r="H348" s="2">
+      <c r="H348" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8515,7 +8489,7 @@
       <c r="G349" t="s">
         <v>175</v>
       </c>
-      <c r="H349" s="2">
+      <c r="H349" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8529,7 +8503,7 @@
       <c r="C350" t="s">
         <v>112</v>
       </c>
-      <c r="H350" s="2">
+      <c r="H350" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8552,7 +8526,7 @@
       <c r="G351" t="s">
         <v>183</v>
       </c>
-      <c r="H351" s="2">
+      <c r="H351" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8566,7 +8540,7 @@
       <c r="C352" t="s">
         <v>112</v>
       </c>
-      <c r="H352" s="2">
+      <c r="H352" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8580,7 +8554,7 @@
       <c r="C353" t="s">
         <v>112</v>
       </c>
-      <c r="H353" s="2">
+      <c r="H353" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8594,7 +8568,7 @@
       <c r="C354" t="s">
         <v>112</v>
       </c>
-      <c r="H354" s="2">
+      <c r="H354" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8608,7 +8582,7 @@
       <c r="C355" t="s">
         <v>116</v>
       </c>
-      <c r="H355" s="2">
+      <c r="H355" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8622,7 +8596,7 @@
       <c r="C356" t="s">
         <v>116</v>
       </c>
-      <c r="H356" s="2">
+      <c r="H356" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8645,7 +8619,7 @@
       <c r="G357" t="s">
         <v>185</v>
       </c>
-      <c r="H357" s="2">
+      <c r="H357" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8659,7 +8633,7 @@
       <c r="C358" t="s">
         <v>112</v>
       </c>
-      <c r="H358" s="2">
+      <c r="H358" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8682,7 +8656,7 @@
       <c r="G359" t="s">
         <v>186</v>
       </c>
-      <c r="H359" s="2">
+      <c r="H359" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8696,7 +8670,7 @@
       <c r="C360" t="s">
         <v>112</v>
       </c>
-      <c r="H360" s="2">
+      <c r="H360" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8710,7 +8684,7 @@
       <c r="C361" t="s">
         <v>112</v>
       </c>
-      <c r="H361" s="2">
+      <c r="H361" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8733,7 +8707,7 @@
       <c r="G362" t="s">
         <v>183</v>
       </c>
-      <c r="H362" s="2">
+      <c r="H362" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8756,7 +8730,7 @@
       <c r="G363" t="s">
         <v>187</v>
       </c>
-      <c r="H363" s="2">
+      <c r="H363" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8770,7 +8744,7 @@
       <c r="C364" t="s">
         <v>112</v>
       </c>
-      <c r="H364" s="2">
+      <c r="H364" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8793,7 +8767,7 @@
       <c r="G365" t="s">
         <v>186</v>
       </c>
-      <c r="H365" s="2">
+      <c r="H365" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8807,7 +8781,7 @@
       <c r="C366" t="s">
         <v>112</v>
       </c>
-      <c r="H366" s="2">
+      <c r="H366" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8821,7 +8795,7 @@
       <c r="C367" t="s">
         <v>112</v>
       </c>
-      <c r="H367" s="2">
+      <c r="H367" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8844,7 +8818,7 @@
       <c r="G368" t="s">
         <v>185</v>
       </c>
-      <c r="H368" s="2">
+      <c r="H368" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8867,7 +8841,7 @@
       <c r="G369" t="s">
         <v>186</v>
       </c>
-      <c r="H369" s="2">
+      <c r="H369" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8884,7 +8858,7 @@
       <c r="D370" t="s">
         <v>168</v>
       </c>
-      <c r="H370" s="2">
+      <c r="H370" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8898,7 +8872,7 @@
       <c r="C371" t="s">
         <v>112</v>
       </c>
-      <c r="H371" s="2">
+      <c r="H371" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8921,7 +8895,7 @@
       <c r="G372" t="s">
         <v>172</v>
       </c>
-      <c r="H372" s="2">
+      <c r="H372" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8938,7 +8912,7 @@
       <c r="D373" t="s">
         <v>129</v>
       </c>
-      <c r="H373" s="2">
+      <c r="H373" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8961,7 +8935,7 @@
       <c r="G374" t="s">
         <v>173</v>
       </c>
-      <c r="H374" s="2">
+      <c r="H374" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8984,7 +8958,7 @@
       <c r="G375" t="s">
         <v>182</v>
       </c>
-      <c r="H375" s="2">
+      <c r="H375" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9007,7 +8981,7 @@
       <c r="G376" t="s">
         <v>174</v>
       </c>
-      <c r="H376" s="2">
+      <c r="H376" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9030,7 +9004,7 @@
       <c r="G377" t="s">
         <v>174</v>
       </c>
-      <c r="H377" s="2">
+      <c r="H377" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9053,7 +9027,7 @@
       <c r="G378" t="s">
         <v>175</v>
       </c>
-      <c r="H378" s="2">
+      <c r="H378" s="1">
         <v>46225</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (23/07/2026 16:16)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -651,16 +651,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -676,7 +668,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -684,30 +676,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1007,72 +981,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1137,7 +1111,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1202,7 +1176,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1267,7 +1241,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1332,7 +1306,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1397,7 +1371,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1462,7 +1436,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1527,7 +1501,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1592,7 +1566,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1657,7 +1631,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1722,7 +1696,7 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>46220</v>
       </c>
       <c r="B12">
@@ -1787,7 +1761,7 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46224</v>
       </c>
       <c r="B13">
@@ -1852,7 +1826,7 @@
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46225</v>
       </c>
       <c r="B14">
@@ -1917,7 +1891,7 @@
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46226</v>
       </c>
       <c r="B15">
@@ -1992,28 +1966,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>74</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>75</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2027,7 +2001,7 @@
       <c r="C2" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2041,7 +2015,7 @@
       <c r="C3" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2064,7 +2038,7 @@
       <c r="G4" t="s">
         <v>174</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2078,7 +2052,7 @@
       <c r="C5" t="s">
         <v>115</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2092,7 +2066,7 @@
       <c r="C6" t="s">
         <v>115</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2109,13 +2083,13 @@
       <c r="D7" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2132,13 +2106,13 @@
       <c r="D8" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>192</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2155,13 +2129,13 @@
       <c r="D9" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>193</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2178,13 +2152,13 @@
       <c r="D10" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>194</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2198,7 +2172,7 @@
       <c r="C11" t="s">
         <v>115</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2212,7 +2186,7 @@
       <c r="C12" t="s">
         <v>115</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2229,13 +2203,13 @@
       <c r="D13" t="s">
         <v>127</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>192</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2249,7 +2223,7 @@
       <c r="C14" t="s">
         <v>119</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2266,13 +2240,13 @@
       <c r="D15" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>195</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2286,7 +2260,7 @@
       <c r="C16" t="s">
         <v>115</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2300,7 +2274,7 @@
       <c r="C17" t="s">
         <v>115</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2317,13 +2291,13 @@
       <c r="D18" t="s">
         <v>129</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>196</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2337,7 +2311,7 @@
       <c r="C19" t="s">
         <v>115</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2354,13 +2328,13 @@
       <c r="D20" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>192</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2383,7 +2357,7 @@
       <c r="G21" t="s">
         <v>175</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2397,7 +2371,7 @@
       <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2411,7 +2385,7 @@
       <c r="C23" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2434,7 +2408,7 @@
       <c r="G24" t="s">
         <v>176</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2451,7 +2425,7 @@
       <c r="D25" t="s">
         <v>132</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2474,7 +2448,7 @@
       <c r="G26" t="s">
         <v>177</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2491,13 +2465,13 @@
       <c r="D27" t="s">
         <v>134</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>197</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2520,7 +2494,7 @@
       <c r="G28" t="s">
         <v>178</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2543,7 +2517,7 @@
       <c r="G29" t="s">
         <v>178</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2566,7 +2540,7 @@
       <c r="G30" t="s">
         <v>179</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2580,7 +2554,7 @@
       <c r="C31" t="s">
         <v>115</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2594,7 +2568,7 @@
       <c r="C32" t="s">
         <v>115</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2617,7 +2591,7 @@
       <c r="G33" t="s">
         <v>180</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2631,7 +2605,7 @@
       <c r="C34" t="s">
         <v>115</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2645,7 +2619,7 @@
       <c r="C35" t="s">
         <v>115</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2662,13 +2636,13 @@
       <c r="D36" t="s">
         <v>123</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>192</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2685,13 +2659,13 @@
       <c r="D37" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>192</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2708,13 +2682,13 @@
       <c r="D38" t="s">
         <v>125</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>193</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2731,13 +2705,13 @@
       <c r="D39" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>194</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2751,7 +2725,7 @@
       <c r="C40" t="s">
         <v>115</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2765,7 +2739,7 @@
       <c r="C41" t="s">
         <v>115</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2782,13 +2756,13 @@
       <c r="D42" t="s">
         <v>127</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>192</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2802,7 +2776,7 @@
       <c r="C43" t="s">
         <v>115</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2819,13 +2793,13 @@
       <c r="D44" t="s">
         <v>128</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>195</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2839,7 +2813,7 @@
       <c r="C45" t="s">
         <v>115</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2853,7 +2827,7 @@
       <c r="C46" t="s">
         <v>115</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="C47" t="s">
         <v>119</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2881,7 +2855,7 @@
       <c r="C48" t="s">
         <v>115</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2898,13 +2872,13 @@
       <c r="D49" t="s">
         <v>139</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>192</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2927,7 +2901,7 @@
       <c r="G50" t="s">
         <v>175</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2941,7 +2915,7 @@
       <c r="C51" t="s">
         <v>119</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2955,7 +2929,7 @@
       <c r="C52" t="s">
         <v>115</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2978,7 +2952,7 @@
       <c r="G53" t="s">
         <v>176</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2995,7 +2969,7 @@
       <c r="D54" t="s">
         <v>132</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3018,7 +2992,7 @@
       <c r="G55" t="s">
         <v>177</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3035,13 +3009,13 @@
       <c r="D56" t="s">
         <v>134</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>197</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3064,7 +3038,7 @@
       <c r="G57" t="s">
         <v>178</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3087,7 +3061,7 @@
       <c r="G58" t="s">
         <v>178</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3110,7 +3084,7 @@
       <c r="G59" t="s">
         <v>179</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3124,7 +3098,7 @@
       <c r="C60" t="s">
         <v>115</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3138,7 +3112,7 @@
       <c r="C61" t="s">
         <v>115</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3155,13 +3129,13 @@
       <c r="D62" t="s">
         <v>138</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>198</v>
       </c>
-      <c r="H62" s="2">
+      <c r="H62" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3175,7 +3149,7 @@
       <c r="C63" t="s">
         <v>115</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3192,13 +3166,13 @@
       <c r="D64" t="s">
         <v>140</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>199</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3212,7 +3186,7 @@
       <c r="C65" t="s">
         <v>115</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3226,7 +3200,7 @@
       <c r="C66" t="s">
         <v>119</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3243,13 +3217,13 @@
       <c r="D67" t="s">
         <v>125</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>193</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3266,13 +3240,13 @@
       <c r="D68" t="s">
         <v>126</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>194</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3286,7 +3260,7 @@
       <c r="C69" t="s">
         <v>115</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3300,7 +3274,7 @@
       <c r="C70" t="s">
         <v>115</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3317,13 +3291,13 @@
       <c r="D71" t="s">
         <v>127</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>198</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3337,7 +3311,7 @@
       <c r="C72" t="s">
         <v>115</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3354,13 +3328,13 @@
       <c r="D73" t="s">
         <v>128</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>195</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3374,7 +3348,7 @@
       <c r="C74" t="s">
         <v>115</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3388,7 +3362,7 @@
       <c r="C75" t="s">
         <v>115</v>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3402,7 +3376,7 @@
       <c r="C76" t="s">
         <v>115</v>
       </c>
-      <c r="H76" s="2">
+      <c r="H76" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3416,7 +3390,7 @@
       <c r="C77" t="s">
         <v>115</v>
       </c>
-      <c r="H77" s="2">
+      <c r="H77" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3433,13 +3407,13 @@
       <c r="D78" t="s">
         <v>139</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="1">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>198</v>
       </c>
-      <c r="H78" s="2">
+      <c r="H78" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3462,7 +3436,7 @@
       <c r="G79" t="s">
         <v>181</v>
       </c>
-      <c r="H79" s="2">
+      <c r="H79" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3476,7 +3450,7 @@
       <c r="C80" t="s">
         <v>119</v>
       </c>
-      <c r="H80" s="2">
+      <c r="H80" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3490,7 +3464,7 @@
       <c r="C81" t="s">
         <v>115</v>
       </c>
-      <c r="H81" s="2">
+      <c r="H81" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3513,7 +3487,7 @@
       <c r="G82" t="s">
         <v>176</v>
       </c>
-      <c r="H82" s="2">
+      <c r="H82" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3530,7 +3504,7 @@
       <c r="D83" t="s">
         <v>132</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3553,7 +3527,7 @@
       <c r="G84" t="s">
         <v>177</v>
       </c>
-      <c r="H84" s="2">
+      <c r="H84" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3570,13 +3544,13 @@
       <c r="D85" t="s">
         <v>134</v>
       </c>
-      <c r="E85" s="2">
+      <c r="E85" s="1">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>197</v>
       </c>
-      <c r="H85" s="2">
+      <c r="H85" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3599,7 +3573,7 @@
       <c r="G86" t="s">
         <v>178</v>
       </c>
-      <c r="H86" s="2">
+      <c r="H86" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3622,7 +3596,7 @@
       <c r="G87" t="s">
         <v>178</v>
       </c>
-      <c r="H87" s="2">
+      <c r="H87" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3645,7 +3619,7 @@
       <c r="G88" t="s">
         <v>179</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3659,7 +3633,7 @@
       <c r="C89" t="s">
         <v>115</v>
       </c>
-      <c r="H89" s="2">
+      <c r="H89" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3676,13 +3650,13 @@
       <c r="D90" t="s">
         <v>142</v>
       </c>
-      <c r="E90" s="2">
+      <c r="E90" s="1">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>199</v>
       </c>
-      <c r="H90" s="2">
+      <c r="H90" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3699,13 +3673,13 @@
       <c r="D91" t="s">
         <v>138</v>
       </c>
-      <c r="E91" s="2">
+      <c r="E91" s="1">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>198</v>
       </c>
-      <c r="H91" s="2">
+      <c r="H91" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3719,7 +3693,7 @@
       <c r="C92" t="s">
         <v>115</v>
       </c>
-      <c r="H92" s="2">
+      <c r="H92" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3736,13 +3710,13 @@
       <c r="D93" t="s">
         <v>140</v>
       </c>
-      <c r="E93" s="2">
+      <c r="E93" s="1">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>199</v>
       </c>
-      <c r="H93" s="2">
+      <c r="H93" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3756,7 +3730,7 @@
       <c r="C94" t="s">
         <v>115</v>
       </c>
-      <c r="H94" s="2">
+      <c r="H94" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3770,7 +3744,7 @@
       <c r="C95" t="s">
         <v>119</v>
       </c>
-      <c r="H95" s="2">
+      <c r="H95" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3787,13 +3761,13 @@
       <c r="D96" t="s">
         <v>125</v>
       </c>
-      <c r="E96" s="2">
+      <c r="E96" s="1">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>193</v>
       </c>
-      <c r="H96" s="2">
+      <c r="H96" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3810,13 +3784,13 @@
       <c r="D97" t="s">
         <v>126</v>
       </c>
-      <c r="E97" s="2">
+      <c r="E97" s="1">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>194</v>
       </c>
-      <c r="H97" s="2">
+      <c r="H97" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3830,7 +3804,7 @@
       <c r="C98" t="s">
         <v>115</v>
       </c>
-      <c r="H98" s="2">
+      <c r="H98" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3847,13 +3821,13 @@
       <c r="D99" t="s">
         <v>143</v>
       </c>
-      <c r="E99" s="2">
+      <c r="E99" s="1">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>194</v>
       </c>
-      <c r="H99" s="2">
+      <c r="H99" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3870,13 +3844,13 @@
       <c r="D100" t="s">
         <v>127</v>
       </c>
-      <c r="E100" s="2">
+      <c r="E100" s="1">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>194</v>
       </c>
-      <c r="H100" s="2">
+      <c r="H100" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3890,7 +3864,7 @@
       <c r="C101" t="s">
         <v>115</v>
       </c>
-      <c r="H101" s="2">
+      <c r="H101" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3907,13 +3881,13 @@
       <c r="D102" t="s">
         <v>128</v>
       </c>
-      <c r="E102" s="2">
+      <c r="E102" s="1">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>195</v>
       </c>
-      <c r="H102" s="2">
+      <c r="H102" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3930,13 +3904,13 @@
       <c r="D103" t="s">
         <v>144</v>
       </c>
-      <c r="E103" s="2">
+      <c r="E103" s="1">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>194</v>
       </c>
-      <c r="H103" s="2">
+      <c r="H103" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3950,7 +3924,7 @@
       <c r="C104" t="s">
         <v>115</v>
       </c>
-      <c r="H104" s="2">
+      <c r="H104" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3964,7 +3938,7 @@
       <c r="C105" t="s">
         <v>115</v>
       </c>
-      <c r="H105" s="2">
+      <c r="H105" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3978,7 +3952,7 @@
       <c r="C106" t="s">
         <v>115</v>
       </c>
-      <c r="H106" s="2">
+      <c r="H106" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3995,13 +3969,13 @@
       <c r="D107" t="s">
         <v>145</v>
       </c>
-      <c r="E107" s="2">
+      <c r="E107" s="1">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>194</v>
       </c>
-      <c r="H107" s="2">
+      <c r="H107" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4024,7 +3998,7 @@
       <c r="G108" t="s">
         <v>181</v>
       </c>
-      <c r="H108" s="2">
+      <c r="H108" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4038,7 +4012,7 @@
       <c r="C109" t="s">
         <v>119</v>
       </c>
-      <c r="H109" s="2">
+      <c r="H109" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4052,7 +4026,7 @@
       <c r="C110" t="s">
         <v>115</v>
       </c>
-      <c r="H110" s="2">
+      <c r="H110" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4075,7 +4049,7 @@
       <c r="G111" t="s">
         <v>176</v>
       </c>
-      <c r="H111" s="2">
+      <c r="H111" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4092,7 +4066,7 @@
       <c r="D112" t="s">
         <v>132</v>
       </c>
-      <c r="H112" s="2">
+      <c r="H112" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4115,7 +4089,7 @@
       <c r="G113" t="s">
         <v>177</v>
       </c>
-      <c r="H113" s="2">
+      <c r="H113" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4132,13 +4106,13 @@
       <c r="D114" t="s">
         <v>134</v>
       </c>
-      <c r="E114" s="2">
+      <c r="E114" s="1">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>197</v>
       </c>
-      <c r="H114" s="2">
+      <c r="H114" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4161,7 +4135,7 @@
       <c r="G115" t="s">
         <v>178</v>
       </c>
-      <c r="H115" s="2">
+      <c r="H115" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4184,7 +4158,7 @@
       <c r="G116" t="s">
         <v>178</v>
       </c>
-      <c r="H116" s="2">
+      <c r="H116" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4207,7 +4181,7 @@
       <c r="G117" t="s">
         <v>179</v>
       </c>
-      <c r="H117" s="2">
+      <c r="H117" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4221,7 +4195,7 @@
       <c r="C118" t="s">
         <v>115</v>
       </c>
-      <c r="H118" s="2">
+      <c r="H118" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4238,13 +4212,13 @@
       <c r="D119" t="s">
         <v>142</v>
       </c>
-      <c r="E119" s="2">
+      <c r="E119" s="1">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>199</v>
       </c>
-      <c r="H119" s="2">
+      <c r="H119" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4258,7 +4232,7 @@
       <c r="C120" t="s">
         <v>119</v>
       </c>
-      <c r="H120" s="2">
+      <c r="H120" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4272,7 +4246,7 @@
       <c r="C121" t="s">
         <v>115</v>
       </c>
-      <c r="H121" s="2">
+      <c r="H121" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4286,7 +4260,7 @@
       <c r="C122" t="s">
         <v>119</v>
       </c>
-      <c r="H122" s="2">
+      <c r="H122" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4300,7 +4274,7 @@
       <c r="C123" t="s">
         <v>119</v>
       </c>
-      <c r="H123" s="2">
+      <c r="H123" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="C124" t="s">
         <v>119</v>
       </c>
-      <c r="H124" s="2">
+      <c r="H124" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4331,13 +4305,13 @@
       <c r="D125" t="s">
         <v>125</v>
       </c>
-      <c r="E125" s="2">
+      <c r="E125" s="1">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>193</v>
       </c>
-      <c r="H125" s="2">
+      <c r="H125" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4354,13 +4328,13 @@
       <c r="D126" t="s">
         <v>126</v>
       </c>
-      <c r="E126" s="2">
+      <c r="E126" s="1">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>194</v>
       </c>
-      <c r="H126" s="2">
+      <c r="H126" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4374,7 +4348,7 @@
       <c r="C127" t="s">
         <v>115</v>
       </c>
-      <c r="H127" s="2">
+      <c r="H127" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4391,13 +4365,13 @@
       <c r="D128" t="s">
         <v>143</v>
       </c>
-      <c r="E128" s="2">
+      <c r="E128" s="1">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>194</v>
       </c>
-      <c r="H128" s="2">
+      <c r="H128" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4414,13 +4388,13 @@
       <c r="D129" t="s">
         <v>127</v>
       </c>
-      <c r="E129" s="2">
+      <c r="E129" s="1">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>194</v>
       </c>
-      <c r="H129" s="2">
+      <c r="H129" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4434,7 +4408,7 @@
       <c r="C130" t="s">
         <v>115</v>
       </c>
-      <c r="H130" s="2">
+      <c r="H130" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4451,13 +4425,13 @@
       <c r="D131" t="s">
         <v>128</v>
       </c>
-      <c r="E131" s="2">
+      <c r="E131" s="1">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>195</v>
       </c>
-      <c r="H131" s="2">
+      <c r="H131" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4474,13 +4448,13 @@
       <c r="D132" t="s">
         <v>144</v>
       </c>
-      <c r="E132" s="2">
+      <c r="E132" s="1">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>194</v>
       </c>
-      <c r="H132" s="2">
+      <c r="H132" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4494,7 +4468,7 @@
       <c r="C133" t="s">
         <v>115</v>
       </c>
-      <c r="H133" s="2">
+      <c r="H133" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4508,7 +4482,7 @@
       <c r="C134" t="s">
         <v>115</v>
       </c>
-      <c r="H134" s="2">
+      <c r="H134" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4522,7 +4496,7 @@
       <c r="C135" t="s">
         <v>115</v>
       </c>
-      <c r="H135" s="2">
+      <c r="H135" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4539,13 +4513,13 @@
       <c r="D136" t="s">
         <v>146</v>
       </c>
-      <c r="E136" s="2">
+      <c r="E136" s="1">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>194</v>
       </c>
-      <c r="H136" s="2">
+      <c r="H136" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4568,7 +4542,7 @@
       <c r="G137" t="s">
         <v>181</v>
       </c>
-      <c r="H137" s="2">
+      <c r="H137" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4582,7 +4556,7 @@
       <c r="C138" t="s">
         <v>119</v>
       </c>
-      <c r="H138" s="2">
+      <c r="H138" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4596,7 +4570,7 @@
       <c r="C139" t="s">
         <v>115</v>
       </c>
-      <c r="H139" s="2">
+      <c r="H139" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4619,7 +4593,7 @@
       <c r="G140" t="s">
         <v>176</v>
       </c>
-      <c r="H140" s="2">
+      <c r="H140" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4636,7 +4610,7 @@
       <c r="D141" t="s">
         <v>132</v>
       </c>
-      <c r="H141" s="2">
+      <c r="H141" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4659,7 +4633,7 @@
       <c r="G142" t="s">
         <v>177</v>
       </c>
-      <c r="H142" s="2">
+      <c r="H142" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4676,13 +4650,13 @@
       <c r="D143" t="s">
         <v>134</v>
       </c>
-      <c r="E143" s="2">
+      <c r="E143" s="1">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>197</v>
       </c>
-      <c r="H143" s="2">
+      <c r="H143" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4705,7 +4679,7 @@
       <c r="G144" t="s">
         <v>178</v>
       </c>
-      <c r="H144" s="2">
+      <c r="H144" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4728,7 +4702,7 @@
       <c r="G145" t="s">
         <v>178</v>
       </c>
-      <c r="H145" s="2">
+      <c r="H145" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4751,7 +4725,7 @@
       <c r="G146" t="s">
         <v>179</v>
       </c>
-      <c r="H146" s="2">
+      <c r="H146" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4765,7 +4739,7 @@
       <c r="C147" t="s">
         <v>115</v>
       </c>
-      <c r="H147" s="2">
+      <c r="H147" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4782,13 +4756,13 @@
       <c r="D148" t="s">
         <v>142</v>
       </c>
-      <c r="E148" s="2">
+      <c r="E148" s="1">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>199</v>
       </c>
-      <c r="H148" s="2">
+      <c r="H148" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4802,7 +4776,7 @@
       <c r="C149" t="s">
         <v>119</v>
       </c>
-      <c r="H149" s="2">
+      <c r="H149" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4816,7 +4790,7 @@
       <c r="C150" t="s">
         <v>115</v>
       </c>
-      <c r="H150" s="2">
+      <c r="H150" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4830,7 +4804,7 @@
       <c r="C151" t="s">
         <v>115</v>
       </c>
-      <c r="H151" s="2">
+      <c r="H151" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4844,7 +4818,7 @@
       <c r="C152" t="s">
         <v>119</v>
       </c>
-      <c r="H152" s="2">
+      <c r="H152" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4858,7 +4832,7 @@
       <c r="C153" t="s">
         <v>119</v>
       </c>
-      <c r="H153" s="2">
+      <c r="H153" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4875,13 +4849,13 @@
       <c r="D154" t="s">
         <v>125</v>
       </c>
-      <c r="E154" s="2">
+      <c r="E154" s="1">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>193</v>
       </c>
-      <c r="H154" s="2">
+      <c r="H154" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4898,13 +4872,13 @@
       <c r="D155" t="s">
         <v>126</v>
       </c>
-      <c r="E155" s="2">
+      <c r="E155" s="1">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>194</v>
       </c>
-      <c r="H155" s="2">
+      <c r="H155" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4918,7 +4892,7 @@
       <c r="C156" t="s">
         <v>115</v>
       </c>
-      <c r="H156" s="2">
+      <c r="H156" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4935,13 +4909,13 @@
       <c r="D157" t="s">
         <v>143</v>
       </c>
-      <c r="E157" s="2">
+      <c r="E157" s="1">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>194</v>
       </c>
-      <c r="H157" s="2">
+      <c r="H157" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4958,13 +4932,13 @@
       <c r="D158" t="s">
         <v>127</v>
       </c>
-      <c r="E158" s="2">
+      <c r="E158" s="1">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>194</v>
       </c>
-      <c r="H158" s="2">
+      <c r="H158" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4981,13 +4955,13 @@
       <c r="D159" t="s">
         <v>147</v>
       </c>
-      <c r="E159" s="2">
+      <c r="E159" s="1">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>200</v>
       </c>
-      <c r="H159" s="2">
+      <c r="H159" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5004,13 +4978,13 @@
       <c r="D160" t="s">
         <v>128</v>
       </c>
-      <c r="E160" s="2">
+      <c r="E160" s="1">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>195</v>
       </c>
-      <c r="H160" s="2">
+      <c r="H160" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5027,13 +5001,13 @@
       <c r="D161" t="s">
         <v>144</v>
       </c>
-      <c r="E161" s="2">
+      <c r="E161" s="1">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>194</v>
       </c>
-      <c r="H161" s="2">
+      <c r="H161" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5047,7 +5021,7 @@
       <c r="C162" t="s">
         <v>115</v>
       </c>
-      <c r="H162" s="2">
+      <c r="H162" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5061,7 +5035,7 @@
       <c r="C163" t="s">
         <v>115</v>
       </c>
-      <c r="H163" s="2">
+      <c r="H163" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5075,7 +5049,7 @@
       <c r="C164" t="s">
         <v>115</v>
       </c>
-      <c r="H164" s="2">
+      <c r="H164" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5092,13 +5066,13 @@
       <c r="D165" t="s">
         <v>146</v>
       </c>
-      <c r="E165" s="2">
+      <c r="E165" s="1">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>194</v>
       </c>
-      <c r="H165" s="2">
+      <c r="H165" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5121,7 +5095,7 @@
       <c r="G166" t="s">
         <v>181</v>
       </c>
-      <c r="H166" s="2">
+      <c r="H166" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5135,7 +5109,7 @@
       <c r="C167" t="s">
         <v>119</v>
       </c>
-      <c r="H167" s="2">
+      <c r="H167" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5149,7 +5123,7 @@
       <c r="C168" t="s">
         <v>115</v>
       </c>
-      <c r="H168" s="2">
+      <c r="H168" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5172,7 +5146,7 @@
       <c r="G169" t="s">
         <v>176</v>
       </c>
-      <c r="H169" s="2">
+      <c r="H169" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5189,7 +5163,7 @@
       <c r="D170" t="s">
         <v>132</v>
       </c>
-      <c r="H170" s="2">
+      <c r="H170" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5212,7 +5186,7 @@
       <c r="G171" t="s">
         <v>177</v>
       </c>
-      <c r="H171" s="2">
+      <c r="H171" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5229,13 +5203,13 @@
       <c r="D172" t="s">
         <v>134</v>
       </c>
-      <c r="E172" s="2">
+      <c r="E172" s="1">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>197</v>
       </c>
-      <c r="H172" s="2">
+      <c r="H172" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5258,7 +5232,7 @@
       <c r="G173" t="s">
         <v>178</v>
       </c>
-      <c r="H173" s="2">
+      <c r="H173" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5281,7 +5255,7 @@
       <c r="G174" t="s">
         <v>178</v>
       </c>
-      <c r="H174" s="2">
+      <c r="H174" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5304,7 +5278,7 @@
       <c r="G175" t="s">
         <v>179</v>
       </c>
-      <c r="H175" s="2">
+      <c r="H175" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5318,7 +5292,7 @@
       <c r="C176" t="s">
         <v>115</v>
       </c>
-      <c r="H176" s="2">
+      <c r="H176" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5335,13 +5309,13 @@
       <c r="D177" t="s">
         <v>148</v>
       </c>
-      <c r="E177" s="2">
+      <c r="E177" s="1">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>199</v>
       </c>
-      <c r="H177" s="2">
+      <c r="H177" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5355,7 +5329,7 @@
       <c r="C178" t="s">
         <v>115</v>
       </c>
-      <c r="H178" s="2">
+      <c r="H178" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5372,13 +5346,13 @@
       <c r="D179" t="s">
         <v>149</v>
       </c>
-      <c r="E179" s="2">
+      <c r="E179" s="1">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>195</v>
       </c>
-      <c r="H179" s="2">
+      <c r="H179" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5392,7 +5366,7 @@
       <c r="C180" t="s">
         <v>115</v>
       </c>
-      <c r="H180" s="2">
+      <c r="H180" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5406,7 +5380,7 @@
       <c r="C181" t="s">
         <v>119</v>
       </c>
-      <c r="H181" s="2">
+      <c r="H181" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5420,7 +5394,7 @@
       <c r="C182" t="s">
         <v>119</v>
       </c>
-      <c r="H182" s="2">
+      <c r="H182" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5437,13 +5411,13 @@
       <c r="D183" t="s">
         <v>125</v>
       </c>
-      <c r="E183" s="2">
+      <c r="E183" s="1">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>193</v>
       </c>
-      <c r="H183" s="2">
+      <c r="H183" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5460,13 +5434,13 @@
       <c r="D184" t="s">
         <v>126</v>
       </c>
-      <c r="E184" s="2">
+      <c r="E184" s="1">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>194</v>
       </c>
-      <c r="H184" s="2">
+      <c r="H184" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5480,7 +5454,7 @@
       <c r="C185" t="s">
         <v>115</v>
       </c>
-      <c r="H185" s="2">
+      <c r="H185" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5497,13 +5471,13 @@
       <c r="D186" t="s">
         <v>143</v>
       </c>
-      <c r="E186" s="2">
+      <c r="E186" s="1">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>194</v>
       </c>
-      <c r="H186" s="2">
+      <c r="H186" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5520,13 +5494,13 @@
       <c r="D187" t="s">
         <v>150</v>
       </c>
-      <c r="E187" s="2">
+      <c r="E187" s="1">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>194</v>
       </c>
-      <c r="H187" s="2">
+      <c r="H187" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5543,13 +5517,13 @@
       <c r="D188" t="s">
         <v>151</v>
       </c>
-      <c r="E188" s="2">
+      <c r="E188" s="1">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>194</v>
       </c>
-      <c r="H188" s="2">
+      <c r="H188" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5566,13 +5540,13 @@
       <c r="D189" t="s">
         <v>128</v>
       </c>
-      <c r="E189" s="2">
+      <c r="E189" s="1">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>195</v>
       </c>
-      <c r="H189" s="2">
+      <c r="H189" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5589,13 +5563,13 @@
       <c r="D190" t="s">
         <v>144</v>
       </c>
-      <c r="E190" s="2">
+      <c r="E190" s="1">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>194</v>
       </c>
-      <c r="H190" s="2">
+      <c r="H190" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5609,7 +5583,7 @@
       <c r="C191" t="s">
         <v>115</v>
       </c>
-      <c r="H191" s="2">
+      <c r="H191" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5623,7 +5597,7 @@
       <c r="C192" t="s">
         <v>115</v>
       </c>
-      <c r="H192" s="2">
+      <c r="H192" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5637,7 +5611,7 @@
       <c r="C193" t="s">
         <v>115</v>
       </c>
-      <c r="H193" s="2">
+      <c r="H193" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5654,13 +5628,13 @@
       <c r="D194" t="s">
         <v>146</v>
       </c>
-      <c r="E194" s="2">
+      <c r="E194" s="1">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>201</v>
       </c>
-      <c r="H194" s="2">
+      <c r="H194" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5683,7 +5657,7 @@
       <c r="G195" t="s">
         <v>181</v>
       </c>
-      <c r="H195" s="2">
+      <c r="H195" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5697,7 +5671,7 @@
       <c r="C196" t="s">
         <v>119</v>
       </c>
-      <c r="H196" s="2">
+      <c r="H196" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5711,7 +5685,7 @@
       <c r="C197" t="s">
         <v>115</v>
       </c>
-      <c r="H197" s="2">
+      <c r="H197" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5734,7 +5708,7 @@
       <c r="G198" t="s">
         <v>176</v>
       </c>
-      <c r="H198" s="2">
+      <c r="H198" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5751,7 +5725,7 @@
       <c r="D199" t="s">
         <v>132</v>
       </c>
-      <c r="H199" s="2">
+      <c r="H199" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5774,7 +5748,7 @@
       <c r="G200" t="s">
         <v>177</v>
       </c>
-      <c r="H200" s="2">
+      <c r="H200" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5791,13 +5765,13 @@
       <c r="D201" t="s">
         <v>134</v>
       </c>
-      <c r="E201" s="2">
+      <c r="E201" s="1">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>197</v>
       </c>
-      <c r="H201" s="2">
+      <c r="H201" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5820,7 +5794,7 @@
       <c r="G202" t="s">
         <v>178</v>
       </c>
-      <c r="H202" s="2">
+      <c r="H202" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5843,7 +5817,7 @@
       <c r="G203" t="s">
         <v>178</v>
       </c>
-      <c r="H203" s="2">
+      <c r="H203" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5866,7 +5840,7 @@
       <c r="G204" t="s">
         <v>179</v>
       </c>
-      <c r="H204" s="2">
+      <c r="H204" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5880,7 +5854,7 @@
       <c r="C205" t="s">
         <v>115</v>
       </c>
-      <c r="H205" s="2">
+      <c r="H205" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5897,13 +5871,13 @@
       <c r="D206" t="s">
         <v>148</v>
       </c>
-      <c r="E206" s="2">
+      <c r="E206" s="1">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>199</v>
       </c>
-      <c r="H206" s="2">
+      <c r="H206" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5917,7 +5891,7 @@
       <c r="C207" t="s">
         <v>115</v>
       </c>
-      <c r="H207" s="2">
+      <c r="H207" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5931,7 +5905,7 @@
       <c r="C208" t="s">
         <v>119</v>
       </c>
-      <c r="H208" s="2">
+      <c r="H208" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5945,7 +5919,7 @@
       <c r="C209" t="s">
         <v>115</v>
       </c>
-      <c r="H209" s="2">
+      <c r="H209" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5959,7 +5933,7 @@
       <c r="C210" t="s">
         <v>119</v>
       </c>
-      <c r="H210" s="2">
+      <c r="H210" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5973,7 +5947,7 @@
       <c r="C211" t="s">
         <v>119</v>
       </c>
-      <c r="H211" s="2">
+      <c r="H211" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5990,13 +5964,13 @@
       <c r="D212" t="s">
         <v>125</v>
       </c>
-      <c r="E212" s="2">
+      <c r="E212" s="1">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>193</v>
       </c>
-      <c r="H212" s="2">
+      <c r="H212" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6010,7 +5984,7 @@
       <c r="C213" t="s">
         <v>119</v>
       </c>
-      <c r="H213" s="2">
+      <c r="H213" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6024,7 +5998,7 @@
       <c r="C214" t="s">
         <v>115</v>
       </c>
-      <c r="H214" s="2">
+      <c r="H214" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6041,13 +6015,13 @@
       <c r="D215" t="s">
         <v>143</v>
       </c>
-      <c r="E215" s="2">
+      <c r="E215" s="1">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>202</v>
       </c>
-      <c r="H215" s="2">
+      <c r="H215" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6064,13 +6038,13 @@
       <c r="D216" t="s">
         <v>150</v>
       </c>
-      <c r="E216" s="2">
+      <c r="E216" s="1">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>195</v>
       </c>
-      <c r="H216" s="2">
+      <c r="H216" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6084,7 +6058,7 @@
       <c r="C217" t="s">
         <v>115</v>
       </c>
-      <c r="H217" s="2">
+      <c r="H217" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6101,13 +6075,13 @@
       <c r="D218" t="s">
         <v>128</v>
       </c>
-      <c r="E218" s="2">
+      <c r="E218" s="1">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>195</v>
       </c>
-      <c r="H218" s="2">
+      <c r="H218" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6121,7 +6095,7 @@
       <c r="C219" t="s">
         <v>115</v>
       </c>
-      <c r="H219" s="2">
+      <c r="H219" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6135,7 +6109,7 @@
       <c r="C220" t="s">
         <v>115</v>
       </c>
-      <c r="H220" s="2">
+      <c r="H220" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6152,13 +6126,13 @@
       <c r="D221" t="s">
         <v>152</v>
       </c>
-      <c r="E221" s="2">
+      <c r="E221" s="1">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>199</v>
       </c>
-      <c r="H221" s="2">
+      <c r="H221" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6172,7 +6146,7 @@
       <c r="C222" t="s">
         <v>115</v>
       </c>
-      <c r="H222" s="2">
+      <c r="H222" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6189,13 +6163,13 @@
       <c r="D223" t="s">
         <v>153</v>
       </c>
-      <c r="E223" s="2">
+      <c r="E223" s="1">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>203</v>
       </c>
-      <c r="H223" s="2">
+      <c r="H223" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6218,7 +6192,7 @@
       <c r="G224" t="s">
         <v>181</v>
       </c>
-      <c r="H224" s="2">
+      <c r="H224" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6232,7 +6206,7 @@
       <c r="C225" t="s">
         <v>119</v>
       </c>
-      <c r="H225" s="2">
+      <c r="H225" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="C226" t="s">
         <v>115</v>
       </c>
-      <c r="H226" s="2">
+      <c r="H226" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6269,7 +6243,7 @@
       <c r="G227" t="s">
         <v>176</v>
       </c>
-      <c r="H227" s="2">
+      <c r="H227" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6286,7 +6260,7 @@
       <c r="D228" t="s">
         <v>132</v>
       </c>
-      <c r="H228" s="2">
+      <c r="H228" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6309,7 +6283,7 @@
       <c r="G229" t="s">
         <v>177</v>
       </c>
-      <c r="H229" s="2">
+      <c r="H229" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6326,13 +6300,13 @@
       <c r="D230" t="s">
         <v>154</v>
       </c>
-      <c r="E230" s="2">
+      <c r="E230" s="1">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>204</v>
       </c>
-      <c r="H230" s="2">
+      <c r="H230" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6355,7 +6329,7 @@
       <c r="G231" t="s">
         <v>178</v>
       </c>
-      <c r="H231" s="2">
+      <c r="H231" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="G232" t="s">
         <v>178</v>
       </c>
-      <c r="H232" s="2">
+      <c r="H232" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6401,7 +6375,7 @@
       <c r="G233" t="s">
         <v>179</v>
       </c>
-      <c r="H233" s="2">
+      <c r="H233" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6415,7 +6389,7 @@
       <c r="C234" t="s">
         <v>115</v>
       </c>
-      <c r="H234" s="2">
+      <c r="H234" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6432,13 +6406,13 @@
       <c r="D235" t="s">
         <v>155</v>
       </c>
-      <c r="E235" s="2">
+      <c r="E235" s="1">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>199</v>
       </c>
-      <c r="H235" s="2">
+      <c r="H235" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6452,7 +6426,7 @@
       <c r="C236" t="s">
         <v>115</v>
       </c>
-      <c r="H236" s="2">
+      <c r="H236" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6466,7 +6440,7 @@
       <c r="C237" t="s">
         <v>119</v>
       </c>
-      <c r="H237" s="2">
+      <c r="H237" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6480,7 +6454,7 @@
       <c r="C238" t="s">
         <v>115</v>
       </c>
-      <c r="H238" s="2">
+      <c r="H238" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6494,7 +6468,7 @@
       <c r="C239" t="s">
         <v>119</v>
       </c>
-      <c r="H239" s="2">
+      <c r="H239" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6508,7 +6482,7 @@
       <c r="C240" t="s">
         <v>119</v>
       </c>
-      <c r="H240" s="2">
+      <c r="H240" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6525,13 +6499,13 @@
       <c r="D241" t="s">
         <v>125</v>
       </c>
-      <c r="E241" s="2">
+      <c r="E241" s="1">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>193</v>
       </c>
-      <c r="H241" s="2">
+      <c r="H241" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6545,7 +6519,7 @@
       <c r="C242" t="s">
         <v>119</v>
       </c>
-      <c r="H242" s="2">
+      <c r="H242" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6562,13 +6536,13 @@
       <c r="D243" t="s">
         <v>156</v>
       </c>
-      <c r="E243" s="2">
+      <c r="E243" s="1">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>205</v>
       </c>
-      <c r="H243" s="2">
+      <c r="H243" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6585,13 +6559,13 @@
       <c r="D244" t="s">
         <v>157</v>
       </c>
-      <c r="E244" s="2">
+      <c r="E244" s="1">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>202</v>
       </c>
-      <c r="H244" s="2">
+      <c r="H244" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6605,7 +6579,7 @@
       <c r="C245" t="s">
         <v>119</v>
       </c>
-      <c r="H245" s="2">
+      <c r="H245" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6619,7 +6593,7 @@
       <c r="C246" t="s">
         <v>115</v>
       </c>
-      <c r="H246" s="2">
+      <c r="H246" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6636,13 +6610,13 @@
       <c r="D247" t="s">
         <v>128</v>
       </c>
-      <c r="E247" s="2">
+      <c r="E247" s="1">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>206</v>
       </c>
-      <c r="H247" s="2">
+      <c r="H247" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6656,7 +6630,7 @@
       <c r="C248" t="s">
         <v>115</v>
       </c>
-      <c r="H248" s="2">
+      <c r="H248" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6670,7 +6644,7 @@
       <c r="C249" t="s">
         <v>115</v>
       </c>
-      <c r="H249" s="2">
+      <c r="H249" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6687,13 +6661,13 @@
       <c r="D250" t="s">
         <v>158</v>
       </c>
-      <c r="E250" s="2">
+      <c r="E250" s="1">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>201</v>
       </c>
-      <c r="H250" s="2">
+      <c r="H250" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6707,7 +6681,7 @@
       <c r="C251" t="s">
         <v>115</v>
       </c>
-      <c r="H251" s="2">
+      <c r="H251" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6724,13 +6698,13 @@
       <c r="D252" t="s">
         <v>159</v>
       </c>
-      <c r="E252" s="2">
+      <c r="E252" s="1">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>203</v>
       </c>
-      <c r="H252" s="2">
+      <c r="H252" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6753,7 +6727,7 @@
       <c r="G253" t="s">
         <v>181</v>
       </c>
-      <c r="H253" s="2">
+      <c r="H253" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6767,7 +6741,7 @@
       <c r="C254" t="s">
         <v>119</v>
       </c>
-      <c r="H254" s="2">
+      <c r="H254" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6781,7 +6755,7 @@
       <c r="C255" t="s">
         <v>115</v>
       </c>
-      <c r="H255" s="2">
+      <c r="H255" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6804,7 +6778,7 @@
       <c r="G256" t="s">
         <v>176</v>
       </c>
-      <c r="H256" s="2">
+      <c r="H256" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6821,7 +6795,7 @@
       <c r="D257" t="s">
         <v>132</v>
       </c>
-      <c r="H257" s="2">
+      <c r="H257" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6844,7 +6818,7 @@
       <c r="G258" t="s">
         <v>177</v>
       </c>
-      <c r="H258" s="2">
+      <c r="H258" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6861,13 +6835,13 @@
       <c r="D259" t="s">
         <v>154</v>
       </c>
-      <c r="E259" s="2">
+      <c r="E259" s="1">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>204</v>
       </c>
-      <c r="H259" s="2">
+      <c r="H259" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6890,7 +6864,7 @@
       <c r="G260" t="s">
         <v>178</v>
       </c>
-      <c r="H260" s="2">
+      <c r="H260" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6913,7 +6887,7 @@
       <c r="G261" t="s">
         <v>178</v>
       </c>
-      <c r="H261" s="2">
+      <c r="H261" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6936,7 +6910,7 @@
       <c r="G262" t="s">
         <v>179</v>
       </c>
-      <c r="H262" s="2">
+      <c r="H262" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6950,7 +6924,7 @@
       <c r="C263" t="s">
         <v>115</v>
       </c>
-      <c r="H263" s="2">
+      <c r="H263" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6967,13 +6941,13 @@
       <c r="D264" t="s">
         <v>155</v>
       </c>
-      <c r="E264" s="2">
+      <c r="E264" s="1">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>199</v>
       </c>
-      <c r="H264" s="2">
+      <c r="H264" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6987,7 +6961,7 @@
       <c r="C265" t="s">
         <v>115</v>
       </c>
-      <c r="H265" s="2">
+      <c r="H265" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7001,7 +6975,7 @@
       <c r="C266" t="s">
         <v>119</v>
       </c>
-      <c r="H266" s="2">
+      <c r="H266" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7015,7 +6989,7 @@
       <c r="C267" t="s">
         <v>115</v>
       </c>
-      <c r="H267" s="2">
+      <c r="H267" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7029,7 +7003,7 @@
       <c r="C268" t="s">
         <v>119</v>
       </c>
-      <c r="H268" s="2">
+      <c r="H268" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7043,7 +7017,7 @@
       <c r="C269" t="s">
         <v>119</v>
       </c>
-      <c r="H269" s="2">
+      <c r="H269" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7060,13 +7034,13 @@
       <c r="D270" t="s">
         <v>125</v>
       </c>
-      <c r="E270" s="2">
+      <c r="E270" s="1">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>193</v>
       </c>
-      <c r="H270" s="2">
+      <c r="H270" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7080,7 +7054,7 @@
       <c r="C271" t="s">
         <v>119</v>
       </c>
-      <c r="H271" s="2">
+      <c r="H271" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7097,13 +7071,13 @@
       <c r="D272" t="s">
         <v>156</v>
       </c>
-      <c r="E272" s="2">
+      <c r="E272" s="1">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>205</v>
       </c>
-      <c r="H272" s="2">
+      <c r="H272" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7120,13 +7094,13 @@
       <c r="D273" t="s">
         <v>157</v>
       </c>
-      <c r="E273" s="2">
+      <c r="E273" s="1">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>207</v>
       </c>
-      <c r="H273" s="2">
+      <c r="H273" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7140,7 +7114,7 @@
       <c r="C274" t="s">
         <v>115</v>
       </c>
-      <c r="H274" s="2">
+      <c r="H274" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7154,7 +7128,7 @@
       <c r="C275" t="s">
         <v>115</v>
       </c>
-      <c r="H275" s="2">
+      <c r="H275" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7171,13 +7145,13 @@
       <c r="D276" t="s">
         <v>128</v>
       </c>
-      <c r="E276" s="2">
+      <c r="E276" s="1">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>206</v>
       </c>
-      <c r="H276" s="2">
+      <c r="H276" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7191,7 +7165,7 @@
       <c r="C277" t="s">
         <v>115</v>
       </c>
-      <c r="H277" s="2">
+      <c r="H277" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7208,13 +7182,13 @@
       <c r="D278" t="s">
         <v>160</v>
       </c>
-      <c r="E278" s="2">
+      <c r="E278" s="1">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>208</v>
       </c>
-      <c r="H278" s="2">
+      <c r="H278" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7231,13 +7205,13 @@
       <c r="D279" t="s">
         <v>158</v>
       </c>
-      <c r="E279" s="2">
+      <c r="E279" s="1">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>207</v>
       </c>
-      <c r="H279" s="2">
+      <c r="H279" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7251,7 +7225,7 @@
       <c r="C280" t="s">
         <v>115</v>
       </c>
-      <c r="H280" s="2">
+      <c r="H280" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7268,13 +7242,13 @@
       <c r="D281" t="s">
         <v>161</v>
       </c>
-      <c r="E281" s="2">
+      <c r="E281" s="1">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>203</v>
       </c>
-      <c r="H281" s="2">
+      <c r="H281" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7297,7 +7271,7 @@
       <c r="G282" t="s">
         <v>181</v>
       </c>
-      <c r="H282" s="2">
+      <c r="H282" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7311,7 +7285,7 @@
       <c r="C283" t="s">
         <v>119</v>
       </c>
-      <c r="H283" s="2">
+      <c r="H283" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7325,7 +7299,7 @@
       <c r="C284" t="s">
         <v>115</v>
       </c>
-      <c r="H284" s="2">
+      <c r="H284" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7348,7 +7322,7 @@
       <c r="G285" t="s">
         <v>176</v>
       </c>
-      <c r="H285" s="2">
+      <c r="H285" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7365,7 +7339,7 @@
       <c r="D286" t="s">
         <v>132</v>
       </c>
-      <c r="H286" s="2">
+      <c r="H286" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7388,7 +7362,7 @@
       <c r="G287" t="s">
         <v>177</v>
       </c>
-      <c r="H287" s="2">
+      <c r="H287" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7405,13 +7379,13 @@
       <c r="D288" t="s">
         <v>154</v>
       </c>
-      <c r="E288" s="2">
+      <c r="E288" s="1">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>204</v>
       </c>
-      <c r="H288" s="2">
+      <c r="H288" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7434,7 +7408,7 @@
       <c r="G289" t="s">
         <v>178</v>
       </c>
-      <c r="H289" s="2">
+      <c r="H289" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7457,7 +7431,7 @@
       <c r="G290" t="s">
         <v>178</v>
       </c>
-      <c r="H290" s="2">
+      <c r="H290" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7480,7 +7454,7 @@
       <c r="G291" t="s">
         <v>179</v>
       </c>
-      <c r="H291" s="2">
+      <c r="H291" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7494,7 +7468,7 @@
       <c r="C292" t="s">
         <v>115</v>
       </c>
-      <c r="H292" s="2">
+      <c r="H292" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7517,7 +7491,7 @@
       <c r="G293" t="s">
         <v>182</v>
       </c>
-      <c r="H293" s="2">
+      <c r="H293" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7531,7 +7505,7 @@
       <c r="C294" t="s">
         <v>115</v>
       </c>
-      <c r="H294" s="2">
+      <c r="H294" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7554,7 +7528,7 @@
       <c r="G295" t="s">
         <v>183</v>
       </c>
-      <c r="H295" s="2">
+      <c r="H295" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7568,7 +7542,7 @@
       <c r="C296" t="s">
         <v>115</v>
       </c>
-      <c r="H296" s="2">
+      <c r="H296" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7582,7 +7556,7 @@
       <c r="C297" t="s">
         <v>119</v>
       </c>
-      <c r="H297" s="2">
+      <c r="H297" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7605,7 +7579,7 @@
       <c r="G298" t="s">
         <v>184</v>
       </c>
-      <c r="H298" s="2">
+      <c r="H298" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7622,13 +7596,13 @@
       <c r="D299" t="s">
         <v>125</v>
       </c>
-      <c r="E299" s="2">
+      <c r="E299" s="1">
         <v>46234</v>
       </c>
       <c r="G299" t="s">
         <v>193</v>
       </c>
-      <c r="H299" s="2">
+      <c r="H299" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7642,7 +7616,7 @@
       <c r="C300" t="s">
         <v>115</v>
       </c>
-      <c r="H300" s="2">
+      <c r="H300" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7659,13 +7633,13 @@
       <c r="D301" t="s">
         <v>156</v>
       </c>
-      <c r="E301" s="2">
+      <c r="E301" s="1">
         <v>46224</v>
       </c>
       <c r="G301" t="s">
         <v>205</v>
       </c>
-      <c r="H301" s="2">
+      <c r="H301" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7682,13 +7656,13 @@
       <c r="D302" t="s">
         <v>157</v>
       </c>
-      <c r="E302" s="2">
+      <c r="E302" s="1">
         <v>46220</v>
       </c>
       <c r="G302" t="s">
         <v>202</v>
       </c>
-      <c r="H302" s="2">
+      <c r="H302" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7702,7 +7676,7 @@
       <c r="C303" t="s">
         <v>115</v>
       </c>
-      <c r="H303" s="2">
+      <c r="H303" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7716,7 +7690,7 @@
       <c r="C304" t="s">
         <v>115</v>
       </c>
-      <c r="H304" s="2">
+      <c r="H304" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7733,13 +7707,13 @@
       <c r="D305" t="s">
         <v>128</v>
       </c>
-      <c r="E305" s="2">
+      <c r="E305" s="1">
         <v>46237</v>
       </c>
       <c r="G305" t="s">
         <v>206</v>
       </c>
-      <c r="H305" s="2">
+      <c r="H305" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7753,7 +7727,7 @@
       <c r="C306" t="s">
         <v>115</v>
       </c>
-      <c r="H306" s="2">
+      <c r="H306" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7770,13 +7744,13 @@
       <c r="D307" t="s">
         <v>160</v>
       </c>
-      <c r="E307" s="2">
+      <c r="E307" s="1">
         <v>46227</v>
       </c>
       <c r="G307" t="s">
         <v>208</v>
       </c>
-      <c r="H307" s="2">
+      <c r="H307" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7790,7 +7764,7 @@
       <c r="C308" t="s">
         <v>119</v>
       </c>
-      <c r="H308" s="2">
+      <c r="H308" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7813,7 +7787,7 @@
       <c r="G309" t="s">
         <v>182</v>
       </c>
-      <c r="H309" s="2">
+      <c r="H309" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7836,7 +7810,7 @@
       <c r="G310" t="s">
         <v>185</v>
       </c>
-      <c r="H310" s="2">
+      <c r="H310" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7853,7 +7827,7 @@
       <c r="D311" t="s">
         <v>166</v>
       </c>
-      <c r="H311" s="2">
+      <c r="H311" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7867,7 +7841,7 @@
       <c r="C312" t="s">
         <v>119</v>
       </c>
-      <c r="H312" s="2">
+      <c r="H312" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7881,7 +7855,7 @@
       <c r="C313" t="s">
         <v>115</v>
       </c>
-      <c r="H313" s="2">
+      <c r="H313" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="G314" t="s">
         <v>176</v>
       </c>
-      <c r="H314" s="2">
+      <c r="H314" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7921,7 +7895,7 @@
       <c r="D315" t="s">
         <v>132</v>
       </c>
-      <c r="H315" s="2">
+      <c r="H315" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7944,7 +7918,7 @@
       <c r="G316" t="s">
         <v>177</v>
       </c>
-      <c r="H316" s="2">
+      <c r="H316" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7967,7 +7941,7 @@
       <c r="G317" t="s">
         <v>186</v>
       </c>
-      <c r="H317" s="2">
+      <c r="H317" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7990,7 +7964,7 @@
       <c r="G318" t="s">
         <v>178</v>
       </c>
-      <c r="H318" s="2">
+      <c r="H318" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -8013,7 +7987,7 @@
       <c r="G319" t="s">
         <v>178</v>
       </c>
-      <c r="H319" s="2">
+      <c r="H319" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -8036,7 +8010,7 @@
       <c r="G320" t="s">
         <v>179</v>
       </c>
-      <c r="H320" s="2">
+      <c r="H320" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -8050,7 +8024,7 @@
       <c r="C321" t="s">
         <v>115</v>
       </c>
-      <c r="H321" s="2">
+      <c r="H321" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8073,7 +8047,7 @@
       <c r="G322" t="s">
         <v>187</v>
       </c>
-      <c r="H322" s="2">
+      <c r="H322" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8087,7 +8061,7 @@
       <c r="C323" t="s">
         <v>115</v>
       </c>
-      <c r="H323" s="2">
+      <c r="H323" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8110,7 +8084,7 @@
       <c r="G324" t="s">
         <v>188</v>
       </c>
-      <c r="H324" s="2">
+      <c r="H324" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8124,7 +8098,7 @@
       <c r="C325" t="s">
         <v>115</v>
       </c>
-      <c r="H325" s="2">
+      <c r="H325" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8138,7 +8112,7 @@
       <c r="C326" t="s">
         <v>119</v>
       </c>
-      <c r="H326" s="2">
+      <c r="H326" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8152,7 +8126,7 @@
       <c r="C327" t="s">
         <v>119</v>
       </c>
-      <c r="H327" s="2">
+      <c r="H327" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8169,13 +8143,13 @@
       <c r="D328" t="s">
         <v>125</v>
       </c>
-      <c r="E328" s="2">
+      <c r="E328" s="1">
         <v>46234</v>
       </c>
       <c r="G328" t="s">
         <v>193</v>
       </c>
-      <c r="H328" s="2">
+      <c r="H328" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8198,7 +8172,7 @@
       <c r="G329" t="s">
         <v>188</v>
       </c>
-      <c r="H329" s="2">
+      <c r="H329" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8221,7 +8195,7 @@
       <c r="G330" t="s">
         <v>188</v>
       </c>
-      <c r="H330" s="2">
+      <c r="H330" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8235,7 +8209,7 @@
       <c r="C331" t="s">
         <v>115</v>
       </c>
-      <c r="H331" s="2">
+      <c r="H331" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8258,7 +8232,7 @@
       <c r="G332" t="s">
         <v>188</v>
       </c>
-      <c r="H332" s="2">
+      <c r="H332" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8281,7 +8255,7 @@
       <c r="G333" t="s">
         <v>187</v>
       </c>
-      <c r="H333" s="2">
+      <c r="H333" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8298,13 +8272,13 @@
       <c r="D334" t="s">
         <v>128</v>
       </c>
-      <c r="E334" s="2">
+      <c r="E334" s="1">
         <v>46237</v>
       </c>
       <c r="G334" t="s">
         <v>206</v>
       </c>
-      <c r="H334" s="2">
+      <c r="H334" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8318,7 +8292,7 @@
       <c r="C335" t="s">
         <v>115</v>
       </c>
-      <c r="H335" s="2">
+      <c r="H335" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8335,13 +8309,13 @@
       <c r="D336" t="s">
         <v>160</v>
       </c>
-      <c r="E336" s="2">
+      <c r="E336" s="1">
         <v>46227</v>
       </c>
       <c r="G336" t="s">
         <v>208</v>
       </c>
-      <c r="H336" s="2">
+      <c r="H336" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8355,7 +8329,7 @@
       <c r="C337" t="s">
         <v>115</v>
       </c>
-      <c r="H337" s="2">
+      <c r="H337" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8369,7 +8343,7 @@
       <c r="C338" t="s">
         <v>115</v>
       </c>
-      <c r="H338" s="2">
+      <c r="H338" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8392,7 +8366,7 @@
       <c r="G339" t="s">
         <v>185</v>
       </c>
-      <c r="H339" s="2">
+      <c r="H339" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8409,7 +8383,7 @@
       <c r="D340" t="s">
         <v>171</v>
       </c>
-      <c r="H340" s="2">
+      <c r="H340" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8423,7 +8397,7 @@
       <c r="C341" t="s">
         <v>119</v>
       </c>
-      <c r="H341" s="2">
+      <c r="H341" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8437,7 +8411,7 @@
       <c r="C342" t="s">
         <v>115</v>
       </c>
-      <c r="H342" s="2">
+      <c r="H342" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8460,7 +8434,7 @@
       <c r="G343" t="s">
         <v>176</v>
       </c>
-      <c r="H343" s="2">
+      <c r="H343" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8477,7 +8451,7 @@
       <c r="D344" t="s">
         <v>132</v>
       </c>
-      <c r="H344" s="2">
+      <c r="H344" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8500,7 +8474,7 @@
       <c r="G345" t="s">
         <v>177</v>
       </c>
-      <c r="H345" s="2">
+      <c r="H345" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8523,7 +8497,7 @@
       <c r="G346" t="s">
         <v>186</v>
       </c>
-      <c r="H346" s="2">
+      <c r="H346" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8546,7 +8520,7 @@
       <c r="G347" t="s">
         <v>178</v>
       </c>
-      <c r="H347" s="2">
+      <c r="H347" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8569,7 +8543,7 @@
       <c r="G348" t="s">
         <v>178</v>
       </c>
-      <c r="H348" s="2">
+      <c r="H348" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8592,7 +8566,7 @@
       <c r="G349" t="s">
         <v>179</v>
       </c>
-      <c r="H349" s="2">
+      <c r="H349" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8606,7 +8580,7 @@
       <c r="C350" t="s">
         <v>115</v>
       </c>
-      <c r="H350" s="2">
+      <c r="H350" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8629,7 +8603,7 @@
       <c r="G351" t="s">
         <v>187</v>
       </c>
-      <c r="H351" s="2">
+      <c r="H351" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8643,7 +8617,7 @@
       <c r="C352" t="s">
         <v>115</v>
       </c>
-      <c r="H352" s="2">
+      <c r="H352" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8657,7 +8631,7 @@
       <c r="C353" t="s">
         <v>115</v>
       </c>
-      <c r="H353" s="2">
+      <c r="H353" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8671,7 +8645,7 @@
       <c r="C354" t="s">
         <v>115</v>
       </c>
-      <c r="H354" s="2">
+      <c r="H354" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8685,7 +8659,7 @@
       <c r="C355" t="s">
         <v>119</v>
       </c>
-      <c r="H355" s="2">
+      <c r="H355" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8699,7 +8673,7 @@
       <c r="C356" t="s">
         <v>119</v>
       </c>
-      <c r="H356" s="2">
+      <c r="H356" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8722,7 +8696,7 @@
       <c r="G357" t="s">
         <v>189</v>
       </c>
-      <c r="H357" s="2">
+      <c r="H357" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8736,7 +8710,7 @@
       <c r="C358" t="s">
         <v>115</v>
       </c>
-      <c r="H358" s="2">
+      <c r="H358" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8759,7 +8733,7 @@
       <c r="G359" t="s">
         <v>190</v>
       </c>
-      <c r="H359" s="2">
+      <c r="H359" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8773,7 +8747,7 @@
       <c r="C360" t="s">
         <v>115</v>
       </c>
-      <c r="H360" s="2">
+      <c r="H360" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8787,7 +8761,7 @@
       <c r="C361" t="s">
         <v>115</v>
       </c>
-      <c r="H361" s="2">
+      <c r="H361" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8810,7 +8784,7 @@
       <c r="G362" t="s">
         <v>187</v>
       </c>
-      <c r="H362" s="2">
+      <c r="H362" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8833,7 +8807,7 @@
       <c r="G363" t="s">
         <v>191</v>
       </c>
-      <c r="H363" s="2">
+      <c r="H363" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8847,7 +8821,7 @@
       <c r="C364" t="s">
         <v>115</v>
       </c>
-      <c r="H364" s="2">
+      <c r="H364" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8870,7 +8844,7 @@
       <c r="G365" t="s">
         <v>190</v>
       </c>
-      <c r="H365" s="2">
+      <c r="H365" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8884,7 +8858,7 @@
       <c r="C366" t="s">
         <v>115</v>
       </c>
-      <c r="H366" s="2">
+      <c r="H366" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8898,7 +8872,7 @@
       <c r="C367" t="s">
         <v>115</v>
       </c>
-      <c r="H367" s="2">
+      <c r="H367" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8921,7 +8895,7 @@
       <c r="G368" t="s">
         <v>189</v>
       </c>
-      <c r="H368" s="2">
+      <c r="H368" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8944,7 +8918,7 @@
       <c r="G369" t="s">
         <v>190</v>
       </c>
-      <c r="H369" s="2">
+      <c r="H369" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8961,7 +8935,7 @@
       <c r="D370" t="s">
         <v>171</v>
       </c>
-      <c r="H370" s="2">
+      <c r="H370" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8975,7 +8949,7 @@
       <c r="C371" t="s">
         <v>115</v>
       </c>
-      <c r="H371" s="2">
+      <c r="H371" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8998,7 +8972,7 @@
       <c r="G372" t="s">
         <v>176</v>
       </c>
-      <c r="H372" s="2">
+      <c r="H372" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9015,7 +8989,7 @@
       <c r="D373" t="s">
         <v>132</v>
       </c>
-      <c r="H373" s="2">
+      <c r="H373" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9038,7 +9012,7 @@
       <c r="G374" t="s">
         <v>177</v>
       </c>
-      <c r="H374" s="2">
+      <c r="H374" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9061,7 +9035,7 @@
       <c r="G375" t="s">
         <v>186</v>
       </c>
-      <c r="H375" s="2">
+      <c r="H375" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9084,7 +9058,7 @@
       <c r="G376" t="s">
         <v>178</v>
       </c>
-      <c r="H376" s="2">
+      <c r="H376" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9107,7 +9081,7 @@
       <c r="G377" t="s">
         <v>178</v>
       </c>
-      <c r="H377" s="2">
+      <c r="H377" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9130,7 +9104,7 @@
       <c r="G378" t="s">
         <v>179</v>
       </c>
-      <c r="H378" s="2">
+      <c r="H378" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9144,7 +9118,7 @@
       <c r="C379" t="s">
         <v>115</v>
       </c>
-      <c r="H379" s="2">
+      <c r="H379" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9167,7 +9141,7 @@
       <c r="G380" t="s">
         <v>190</v>
       </c>
-      <c r="H380" s="2">
+      <c r="H380" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9181,7 +9155,7 @@
       <c r="C381" t="s">
         <v>115</v>
       </c>
-      <c r="H381" s="2">
+      <c r="H381" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9195,7 +9169,7 @@
       <c r="C382" t="s">
         <v>115</v>
       </c>
-      <c r="H382" s="2">
+      <c r="H382" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9209,7 +9183,7 @@
       <c r="C383" t="s">
         <v>115</v>
       </c>
-      <c r="H383" s="2">
+      <c r="H383" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9223,7 +9197,7 @@
       <c r="C384" t="s">
         <v>119</v>
       </c>
-      <c r="H384" s="2">
+      <c r="H384" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9237,7 +9211,7 @@
       <c r="C385" t="s">
         <v>119</v>
       </c>
-      <c r="H385" s="2">
+      <c r="H385" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9260,7 +9234,7 @@
       <c r="G386" t="s">
         <v>189</v>
       </c>
-      <c r="H386" s="2">
+      <c r="H386" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9274,7 +9248,7 @@
       <c r="C387" t="s">
         <v>115</v>
       </c>
-      <c r="H387" s="2">
+      <c r="H387" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9288,7 +9262,7 @@
       <c r="C388" t="s">
         <v>119</v>
       </c>
-      <c r="H388" s="2">
+      <c r="H388" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9302,7 +9276,7 @@
       <c r="C389" t="s">
         <v>115</v>
       </c>
-      <c r="H389" s="2">
+      <c r="H389" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9316,7 +9290,7 @@
       <c r="C390" t="s">
         <v>115</v>
       </c>
-      <c r="H390" s="2">
+      <c r="H390" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9339,7 +9313,7 @@
       <c r="G391" t="s">
         <v>190</v>
       </c>
-      <c r="H391" s="2">
+      <c r="H391" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9362,7 +9336,7 @@
       <c r="G392" t="s">
         <v>191</v>
       </c>
-      <c r="H392" s="2">
+      <c r="H392" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9376,7 +9350,7 @@
       <c r="C393" t="s">
         <v>115</v>
       </c>
-      <c r="H393" s="2">
+      <c r="H393" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9399,7 +9373,7 @@
       <c r="G394" t="s">
         <v>190</v>
       </c>
-      <c r="H394" s="2">
+      <c r="H394" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9413,7 +9387,7 @@
       <c r="C395" t="s">
         <v>115</v>
       </c>
-      <c r="H395" s="2">
+      <c r="H395" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9427,7 +9401,7 @@
       <c r="C396" t="s">
         <v>115</v>
       </c>
-      <c r="H396" s="2">
+      <c r="H396" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9450,7 +9424,7 @@
       <c r="G397" t="s">
         <v>189</v>
       </c>
-      <c r="H397" s="2">
+      <c r="H397" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9473,7 +9447,7 @@
       <c r="G398" t="s">
         <v>190</v>
       </c>
-      <c r="H398" s="2">
+      <c r="H398" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9490,7 +9464,7 @@
       <c r="D399" t="s">
         <v>171</v>
       </c>
-      <c r="H399" s="2">
+      <c r="H399" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9504,7 +9478,7 @@
       <c r="C400" t="s">
         <v>115</v>
       </c>
-      <c r="H400" s="2">
+      <c r="H400" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9527,7 +9501,7 @@
       <c r="G401" t="s">
         <v>176</v>
       </c>
-      <c r="H401" s="2">
+      <c r="H401" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9544,7 +9518,7 @@
       <c r="D402" t="s">
         <v>132</v>
       </c>
-      <c r="H402" s="2">
+      <c r="H402" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9567,7 +9541,7 @@
       <c r="G403" t="s">
         <v>177</v>
       </c>
-      <c r="H403" s="2">
+      <c r="H403" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9590,7 +9564,7 @@
       <c r="G404" t="s">
         <v>186</v>
       </c>
-      <c r="H404" s="2">
+      <c r="H404" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9613,7 +9587,7 @@
       <c r="G405" t="s">
         <v>178</v>
       </c>
-      <c r="H405" s="2">
+      <c r="H405" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9636,7 +9610,7 @@
       <c r="G406" t="s">
         <v>178</v>
       </c>
-      <c r="H406" s="2">
+      <c r="H406" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9659,7 +9633,7 @@
       <c r="G407" t="s">
         <v>179</v>
       </c>
-      <c r="H407" s="2">
+      <c r="H407" s="1">
         <v>46226</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Registra verificação do Drive (Disponibilidade Diária) do teste pós-rebase
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -651,8 +651,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -668,7 +676,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -676,12 +684,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -981,72 +1007,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1111,7 +1137,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1176,7 +1202,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1241,7 +1267,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1306,7 +1332,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1371,7 +1397,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1436,7 +1462,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1501,7 +1527,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1566,7 +1592,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1631,7 +1657,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1696,7 +1722,7 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>46220</v>
       </c>
       <c r="B12">
@@ -1761,7 +1787,7 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46224</v>
       </c>
       <c r="B13">
@@ -1826,7 +1852,7 @@
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46225</v>
       </c>
       <c r="B14">
@@ -1891,7 +1917,7 @@
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46226</v>
       </c>
       <c r="B15">
@@ -1966,28 +1992,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2001,7 +2027,7 @@
       <c r="C2" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2015,7 +2041,7 @@
       <c r="C3" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2038,7 +2064,7 @@
       <c r="G4" t="s">
         <v>174</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2052,7 +2078,7 @@
       <c r="C5" t="s">
         <v>115</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2066,7 +2092,7 @@
       <c r="C6" t="s">
         <v>115</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2083,13 +2109,13 @@
       <c r="D7" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2106,13 +2132,13 @@
       <c r="D8" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>192</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2129,13 +2155,13 @@
       <c r="D9" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>193</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2152,13 +2178,13 @@
       <c r="D10" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>194</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2172,7 +2198,7 @@
       <c r="C11" t="s">
         <v>115</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2186,7 +2212,7 @@
       <c r="C12" t="s">
         <v>115</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2203,13 +2229,13 @@
       <c r="D13" t="s">
         <v>127</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>192</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2223,7 +2249,7 @@
       <c r="C14" t="s">
         <v>119</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2240,13 +2266,13 @@
       <c r="D15" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>195</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2260,7 +2286,7 @@
       <c r="C16" t="s">
         <v>115</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2274,7 +2300,7 @@
       <c r="C17" t="s">
         <v>115</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2291,13 +2317,13 @@
       <c r="D18" t="s">
         <v>129</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>196</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2311,7 +2337,7 @@
       <c r="C19" t="s">
         <v>115</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2328,13 +2354,13 @@
       <c r="D20" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>192</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2357,7 +2383,7 @@
       <c r="G21" t="s">
         <v>175</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2371,7 +2397,7 @@
       <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2385,7 +2411,7 @@
       <c r="C23" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2408,7 +2434,7 @@
       <c r="G24" t="s">
         <v>176</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2425,7 +2451,7 @@
       <c r="D25" t="s">
         <v>132</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2448,7 +2474,7 @@
       <c r="G26" t="s">
         <v>177</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2465,13 +2491,13 @@
       <c r="D27" t="s">
         <v>134</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>197</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2494,7 +2520,7 @@
       <c r="G28" t="s">
         <v>178</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2517,7 +2543,7 @@
       <c r="G29" t="s">
         <v>178</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2540,7 +2566,7 @@
       <c r="G30" t="s">
         <v>179</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2554,7 +2580,7 @@
       <c r="C31" t="s">
         <v>115</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2568,7 +2594,7 @@
       <c r="C32" t="s">
         <v>115</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2591,7 +2617,7 @@
       <c r="G33" t="s">
         <v>180</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2605,7 +2631,7 @@
       <c r="C34" t="s">
         <v>115</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2619,7 +2645,7 @@
       <c r="C35" t="s">
         <v>115</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2636,13 +2662,13 @@
       <c r="D36" t="s">
         <v>123</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>192</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2659,13 +2685,13 @@
       <c r="D37" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="2">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>192</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2682,13 +2708,13 @@
       <c r="D38" t="s">
         <v>125</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38" s="2">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>193</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2705,13 +2731,13 @@
       <c r="D39" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39" s="2">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>194</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2725,7 +2751,7 @@
       <c r="C40" t="s">
         <v>115</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2739,7 +2765,7 @@
       <c r="C41" t="s">
         <v>115</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2756,13 +2782,13 @@
       <c r="D42" t="s">
         <v>127</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42" s="2">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>192</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2776,7 +2802,7 @@
       <c r="C43" t="s">
         <v>115</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2793,13 +2819,13 @@
       <c r="D44" t="s">
         <v>128</v>
       </c>
-      <c r="E44" s="1">
+      <c r="E44" s="2">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>195</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2813,7 +2839,7 @@
       <c r="C45" t="s">
         <v>115</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2827,7 +2853,7 @@
       <c r="C46" t="s">
         <v>115</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="C47" t="s">
         <v>119</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2855,7 +2881,7 @@
       <c r="C48" t="s">
         <v>115</v>
       </c>
-      <c r="H48" s="1">
+      <c r="H48" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2872,13 +2898,13 @@
       <c r="D49" t="s">
         <v>139</v>
       </c>
-      <c r="E49" s="1">
+      <c r="E49" s="2">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>192</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2901,7 +2927,7 @@
       <c r="G50" t="s">
         <v>175</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2915,7 +2941,7 @@
       <c r="C51" t="s">
         <v>119</v>
       </c>
-      <c r="H51" s="1">
+      <c r="H51" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2929,7 +2955,7 @@
       <c r="C52" t="s">
         <v>115</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2952,7 +2978,7 @@
       <c r="G53" t="s">
         <v>176</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2969,7 +2995,7 @@
       <c r="D54" t="s">
         <v>132</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2992,7 +3018,7 @@
       <c r="G55" t="s">
         <v>177</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3009,13 +3035,13 @@
       <c r="D56" t="s">
         <v>134</v>
       </c>
-      <c r="E56" s="1">
+      <c r="E56" s="2">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>197</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3038,7 +3064,7 @@
       <c r="G57" t="s">
         <v>178</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3061,7 +3087,7 @@
       <c r="G58" t="s">
         <v>178</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3084,7 +3110,7 @@
       <c r="G59" t="s">
         <v>179</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3098,7 +3124,7 @@
       <c r="C60" t="s">
         <v>115</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3112,7 +3138,7 @@
       <c r="C61" t="s">
         <v>115</v>
       </c>
-      <c r="H61" s="1">
+      <c r="H61" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3129,13 +3155,13 @@
       <c r="D62" t="s">
         <v>138</v>
       </c>
-      <c r="E62" s="1">
+      <c r="E62" s="2">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>198</v>
       </c>
-      <c r="H62" s="1">
+      <c r="H62" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3149,7 +3175,7 @@
       <c r="C63" t="s">
         <v>115</v>
       </c>
-      <c r="H63" s="1">
+      <c r="H63" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3166,13 +3192,13 @@
       <c r="D64" t="s">
         <v>140</v>
       </c>
-      <c r="E64" s="1">
+      <c r="E64" s="2">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>199</v>
       </c>
-      <c r="H64" s="1">
+      <c r="H64" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3186,7 +3212,7 @@
       <c r="C65" t="s">
         <v>115</v>
       </c>
-      <c r="H65" s="1">
+      <c r="H65" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3200,7 +3226,7 @@
       <c r="C66" t="s">
         <v>119</v>
       </c>
-      <c r="H66" s="1">
+      <c r="H66" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3217,13 +3243,13 @@
       <c r="D67" t="s">
         <v>125</v>
       </c>
-      <c r="E67" s="1">
+      <c r="E67" s="2">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>193</v>
       </c>
-      <c r="H67" s="1">
+      <c r="H67" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3240,13 +3266,13 @@
       <c r="D68" t="s">
         <v>126</v>
       </c>
-      <c r="E68" s="1">
+      <c r="E68" s="2">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>194</v>
       </c>
-      <c r="H68" s="1">
+      <c r="H68" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3260,7 +3286,7 @@
       <c r="C69" t="s">
         <v>115</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3274,7 +3300,7 @@
       <c r="C70" t="s">
         <v>115</v>
       </c>
-      <c r="H70" s="1">
+      <c r="H70" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3291,13 +3317,13 @@
       <c r="D71" t="s">
         <v>127</v>
       </c>
-      <c r="E71" s="1">
+      <c r="E71" s="2">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>198</v>
       </c>
-      <c r="H71" s="1">
+      <c r="H71" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3311,7 +3337,7 @@
       <c r="C72" t="s">
         <v>115</v>
       </c>
-      <c r="H72" s="1">
+      <c r="H72" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3328,13 +3354,13 @@
       <c r="D73" t="s">
         <v>128</v>
       </c>
-      <c r="E73" s="1">
+      <c r="E73" s="2">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>195</v>
       </c>
-      <c r="H73" s="1">
+      <c r="H73" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3348,7 +3374,7 @@
       <c r="C74" t="s">
         <v>115</v>
       </c>
-      <c r="H74" s="1">
+      <c r="H74" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3362,7 +3388,7 @@
       <c r="C75" t="s">
         <v>115</v>
       </c>
-      <c r="H75" s="1">
+      <c r="H75" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3376,7 +3402,7 @@
       <c r="C76" t="s">
         <v>115</v>
       </c>
-      <c r="H76" s="1">
+      <c r="H76" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3390,7 +3416,7 @@
       <c r="C77" t="s">
         <v>115</v>
       </c>
-      <c r="H77" s="1">
+      <c r="H77" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3407,13 +3433,13 @@
       <c r="D78" t="s">
         <v>139</v>
       </c>
-      <c r="E78" s="1">
+      <c r="E78" s="2">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>198</v>
       </c>
-      <c r="H78" s="1">
+      <c r="H78" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3436,7 +3462,7 @@
       <c r="G79" t="s">
         <v>181</v>
       </c>
-      <c r="H79" s="1">
+      <c r="H79" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3450,7 +3476,7 @@
       <c r="C80" t="s">
         <v>119</v>
       </c>
-      <c r="H80" s="1">
+      <c r="H80" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3464,7 +3490,7 @@
       <c r="C81" t="s">
         <v>115</v>
       </c>
-      <c r="H81" s="1">
+      <c r="H81" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3487,7 +3513,7 @@
       <c r="G82" t="s">
         <v>176</v>
       </c>
-      <c r="H82" s="1">
+      <c r="H82" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3504,7 +3530,7 @@
       <c r="D83" t="s">
         <v>132</v>
       </c>
-      <c r="H83" s="1">
+      <c r="H83" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3527,7 +3553,7 @@
       <c r="G84" t="s">
         <v>177</v>
       </c>
-      <c r="H84" s="1">
+      <c r="H84" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3544,13 +3570,13 @@
       <c r="D85" t="s">
         <v>134</v>
       </c>
-      <c r="E85" s="1">
+      <c r="E85" s="2">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>197</v>
       </c>
-      <c r="H85" s="1">
+      <c r="H85" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3573,7 +3599,7 @@
       <c r="G86" t="s">
         <v>178</v>
       </c>
-      <c r="H86" s="1">
+      <c r="H86" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3596,7 +3622,7 @@
       <c r="G87" t="s">
         <v>178</v>
       </c>
-      <c r="H87" s="1">
+      <c r="H87" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3619,7 +3645,7 @@
       <c r="G88" t="s">
         <v>179</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3633,7 +3659,7 @@
       <c r="C89" t="s">
         <v>115</v>
       </c>
-      <c r="H89" s="1">
+      <c r="H89" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3650,13 +3676,13 @@
       <c r="D90" t="s">
         <v>142</v>
       </c>
-      <c r="E90" s="1">
+      <c r="E90" s="2">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>199</v>
       </c>
-      <c r="H90" s="1">
+      <c r="H90" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3673,13 +3699,13 @@
       <c r="D91" t="s">
         <v>138</v>
       </c>
-      <c r="E91" s="1">
+      <c r="E91" s="2">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>198</v>
       </c>
-      <c r="H91" s="1">
+      <c r="H91" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3693,7 +3719,7 @@
       <c r="C92" t="s">
         <v>115</v>
       </c>
-      <c r="H92" s="1">
+      <c r="H92" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3710,13 +3736,13 @@
       <c r="D93" t="s">
         <v>140</v>
       </c>
-      <c r="E93" s="1">
+      <c r="E93" s="2">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>199</v>
       </c>
-      <c r="H93" s="1">
+      <c r="H93" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3730,7 +3756,7 @@
       <c r="C94" t="s">
         <v>115</v>
       </c>
-      <c r="H94" s="1">
+      <c r="H94" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3744,7 +3770,7 @@
       <c r="C95" t="s">
         <v>119</v>
       </c>
-      <c r="H95" s="1">
+      <c r="H95" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3761,13 +3787,13 @@
       <c r="D96" t="s">
         <v>125</v>
       </c>
-      <c r="E96" s="1">
+      <c r="E96" s="2">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>193</v>
       </c>
-      <c r="H96" s="1">
+      <c r="H96" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3784,13 +3810,13 @@
       <c r="D97" t="s">
         <v>126</v>
       </c>
-      <c r="E97" s="1">
+      <c r="E97" s="2">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>194</v>
       </c>
-      <c r="H97" s="1">
+      <c r="H97" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3804,7 +3830,7 @@
       <c r="C98" t="s">
         <v>115</v>
       </c>
-      <c r="H98" s="1">
+      <c r="H98" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3821,13 +3847,13 @@
       <c r="D99" t="s">
         <v>143</v>
       </c>
-      <c r="E99" s="1">
+      <c r="E99" s="2">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>194</v>
       </c>
-      <c r="H99" s="1">
+      <c r="H99" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3844,13 +3870,13 @@
       <c r="D100" t="s">
         <v>127</v>
       </c>
-      <c r="E100" s="1">
+      <c r="E100" s="2">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>194</v>
       </c>
-      <c r="H100" s="1">
+      <c r="H100" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3864,7 +3890,7 @@
       <c r="C101" t="s">
         <v>115</v>
       </c>
-      <c r="H101" s="1">
+      <c r="H101" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3881,13 +3907,13 @@
       <c r="D102" t="s">
         <v>128</v>
       </c>
-      <c r="E102" s="1">
+      <c r="E102" s="2">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>195</v>
       </c>
-      <c r="H102" s="1">
+      <c r="H102" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3904,13 +3930,13 @@
       <c r="D103" t="s">
         <v>144</v>
       </c>
-      <c r="E103" s="1">
+      <c r="E103" s="2">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>194</v>
       </c>
-      <c r="H103" s="1">
+      <c r="H103" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3924,7 +3950,7 @@
       <c r="C104" t="s">
         <v>115</v>
       </c>
-      <c r="H104" s="1">
+      <c r="H104" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3938,7 +3964,7 @@
       <c r="C105" t="s">
         <v>115</v>
       </c>
-      <c r="H105" s="1">
+      <c r="H105" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3952,7 +3978,7 @@
       <c r="C106" t="s">
         <v>115</v>
       </c>
-      <c r="H106" s="1">
+      <c r="H106" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3969,13 +3995,13 @@
       <c r="D107" t="s">
         <v>145</v>
       </c>
-      <c r="E107" s="1">
+      <c r="E107" s="2">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>194</v>
       </c>
-      <c r="H107" s="1">
+      <c r="H107" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3998,7 +4024,7 @@
       <c r="G108" t="s">
         <v>181</v>
       </c>
-      <c r="H108" s="1">
+      <c r="H108" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4012,7 +4038,7 @@
       <c r="C109" t="s">
         <v>119</v>
       </c>
-      <c r="H109" s="1">
+      <c r="H109" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4026,7 +4052,7 @@
       <c r="C110" t="s">
         <v>115</v>
       </c>
-      <c r="H110" s="1">
+      <c r="H110" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4049,7 +4075,7 @@
       <c r="G111" t="s">
         <v>176</v>
       </c>
-      <c r="H111" s="1">
+      <c r="H111" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4066,7 +4092,7 @@
       <c r="D112" t="s">
         <v>132</v>
       </c>
-      <c r="H112" s="1">
+      <c r="H112" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4089,7 +4115,7 @@
       <c r="G113" t="s">
         <v>177</v>
       </c>
-      <c r="H113" s="1">
+      <c r="H113" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4106,13 +4132,13 @@
       <c r="D114" t="s">
         <v>134</v>
       </c>
-      <c r="E114" s="1">
+      <c r="E114" s="2">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>197</v>
       </c>
-      <c r="H114" s="1">
+      <c r="H114" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4135,7 +4161,7 @@
       <c r="G115" t="s">
         <v>178</v>
       </c>
-      <c r="H115" s="1">
+      <c r="H115" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4158,7 +4184,7 @@
       <c r="G116" t="s">
         <v>178</v>
       </c>
-      <c r="H116" s="1">
+      <c r="H116" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4181,7 +4207,7 @@
       <c r="G117" t="s">
         <v>179</v>
       </c>
-      <c r="H117" s="1">
+      <c r="H117" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4195,7 +4221,7 @@
       <c r="C118" t="s">
         <v>115</v>
       </c>
-      <c r="H118" s="1">
+      <c r="H118" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4212,13 +4238,13 @@
       <c r="D119" t="s">
         <v>142</v>
       </c>
-      <c r="E119" s="1">
+      <c r="E119" s="2">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>199</v>
       </c>
-      <c r="H119" s="1">
+      <c r="H119" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4232,7 +4258,7 @@
       <c r="C120" t="s">
         <v>119</v>
       </c>
-      <c r="H120" s="1">
+      <c r="H120" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4246,7 +4272,7 @@
       <c r="C121" t="s">
         <v>115</v>
       </c>
-      <c r="H121" s="1">
+      <c r="H121" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4260,7 +4286,7 @@
       <c r="C122" t="s">
         <v>119</v>
       </c>
-      <c r="H122" s="1">
+      <c r="H122" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4274,7 +4300,7 @@
       <c r="C123" t="s">
         <v>119</v>
       </c>
-      <c r="H123" s="1">
+      <c r="H123" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="C124" t="s">
         <v>119</v>
       </c>
-      <c r="H124" s="1">
+      <c r="H124" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4305,13 +4331,13 @@
       <c r="D125" t="s">
         <v>125</v>
       </c>
-      <c r="E125" s="1">
+      <c r="E125" s="2">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>193</v>
       </c>
-      <c r="H125" s="1">
+      <c r="H125" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4328,13 +4354,13 @@
       <c r="D126" t="s">
         <v>126</v>
       </c>
-      <c r="E126" s="1">
+      <c r="E126" s="2">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>194</v>
       </c>
-      <c r="H126" s="1">
+      <c r="H126" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4348,7 +4374,7 @@
       <c r="C127" t="s">
         <v>115</v>
       </c>
-      <c r="H127" s="1">
+      <c r="H127" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4365,13 +4391,13 @@
       <c r="D128" t="s">
         <v>143</v>
       </c>
-      <c r="E128" s="1">
+      <c r="E128" s="2">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>194</v>
       </c>
-      <c r="H128" s="1">
+      <c r="H128" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4388,13 +4414,13 @@
       <c r="D129" t="s">
         <v>127</v>
       </c>
-      <c r="E129" s="1">
+      <c r="E129" s="2">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>194</v>
       </c>
-      <c r="H129" s="1">
+      <c r="H129" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4408,7 +4434,7 @@
       <c r="C130" t="s">
         <v>115</v>
       </c>
-      <c r="H130" s="1">
+      <c r="H130" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4425,13 +4451,13 @@
       <c r="D131" t="s">
         <v>128</v>
       </c>
-      <c r="E131" s="1">
+      <c r="E131" s="2">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>195</v>
       </c>
-      <c r="H131" s="1">
+      <c r="H131" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4448,13 +4474,13 @@
       <c r="D132" t="s">
         <v>144</v>
       </c>
-      <c r="E132" s="1">
+      <c r="E132" s="2">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>194</v>
       </c>
-      <c r="H132" s="1">
+      <c r="H132" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4468,7 +4494,7 @@
       <c r="C133" t="s">
         <v>115</v>
       </c>
-      <c r="H133" s="1">
+      <c r="H133" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4482,7 +4508,7 @@
       <c r="C134" t="s">
         <v>115</v>
       </c>
-      <c r="H134" s="1">
+      <c r="H134" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4496,7 +4522,7 @@
       <c r="C135" t="s">
         <v>115</v>
       </c>
-      <c r="H135" s="1">
+      <c r="H135" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4513,13 +4539,13 @@
       <c r="D136" t="s">
         <v>146</v>
       </c>
-      <c r="E136" s="1">
+      <c r="E136" s="2">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>194</v>
       </c>
-      <c r="H136" s="1">
+      <c r="H136" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4542,7 +4568,7 @@
       <c r="G137" t="s">
         <v>181</v>
       </c>
-      <c r="H137" s="1">
+      <c r="H137" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4556,7 +4582,7 @@
       <c r="C138" t="s">
         <v>119</v>
       </c>
-      <c r="H138" s="1">
+      <c r="H138" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4570,7 +4596,7 @@
       <c r="C139" t="s">
         <v>115</v>
       </c>
-      <c r="H139" s="1">
+      <c r="H139" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4593,7 +4619,7 @@
       <c r="G140" t="s">
         <v>176</v>
       </c>
-      <c r="H140" s="1">
+      <c r="H140" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4610,7 +4636,7 @@
       <c r="D141" t="s">
         <v>132</v>
       </c>
-      <c r="H141" s="1">
+      <c r="H141" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4633,7 +4659,7 @@
       <c r="G142" t="s">
         <v>177</v>
       </c>
-      <c r="H142" s="1">
+      <c r="H142" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4650,13 +4676,13 @@
       <c r="D143" t="s">
         <v>134</v>
       </c>
-      <c r="E143" s="1">
+      <c r="E143" s="2">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>197</v>
       </c>
-      <c r="H143" s="1">
+      <c r="H143" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4679,7 +4705,7 @@
       <c r="G144" t="s">
         <v>178</v>
       </c>
-      <c r="H144" s="1">
+      <c r="H144" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4702,7 +4728,7 @@
       <c r="G145" t="s">
         <v>178</v>
       </c>
-      <c r="H145" s="1">
+      <c r="H145" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4725,7 +4751,7 @@
       <c r="G146" t="s">
         <v>179</v>
       </c>
-      <c r="H146" s="1">
+      <c r="H146" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4739,7 +4765,7 @@
       <c r="C147" t="s">
         <v>115</v>
       </c>
-      <c r="H147" s="1">
+      <c r="H147" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4756,13 +4782,13 @@
       <c r="D148" t="s">
         <v>142</v>
       </c>
-      <c r="E148" s="1">
+      <c r="E148" s="2">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>199</v>
       </c>
-      <c r="H148" s="1">
+      <c r="H148" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4776,7 +4802,7 @@
       <c r="C149" t="s">
         <v>119</v>
       </c>
-      <c r="H149" s="1">
+      <c r="H149" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4790,7 +4816,7 @@
       <c r="C150" t="s">
         <v>115</v>
       </c>
-      <c r="H150" s="1">
+      <c r="H150" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4804,7 +4830,7 @@
       <c r="C151" t="s">
         <v>115</v>
       </c>
-      <c r="H151" s="1">
+      <c r="H151" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4818,7 +4844,7 @@
       <c r="C152" t="s">
         <v>119</v>
       </c>
-      <c r="H152" s="1">
+      <c r="H152" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4832,7 +4858,7 @@
       <c r="C153" t="s">
         <v>119</v>
       </c>
-      <c r="H153" s="1">
+      <c r="H153" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4849,13 +4875,13 @@
       <c r="D154" t="s">
         <v>125</v>
       </c>
-      <c r="E154" s="1">
+      <c r="E154" s="2">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>193</v>
       </c>
-      <c r="H154" s="1">
+      <c r="H154" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4872,13 +4898,13 @@
       <c r="D155" t="s">
         <v>126</v>
       </c>
-      <c r="E155" s="1">
+      <c r="E155" s="2">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>194</v>
       </c>
-      <c r="H155" s="1">
+      <c r="H155" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4892,7 +4918,7 @@
       <c r="C156" t="s">
         <v>115</v>
       </c>
-      <c r="H156" s="1">
+      <c r="H156" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4909,13 +4935,13 @@
       <c r="D157" t="s">
         <v>143</v>
       </c>
-      <c r="E157" s="1">
+      <c r="E157" s="2">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>194</v>
       </c>
-      <c r="H157" s="1">
+      <c r="H157" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4932,13 +4958,13 @@
       <c r="D158" t="s">
         <v>127</v>
       </c>
-      <c r="E158" s="1">
+      <c r="E158" s="2">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>194</v>
       </c>
-      <c r="H158" s="1">
+      <c r="H158" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4955,13 +4981,13 @@
       <c r="D159" t="s">
         <v>147</v>
       </c>
-      <c r="E159" s="1">
+      <c r="E159" s="2">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>200</v>
       </c>
-      <c r="H159" s="1">
+      <c r="H159" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4978,13 +5004,13 @@
       <c r="D160" t="s">
         <v>128</v>
       </c>
-      <c r="E160" s="1">
+      <c r="E160" s="2">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>195</v>
       </c>
-      <c r="H160" s="1">
+      <c r="H160" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5001,13 +5027,13 @@
       <c r="D161" t="s">
         <v>144</v>
       </c>
-      <c r="E161" s="1">
+      <c r="E161" s="2">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>194</v>
       </c>
-      <c r="H161" s="1">
+      <c r="H161" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5021,7 +5047,7 @@
       <c r="C162" t="s">
         <v>115</v>
       </c>
-      <c r="H162" s="1">
+      <c r="H162" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5035,7 +5061,7 @@
       <c r="C163" t="s">
         <v>115</v>
       </c>
-      <c r="H163" s="1">
+      <c r="H163" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5049,7 +5075,7 @@
       <c r="C164" t="s">
         <v>115</v>
       </c>
-      <c r="H164" s="1">
+      <c r="H164" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5066,13 +5092,13 @@
       <c r="D165" t="s">
         <v>146</v>
       </c>
-      <c r="E165" s="1">
+      <c r="E165" s="2">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>194</v>
       </c>
-      <c r="H165" s="1">
+      <c r="H165" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5095,7 +5121,7 @@
       <c r="G166" t="s">
         <v>181</v>
       </c>
-      <c r="H166" s="1">
+      <c r="H166" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5109,7 +5135,7 @@
       <c r="C167" t="s">
         <v>119</v>
       </c>
-      <c r="H167" s="1">
+      <c r="H167" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5123,7 +5149,7 @@
       <c r="C168" t="s">
         <v>115</v>
       </c>
-      <c r="H168" s="1">
+      <c r="H168" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5146,7 +5172,7 @@
       <c r="G169" t="s">
         <v>176</v>
       </c>
-      <c r="H169" s="1">
+      <c r="H169" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5163,7 +5189,7 @@
       <c r="D170" t="s">
         <v>132</v>
       </c>
-      <c r="H170" s="1">
+      <c r="H170" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5186,7 +5212,7 @@
       <c r="G171" t="s">
         <v>177</v>
       </c>
-      <c r="H171" s="1">
+      <c r="H171" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5203,13 +5229,13 @@
       <c r="D172" t="s">
         <v>134</v>
       </c>
-      <c r="E172" s="1">
+      <c r="E172" s="2">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>197</v>
       </c>
-      <c r="H172" s="1">
+      <c r="H172" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5232,7 +5258,7 @@
       <c r="G173" t="s">
         <v>178</v>
       </c>
-      <c r="H173" s="1">
+      <c r="H173" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5255,7 +5281,7 @@
       <c r="G174" t="s">
         <v>178</v>
       </c>
-      <c r="H174" s="1">
+      <c r="H174" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="G175" t="s">
         <v>179</v>
       </c>
-      <c r="H175" s="1">
+      <c r="H175" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5292,7 +5318,7 @@
       <c r="C176" t="s">
         <v>115</v>
       </c>
-      <c r="H176" s="1">
+      <c r="H176" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5309,13 +5335,13 @@
       <c r="D177" t="s">
         <v>148</v>
       </c>
-      <c r="E177" s="1">
+      <c r="E177" s="2">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>199</v>
       </c>
-      <c r="H177" s="1">
+      <c r="H177" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5329,7 +5355,7 @@
       <c r="C178" t="s">
         <v>115</v>
       </c>
-      <c r="H178" s="1">
+      <c r="H178" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5346,13 +5372,13 @@
       <c r="D179" t="s">
         <v>149</v>
       </c>
-      <c r="E179" s="1">
+      <c r="E179" s="2">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>195</v>
       </c>
-      <c r="H179" s="1">
+      <c r="H179" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5366,7 +5392,7 @@
       <c r="C180" t="s">
         <v>115</v>
       </c>
-      <c r="H180" s="1">
+      <c r="H180" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5380,7 +5406,7 @@
       <c r="C181" t="s">
         <v>119</v>
       </c>
-      <c r="H181" s="1">
+      <c r="H181" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5394,7 +5420,7 @@
       <c r="C182" t="s">
         <v>119</v>
       </c>
-      <c r="H182" s="1">
+      <c r="H182" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5411,13 +5437,13 @@
       <c r="D183" t="s">
         <v>125</v>
       </c>
-      <c r="E183" s="1">
+      <c r="E183" s="2">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>193</v>
       </c>
-      <c r="H183" s="1">
+      <c r="H183" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5434,13 +5460,13 @@
       <c r="D184" t="s">
         <v>126</v>
       </c>
-      <c r="E184" s="1">
+      <c r="E184" s="2">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>194</v>
       </c>
-      <c r="H184" s="1">
+      <c r="H184" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5454,7 +5480,7 @@
       <c r="C185" t="s">
         <v>115</v>
       </c>
-      <c r="H185" s="1">
+      <c r="H185" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5471,13 +5497,13 @@
       <c r="D186" t="s">
         <v>143</v>
       </c>
-      <c r="E186" s="1">
+      <c r="E186" s="2">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>194</v>
       </c>
-      <c r="H186" s="1">
+      <c r="H186" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5494,13 +5520,13 @@
       <c r="D187" t="s">
         <v>150</v>
       </c>
-      <c r="E187" s="1">
+      <c r="E187" s="2">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>194</v>
       </c>
-      <c r="H187" s="1">
+      <c r="H187" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5517,13 +5543,13 @@
       <c r="D188" t="s">
         <v>151</v>
       </c>
-      <c r="E188" s="1">
+      <c r="E188" s="2">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>194</v>
       </c>
-      <c r="H188" s="1">
+      <c r="H188" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5540,13 +5566,13 @@
       <c r="D189" t="s">
         <v>128</v>
       </c>
-      <c r="E189" s="1">
+      <c r="E189" s="2">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>195</v>
       </c>
-      <c r="H189" s="1">
+      <c r="H189" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5563,13 +5589,13 @@
       <c r="D190" t="s">
         <v>144</v>
       </c>
-      <c r="E190" s="1">
+      <c r="E190" s="2">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>194</v>
       </c>
-      <c r="H190" s="1">
+      <c r="H190" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5583,7 +5609,7 @@
       <c r="C191" t="s">
         <v>115</v>
       </c>
-      <c r="H191" s="1">
+      <c r="H191" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5597,7 +5623,7 @@
       <c r="C192" t="s">
         <v>115</v>
       </c>
-      <c r="H192" s="1">
+      <c r="H192" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5611,7 +5637,7 @@
       <c r="C193" t="s">
         <v>115</v>
       </c>
-      <c r="H193" s="1">
+      <c r="H193" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5628,13 +5654,13 @@
       <c r="D194" t="s">
         <v>146</v>
       </c>
-      <c r="E194" s="1">
+      <c r="E194" s="2">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>201</v>
       </c>
-      <c r="H194" s="1">
+      <c r="H194" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5657,7 +5683,7 @@
       <c r="G195" t="s">
         <v>181</v>
       </c>
-      <c r="H195" s="1">
+      <c r="H195" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5671,7 +5697,7 @@
       <c r="C196" t="s">
         <v>119</v>
       </c>
-      <c r="H196" s="1">
+      <c r="H196" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5685,7 +5711,7 @@
       <c r="C197" t="s">
         <v>115</v>
       </c>
-      <c r="H197" s="1">
+      <c r="H197" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5708,7 +5734,7 @@
       <c r="G198" t="s">
         <v>176</v>
       </c>
-      <c r="H198" s="1">
+      <c r="H198" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5725,7 +5751,7 @@
       <c r="D199" t="s">
         <v>132</v>
       </c>
-      <c r="H199" s="1">
+      <c r="H199" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5748,7 +5774,7 @@
       <c r="G200" t="s">
         <v>177</v>
       </c>
-      <c r="H200" s="1">
+      <c r="H200" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5765,13 +5791,13 @@
       <c r="D201" t="s">
         <v>134</v>
       </c>
-      <c r="E201" s="1">
+      <c r="E201" s="2">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>197</v>
       </c>
-      <c r="H201" s="1">
+      <c r="H201" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5794,7 +5820,7 @@
       <c r="G202" t="s">
         <v>178</v>
       </c>
-      <c r="H202" s="1">
+      <c r="H202" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5817,7 +5843,7 @@
       <c r="G203" t="s">
         <v>178</v>
       </c>
-      <c r="H203" s="1">
+      <c r="H203" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5840,7 +5866,7 @@
       <c r="G204" t="s">
         <v>179</v>
       </c>
-      <c r="H204" s="1">
+      <c r="H204" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5854,7 +5880,7 @@
       <c r="C205" t="s">
         <v>115</v>
       </c>
-      <c r="H205" s="1">
+      <c r="H205" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5871,13 +5897,13 @@
       <c r="D206" t="s">
         <v>148</v>
       </c>
-      <c r="E206" s="1">
+      <c r="E206" s="2">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>199</v>
       </c>
-      <c r="H206" s="1">
+      <c r="H206" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5891,7 +5917,7 @@
       <c r="C207" t="s">
         <v>115</v>
       </c>
-      <c r="H207" s="1">
+      <c r="H207" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5905,7 +5931,7 @@
       <c r="C208" t="s">
         <v>119</v>
       </c>
-      <c r="H208" s="1">
+      <c r="H208" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5919,7 +5945,7 @@
       <c r="C209" t="s">
         <v>115</v>
       </c>
-      <c r="H209" s="1">
+      <c r="H209" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5933,7 +5959,7 @@
       <c r="C210" t="s">
         <v>119</v>
       </c>
-      <c r="H210" s="1">
+      <c r="H210" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5947,7 +5973,7 @@
       <c r="C211" t="s">
         <v>119</v>
       </c>
-      <c r="H211" s="1">
+      <c r="H211" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5964,13 +5990,13 @@
       <c r="D212" t="s">
         <v>125</v>
       </c>
-      <c r="E212" s="1">
+      <c r="E212" s="2">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>193</v>
       </c>
-      <c r="H212" s="1">
+      <c r="H212" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5984,7 +6010,7 @@
       <c r="C213" t="s">
         <v>119</v>
       </c>
-      <c r="H213" s="1">
+      <c r="H213" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5998,7 +6024,7 @@
       <c r="C214" t="s">
         <v>115</v>
       </c>
-      <c r="H214" s="1">
+      <c r="H214" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6015,13 +6041,13 @@
       <c r="D215" t="s">
         <v>143</v>
       </c>
-      <c r="E215" s="1">
+      <c r="E215" s="2">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>202</v>
       </c>
-      <c r="H215" s="1">
+      <c r="H215" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6038,13 +6064,13 @@
       <c r="D216" t="s">
         <v>150</v>
       </c>
-      <c r="E216" s="1">
+      <c r="E216" s="2">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>195</v>
       </c>
-      <c r="H216" s="1">
+      <c r="H216" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6058,7 +6084,7 @@
       <c r="C217" t="s">
         <v>115</v>
       </c>
-      <c r="H217" s="1">
+      <c r="H217" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6075,13 +6101,13 @@
       <c r="D218" t="s">
         <v>128</v>
       </c>
-      <c r="E218" s="1">
+      <c r="E218" s="2">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>195</v>
       </c>
-      <c r="H218" s="1">
+      <c r="H218" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6095,7 +6121,7 @@
       <c r="C219" t="s">
         <v>115</v>
       </c>
-      <c r="H219" s="1">
+      <c r="H219" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6109,7 +6135,7 @@
       <c r="C220" t="s">
         <v>115</v>
       </c>
-      <c r="H220" s="1">
+      <c r="H220" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6126,13 +6152,13 @@
       <c r="D221" t="s">
         <v>152</v>
       </c>
-      <c r="E221" s="1">
+      <c r="E221" s="2">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>199</v>
       </c>
-      <c r="H221" s="1">
+      <c r="H221" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6146,7 +6172,7 @@
       <c r="C222" t="s">
         <v>115</v>
       </c>
-      <c r="H222" s="1">
+      <c r="H222" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6163,13 +6189,13 @@
       <c r="D223" t="s">
         <v>153</v>
       </c>
-      <c r="E223" s="1">
+      <c r="E223" s="2">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>203</v>
       </c>
-      <c r="H223" s="1">
+      <c r="H223" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6192,7 +6218,7 @@
       <c r="G224" t="s">
         <v>181</v>
       </c>
-      <c r="H224" s="1">
+      <c r="H224" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6206,7 +6232,7 @@
       <c r="C225" t="s">
         <v>119</v>
       </c>
-      <c r="H225" s="1">
+      <c r="H225" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="C226" t="s">
         <v>115</v>
       </c>
-      <c r="H226" s="1">
+      <c r="H226" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6243,7 +6269,7 @@
       <c r="G227" t="s">
         <v>176</v>
       </c>
-      <c r="H227" s="1">
+      <c r="H227" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6260,7 +6286,7 @@
       <c r="D228" t="s">
         <v>132</v>
       </c>
-      <c r="H228" s="1">
+      <c r="H228" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6283,7 +6309,7 @@
       <c r="G229" t="s">
         <v>177</v>
       </c>
-      <c r="H229" s="1">
+      <c r="H229" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6300,13 +6326,13 @@
       <c r="D230" t="s">
         <v>154</v>
       </c>
-      <c r="E230" s="1">
+      <c r="E230" s="2">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>204</v>
       </c>
-      <c r="H230" s="1">
+      <c r="H230" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6329,7 +6355,7 @@
       <c r="G231" t="s">
         <v>178</v>
       </c>
-      <c r="H231" s="1">
+      <c r="H231" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="G232" t="s">
         <v>178</v>
       </c>
-      <c r="H232" s="1">
+      <c r="H232" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6375,7 +6401,7 @@
       <c r="G233" t="s">
         <v>179</v>
       </c>
-      <c r="H233" s="1">
+      <c r="H233" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6389,7 +6415,7 @@
       <c r="C234" t="s">
         <v>115</v>
       </c>
-      <c r="H234" s="1">
+      <c r="H234" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6406,13 +6432,13 @@
       <c r="D235" t="s">
         <v>155</v>
       </c>
-      <c r="E235" s="1">
+      <c r="E235" s="2">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>199</v>
       </c>
-      <c r="H235" s="1">
+      <c r="H235" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6426,7 +6452,7 @@
       <c r="C236" t="s">
         <v>115</v>
       </c>
-      <c r="H236" s="1">
+      <c r="H236" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6440,7 +6466,7 @@
       <c r="C237" t="s">
         <v>119</v>
       </c>
-      <c r="H237" s="1">
+      <c r="H237" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6454,7 +6480,7 @@
       <c r="C238" t="s">
         <v>115</v>
       </c>
-      <c r="H238" s="1">
+      <c r="H238" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6468,7 +6494,7 @@
       <c r="C239" t="s">
         <v>119</v>
       </c>
-      <c r="H239" s="1">
+      <c r="H239" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6482,7 +6508,7 @@
       <c r="C240" t="s">
         <v>119</v>
       </c>
-      <c r="H240" s="1">
+      <c r="H240" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6499,13 +6525,13 @@
       <c r="D241" t="s">
         <v>125</v>
       </c>
-      <c r="E241" s="1">
+      <c r="E241" s="2">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>193</v>
       </c>
-      <c r="H241" s="1">
+      <c r="H241" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6519,7 +6545,7 @@
       <c r="C242" t="s">
         <v>119</v>
       </c>
-      <c r="H242" s="1">
+      <c r="H242" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6536,13 +6562,13 @@
       <c r="D243" t="s">
         <v>156</v>
       </c>
-      <c r="E243" s="1">
+      <c r="E243" s="2">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>205</v>
       </c>
-      <c r="H243" s="1">
+      <c r="H243" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6559,13 +6585,13 @@
       <c r="D244" t="s">
         <v>157</v>
       </c>
-      <c r="E244" s="1">
+      <c r="E244" s="2">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>202</v>
       </c>
-      <c r="H244" s="1">
+      <c r="H244" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6579,7 +6605,7 @@
       <c r="C245" t="s">
         <v>119</v>
       </c>
-      <c r="H245" s="1">
+      <c r="H245" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6593,7 +6619,7 @@
       <c r="C246" t="s">
         <v>115</v>
       </c>
-      <c r="H246" s="1">
+      <c r="H246" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6610,13 +6636,13 @@
       <c r="D247" t="s">
         <v>128</v>
       </c>
-      <c r="E247" s="1">
+      <c r="E247" s="2">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>206</v>
       </c>
-      <c r="H247" s="1">
+      <c r="H247" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6630,7 +6656,7 @@
       <c r="C248" t="s">
         <v>115</v>
       </c>
-      <c r="H248" s="1">
+      <c r="H248" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6644,7 +6670,7 @@
       <c r="C249" t="s">
         <v>115</v>
       </c>
-      <c r="H249" s="1">
+      <c r="H249" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6661,13 +6687,13 @@
       <c r="D250" t="s">
         <v>158</v>
       </c>
-      <c r="E250" s="1">
+      <c r="E250" s="2">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>201</v>
       </c>
-      <c r="H250" s="1">
+      <c r="H250" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6681,7 +6707,7 @@
       <c r="C251" t="s">
         <v>115</v>
       </c>
-      <c r="H251" s="1">
+      <c r="H251" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6698,13 +6724,13 @@
       <c r="D252" t="s">
         <v>159</v>
       </c>
-      <c r="E252" s="1">
+      <c r="E252" s="2">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>203</v>
       </c>
-      <c r="H252" s="1">
+      <c r="H252" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6727,7 +6753,7 @@
       <c r="G253" t="s">
         <v>181</v>
       </c>
-      <c r="H253" s="1">
+      <c r="H253" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6741,7 +6767,7 @@
       <c r="C254" t="s">
         <v>119</v>
       </c>
-      <c r="H254" s="1">
+      <c r="H254" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6755,7 +6781,7 @@
       <c r="C255" t="s">
         <v>115</v>
       </c>
-      <c r="H255" s="1">
+      <c r="H255" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6778,7 +6804,7 @@
       <c r="G256" t="s">
         <v>176</v>
       </c>
-      <c r="H256" s="1">
+      <c r="H256" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6795,7 +6821,7 @@
       <c r="D257" t="s">
         <v>132</v>
       </c>
-      <c r="H257" s="1">
+      <c r="H257" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6818,7 +6844,7 @@
       <c r="G258" t="s">
         <v>177</v>
       </c>
-      <c r="H258" s="1">
+      <c r="H258" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6835,13 +6861,13 @@
       <c r="D259" t="s">
         <v>154</v>
       </c>
-      <c r="E259" s="1">
+      <c r="E259" s="2">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>204</v>
       </c>
-      <c r="H259" s="1">
+      <c r="H259" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6864,7 +6890,7 @@
       <c r="G260" t="s">
         <v>178</v>
       </c>
-      <c r="H260" s="1">
+      <c r="H260" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6887,7 +6913,7 @@
       <c r="G261" t="s">
         <v>178</v>
       </c>
-      <c r="H261" s="1">
+      <c r="H261" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6910,7 +6936,7 @@
       <c r="G262" t="s">
         <v>179</v>
       </c>
-      <c r="H262" s="1">
+      <c r="H262" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6924,7 +6950,7 @@
       <c r="C263" t="s">
         <v>115</v>
       </c>
-      <c r="H263" s="1">
+      <c r="H263" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6941,13 +6967,13 @@
       <c r="D264" t="s">
         <v>155</v>
       </c>
-      <c r="E264" s="1">
+      <c r="E264" s="2">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>199</v>
       </c>
-      <c r="H264" s="1">
+      <c r="H264" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6961,7 +6987,7 @@
       <c r="C265" t="s">
         <v>115</v>
       </c>
-      <c r="H265" s="1">
+      <c r="H265" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6975,7 +7001,7 @@
       <c r="C266" t="s">
         <v>119</v>
       </c>
-      <c r="H266" s="1">
+      <c r="H266" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6989,7 +7015,7 @@
       <c r="C267" t="s">
         <v>115</v>
       </c>
-      <c r="H267" s="1">
+      <c r="H267" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7003,7 +7029,7 @@
       <c r="C268" t="s">
         <v>119</v>
       </c>
-      <c r="H268" s="1">
+      <c r="H268" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7017,7 +7043,7 @@
       <c r="C269" t="s">
         <v>119</v>
       </c>
-      <c r="H269" s="1">
+      <c r="H269" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7034,13 +7060,13 @@
       <c r="D270" t="s">
         <v>125</v>
       </c>
-      <c r="E270" s="1">
+      <c r="E270" s="2">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>193</v>
       </c>
-      <c r="H270" s="1">
+      <c r="H270" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7054,7 +7080,7 @@
       <c r="C271" t="s">
         <v>119</v>
       </c>
-      <c r="H271" s="1">
+      <c r="H271" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7071,13 +7097,13 @@
       <c r="D272" t="s">
         <v>156</v>
       </c>
-      <c r="E272" s="1">
+      <c r="E272" s="2">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>205</v>
       </c>
-      <c r="H272" s="1">
+      <c r="H272" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7094,13 +7120,13 @@
       <c r="D273" t="s">
         <v>157</v>
       </c>
-      <c r="E273" s="1">
+      <c r="E273" s="2">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>207</v>
       </c>
-      <c r="H273" s="1">
+      <c r="H273" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7114,7 +7140,7 @@
       <c r="C274" t="s">
         <v>115</v>
       </c>
-      <c r="H274" s="1">
+      <c r="H274" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7128,7 +7154,7 @@
       <c r="C275" t="s">
         <v>115</v>
       </c>
-      <c r="H275" s="1">
+      <c r="H275" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7145,13 +7171,13 @@
       <c r="D276" t="s">
         <v>128</v>
       </c>
-      <c r="E276" s="1">
+      <c r="E276" s="2">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>206</v>
       </c>
-      <c r="H276" s="1">
+      <c r="H276" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7165,7 +7191,7 @@
       <c r="C277" t="s">
         <v>115</v>
       </c>
-      <c r="H277" s="1">
+      <c r="H277" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7182,13 +7208,13 @@
       <c r="D278" t="s">
         <v>160</v>
       </c>
-      <c r="E278" s="1">
+      <c r="E278" s="2">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>208</v>
       </c>
-      <c r="H278" s="1">
+      <c r="H278" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7205,13 +7231,13 @@
       <c r="D279" t="s">
         <v>158</v>
       </c>
-      <c r="E279" s="1">
+      <c r="E279" s="2">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>207</v>
       </c>
-      <c r="H279" s="1">
+      <c r="H279" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7225,7 +7251,7 @@
       <c r="C280" t="s">
         <v>115</v>
       </c>
-      <c r="H280" s="1">
+      <c r="H280" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7242,13 +7268,13 @@
       <c r="D281" t="s">
         <v>161</v>
       </c>
-      <c r="E281" s="1">
+      <c r="E281" s="2">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>203</v>
       </c>
-      <c r="H281" s="1">
+      <c r="H281" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7271,7 +7297,7 @@
       <c r="G282" t="s">
         <v>181</v>
       </c>
-      <c r="H282" s="1">
+      <c r="H282" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7285,7 +7311,7 @@
       <c r="C283" t="s">
         <v>119</v>
       </c>
-      <c r="H283" s="1">
+      <c r="H283" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7299,7 +7325,7 @@
       <c r="C284" t="s">
         <v>115</v>
       </c>
-      <c r="H284" s="1">
+      <c r="H284" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7322,7 +7348,7 @@
       <c r="G285" t="s">
         <v>176</v>
       </c>
-      <c r="H285" s="1">
+      <c r="H285" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7339,7 +7365,7 @@
       <c r="D286" t="s">
         <v>132</v>
       </c>
-      <c r="H286" s="1">
+      <c r="H286" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7362,7 +7388,7 @@
       <c r="G287" t="s">
         <v>177</v>
       </c>
-      <c r="H287" s="1">
+      <c r="H287" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7379,13 +7405,13 @@
       <c r="D288" t="s">
         <v>154</v>
       </c>
-      <c r="E288" s="1">
+      <c r="E288" s="2">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>204</v>
       </c>
-      <c r="H288" s="1">
+      <c r="H288" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7408,7 +7434,7 @@
       <c r="G289" t="s">
         <v>178</v>
       </c>
-      <c r="H289" s="1">
+      <c r="H289" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7431,7 +7457,7 @@
       <c r="G290" t="s">
         <v>178</v>
       </c>
-      <c r="H290" s="1">
+      <c r="H290" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7454,7 +7480,7 @@
       <c r="G291" t="s">
         <v>179</v>
       </c>
-      <c r="H291" s="1">
+      <c r="H291" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7468,7 +7494,7 @@
       <c r="C292" t="s">
         <v>115</v>
       </c>
-      <c r="H292" s="1">
+      <c r="H292" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7491,7 +7517,7 @@
       <c r="G293" t="s">
         <v>182</v>
       </c>
-      <c r="H293" s="1">
+      <c r="H293" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7505,7 +7531,7 @@
       <c r="C294" t="s">
         <v>115</v>
       </c>
-      <c r="H294" s="1">
+      <c r="H294" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7528,7 +7554,7 @@
       <c r="G295" t="s">
         <v>183</v>
       </c>
-      <c r="H295" s="1">
+      <c r="H295" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7542,7 +7568,7 @@
       <c r="C296" t="s">
         <v>115</v>
       </c>
-      <c r="H296" s="1">
+      <c r="H296" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7556,7 +7582,7 @@
       <c r="C297" t="s">
         <v>119</v>
       </c>
-      <c r="H297" s="1">
+      <c r="H297" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7579,7 +7605,7 @@
       <c r="G298" t="s">
         <v>184</v>
       </c>
-      <c r="H298" s="1">
+      <c r="H298" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7596,13 +7622,13 @@
       <c r="D299" t="s">
         <v>125</v>
       </c>
-      <c r="E299" s="1">
+      <c r="E299" s="2">
         <v>46234</v>
       </c>
       <c r="G299" t="s">
         <v>193</v>
       </c>
-      <c r="H299" s="1">
+      <c r="H299" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7616,7 +7642,7 @@
       <c r="C300" t="s">
         <v>115</v>
       </c>
-      <c r="H300" s="1">
+      <c r="H300" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7633,13 +7659,13 @@
       <c r="D301" t="s">
         <v>156</v>
       </c>
-      <c r="E301" s="1">
+      <c r="E301" s="2">
         <v>46224</v>
       </c>
       <c r="G301" t="s">
         <v>205</v>
       </c>
-      <c r="H301" s="1">
+      <c r="H301" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7656,13 +7682,13 @@
       <c r="D302" t="s">
         <v>157</v>
       </c>
-      <c r="E302" s="1">
+      <c r="E302" s="2">
         <v>46220</v>
       </c>
       <c r="G302" t="s">
         <v>202</v>
       </c>
-      <c r="H302" s="1">
+      <c r="H302" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7676,7 +7702,7 @@
       <c r="C303" t="s">
         <v>115</v>
       </c>
-      <c r="H303" s="1">
+      <c r="H303" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7690,7 +7716,7 @@
       <c r="C304" t="s">
         <v>115</v>
       </c>
-      <c r="H304" s="1">
+      <c r="H304" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7707,13 +7733,13 @@
       <c r="D305" t="s">
         <v>128</v>
       </c>
-      <c r="E305" s="1">
+      <c r="E305" s="2">
         <v>46237</v>
       </c>
       <c r="G305" t="s">
         <v>206</v>
       </c>
-      <c r="H305" s="1">
+      <c r="H305" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7727,7 +7753,7 @@
       <c r="C306" t="s">
         <v>115</v>
       </c>
-      <c r="H306" s="1">
+      <c r="H306" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7744,13 +7770,13 @@
       <c r="D307" t="s">
         <v>160</v>
       </c>
-      <c r="E307" s="1">
+      <c r="E307" s="2">
         <v>46227</v>
       </c>
       <c r="G307" t="s">
         <v>208</v>
       </c>
-      <c r="H307" s="1">
+      <c r="H307" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7764,7 +7790,7 @@
       <c r="C308" t="s">
         <v>119</v>
       </c>
-      <c r="H308" s="1">
+      <c r="H308" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7787,7 +7813,7 @@
       <c r="G309" t="s">
         <v>182</v>
       </c>
-      <c r="H309" s="1">
+      <c r="H309" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7810,7 +7836,7 @@
       <c r="G310" t="s">
         <v>185</v>
       </c>
-      <c r="H310" s="1">
+      <c r="H310" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7827,7 +7853,7 @@
       <c r="D311" t="s">
         <v>166</v>
       </c>
-      <c r="H311" s="1">
+      <c r="H311" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7841,7 +7867,7 @@
       <c r="C312" t="s">
         <v>119</v>
       </c>
-      <c r="H312" s="1">
+      <c r="H312" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7855,7 +7881,7 @@
       <c r="C313" t="s">
         <v>115</v>
       </c>
-      <c r="H313" s="1">
+      <c r="H313" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7878,7 +7904,7 @@
       <c r="G314" t="s">
         <v>176</v>
       </c>
-      <c r="H314" s="1">
+      <c r="H314" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7895,7 +7921,7 @@
       <c r="D315" t="s">
         <v>132</v>
       </c>
-      <c r="H315" s="1">
+      <c r="H315" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7918,7 +7944,7 @@
       <c r="G316" t="s">
         <v>177</v>
       </c>
-      <c r="H316" s="1">
+      <c r="H316" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7941,7 +7967,7 @@
       <c r="G317" t="s">
         <v>186</v>
       </c>
-      <c r="H317" s="1">
+      <c r="H317" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7964,7 +7990,7 @@
       <c r="G318" t="s">
         <v>178</v>
       </c>
-      <c r="H318" s="1">
+      <c r="H318" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7987,7 +8013,7 @@
       <c r="G319" t="s">
         <v>178</v>
       </c>
-      <c r="H319" s="1">
+      <c r="H319" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -8010,7 +8036,7 @@
       <c r="G320" t="s">
         <v>179</v>
       </c>
-      <c r="H320" s="1">
+      <c r="H320" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -8024,7 +8050,7 @@
       <c r="C321" t="s">
         <v>115</v>
       </c>
-      <c r="H321" s="1">
+      <c r="H321" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8047,7 +8073,7 @@
       <c r="G322" t="s">
         <v>187</v>
       </c>
-      <c r="H322" s="1">
+      <c r="H322" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8061,7 +8087,7 @@
       <c r="C323" t="s">
         <v>115</v>
       </c>
-      <c r="H323" s="1">
+      <c r="H323" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8084,7 +8110,7 @@
       <c r="G324" t="s">
         <v>188</v>
       </c>
-      <c r="H324" s="1">
+      <c r="H324" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8098,7 +8124,7 @@
       <c r="C325" t="s">
         <v>115</v>
       </c>
-      <c r="H325" s="1">
+      <c r="H325" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8112,7 +8138,7 @@
       <c r="C326" t="s">
         <v>119</v>
       </c>
-      <c r="H326" s="1">
+      <c r="H326" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8126,7 +8152,7 @@
       <c r="C327" t="s">
         <v>119</v>
       </c>
-      <c r="H327" s="1">
+      <c r="H327" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8143,13 +8169,13 @@
       <c r="D328" t="s">
         <v>125</v>
       </c>
-      <c r="E328" s="1">
+      <c r="E328" s="2">
         <v>46234</v>
       </c>
       <c r="G328" t="s">
         <v>193</v>
       </c>
-      <c r="H328" s="1">
+      <c r="H328" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8172,7 +8198,7 @@
       <c r="G329" t="s">
         <v>188</v>
       </c>
-      <c r="H329" s="1">
+      <c r="H329" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8195,7 +8221,7 @@
       <c r="G330" t="s">
         <v>188</v>
       </c>
-      <c r="H330" s="1">
+      <c r="H330" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8209,7 +8235,7 @@
       <c r="C331" t="s">
         <v>115</v>
       </c>
-      <c r="H331" s="1">
+      <c r="H331" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8232,7 +8258,7 @@
       <c r="G332" t="s">
         <v>188</v>
       </c>
-      <c r="H332" s="1">
+      <c r="H332" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8255,7 +8281,7 @@
       <c r="G333" t="s">
         <v>187</v>
       </c>
-      <c r="H333" s="1">
+      <c r="H333" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8272,13 +8298,13 @@
       <c r="D334" t="s">
         <v>128</v>
       </c>
-      <c r="E334" s="1">
+      <c r="E334" s="2">
         <v>46237</v>
       </c>
       <c r="G334" t="s">
         <v>206</v>
       </c>
-      <c r="H334" s="1">
+      <c r="H334" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8292,7 +8318,7 @@
       <c r="C335" t="s">
         <v>115</v>
       </c>
-      <c r="H335" s="1">
+      <c r="H335" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8309,13 +8335,13 @@
       <c r="D336" t="s">
         <v>160</v>
       </c>
-      <c r="E336" s="1">
+      <c r="E336" s="2">
         <v>46227</v>
       </c>
       <c r="G336" t="s">
         <v>208</v>
       </c>
-      <c r="H336" s="1">
+      <c r="H336" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8329,7 +8355,7 @@
       <c r="C337" t="s">
         <v>115</v>
       </c>
-      <c r="H337" s="1">
+      <c r="H337" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8343,7 +8369,7 @@
       <c r="C338" t="s">
         <v>115</v>
       </c>
-      <c r="H338" s="1">
+      <c r="H338" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8366,7 +8392,7 @@
       <c r="G339" t="s">
         <v>185</v>
       </c>
-      <c r="H339" s="1">
+      <c r="H339" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8383,7 +8409,7 @@
       <c r="D340" t="s">
         <v>171</v>
       </c>
-      <c r="H340" s="1">
+      <c r="H340" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8397,7 +8423,7 @@
       <c r="C341" t="s">
         <v>119</v>
       </c>
-      <c r="H341" s="1">
+      <c r="H341" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8411,7 +8437,7 @@
       <c r="C342" t="s">
         <v>115</v>
       </c>
-      <c r="H342" s="1">
+      <c r="H342" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8434,7 +8460,7 @@
       <c r="G343" t="s">
         <v>176</v>
       </c>
-      <c r="H343" s="1">
+      <c r="H343" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8451,7 +8477,7 @@
       <c r="D344" t="s">
         <v>132</v>
       </c>
-      <c r="H344" s="1">
+      <c r="H344" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8474,7 +8500,7 @@
       <c r="G345" t="s">
         <v>177</v>
       </c>
-      <c r="H345" s="1">
+      <c r="H345" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8497,7 +8523,7 @@
       <c r="G346" t="s">
         <v>186</v>
       </c>
-      <c r="H346" s="1">
+      <c r="H346" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8520,7 +8546,7 @@
       <c r="G347" t="s">
         <v>178</v>
       </c>
-      <c r="H347" s="1">
+      <c r="H347" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8543,7 +8569,7 @@
       <c r="G348" t="s">
         <v>178</v>
       </c>
-      <c r="H348" s="1">
+      <c r="H348" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8566,7 +8592,7 @@
       <c r="G349" t="s">
         <v>179</v>
       </c>
-      <c r="H349" s="1">
+      <c r="H349" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8580,7 +8606,7 @@
       <c r="C350" t="s">
         <v>115</v>
       </c>
-      <c r="H350" s="1">
+      <c r="H350" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8603,7 +8629,7 @@
       <c r="G351" t="s">
         <v>187</v>
       </c>
-      <c r="H351" s="1">
+      <c r="H351" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8617,7 +8643,7 @@
       <c r="C352" t="s">
         <v>115</v>
       </c>
-      <c r="H352" s="1">
+      <c r="H352" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8631,7 +8657,7 @@
       <c r="C353" t="s">
         <v>115</v>
       </c>
-      <c r="H353" s="1">
+      <c r="H353" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8645,7 +8671,7 @@
       <c r="C354" t="s">
         <v>115</v>
       </c>
-      <c r="H354" s="1">
+      <c r="H354" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8659,7 +8685,7 @@
       <c r="C355" t="s">
         <v>119</v>
       </c>
-      <c r="H355" s="1">
+      <c r="H355" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8673,7 +8699,7 @@
       <c r="C356" t="s">
         <v>119</v>
       </c>
-      <c r="H356" s="1">
+      <c r="H356" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8696,7 +8722,7 @@
       <c r="G357" t="s">
         <v>189</v>
       </c>
-      <c r="H357" s="1">
+      <c r="H357" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8710,7 +8736,7 @@
       <c r="C358" t="s">
         <v>115</v>
       </c>
-      <c r="H358" s="1">
+      <c r="H358" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8733,7 +8759,7 @@
       <c r="G359" t="s">
         <v>190</v>
       </c>
-      <c r="H359" s="1">
+      <c r="H359" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8747,7 +8773,7 @@
       <c r="C360" t="s">
         <v>115</v>
       </c>
-      <c r="H360" s="1">
+      <c r="H360" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8761,7 +8787,7 @@
       <c r="C361" t="s">
         <v>115</v>
       </c>
-      <c r="H361" s="1">
+      <c r="H361" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8784,7 +8810,7 @@
       <c r="G362" t="s">
         <v>187</v>
       </c>
-      <c r="H362" s="1">
+      <c r="H362" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8807,7 +8833,7 @@
       <c r="G363" t="s">
         <v>191</v>
       </c>
-      <c r="H363" s="1">
+      <c r="H363" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8821,7 +8847,7 @@
       <c r="C364" t="s">
         <v>115</v>
       </c>
-      <c r="H364" s="1">
+      <c r="H364" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8844,7 +8870,7 @@
       <c r="G365" t="s">
         <v>190</v>
       </c>
-      <c r="H365" s="1">
+      <c r="H365" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8858,7 +8884,7 @@
       <c r="C366" t="s">
         <v>115</v>
       </c>
-      <c r="H366" s="1">
+      <c r="H366" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8872,7 +8898,7 @@
       <c r="C367" t="s">
         <v>115</v>
       </c>
-      <c r="H367" s="1">
+      <c r="H367" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8895,7 +8921,7 @@
       <c r="G368" t="s">
         <v>189</v>
       </c>
-      <c r="H368" s="1">
+      <c r="H368" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8918,7 +8944,7 @@
       <c r="G369" t="s">
         <v>190</v>
       </c>
-      <c r="H369" s="1">
+      <c r="H369" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8935,7 +8961,7 @@
       <c r="D370" t="s">
         <v>171</v>
       </c>
-      <c r="H370" s="1">
+      <c r="H370" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8949,7 +8975,7 @@
       <c r="C371" t="s">
         <v>115</v>
       </c>
-      <c r="H371" s="1">
+      <c r="H371" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8972,7 +8998,7 @@
       <c r="G372" t="s">
         <v>176</v>
       </c>
-      <c r="H372" s="1">
+      <c r="H372" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8989,7 +9015,7 @@
       <c r="D373" t="s">
         <v>132</v>
       </c>
-      <c r="H373" s="1">
+      <c r="H373" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9012,7 +9038,7 @@
       <c r="G374" t="s">
         <v>177</v>
       </c>
-      <c r="H374" s="1">
+      <c r="H374" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9035,7 +9061,7 @@
       <c r="G375" t="s">
         <v>186</v>
       </c>
-      <c r="H375" s="1">
+      <c r="H375" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9058,7 +9084,7 @@
       <c r="G376" t="s">
         <v>178</v>
       </c>
-      <c r="H376" s="1">
+      <c r="H376" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9081,7 +9107,7 @@
       <c r="G377" t="s">
         <v>178</v>
       </c>
-      <c r="H377" s="1">
+      <c r="H377" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9104,7 +9130,7 @@
       <c r="G378" t="s">
         <v>179</v>
       </c>
-      <c r="H378" s="1">
+      <c r="H378" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9118,7 +9144,7 @@
       <c r="C379" t="s">
         <v>115</v>
       </c>
-      <c r="H379" s="1">
+      <c r="H379" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9141,7 +9167,7 @@
       <c r="G380" t="s">
         <v>190</v>
       </c>
-      <c r="H380" s="1">
+      <c r="H380" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9155,7 +9181,7 @@
       <c r="C381" t="s">
         <v>115</v>
       </c>
-      <c r="H381" s="1">
+      <c r="H381" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9169,7 +9195,7 @@
       <c r="C382" t="s">
         <v>115</v>
       </c>
-      <c r="H382" s="1">
+      <c r="H382" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9183,7 +9209,7 @@
       <c r="C383" t="s">
         <v>115</v>
       </c>
-      <c r="H383" s="1">
+      <c r="H383" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9197,7 +9223,7 @@
       <c r="C384" t="s">
         <v>119</v>
       </c>
-      <c r="H384" s="1">
+      <c r="H384" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9211,7 +9237,7 @@
       <c r="C385" t="s">
         <v>119</v>
       </c>
-      <c r="H385" s="1">
+      <c r="H385" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9234,7 +9260,7 @@
       <c r="G386" t="s">
         <v>189</v>
       </c>
-      <c r="H386" s="1">
+      <c r="H386" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9248,7 +9274,7 @@
       <c r="C387" t="s">
         <v>115</v>
       </c>
-      <c r="H387" s="1">
+      <c r="H387" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9262,7 +9288,7 @@
       <c r="C388" t="s">
         <v>119</v>
       </c>
-      <c r="H388" s="1">
+      <c r="H388" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9276,7 +9302,7 @@
       <c r="C389" t="s">
         <v>115</v>
       </c>
-      <c r="H389" s="1">
+      <c r="H389" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9290,7 +9316,7 @@
       <c r="C390" t="s">
         <v>115</v>
       </c>
-      <c r="H390" s="1">
+      <c r="H390" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9313,7 +9339,7 @@
       <c r="G391" t="s">
         <v>190</v>
       </c>
-      <c r="H391" s="1">
+      <c r="H391" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9336,7 +9362,7 @@
       <c r="G392" t="s">
         <v>191</v>
       </c>
-      <c r="H392" s="1">
+      <c r="H392" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9350,7 +9376,7 @@
       <c r="C393" t="s">
         <v>115</v>
       </c>
-      <c r="H393" s="1">
+      <c r="H393" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9373,7 +9399,7 @@
       <c r="G394" t="s">
         <v>190</v>
       </c>
-      <c r="H394" s="1">
+      <c r="H394" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9387,7 +9413,7 @@
       <c r="C395" t="s">
         <v>115</v>
       </c>
-      <c r="H395" s="1">
+      <c r="H395" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9401,7 +9427,7 @@
       <c r="C396" t="s">
         <v>115</v>
       </c>
-      <c r="H396" s="1">
+      <c r="H396" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9424,7 +9450,7 @@
       <c r="G397" t="s">
         <v>189</v>
       </c>
-      <c r="H397" s="1">
+      <c r="H397" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9447,7 +9473,7 @@
       <c r="G398" t="s">
         <v>190</v>
       </c>
-      <c r="H398" s="1">
+      <c r="H398" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9464,7 +9490,7 @@
       <c r="D399" t="s">
         <v>171</v>
       </c>
-      <c r="H399" s="1">
+      <c r="H399" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9478,7 +9504,7 @@
       <c r="C400" t="s">
         <v>115</v>
       </c>
-      <c r="H400" s="1">
+      <c r="H400" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9501,7 +9527,7 @@
       <c r="G401" t="s">
         <v>176</v>
       </c>
-      <c r="H401" s="1">
+      <c r="H401" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9518,7 +9544,7 @@
       <c r="D402" t="s">
         <v>132</v>
       </c>
-      <c r="H402" s="1">
+      <c r="H402" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9541,7 +9567,7 @@
       <c r="G403" t="s">
         <v>177</v>
       </c>
-      <c r="H403" s="1">
+      <c r="H403" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9564,7 +9590,7 @@
       <c r="G404" t="s">
         <v>186</v>
       </c>
-      <c r="H404" s="1">
+      <c r="H404" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9587,7 +9613,7 @@
       <c r="G405" t="s">
         <v>178</v>
       </c>
-      <c r="H405" s="1">
+      <c r="H405" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9610,7 +9636,7 @@
       <c r="G406" t="s">
         <v>178</v>
       </c>
-      <c r="H406" s="1">
+      <c r="H406" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9633,7 +9659,7 @@
       <c r="G407" t="s">
         <v>179</v>
       </c>
-      <c r="H407" s="1">
+      <c r="H407" s="2">
         <v>46226</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: disponibilidade_diaria (23/07/2026 20:40)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -651,16 +651,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -676,7 +668,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -684,30 +676,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1007,72 +981,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1137,7 +1111,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1202,7 +1176,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1267,7 +1241,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1332,7 +1306,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1397,7 +1371,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1462,7 +1436,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1527,7 +1501,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1592,7 +1566,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1657,7 +1631,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1722,7 +1696,7 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>46220</v>
       </c>
       <c r="B12">
@@ -1787,7 +1761,7 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46224</v>
       </c>
       <c r="B13">
@@ -1852,7 +1826,7 @@
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46225</v>
       </c>
       <c r="B14">
@@ -1917,7 +1891,7 @@
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46226</v>
       </c>
       <c r="B15">
@@ -1992,28 +1966,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>74</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>75</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2027,7 +2001,7 @@
       <c r="C2" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2041,7 +2015,7 @@
       <c r="C3" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2064,7 +2038,7 @@
       <c r="G4" t="s">
         <v>174</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2078,7 +2052,7 @@
       <c r="C5" t="s">
         <v>115</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2092,7 +2066,7 @@
       <c r="C6" t="s">
         <v>115</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2109,13 +2083,13 @@
       <c r="D7" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2132,13 +2106,13 @@
       <c r="D8" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>192</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2155,13 +2129,13 @@
       <c r="D9" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>193</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2178,13 +2152,13 @@
       <c r="D10" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>194</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2198,7 +2172,7 @@
       <c r="C11" t="s">
         <v>115</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2212,7 +2186,7 @@
       <c r="C12" t="s">
         <v>115</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2229,13 +2203,13 @@
       <c r="D13" t="s">
         <v>127</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>192</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2249,7 +2223,7 @@
       <c r="C14" t="s">
         <v>119</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2266,13 +2240,13 @@
       <c r="D15" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>195</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2286,7 +2260,7 @@
       <c r="C16" t="s">
         <v>115</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2300,7 +2274,7 @@
       <c r="C17" t="s">
         <v>115</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2317,13 +2291,13 @@
       <c r="D18" t="s">
         <v>129</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>196</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2337,7 +2311,7 @@
       <c r="C19" t="s">
         <v>115</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2354,13 +2328,13 @@
       <c r="D20" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>192</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2383,7 +2357,7 @@
       <c r="G21" t="s">
         <v>175</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2397,7 +2371,7 @@
       <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2411,7 +2385,7 @@
       <c r="C23" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2434,7 +2408,7 @@
       <c r="G24" t="s">
         <v>176</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2451,7 +2425,7 @@
       <c r="D25" t="s">
         <v>132</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2474,7 +2448,7 @@
       <c r="G26" t="s">
         <v>177</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2491,13 +2465,13 @@
       <c r="D27" t="s">
         <v>134</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>197</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2520,7 +2494,7 @@
       <c r="G28" t="s">
         <v>178</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2543,7 +2517,7 @@
       <c r="G29" t="s">
         <v>178</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2566,7 +2540,7 @@
       <c r="G30" t="s">
         <v>179</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46204</v>
       </c>
     </row>
@@ -2580,7 +2554,7 @@
       <c r="C31" t="s">
         <v>115</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2594,7 +2568,7 @@
       <c r="C32" t="s">
         <v>115</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2617,7 +2591,7 @@
       <c r="G33" t="s">
         <v>180</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2631,7 +2605,7 @@
       <c r="C34" t="s">
         <v>115</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2645,7 +2619,7 @@
       <c r="C35" t="s">
         <v>115</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2662,13 +2636,13 @@
       <c r="D36" t="s">
         <v>123</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>192</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2685,13 +2659,13 @@
       <c r="D37" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>192</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2708,13 +2682,13 @@
       <c r="D38" t="s">
         <v>125</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="1">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>193</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2731,13 +2705,13 @@
       <c r="D39" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39" s="1">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>194</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2751,7 +2725,7 @@
       <c r="C40" t="s">
         <v>115</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2765,7 +2739,7 @@
       <c r="C41" t="s">
         <v>115</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2782,13 +2756,13 @@
       <c r="D42" t="s">
         <v>127</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42" s="1">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>192</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2802,7 +2776,7 @@
       <c r="C43" t="s">
         <v>115</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2819,13 +2793,13 @@
       <c r="D44" t="s">
         <v>128</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44" s="1">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>195</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2839,7 +2813,7 @@
       <c r="C45" t="s">
         <v>115</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2853,7 +2827,7 @@
       <c r="C46" t="s">
         <v>115</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2867,7 +2841,7 @@
       <c r="C47" t="s">
         <v>119</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2881,7 +2855,7 @@
       <c r="C48" t="s">
         <v>115</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2898,13 +2872,13 @@
       <c r="D49" t="s">
         <v>139</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="1">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>192</v>
       </c>
-      <c r="H49" s="2">
+      <c r="H49" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2927,7 +2901,7 @@
       <c r="G50" t="s">
         <v>175</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2941,7 +2915,7 @@
       <c r="C51" t="s">
         <v>119</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2955,7 +2929,7 @@
       <c r="C52" t="s">
         <v>115</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2978,7 +2952,7 @@
       <c r="G53" t="s">
         <v>176</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -2995,7 +2969,7 @@
       <c r="D54" t="s">
         <v>132</v>
       </c>
-      <c r="H54" s="2">
+      <c r="H54" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3018,7 +2992,7 @@
       <c r="G55" t="s">
         <v>177</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3035,13 +3009,13 @@
       <c r="D56" t="s">
         <v>134</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56" s="1">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>197</v>
       </c>
-      <c r="H56" s="2">
+      <c r="H56" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3064,7 +3038,7 @@
       <c r="G57" t="s">
         <v>178</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3087,7 +3061,7 @@
       <c r="G58" t="s">
         <v>178</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3110,7 +3084,7 @@
       <c r="G59" t="s">
         <v>179</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="1">
         <v>46205</v>
       </c>
     </row>
@@ -3124,7 +3098,7 @@
       <c r="C60" t="s">
         <v>115</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3138,7 +3112,7 @@
       <c r="C61" t="s">
         <v>115</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3155,13 +3129,13 @@
       <c r="D62" t="s">
         <v>138</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="1">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>198</v>
       </c>
-      <c r="H62" s="2">
+      <c r="H62" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3175,7 +3149,7 @@
       <c r="C63" t="s">
         <v>115</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3192,13 +3166,13 @@
       <c r="D64" t="s">
         <v>140</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64" s="1">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>199</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3212,7 +3186,7 @@
       <c r="C65" t="s">
         <v>115</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3226,7 +3200,7 @@
       <c r="C66" t="s">
         <v>119</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3243,13 +3217,13 @@
       <c r="D67" t="s">
         <v>125</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67" s="1">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>193</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3266,13 +3240,13 @@
       <c r="D68" t="s">
         <v>126</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68" s="1">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>194</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3286,7 +3260,7 @@
       <c r="C69" t="s">
         <v>115</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3300,7 +3274,7 @@
       <c r="C70" t="s">
         <v>115</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3317,13 +3291,13 @@
       <c r="D71" t="s">
         <v>127</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71" s="1">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>198</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3337,7 +3311,7 @@
       <c r="C72" t="s">
         <v>115</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3354,13 +3328,13 @@
       <c r="D73" t="s">
         <v>128</v>
       </c>
-      <c r="E73" s="2">
+      <c r="E73" s="1">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>195</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3374,7 +3348,7 @@
       <c r="C74" t="s">
         <v>115</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3388,7 +3362,7 @@
       <c r="C75" t="s">
         <v>115</v>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3402,7 +3376,7 @@
       <c r="C76" t="s">
         <v>115</v>
       </c>
-      <c r="H76" s="2">
+      <c r="H76" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3416,7 +3390,7 @@
       <c r="C77" t="s">
         <v>115</v>
       </c>
-      <c r="H77" s="2">
+      <c r="H77" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3433,13 +3407,13 @@
       <c r="D78" t="s">
         <v>139</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78" s="1">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>198</v>
       </c>
-      <c r="H78" s="2">
+      <c r="H78" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3462,7 +3436,7 @@
       <c r="G79" t="s">
         <v>181</v>
       </c>
-      <c r="H79" s="2">
+      <c r="H79" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3476,7 +3450,7 @@
       <c r="C80" t="s">
         <v>119</v>
       </c>
-      <c r="H80" s="2">
+      <c r="H80" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3490,7 +3464,7 @@
       <c r="C81" t="s">
         <v>115</v>
       </c>
-      <c r="H81" s="2">
+      <c r="H81" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3513,7 +3487,7 @@
       <c r="G82" t="s">
         <v>176</v>
       </c>
-      <c r="H82" s="2">
+      <c r="H82" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3530,7 +3504,7 @@
       <c r="D83" t="s">
         <v>132</v>
       </c>
-      <c r="H83" s="2">
+      <c r="H83" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3553,7 +3527,7 @@
       <c r="G84" t="s">
         <v>177</v>
       </c>
-      <c r="H84" s="2">
+      <c r="H84" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3570,13 +3544,13 @@
       <c r="D85" t="s">
         <v>134</v>
       </c>
-      <c r="E85" s="2">
+      <c r="E85" s="1">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>197</v>
       </c>
-      <c r="H85" s="2">
+      <c r="H85" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3599,7 +3573,7 @@
       <c r="G86" t="s">
         <v>178</v>
       </c>
-      <c r="H86" s="2">
+      <c r="H86" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3622,7 +3596,7 @@
       <c r="G87" t="s">
         <v>178</v>
       </c>
-      <c r="H87" s="2">
+      <c r="H87" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3645,7 +3619,7 @@
       <c r="G88" t="s">
         <v>179</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -3659,7 +3633,7 @@
       <c r="C89" t="s">
         <v>115</v>
       </c>
-      <c r="H89" s="2">
+      <c r="H89" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3676,13 +3650,13 @@
       <c r="D90" t="s">
         <v>142</v>
       </c>
-      <c r="E90" s="2">
+      <c r="E90" s="1">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>199</v>
       </c>
-      <c r="H90" s="2">
+      <c r="H90" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3699,13 +3673,13 @@
       <c r="D91" t="s">
         <v>138</v>
       </c>
-      <c r="E91" s="2">
+      <c r="E91" s="1">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>198</v>
       </c>
-      <c r="H91" s="2">
+      <c r="H91" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3719,7 +3693,7 @@
       <c r="C92" t="s">
         <v>115</v>
       </c>
-      <c r="H92" s="2">
+      <c r="H92" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3736,13 +3710,13 @@
       <c r="D93" t="s">
         <v>140</v>
       </c>
-      <c r="E93" s="2">
+      <c r="E93" s="1">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>199</v>
       </c>
-      <c r="H93" s="2">
+      <c r="H93" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3756,7 +3730,7 @@
       <c r="C94" t="s">
         <v>115</v>
       </c>
-      <c r="H94" s="2">
+      <c r="H94" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3770,7 +3744,7 @@
       <c r="C95" t="s">
         <v>119</v>
       </c>
-      <c r="H95" s="2">
+      <c r="H95" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3787,13 +3761,13 @@
       <c r="D96" t="s">
         <v>125</v>
       </c>
-      <c r="E96" s="2">
+      <c r="E96" s="1">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>193</v>
       </c>
-      <c r="H96" s="2">
+      <c r="H96" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3810,13 +3784,13 @@
       <c r="D97" t="s">
         <v>126</v>
       </c>
-      <c r="E97" s="2">
+      <c r="E97" s="1">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>194</v>
       </c>
-      <c r="H97" s="2">
+      <c r="H97" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3830,7 +3804,7 @@
       <c r="C98" t="s">
         <v>115</v>
       </c>
-      <c r="H98" s="2">
+      <c r="H98" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3847,13 +3821,13 @@
       <c r="D99" t="s">
         <v>143</v>
       </c>
-      <c r="E99" s="2">
+      <c r="E99" s="1">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>194</v>
       </c>
-      <c r="H99" s="2">
+      <c r="H99" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3870,13 +3844,13 @@
       <c r="D100" t="s">
         <v>127</v>
       </c>
-      <c r="E100" s="2">
+      <c r="E100" s="1">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>194</v>
       </c>
-      <c r="H100" s="2">
+      <c r="H100" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3890,7 +3864,7 @@
       <c r="C101" t="s">
         <v>115</v>
       </c>
-      <c r="H101" s="2">
+      <c r="H101" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3907,13 +3881,13 @@
       <c r="D102" t="s">
         <v>128</v>
       </c>
-      <c r="E102" s="2">
+      <c r="E102" s="1">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>195</v>
       </c>
-      <c r="H102" s="2">
+      <c r="H102" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3930,13 +3904,13 @@
       <c r="D103" t="s">
         <v>144</v>
       </c>
-      <c r="E103" s="2">
+      <c r="E103" s="1">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>194</v>
       </c>
-      <c r="H103" s="2">
+      <c r="H103" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3950,7 +3924,7 @@
       <c r="C104" t="s">
         <v>115</v>
       </c>
-      <c r="H104" s="2">
+      <c r="H104" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3964,7 +3938,7 @@
       <c r="C105" t="s">
         <v>115</v>
       </c>
-      <c r="H105" s="2">
+      <c r="H105" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3978,7 +3952,7 @@
       <c r="C106" t="s">
         <v>115</v>
       </c>
-      <c r="H106" s="2">
+      <c r="H106" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -3995,13 +3969,13 @@
       <c r="D107" t="s">
         <v>145</v>
       </c>
-      <c r="E107" s="2">
+      <c r="E107" s="1">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>194</v>
       </c>
-      <c r="H107" s="2">
+      <c r="H107" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4024,7 +3998,7 @@
       <c r="G108" t="s">
         <v>181</v>
       </c>
-      <c r="H108" s="2">
+      <c r="H108" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4038,7 +4012,7 @@
       <c r="C109" t="s">
         <v>119</v>
       </c>
-      <c r="H109" s="2">
+      <c r="H109" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4052,7 +4026,7 @@
       <c r="C110" t="s">
         <v>115</v>
       </c>
-      <c r="H110" s="2">
+      <c r="H110" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4075,7 +4049,7 @@
       <c r="G111" t="s">
         <v>176</v>
       </c>
-      <c r="H111" s="2">
+      <c r="H111" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4092,7 +4066,7 @@
       <c r="D112" t="s">
         <v>132</v>
       </c>
-      <c r="H112" s="2">
+      <c r="H112" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4115,7 +4089,7 @@
       <c r="G113" t="s">
         <v>177</v>
       </c>
-      <c r="H113" s="2">
+      <c r="H113" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4132,13 +4106,13 @@
       <c r="D114" t="s">
         <v>134</v>
       </c>
-      <c r="E114" s="2">
+      <c r="E114" s="1">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>197</v>
       </c>
-      <c r="H114" s="2">
+      <c r="H114" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4161,7 +4135,7 @@
       <c r="G115" t="s">
         <v>178</v>
       </c>
-      <c r="H115" s="2">
+      <c r="H115" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4184,7 +4158,7 @@
       <c r="G116" t="s">
         <v>178</v>
       </c>
-      <c r="H116" s="2">
+      <c r="H116" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4207,7 +4181,7 @@
       <c r="G117" t="s">
         <v>179</v>
       </c>
-      <c r="H117" s="2">
+      <c r="H117" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -4221,7 +4195,7 @@
       <c r="C118" t="s">
         <v>115</v>
       </c>
-      <c r="H118" s="2">
+      <c r="H118" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4238,13 +4212,13 @@
       <c r="D119" t="s">
         <v>142</v>
       </c>
-      <c r="E119" s="2">
+      <c r="E119" s="1">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>199</v>
       </c>
-      <c r="H119" s="2">
+      <c r="H119" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4258,7 +4232,7 @@
       <c r="C120" t="s">
         <v>119</v>
       </c>
-      <c r="H120" s="2">
+      <c r="H120" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4272,7 +4246,7 @@
       <c r="C121" t="s">
         <v>115</v>
       </c>
-      <c r="H121" s="2">
+      <c r="H121" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4286,7 +4260,7 @@
       <c r="C122" t="s">
         <v>119</v>
       </c>
-      <c r="H122" s="2">
+      <c r="H122" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4300,7 +4274,7 @@
       <c r="C123" t="s">
         <v>119</v>
       </c>
-      <c r="H123" s="2">
+      <c r="H123" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4314,7 +4288,7 @@
       <c r="C124" t="s">
         <v>119</v>
       </c>
-      <c r="H124" s="2">
+      <c r="H124" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4331,13 +4305,13 @@
       <c r="D125" t="s">
         <v>125</v>
       </c>
-      <c r="E125" s="2">
+      <c r="E125" s="1">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>193</v>
       </c>
-      <c r="H125" s="2">
+      <c r="H125" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4354,13 +4328,13 @@
       <c r="D126" t="s">
         <v>126</v>
       </c>
-      <c r="E126" s="2">
+      <c r="E126" s="1">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>194</v>
       </c>
-      <c r="H126" s="2">
+      <c r="H126" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4374,7 +4348,7 @@
       <c r="C127" t="s">
         <v>115</v>
       </c>
-      <c r="H127" s="2">
+      <c r="H127" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4391,13 +4365,13 @@
       <c r="D128" t="s">
         <v>143</v>
       </c>
-      <c r="E128" s="2">
+      <c r="E128" s="1">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>194</v>
       </c>
-      <c r="H128" s="2">
+      <c r="H128" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4414,13 +4388,13 @@
       <c r="D129" t="s">
         <v>127</v>
       </c>
-      <c r="E129" s="2">
+      <c r="E129" s="1">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>194</v>
       </c>
-      <c r="H129" s="2">
+      <c r="H129" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4434,7 +4408,7 @@
       <c r="C130" t="s">
         <v>115</v>
       </c>
-      <c r="H130" s="2">
+      <c r="H130" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4451,13 +4425,13 @@
       <c r="D131" t="s">
         <v>128</v>
       </c>
-      <c r="E131" s="2">
+      <c r="E131" s="1">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>195</v>
       </c>
-      <c r="H131" s="2">
+      <c r="H131" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4474,13 +4448,13 @@
       <c r="D132" t="s">
         <v>144</v>
       </c>
-      <c r="E132" s="2">
+      <c r="E132" s="1">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>194</v>
       </c>
-      <c r="H132" s="2">
+      <c r="H132" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4494,7 +4468,7 @@
       <c r="C133" t="s">
         <v>115</v>
       </c>
-      <c r="H133" s="2">
+      <c r="H133" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4508,7 +4482,7 @@
       <c r="C134" t="s">
         <v>115</v>
       </c>
-      <c r="H134" s="2">
+      <c r="H134" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4522,7 +4496,7 @@
       <c r="C135" t="s">
         <v>115</v>
       </c>
-      <c r="H135" s="2">
+      <c r="H135" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4539,13 +4513,13 @@
       <c r="D136" t="s">
         <v>146</v>
       </c>
-      <c r="E136" s="2">
+      <c r="E136" s="1">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>194</v>
       </c>
-      <c r="H136" s="2">
+      <c r="H136" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4568,7 +4542,7 @@
       <c r="G137" t="s">
         <v>181</v>
       </c>
-      <c r="H137" s="2">
+      <c r="H137" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4582,7 +4556,7 @@
       <c r="C138" t="s">
         <v>119</v>
       </c>
-      <c r="H138" s="2">
+      <c r="H138" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4596,7 +4570,7 @@
       <c r="C139" t="s">
         <v>115</v>
       </c>
-      <c r="H139" s="2">
+      <c r="H139" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4619,7 +4593,7 @@
       <c r="G140" t="s">
         <v>176</v>
       </c>
-      <c r="H140" s="2">
+      <c r="H140" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4636,7 +4610,7 @@
       <c r="D141" t="s">
         <v>132</v>
       </c>
-      <c r="H141" s="2">
+      <c r="H141" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4659,7 +4633,7 @@
       <c r="G142" t="s">
         <v>177</v>
       </c>
-      <c r="H142" s="2">
+      <c r="H142" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4676,13 +4650,13 @@
       <c r="D143" t="s">
         <v>134</v>
       </c>
-      <c r="E143" s="2">
+      <c r="E143" s="1">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>197</v>
       </c>
-      <c r="H143" s="2">
+      <c r="H143" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4705,7 +4679,7 @@
       <c r="G144" t="s">
         <v>178</v>
       </c>
-      <c r="H144" s="2">
+      <c r="H144" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4728,7 +4702,7 @@
       <c r="G145" t="s">
         <v>178</v>
       </c>
-      <c r="H145" s="2">
+      <c r="H145" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4751,7 +4725,7 @@
       <c r="G146" t="s">
         <v>179</v>
       </c>
-      <c r="H146" s="2">
+      <c r="H146" s="1">
         <v>46211</v>
       </c>
     </row>
@@ -4765,7 +4739,7 @@
       <c r="C147" t="s">
         <v>115</v>
       </c>
-      <c r="H147" s="2">
+      <c r="H147" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4782,13 +4756,13 @@
       <c r="D148" t="s">
         <v>142</v>
       </c>
-      <c r="E148" s="2">
+      <c r="E148" s="1">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>199</v>
       </c>
-      <c r="H148" s="2">
+      <c r="H148" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4802,7 +4776,7 @@
       <c r="C149" t="s">
         <v>119</v>
       </c>
-      <c r="H149" s="2">
+      <c r="H149" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4816,7 +4790,7 @@
       <c r="C150" t="s">
         <v>115</v>
       </c>
-      <c r="H150" s="2">
+      <c r="H150" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4830,7 +4804,7 @@
       <c r="C151" t="s">
         <v>115</v>
       </c>
-      <c r="H151" s="2">
+      <c r="H151" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4844,7 +4818,7 @@
       <c r="C152" t="s">
         <v>119</v>
       </c>
-      <c r="H152" s="2">
+      <c r="H152" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4858,7 +4832,7 @@
       <c r="C153" t="s">
         <v>119</v>
       </c>
-      <c r="H153" s="2">
+      <c r="H153" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4875,13 +4849,13 @@
       <c r="D154" t="s">
         <v>125</v>
       </c>
-      <c r="E154" s="2">
+      <c r="E154" s="1">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>193</v>
       </c>
-      <c r="H154" s="2">
+      <c r="H154" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4898,13 +4872,13 @@
       <c r="D155" t="s">
         <v>126</v>
       </c>
-      <c r="E155" s="2">
+      <c r="E155" s="1">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>194</v>
       </c>
-      <c r="H155" s="2">
+      <c r="H155" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4918,7 +4892,7 @@
       <c r="C156" t="s">
         <v>115</v>
       </c>
-      <c r="H156" s="2">
+      <c r="H156" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4935,13 +4909,13 @@
       <c r="D157" t="s">
         <v>143</v>
       </c>
-      <c r="E157" s="2">
+      <c r="E157" s="1">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>194</v>
       </c>
-      <c r="H157" s="2">
+      <c r="H157" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4958,13 +4932,13 @@
       <c r="D158" t="s">
         <v>127</v>
       </c>
-      <c r="E158" s="2">
+      <c r="E158" s="1">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>194</v>
       </c>
-      <c r="H158" s="2">
+      <c r="H158" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -4981,13 +4955,13 @@
       <c r="D159" t="s">
         <v>147</v>
       </c>
-      <c r="E159" s="2">
+      <c r="E159" s="1">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>200</v>
       </c>
-      <c r="H159" s="2">
+      <c r="H159" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5004,13 +4978,13 @@
       <c r="D160" t="s">
         <v>128</v>
       </c>
-      <c r="E160" s="2">
+      <c r="E160" s="1">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>195</v>
       </c>
-      <c r="H160" s="2">
+      <c r="H160" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5027,13 +5001,13 @@
       <c r="D161" t="s">
         <v>144</v>
       </c>
-      <c r="E161" s="2">
+      <c r="E161" s="1">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>194</v>
       </c>
-      <c r="H161" s="2">
+      <c r="H161" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5047,7 +5021,7 @@
       <c r="C162" t="s">
         <v>115</v>
       </c>
-      <c r="H162" s="2">
+      <c r="H162" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5061,7 +5035,7 @@
       <c r="C163" t="s">
         <v>115</v>
       </c>
-      <c r="H163" s="2">
+      <c r="H163" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5075,7 +5049,7 @@
       <c r="C164" t="s">
         <v>115</v>
       </c>
-      <c r="H164" s="2">
+      <c r="H164" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5092,13 +5066,13 @@
       <c r="D165" t="s">
         <v>146</v>
       </c>
-      <c r="E165" s="2">
+      <c r="E165" s="1">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>194</v>
       </c>
-      <c r="H165" s="2">
+      <c r="H165" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5121,7 +5095,7 @@
       <c r="G166" t="s">
         <v>181</v>
       </c>
-      <c r="H166" s="2">
+      <c r="H166" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5135,7 +5109,7 @@
       <c r="C167" t="s">
         <v>119</v>
       </c>
-      <c r="H167" s="2">
+      <c r="H167" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5149,7 +5123,7 @@
       <c r="C168" t="s">
         <v>115</v>
       </c>
-      <c r="H168" s="2">
+      <c r="H168" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5172,7 +5146,7 @@
       <c r="G169" t="s">
         <v>176</v>
       </c>
-      <c r="H169" s="2">
+      <c r="H169" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5189,7 +5163,7 @@
       <c r="D170" t="s">
         <v>132</v>
       </c>
-      <c r="H170" s="2">
+      <c r="H170" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5212,7 +5186,7 @@
       <c r="G171" t="s">
         <v>177</v>
       </c>
-      <c r="H171" s="2">
+      <c r="H171" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5229,13 +5203,13 @@
       <c r="D172" t="s">
         <v>134</v>
       </c>
-      <c r="E172" s="2">
+      <c r="E172" s="1">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>197</v>
       </c>
-      <c r="H172" s="2">
+      <c r="H172" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5258,7 +5232,7 @@
       <c r="G173" t="s">
         <v>178</v>
       </c>
-      <c r="H173" s="2">
+      <c r="H173" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5281,7 +5255,7 @@
       <c r="G174" t="s">
         <v>178</v>
       </c>
-      <c r="H174" s="2">
+      <c r="H174" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5304,7 +5278,7 @@
       <c r="G175" t="s">
         <v>179</v>
       </c>
-      <c r="H175" s="2">
+      <c r="H175" s="1">
         <v>46212</v>
       </c>
     </row>
@@ -5318,7 +5292,7 @@
       <c r="C176" t="s">
         <v>115</v>
       </c>
-      <c r="H176" s="2">
+      <c r="H176" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5335,13 +5309,13 @@
       <c r="D177" t="s">
         <v>148</v>
       </c>
-      <c r="E177" s="2">
+      <c r="E177" s="1">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>199</v>
       </c>
-      <c r="H177" s="2">
+      <c r="H177" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5355,7 +5329,7 @@
       <c r="C178" t="s">
         <v>115</v>
       </c>
-      <c r="H178" s="2">
+      <c r="H178" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5372,13 +5346,13 @@
       <c r="D179" t="s">
         <v>149</v>
       </c>
-      <c r="E179" s="2">
+      <c r="E179" s="1">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>195</v>
       </c>
-      <c r="H179" s="2">
+      <c r="H179" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5392,7 +5366,7 @@
       <c r="C180" t="s">
         <v>115</v>
       </c>
-      <c r="H180" s="2">
+      <c r="H180" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5406,7 +5380,7 @@
       <c r="C181" t="s">
         <v>119</v>
       </c>
-      <c r="H181" s="2">
+      <c r="H181" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5420,7 +5394,7 @@
       <c r="C182" t="s">
         <v>119</v>
       </c>
-      <c r="H182" s="2">
+      <c r="H182" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5437,13 +5411,13 @@
       <c r="D183" t="s">
         <v>125</v>
       </c>
-      <c r="E183" s="2">
+      <c r="E183" s="1">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>193</v>
       </c>
-      <c r="H183" s="2">
+      <c r="H183" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5460,13 +5434,13 @@
       <c r="D184" t="s">
         <v>126</v>
       </c>
-      <c r="E184" s="2">
+      <c r="E184" s="1">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>194</v>
       </c>
-      <c r="H184" s="2">
+      <c r="H184" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5480,7 +5454,7 @@
       <c r="C185" t="s">
         <v>115</v>
       </c>
-      <c r="H185" s="2">
+      <c r="H185" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5497,13 +5471,13 @@
       <c r="D186" t="s">
         <v>143</v>
       </c>
-      <c r="E186" s="2">
+      <c r="E186" s="1">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>194</v>
       </c>
-      <c r="H186" s="2">
+      <c r="H186" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5520,13 +5494,13 @@
       <c r="D187" t="s">
         <v>150</v>
       </c>
-      <c r="E187" s="2">
+      <c r="E187" s="1">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>194</v>
       </c>
-      <c r="H187" s="2">
+      <c r="H187" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5543,13 +5517,13 @@
       <c r="D188" t="s">
         <v>151</v>
       </c>
-      <c r="E188" s="2">
+      <c r="E188" s="1">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>194</v>
       </c>
-      <c r="H188" s="2">
+      <c r="H188" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5566,13 +5540,13 @@
       <c r="D189" t="s">
         <v>128</v>
       </c>
-      <c r="E189" s="2">
+      <c r="E189" s="1">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>195</v>
       </c>
-      <c r="H189" s="2">
+      <c r="H189" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5589,13 +5563,13 @@
       <c r="D190" t="s">
         <v>144</v>
       </c>
-      <c r="E190" s="2">
+      <c r="E190" s="1">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>194</v>
       </c>
-      <c r="H190" s="2">
+      <c r="H190" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5609,7 +5583,7 @@
       <c r="C191" t="s">
         <v>115</v>
       </c>
-      <c r="H191" s="2">
+      <c r="H191" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5623,7 +5597,7 @@
       <c r="C192" t="s">
         <v>115</v>
       </c>
-      <c r="H192" s="2">
+      <c r="H192" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5637,7 +5611,7 @@
       <c r="C193" t="s">
         <v>115</v>
       </c>
-      <c r="H193" s="2">
+      <c r="H193" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5654,13 +5628,13 @@
       <c r="D194" t="s">
         <v>146</v>
       </c>
-      <c r="E194" s="2">
+      <c r="E194" s="1">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>201</v>
       </c>
-      <c r="H194" s="2">
+      <c r="H194" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5683,7 +5657,7 @@
       <c r="G195" t="s">
         <v>181</v>
       </c>
-      <c r="H195" s="2">
+      <c r="H195" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5697,7 +5671,7 @@
       <c r="C196" t="s">
         <v>119</v>
       </c>
-      <c r="H196" s="2">
+      <c r="H196" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5711,7 +5685,7 @@
       <c r="C197" t="s">
         <v>115</v>
       </c>
-      <c r="H197" s="2">
+      <c r="H197" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5734,7 +5708,7 @@
       <c r="G198" t="s">
         <v>176</v>
       </c>
-      <c r="H198" s="2">
+      <c r="H198" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5751,7 +5725,7 @@
       <c r="D199" t="s">
         <v>132</v>
       </c>
-      <c r="H199" s="2">
+      <c r="H199" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5774,7 +5748,7 @@
       <c r="G200" t="s">
         <v>177</v>
       </c>
-      <c r="H200" s="2">
+      <c r="H200" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5791,13 +5765,13 @@
       <c r="D201" t="s">
         <v>134</v>
       </c>
-      <c r="E201" s="2">
+      <c r="E201" s="1">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>197</v>
       </c>
-      <c r="H201" s="2">
+      <c r="H201" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5820,7 +5794,7 @@
       <c r="G202" t="s">
         <v>178</v>
       </c>
-      <c r="H202" s="2">
+      <c r="H202" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5843,7 +5817,7 @@
       <c r="G203" t="s">
         <v>178</v>
       </c>
-      <c r="H203" s="2">
+      <c r="H203" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5866,7 +5840,7 @@
       <c r="G204" t="s">
         <v>179</v>
       </c>
-      <c r="H204" s="2">
+      <c r="H204" s="1">
         <v>46213</v>
       </c>
     </row>
@@ -5880,7 +5854,7 @@
       <c r="C205" t="s">
         <v>115</v>
       </c>
-      <c r="H205" s="2">
+      <c r="H205" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5897,13 +5871,13 @@
       <c r="D206" t="s">
         <v>148</v>
       </c>
-      <c r="E206" s="2">
+      <c r="E206" s="1">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>199</v>
       </c>
-      <c r="H206" s="2">
+      <c r="H206" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5917,7 +5891,7 @@
       <c r="C207" t="s">
         <v>115</v>
       </c>
-      <c r="H207" s="2">
+      <c r="H207" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5931,7 +5905,7 @@
       <c r="C208" t="s">
         <v>119</v>
       </c>
-      <c r="H208" s="2">
+      <c r="H208" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5945,7 +5919,7 @@
       <c r="C209" t="s">
         <v>115</v>
       </c>
-      <c r="H209" s="2">
+      <c r="H209" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5959,7 +5933,7 @@
       <c r="C210" t="s">
         <v>119</v>
       </c>
-      <c r="H210" s="2">
+      <c r="H210" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5973,7 +5947,7 @@
       <c r="C211" t="s">
         <v>119</v>
       </c>
-      <c r="H211" s="2">
+      <c r="H211" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -5990,13 +5964,13 @@
       <c r="D212" t="s">
         <v>125</v>
       </c>
-      <c r="E212" s="2">
+      <c r="E212" s="1">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>193</v>
       </c>
-      <c r="H212" s="2">
+      <c r="H212" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6010,7 +5984,7 @@
       <c r="C213" t="s">
         <v>119</v>
       </c>
-      <c r="H213" s="2">
+      <c r="H213" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6024,7 +5998,7 @@
       <c r="C214" t="s">
         <v>115</v>
       </c>
-      <c r="H214" s="2">
+      <c r="H214" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6041,13 +6015,13 @@
       <c r="D215" t="s">
         <v>143</v>
       </c>
-      <c r="E215" s="2">
+      <c r="E215" s="1">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>202</v>
       </c>
-      <c r="H215" s="2">
+      <c r="H215" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6064,13 +6038,13 @@
       <c r="D216" t="s">
         <v>150</v>
       </c>
-      <c r="E216" s="2">
+      <c r="E216" s="1">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>195</v>
       </c>
-      <c r="H216" s="2">
+      <c r="H216" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6084,7 +6058,7 @@
       <c r="C217" t="s">
         <v>115</v>
       </c>
-      <c r="H217" s="2">
+      <c r="H217" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6101,13 +6075,13 @@
       <c r="D218" t="s">
         <v>128</v>
       </c>
-      <c r="E218" s="2">
+      <c r="E218" s="1">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>195</v>
       </c>
-      <c r="H218" s="2">
+      <c r="H218" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6121,7 +6095,7 @@
       <c r="C219" t="s">
         <v>115</v>
       </c>
-      <c r="H219" s="2">
+      <c r="H219" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6135,7 +6109,7 @@
       <c r="C220" t="s">
         <v>115</v>
       </c>
-      <c r="H220" s="2">
+      <c r="H220" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6152,13 +6126,13 @@
       <c r="D221" t="s">
         <v>152</v>
       </c>
-      <c r="E221" s="2">
+      <c r="E221" s="1">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>199</v>
       </c>
-      <c r="H221" s="2">
+      <c r="H221" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6172,7 +6146,7 @@
       <c r="C222" t="s">
         <v>115</v>
       </c>
-      <c r="H222" s="2">
+      <c r="H222" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6189,13 +6163,13 @@
       <c r="D223" t="s">
         <v>153</v>
       </c>
-      <c r="E223" s="2">
+      <c r="E223" s="1">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>203</v>
       </c>
-      <c r="H223" s="2">
+      <c r="H223" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6218,7 +6192,7 @@
       <c r="G224" t="s">
         <v>181</v>
       </c>
-      <c r="H224" s="2">
+      <c r="H224" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6232,7 +6206,7 @@
       <c r="C225" t="s">
         <v>119</v>
       </c>
-      <c r="H225" s="2">
+      <c r="H225" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="C226" t="s">
         <v>115</v>
       </c>
-      <c r="H226" s="2">
+      <c r="H226" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6269,7 +6243,7 @@
       <c r="G227" t="s">
         <v>176</v>
       </c>
-      <c r="H227" s="2">
+      <c r="H227" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6286,7 +6260,7 @@
       <c r="D228" t="s">
         <v>132</v>
       </c>
-      <c r="H228" s="2">
+      <c r="H228" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6309,7 +6283,7 @@
       <c r="G229" t="s">
         <v>177</v>
       </c>
-      <c r="H229" s="2">
+      <c r="H229" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6326,13 +6300,13 @@
       <c r="D230" t="s">
         <v>154</v>
       </c>
-      <c r="E230" s="2">
+      <c r="E230" s="1">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>204</v>
       </c>
-      <c r="H230" s="2">
+      <c r="H230" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6355,7 +6329,7 @@
       <c r="G231" t="s">
         <v>178</v>
       </c>
-      <c r="H231" s="2">
+      <c r="H231" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6378,7 +6352,7 @@
       <c r="G232" t="s">
         <v>178</v>
       </c>
-      <c r="H232" s="2">
+      <c r="H232" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6401,7 +6375,7 @@
       <c r="G233" t="s">
         <v>179</v>
       </c>
-      <c r="H233" s="2">
+      <c r="H233" s="1">
         <v>46216</v>
       </c>
     </row>
@@ -6415,7 +6389,7 @@
       <c r="C234" t="s">
         <v>115</v>
       </c>
-      <c r="H234" s="2">
+      <c r="H234" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6432,13 +6406,13 @@
       <c r="D235" t="s">
         <v>155</v>
       </c>
-      <c r="E235" s="2">
+      <c r="E235" s="1">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>199</v>
       </c>
-      <c r="H235" s="2">
+      <c r="H235" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6452,7 +6426,7 @@
       <c r="C236" t="s">
         <v>115</v>
       </c>
-      <c r="H236" s="2">
+      <c r="H236" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6466,7 +6440,7 @@
       <c r="C237" t="s">
         <v>119</v>
       </c>
-      <c r="H237" s="2">
+      <c r="H237" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6480,7 +6454,7 @@
       <c r="C238" t="s">
         <v>115</v>
       </c>
-      <c r="H238" s="2">
+      <c r="H238" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6494,7 +6468,7 @@
       <c r="C239" t="s">
         <v>119</v>
       </c>
-      <c r="H239" s="2">
+      <c r="H239" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6508,7 +6482,7 @@
       <c r="C240" t="s">
         <v>119</v>
       </c>
-      <c r="H240" s="2">
+      <c r="H240" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6525,13 +6499,13 @@
       <c r="D241" t="s">
         <v>125</v>
       </c>
-      <c r="E241" s="2">
+      <c r="E241" s="1">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>193</v>
       </c>
-      <c r="H241" s="2">
+      <c r="H241" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6545,7 +6519,7 @@
       <c r="C242" t="s">
         <v>119</v>
       </c>
-      <c r="H242" s="2">
+      <c r="H242" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6562,13 +6536,13 @@
       <c r="D243" t="s">
         <v>156</v>
       </c>
-      <c r="E243" s="2">
+      <c r="E243" s="1">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>205</v>
       </c>
-      <c r="H243" s="2">
+      <c r="H243" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6585,13 +6559,13 @@
       <c r="D244" t="s">
         <v>157</v>
       </c>
-      <c r="E244" s="2">
+      <c r="E244" s="1">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>202</v>
       </c>
-      <c r="H244" s="2">
+      <c r="H244" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6605,7 +6579,7 @@
       <c r="C245" t="s">
         <v>119</v>
       </c>
-      <c r="H245" s="2">
+      <c r="H245" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6619,7 +6593,7 @@
       <c r="C246" t="s">
         <v>115</v>
       </c>
-      <c r="H246" s="2">
+      <c r="H246" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6636,13 +6610,13 @@
       <c r="D247" t="s">
         <v>128</v>
       </c>
-      <c r="E247" s="2">
+      <c r="E247" s="1">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>206</v>
       </c>
-      <c r="H247" s="2">
+      <c r="H247" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6656,7 +6630,7 @@
       <c r="C248" t="s">
         <v>115</v>
       </c>
-      <c r="H248" s="2">
+      <c r="H248" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6670,7 +6644,7 @@
       <c r="C249" t="s">
         <v>115</v>
       </c>
-      <c r="H249" s="2">
+      <c r="H249" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6687,13 +6661,13 @@
       <c r="D250" t="s">
         <v>158</v>
       </c>
-      <c r="E250" s="2">
+      <c r="E250" s="1">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>201</v>
       </c>
-      <c r="H250" s="2">
+      <c r="H250" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6707,7 +6681,7 @@
       <c r="C251" t="s">
         <v>115</v>
       </c>
-      <c r="H251" s="2">
+      <c r="H251" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6724,13 +6698,13 @@
       <c r="D252" t="s">
         <v>159</v>
       </c>
-      <c r="E252" s="2">
+      <c r="E252" s="1">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>203</v>
       </c>
-      <c r="H252" s="2">
+      <c r="H252" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6753,7 +6727,7 @@
       <c r="G253" t="s">
         <v>181</v>
       </c>
-      <c r="H253" s="2">
+      <c r="H253" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6767,7 +6741,7 @@
       <c r="C254" t="s">
         <v>119</v>
       </c>
-      <c r="H254" s="2">
+      <c r="H254" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6781,7 +6755,7 @@
       <c r="C255" t="s">
         <v>115</v>
       </c>
-      <c r="H255" s="2">
+      <c r="H255" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6804,7 +6778,7 @@
       <c r="G256" t="s">
         <v>176</v>
       </c>
-      <c r="H256" s="2">
+      <c r="H256" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6821,7 +6795,7 @@
       <c r="D257" t="s">
         <v>132</v>
       </c>
-      <c r="H257" s="2">
+      <c r="H257" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6844,7 +6818,7 @@
       <c r="G258" t="s">
         <v>177</v>
       </c>
-      <c r="H258" s="2">
+      <c r="H258" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6861,13 +6835,13 @@
       <c r="D259" t="s">
         <v>154</v>
       </c>
-      <c r="E259" s="2">
+      <c r="E259" s="1">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>204</v>
       </c>
-      <c r="H259" s="2">
+      <c r="H259" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6890,7 +6864,7 @@
       <c r="G260" t="s">
         <v>178</v>
       </c>
-      <c r="H260" s="2">
+      <c r="H260" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6913,7 +6887,7 @@
       <c r="G261" t="s">
         <v>178</v>
       </c>
-      <c r="H261" s="2">
+      <c r="H261" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6936,7 +6910,7 @@
       <c r="G262" t="s">
         <v>179</v>
       </c>
-      <c r="H262" s="2">
+      <c r="H262" s="1">
         <v>46217</v>
       </c>
     </row>
@@ -6950,7 +6924,7 @@
       <c r="C263" t="s">
         <v>115</v>
       </c>
-      <c r="H263" s="2">
+      <c r="H263" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6967,13 +6941,13 @@
       <c r="D264" t="s">
         <v>155</v>
       </c>
-      <c r="E264" s="2">
+      <c r="E264" s="1">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>199</v>
       </c>
-      <c r="H264" s="2">
+      <c r="H264" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -6987,7 +6961,7 @@
       <c r="C265" t="s">
         <v>115</v>
       </c>
-      <c r="H265" s="2">
+      <c r="H265" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7001,7 +6975,7 @@
       <c r="C266" t="s">
         <v>119</v>
       </c>
-      <c r="H266" s="2">
+      <c r="H266" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7015,7 +6989,7 @@
       <c r="C267" t="s">
         <v>115</v>
       </c>
-      <c r="H267" s="2">
+      <c r="H267" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7029,7 +7003,7 @@
       <c r="C268" t="s">
         <v>119</v>
       </c>
-      <c r="H268" s="2">
+      <c r="H268" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7043,7 +7017,7 @@
       <c r="C269" t="s">
         <v>119</v>
       </c>
-      <c r="H269" s="2">
+      <c r="H269" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7060,13 +7034,13 @@
       <c r="D270" t="s">
         <v>125</v>
       </c>
-      <c r="E270" s="2">
+      <c r="E270" s="1">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>193</v>
       </c>
-      <c r="H270" s="2">
+      <c r="H270" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7080,7 +7054,7 @@
       <c r="C271" t="s">
         <v>119</v>
       </c>
-      <c r="H271" s="2">
+      <c r="H271" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7097,13 +7071,13 @@
       <c r="D272" t="s">
         <v>156</v>
       </c>
-      <c r="E272" s="2">
+      <c r="E272" s="1">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>205</v>
       </c>
-      <c r="H272" s="2">
+      <c r="H272" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7120,13 +7094,13 @@
       <c r="D273" t="s">
         <v>157</v>
       </c>
-      <c r="E273" s="2">
+      <c r="E273" s="1">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>207</v>
       </c>
-      <c r="H273" s="2">
+      <c r="H273" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7140,7 +7114,7 @@
       <c r="C274" t="s">
         <v>115</v>
       </c>
-      <c r="H274" s="2">
+      <c r="H274" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7154,7 +7128,7 @@
       <c r="C275" t="s">
         <v>115</v>
       </c>
-      <c r="H275" s="2">
+      <c r="H275" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7171,13 +7145,13 @@
       <c r="D276" t="s">
         <v>128</v>
       </c>
-      <c r="E276" s="2">
+      <c r="E276" s="1">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>206</v>
       </c>
-      <c r="H276" s="2">
+      <c r="H276" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7191,7 +7165,7 @@
       <c r="C277" t="s">
         <v>115</v>
       </c>
-      <c r="H277" s="2">
+      <c r="H277" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7208,13 +7182,13 @@
       <c r="D278" t="s">
         <v>160</v>
       </c>
-      <c r="E278" s="2">
+      <c r="E278" s="1">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>208</v>
       </c>
-      <c r="H278" s="2">
+      <c r="H278" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7231,13 +7205,13 @@
       <c r="D279" t="s">
         <v>158</v>
       </c>
-      <c r="E279" s="2">
+      <c r="E279" s="1">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>207</v>
       </c>
-      <c r="H279" s="2">
+      <c r="H279" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7251,7 +7225,7 @@
       <c r="C280" t="s">
         <v>115</v>
       </c>
-      <c r="H280" s="2">
+      <c r="H280" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7268,13 +7242,13 @@
       <c r="D281" t="s">
         <v>161</v>
       </c>
-      <c r="E281" s="2">
+      <c r="E281" s="1">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>203</v>
       </c>
-      <c r="H281" s="2">
+      <c r="H281" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7297,7 +7271,7 @@
       <c r="G282" t="s">
         <v>181</v>
       </c>
-      <c r="H282" s="2">
+      <c r="H282" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7311,7 +7285,7 @@
       <c r="C283" t="s">
         <v>119</v>
       </c>
-      <c r="H283" s="2">
+      <c r="H283" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7325,7 +7299,7 @@
       <c r="C284" t="s">
         <v>115</v>
       </c>
-      <c r="H284" s="2">
+      <c r="H284" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7348,7 +7322,7 @@
       <c r="G285" t="s">
         <v>176</v>
       </c>
-      <c r="H285" s="2">
+      <c r="H285" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7365,7 +7339,7 @@
       <c r="D286" t="s">
         <v>132</v>
       </c>
-      <c r="H286" s="2">
+      <c r="H286" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7388,7 +7362,7 @@
       <c r="G287" t="s">
         <v>177</v>
       </c>
-      <c r="H287" s="2">
+      <c r="H287" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7405,13 +7379,13 @@
       <c r="D288" t="s">
         <v>154</v>
       </c>
-      <c r="E288" s="2">
+      <c r="E288" s="1">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>204</v>
       </c>
-      <c r="H288" s="2">
+      <c r="H288" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7434,7 +7408,7 @@
       <c r="G289" t="s">
         <v>178</v>
       </c>
-      <c r="H289" s="2">
+      <c r="H289" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7457,7 +7431,7 @@
       <c r="G290" t="s">
         <v>178</v>
       </c>
-      <c r="H290" s="2">
+      <c r="H290" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7480,7 +7454,7 @@
       <c r="G291" t="s">
         <v>179</v>
       </c>
-      <c r="H291" s="2">
+      <c r="H291" s="1">
         <v>46218</v>
       </c>
     </row>
@@ -7494,7 +7468,7 @@
       <c r="C292" t="s">
         <v>115</v>
       </c>
-      <c r="H292" s="2">
+      <c r="H292" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7517,7 +7491,7 @@
       <c r="G293" t="s">
         <v>182</v>
       </c>
-      <c r="H293" s="2">
+      <c r="H293" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7531,7 +7505,7 @@
       <c r="C294" t="s">
         <v>115</v>
       </c>
-      <c r="H294" s="2">
+      <c r="H294" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7554,7 +7528,7 @@
       <c r="G295" t="s">
         <v>183</v>
       </c>
-      <c r="H295" s="2">
+      <c r="H295" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7568,7 +7542,7 @@
       <c r="C296" t="s">
         <v>115</v>
       </c>
-      <c r="H296" s="2">
+      <c r="H296" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7582,7 +7556,7 @@
       <c r="C297" t="s">
         <v>119</v>
       </c>
-      <c r="H297" s="2">
+      <c r="H297" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7605,7 +7579,7 @@
       <c r="G298" t="s">
         <v>184</v>
       </c>
-      <c r="H298" s="2">
+      <c r="H298" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7622,13 +7596,13 @@
       <c r="D299" t="s">
         <v>125</v>
       </c>
-      <c r="E299" s="2">
+      <c r="E299" s="1">
         <v>46234</v>
       </c>
       <c r="G299" t="s">
         <v>193</v>
       </c>
-      <c r="H299" s="2">
+      <c r="H299" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7642,7 +7616,7 @@
       <c r="C300" t="s">
         <v>115</v>
       </c>
-      <c r="H300" s="2">
+      <c r="H300" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7659,13 +7633,13 @@
       <c r="D301" t="s">
         <v>156</v>
       </c>
-      <c r="E301" s="2">
+      <c r="E301" s="1">
         <v>46224</v>
       </c>
       <c r="G301" t="s">
         <v>205</v>
       </c>
-      <c r="H301" s="2">
+      <c r="H301" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7682,13 +7656,13 @@
       <c r="D302" t="s">
         <v>157</v>
       </c>
-      <c r="E302" s="2">
+      <c r="E302" s="1">
         <v>46220</v>
       </c>
       <c r="G302" t="s">
         <v>202</v>
       </c>
-      <c r="H302" s="2">
+      <c r="H302" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7702,7 +7676,7 @@
       <c r="C303" t="s">
         <v>115</v>
       </c>
-      <c r="H303" s="2">
+      <c r="H303" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7716,7 +7690,7 @@
       <c r="C304" t="s">
         <v>115</v>
       </c>
-      <c r="H304" s="2">
+      <c r="H304" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7733,13 +7707,13 @@
       <c r="D305" t="s">
         <v>128</v>
       </c>
-      <c r="E305" s="2">
+      <c r="E305" s="1">
         <v>46237</v>
       </c>
       <c r="G305" t="s">
         <v>206</v>
       </c>
-      <c r="H305" s="2">
+      <c r="H305" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7753,7 +7727,7 @@
       <c r="C306" t="s">
         <v>115</v>
       </c>
-      <c r="H306" s="2">
+      <c r="H306" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7770,13 +7744,13 @@
       <c r="D307" t="s">
         <v>160</v>
       </c>
-      <c r="E307" s="2">
+      <c r="E307" s="1">
         <v>46227</v>
       </c>
       <c r="G307" t="s">
         <v>208</v>
       </c>
-      <c r="H307" s="2">
+      <c r="H307" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7790,7 +7764,7 @@
       <c r="C308" t="s">
         <v>119</v>
       </c>
-      <c r="H308" s="2">
+      <c r="H308" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7813,7 +7787,7 @@
       <c r="G309" t="s">
         <v>182</v>
       </c>
-      <c r="H309" s="2">
+      <c r="H309" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7836,7 +7810,7 @@
       <c r="G310" t="s">
         <v>185</v>
       </c>
-      <c r="H310" s="2">
+      <c r="H310" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7853,7 +7827,7 @@
       <c r="D311" t="s">
         <v>166</v>
       </c>
-      <c r="H311" s="2">
+      <c r="H311" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7867,7 +7841,7 @@
       <c r="C312" t="s">
         <v>119</v>
       </c>
-      <c r="H312" s="2">
+      <c r="H312" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7881,7 +7855,7 @@
       <c r="C313" t="s">
         <v>115</v>
       </c>
-      <c r="H313" s="2">
+      <c r="H313" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="G314" t="s">
         <v>176</v>
       </c>
-      <c r="H314" s="2">
+      <c r="H314" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7921,7 +7895,7 @@
       <c r="D315" t="s">
         <v>132</v>
       </c>
-      <c r="H315" s="2">
+      <c r="H315" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7944,7 +7918,7 @@
       <c r="G316" t="s">
         <v>177</v>
       </c>
-      <c r="H316" s="2">
+      <c r="H316" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7967,7 +7941,7 @@
       <c r="G317" t="s">
         <v>186</v>
       </c>
-      <c r="H317" s="2">
+      <c r="H317" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -7990,7 +7964,7 @@
       <c r="G318" t="s">
         <v>178</v>
       </c>
-      <c r="H318" s="2">
+      <c r="H318" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -8013,7 +7987,7 @@
       <c r="G319" t="s">
         <v>178</v>
       </c>
-      <c r="H319" s="2">
+      <c r="H319" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -8036,7 +8010,7 @@
       <c r="G320" t="s">
         <v>179</v>
       </c>
-      <c r="H320" s="2">
+      <c r="H320" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -8050,7 +8024,7 @@
       <c r="C321" t="s">
         <v>115</v>
       </c>
-      <c r="H321" s="2">
+      <c r="H321" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8073,7 +8047,7 @@
       <c r="G322" t="s">
         <v>187</v>
       </c>
-      <c r="H322" s="2">
+      <c r="H322" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8087,7 +8061,7 @@
       <c r="C323" t="s">
         <v>115</v>
       </c>
-      <c r="H323" s="2">
+      <c r="H323" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8110,7 +8084,7 @@
       <c r="G324" t="s">
         <v>188</v>
       </c>
-      <c r="H324" s="2">
+      <c r="H324" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8124,7 +8098,7 @@
       <c r="C325" t="s">
         <v>115</v>
       </c>
-      <c r="H325" s="2">
+      <c r="H325" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8138,7 +8112,7 @@
       <c r="C326" t="s">
         <v>119</v>
       </c>
-      <c r="H326" s="2">
+      <c r="H326" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8152,7 +8126,7 @@
       <c r="C327" t="s">
         <v>119</v>
       </c>
-      <c r="H327" s="2">
+      <c r="H327" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8169,13 +8143,13 @@
       <c r="D328" t="s">
         <v>125</v>
       </c>
-      <c r="E328" s="2">
+      <c r="E328" s="1">
         <v>46234</v>
       </c>
       <c r="G328" t="s">
         <v>193</v>
       </c>
-      <c r="H328" s="2">
+      <c r="H328" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8198,7 +8172,7 @@
       <c r="G329" t="s">
         <v>188</v>
       </c>
-      <c r="H329" s="2">
+      <c r="H329" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8221,7 +8195,7 @@
       <c r="G330" t="s">
         <v>188</v>
       </c>
-      <c r="H330" s="2">
+      <c r="H330" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8235,7 +8209,7 @@
       <c r="C331" t="s">
         <v>115</v>
       </c>
-      <c r="H331" s="2">
+      <c r="H331" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8258,7 +8232,7 @@
       <c r="G332" t="s">
         <v>188</v>
       </c>
-      <c r="H332" s="2">
+      <c r="H332" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8281,7 +8255,7 @@
       <c r="G333" t="s">
         <v>187</v>
       </c>
-      <c r="H333" s="2">
+      <c r="H333" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8298,13 +8272,13 @@
       <c r="D334" t="s">
         <v>128</v>
       </c>
-      <c r="E334" s="2">
+      <c r="E334" s="1">
         <v>46237</v>
       </c>
       <c r="G334" t="s">
         <v>206</v>
       </c>
-      <c r="H334" s="2">
+      <c r="H334" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8318,7 +8292,7 @@
       <c r="C335" t="s">
         <v>115</v>
       </c>
-      <c r="H335" s="2">
+      <c r="H335" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8335,13 +8309,13 @@
       <c r="D336" t="s">
         <v>160</v>
       </c>
-      <c r="E336" s="2">
+      <c r="E336" s="1">
         <v>46227</v>
       </c>
       <c r="G336" t="s">
         <v>208</v>
       </c>
-      <c r="H336" s="2">
+      <c r="H336" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8355,7 +8329,7 @@
       <c r="C337" t="s">
         <v>115</v>
       </c>
-      <c r="H337" s="2">
+      <c r="H337" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8369,7 +8343,7 @@
       <c r="C338" t="s">
         <v>115</v>
       </c>
-      <c r="H338" s="2">
+      <c r="H338" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8392,7 +8366,7 @@
       <c r="G339" t="s">
         <v>185</v>
       </c>
-      <c r="H339" s="2">
+      <c r="H339" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8409,7 +8383,7 @@
       <c r="D340" t="s">
         <v>171</v>
       </c>
-      <c r="H340" s="2">
+      <c r="H340" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8423,7 +8397,7 @@
       <c r="C341" t="s">
         <v>119</v>
       </c>
-      <c r="H341" s="2">
+      <c r="H341" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8437,7 +8411,7 @@
       <c r="C342" t="s">
         <v>115</v>
       </c>
-      <c r="H342" s="2">
+      <c r="H342" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8460,7 +8434,7 @@
       <c r="G343" t="s">
         <v>176</v>
       </c>
-      <c r="H343" s="2">
+      <c r="H343" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8477,7 +8451,7 @@
       <c r="D344" t="s">
         <v>132</v>
       </c>
-      <c r="H344" s="2">
+      <c r="H344" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8500,7 +8474,7 @@
       <c r="G345" t="s">
         <v>177</v>
       </c>
-      <c r="H345" s="2">
+      <c r="H345" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8523,7 +8497,7 @@
       <c r="G346" t="s">
         <v>186</v>
       </c>
-      <c r="H346" s="2">
+      <c r="H346" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8546,7 +8520,7 @@
       <c r="G347" t="s">
         <v>178</v>
       </c>
-      <c r="H347" s="2">
+      <c r="H347" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8569,7 +8543,7 @@
       <c r="G348" t="s">
         <v>178</v>
       </c>
-      <c r="H348" s="2">
+      <c r="H348" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8592,7 +8566,7 @@
       <c r="G349" t="s">
         <v>179</v>
       </c>
-      <c r="H349" s="2">
+      <c r="H349" s="1">
         <v>46224</v>
       </c>
     </row>
@@ -8606,7 +8580,7 @@
       <c r="C350" t="s">
         <v>115</v>
       </c>
-      <c r="H350" s="2">
+      <c r="H350" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8629,7 +8603,7 @@
       <c r="G351" t="s">
         <v>187</v>
       </c>
-      <c r="H351" s="2">
+      <c r="H351" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8643,7 +8617,7 @@
       <c r="C352" t="s">
         <v>115</v>
       </c>
-      <c r="H352" s="2">
+      <c r="H352" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8657,7 +8631,7 @@
       <c r="C353" t="s">
         <v>115</v>
       </c>
-      <c r="H353" s="2">
+      <c r="H353" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8671,7 +8645,7 @@
       <c r="C354" t="s">
         <v>115</v>
       </c>
-      <c r="H354" s="2">
+      <c r="H354" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8685,7 +8659,7 @@
       <c r="C355" t="s">
         <v>119</v>
       </c>
-      <c r="H355" s="2">
+      <c r="H355" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8699,7 +8673,7 @@
       <c r="C356" t="s">
         <v>119</v>
       </c>
-      <c r="H356" s="2">
+      <c r="H356" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8722,7 +8696,7 @@
       <c r="G357" t="s">
         <v>189</v>
       </c>
-      <c r="H357" s="2">
+      <c r="H357" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8736,7 +8710,7 @@
       <c r="C358" t="s">
         <v>115</v>
       </c>
-      <c r="H358" s="2">
+      <c r="H358" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8759,7 +8733,7 @@
       <c r="G359" t="s">
         <v>190</v>
       </c>
-      <c r="H359" s="2">
+      <c r="H359" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8773,7 +8747,7 @@
       <c r="C360" t="s">
         <v>115</v>
       </c>
-      <c r="H360" s="2">
+      <c r="H360" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8787,7 +8761,7 @@
       <c r="C361" t="s">
         <v>115</v>
       </c>
-      <c r="H361" s="2">
+      <c r="H361" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8810,7 +8784,7 @@
       <c r="G362" t="s">
         <v>187</v>
       </c>
-      <c r="H362" s="2">
+      <c r="H362" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8833,7 +8807,7 @@
       <c r="G363" t="s">
         <v>191</v>
       </c>
-      <c r="H363" s="2">
+      <c r="H363" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8847,7 +8821,7 @@
       <c r="C364" t="s">
         <v>115</v>
       </c>
-      <c r="H364" s="2">
+      <c r="H364" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8870,7 +8844,7 @@
       <c r="G365" t="s">
         <v>190</v>
       </c>
-      <c r="H365" s="2">
+      <c r="H365" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8884,7 +8858,7 @@
       <c r="C366" t="s">
         <v>115</v>
       </c>
-      <c r="H366" s="2">
+      <c r="H366" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8898,7 +8872,7 @@
       <c r="C367" t="s">
         <v>115</v>
       </c>
-      <c r="H367" s="2">
+      <c r="H367" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8921,7 +8895,7 @@
       <c r="G368" t="s">
         <v>189</v>
       </c>
-      <c r="H368" s="2">
+      <c r="H368" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8944,7 +8918,7 @@
       <c r="G369" t="s">
         <v>190</v>
       </c>
-      <c r="H369" s="2">
+      <c r="H369" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8961,7 +8935,7 @@
       <c r="D370" t="s">
         <v>171</v>
       </c>
-      <c r="H370" s="2">
+      <c r="H370" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8975,7 +8949,7 @@
       <c r="C371" t="s">
         <v>115</v>
       </c>
-      <c r="H371" s="2">
+      <c r="H371" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -8998,7 +8972,7 @@
       <c r="G372" t="s">
         <v>176</v>
       </c>
-      <c r="H372" s="2">
+      <c r="H372" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9015,7 +8989,7 @@
       <c r="D373" t="s">
         <v>132</v>
       </c>
-      <c r="H373" s="2">
+      <c r="H373" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9038,7 +9012,7 @@
       <c r="G374" t="s">
         <v>177</v>
       </c>
-      <c r="H374" s="2">
+      <c r="H374" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9061,7 +9035,7 @@
       <c r="G375" t="s">
         <v>186</v>
       </c>
-      <c r="H375" s="2">
+      <c r="H375" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9084,7 +9058,7 @@
       <c r="G376" t="s">
         <v>178</v>
       </c>
-      <c r="H376" s="2">
+      <c r="H376" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9107,7 +9081,7 @@
       <c r="G377" t="s">
         <v>178</v>
       </c>
-      <c r="H377" s="2">
+      <c r="H377" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9130,7 +9104,7 @@
       <c r="G378" t="s">
         <v>179</v>
       </c>
-      <c r="H378" s="2">
+      <c r="H378" s="1">
         <v>46225</v>
       </c>
     </row>
@@ -9144,7 +9118,7 @@
       <c r="C379" t="s">
         <v>115</v>
       </c>
-      <c r="H379" s="2">
+      <c r="H379" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9167,7 +9141,7 @@
       <c r="G380" t="s">
         <v>190</v>
       </c>
-      <c r="H380" s="2">
+      <c r="H380" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9181,7 +9155,7 @@
       <c r="C381" t="s">
         <v>115</v>
       </c>
-      <c r="H381" s="2">
+      <c r="H381" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9195,7 +9169,7 @@
       <c r="C382" t="s">
         <v>115</v>
       </c>
-      <c r="H382" s="2">
+      <c r="H382" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9209,7 +9183,7 @@
       <c r="C383" t="s">
         <v>115</v>
       </c>
-      <c r="H383" s="2">
+      <c r="H383" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9223,7 +9197,7 @@
       <c r="C384" t="s">
         <v>119</v>
       </c>
-      <c r="H384" s="2">
+      <c r="H384" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9237,7 +9211,7 @@
       <c r="C385" t="s">
         <v>119</v>
       </c>
-      <c r="H385" s="2">
+      <c r="H385" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9260,7 +9234,7 @@
       <c r="G386" t="s">
         <v>189</v>
       </c>
-      <c r="H386" s="2">
+      <c r="H386" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9274,7 +9248,7 @@
       <c r="C387" t="s">
         <v>115</v>
       </c>
-      <c r="H387" s="2">
+      <c r="H387" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9288,7 +9262,7 @@
       <c r="C388" t="s">
         <v>119</v>
       </c>
-      <c r="H388" s="2">
+      <c r="H388" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9302,7 +9276,7 @@
       <c r="C389" t="s">
         <v>115</v>
       </c>
-      <c r="H389" s="2">
+      <c r="H389" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9316,7 +9290,7 @@
       <c r="C390" t="s">
         <v>115</v>
       </c>
-      <c r="H390" s="2">
+      <c r="H390" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9339,7 +9313,7 @@
       <c r="G391" t="s">
         <v>190</v>
       </c>
-      <c r="H391" s="2">
+      <c r="H391" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9362,7 +9336,7 @@
       <c r="G392" t="s">
         <v>191</v>
       </c>
-      <c r="H392" s="2">
+      <c r="H392" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9376,7 +9350,7 @@
       <c r="C393" t="s">
         <v>115</v>
       </c>
-      <c r="H393" s="2">
+      <c r="H393" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9399,7 +9373,7 @@
       <c r="G394" t="s">
         <v>190</v>
       </c>
-      <c r="H394" s="2">
+      <c r="H394" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9413,7 +9387,7 @@
       <c r="C395" t="s">
         <v>115</v>
       </c>
-      <c r="H395" s="2">
+      <c r="H395" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9427,7 +9401,7 @@
       <c r="C396" t="s">
         <v>115</v>
       </c>
-      <c r="H396" s="2">
+      <c r="H396" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9450,7 +9424,7 @@
       <c r="G397" t="s">
         <v>189</v>
       </c>
-      <c r="H397" s="2">
+      <c r="H397" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9473,7 +9447,7 @@
       <c r="G398" t="s">
         <v>190</v>
       </c>
-      <c r="H398" s="2">
+      <c r="H398" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9490,7 +9464,7 @@
       <c r="D399" t="s">
         <v>171</v>
       </c>
-      <c r="H399" s="2">
+      <c r="H399" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9504,7 +9478,7 @@
       <c r="C400" t="s">
         <v>115</v>
       </c>
-      <c r="H400" s="2">
+      <c r="H400" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9527,7 +9501,7 @@
       <c r="G401" t="s">
         <v>176</v>
       </c>
-      <c r="H401" s="2">
+      <c r="H401" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9544,7 +9518,7 @@
       <c r="D402" t="s">
         <v>132</v>
       </c>
-      <c r="H402" s="2">
+      <c r="H402" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9567,7 +9541,7 @@
       <c r="G403" t="s">
         <v>177</v>
       </c>
-      <c r="H403" s="2">
+      <c r="H403" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9590,7 +9564,7 @@
       <c r="G404" t="s">
         <v>186</v>
       </c>
-      <c r="H404" s="2">
+      <c r="H404" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9613,7 +9587,7 @@
       <c r="G405" t="s">
         <v>178</v>
       </c>
-      <c r="H405" s="2">
+      <c r="H405" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9636,7 +9610,7 @@
       <c r="G406" t="s">
         <v>178</v>
       </c>
-      <c r="H406" s="2">
+      <c r="H406" s="1">
         <v>46226</v>
       </c>
     </row>
@@ -9659,7 +9633,7 @@
       <c r="G407" t="s">
         <v>179</v>
       </c>
-      <c r="H407" s="2">
+      <c r="H407" s="1">
         <v>46226</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Registra verificação do Drive (Disponibilidade Diária) do teste final
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -651,8 +651,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -668,7 +676,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -676,12 +684,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -981,72 +1007,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>46204</v>
       </c>
       <c r="B2">
@@ -1111,7 +1137,7 @@
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>46205</v>
       </c>
       <c r="B3">
@@ -1176,7 +1202,7 @@
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>46209</v>
       </c>
       <c r="B4">
@@ -1241,7 +1267,7 @@
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>46210</v>
       </c>
       <c r="B5">
@@ -1306,7 +1332,7 @@
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>46211</v>
       </c>
       <c r="B6">
@@ -1371,7 +1397,7 @@
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>46212</v>
       </c>
       <c r="B7">
@@ -1436,7 +1462,7 @@
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>46213</v>
       </c>
       <c r="B8">
@@ -1501,7 +1527,7 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>46216</v>
       </c>
       <c r="B9">
@@ -1566,7 +1592,7 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>46217</v>
       </c>
       <c r="B10">
@@ -1631,7 +1657,7 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>46218</v>
       </c>
       <c r="B11">
@@ -1696,7 +1722,7 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>46220</v>
       </c>
       <c r="B12">
@@ -1761,7 +1787,7 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46224</v>
       </c>
       <c r="B13">
@@ -1826,7 +1852,7 @@
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46225</v>
       </c>
       <c r="B14">
@@ -1891,7 +1917,7 @@
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46226</v>
       </c>
       <c r="B15">
@@ -1966,28 +1992,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2001,7 +2027,7 @@
       <c r="C2" t="s">
         <v>115</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2015,7 +2041,7 @@
       <c r="C3" t="s">
         <v>115</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2038,7 +2064,7 @@
       <c r="G4" t="s">
         <v>174</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2052,7 +2078,7 @@
       <c r="C5" t="s">
         <v>115</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2066,7 +2092,7 @@
       <c r="C6" t="s">
         <v>115</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2083,13 +2109,13 @@
       <c r="D7" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>46206</v>
       </c>
       <c r="G7" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2106,13 +2132,13 @@
       <c r="D8" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>46206</v>
       </c>
       <c r="G8" t="s">
         <v>192</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2129,13 +2155,13 @@
       <c r="D9" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>46234</v>
       </c>
       <c r="G9" t="s">
         <v>193</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2152,13 +2178,13 @@
       <c r="D10" t="s">
         <v>126</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>46213</v>
       </c>
       <c r="G10" t="s">
         <v>194</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2172,7 +2198,7 @@
       <c r="C11" t="s">
         <v>115</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2186,7 +2212,7 @@
       <c r="C12" t="s">
         <v>115</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2203,13 +2229,13 @@
       <c r="D13" t="s">
         <v>127</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46206</v>
       </c>
       <c r="G13" t="s">
         <v>192</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2223,7 +2249,7 @@
       <c r="C14" t="s">
         <v>119</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2240,13 +2266,13 @@
       <c r="D15" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46216</v>
       </c>
       <c r="G15" t="s">
         <v>195</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2260,7 +2286,7 @@
       <c r="C16" t="s">
         <v>115</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2274,7 +2300,7 @@
       <c r="C17" t="s">
         <v>115</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2291,13 +2317,13 @@
       <c r="D18" t="s">
         <v>129</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46204</v>
       </c>
       <c r="G18" t="s">
         <v>196</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2311,7 +2337,7 @@
       <c r="C19" t="s">
         <v>115</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2328,13 +2354,13 @@
       <c r="D20" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46206</v>
       </c>
       <c r="G20" t="s">
         <v>192</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2357,7 +2383,7 @@
       <c r="G21" t="s">
         <v>175</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2371,7 +2397,7 @@
       <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2385,7 +2411,7 @@
       <c r="C23" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2408,7 +2434,7 @@
       <c r="G24" t="s">
         <v>176</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2425,7 +2451,7 @@
       <c r="D25" t="s">
         <v>132</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2448,7 +2474,7 @@
       <c r="G26" t="s">
         <v>177</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2465,13 +2491,13 @@
       <c r="D27" t="s">
         <v>134</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46209</v>
       </c>
       <c r="G27" t="s">
         <v>197</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2494,7 +2520,7 @@
       <c r="G28" t="s">
         <v>178</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2517,7 +2543,7 @@
       <c r="G29" t="s">
         <v>178</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2540,7 +2566,7 @@
       <c r="G30" t="s">
         <v>179</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46204</v>
       </c>
     </row>
@@ -2554,7 +2580,7 @@
       <c r="C31" t="s">
         <v>115</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2568,7 +2594,7 @@
       <c r="C32" t="s">
         <v>115</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2591,7 +2617,7 @@
       <c r="G33" t="s">
         <v>180</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2605,7 +2631,7 @@
       <c r="C34" t="s">
         <v>115</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2619,7 +2645,7 @@
       <c r="C35" t="s">
         <v>115</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2636,13 +2662,13 @@
       <c r="D36" t="s">
         <v>123</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46206</v>
       </c>
       <c r="G36" t="s">
         <v>192</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2659,13 +2685,13 @@
       <c r="D37" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="2">
         <v>46206</v>
       </c>
       <c r="G37" t="s">
         <v>192</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2682,13 +2708,13 @@
       <c r="D38" t="s">
         <v>125</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38" s="2">
         <v>46234</v>
       </c>
       <c r="G38" t="s">
         <v>193</v>
       </c>
-      <c r="H38" s="1">
+      <c r="H38" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2705,13 +2731,13 @@
       <c r="D39" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39" s="2">
         <v>46213</v>
       </c>
       <c r="G39" t="s">
         <v>194</v>
       </c>
-      <c r="H39" s="1">
+      <c r="H39" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2725,7 +2751,7 @@
       <c r="C40" t="s">
         <v>115</v>
       </c>
-      <c r="H40" s="1">
+      <c r="H40" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2739,7 +2765,7 @@
       <c r="C41" t="s">
         <v>115</v>
       </c>
-      <c r="H41" s="1">
+      <c r="H41" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2756,13 +2782,13 @@
       <c r="D42" t="s">
         <v>127</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42" s="2">
         <v>46206</v>
       </c>
       <c r="G42" t="s">
         <v>192</v>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2776,7 +2802,7 @@
       <c r="C43" t="s">
         <v>115</v>
       </c>
-      <c r="H43" s="1">
+      <c r="H43" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2793,13 +2819,13 @@
       <c r="D44" t="s">
         <v>128</v>
       </c>
-      <c r="E44" s="1">
+      <c r="E44" s="2">
         <v>46216</v>
       </c>
       <c r="G44" t="s">
         <v>195</v>
       </c>
-      <c r="H44" s="1">
+      <c r="H44" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2813,7 +2839,7 @@
       <c r="C45" t="s">
         <v>115</v>
       </c>
-      <c r="H45" s="1">
+      <c r="H45" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2827,7 +2853,7 @@
       <c r="C46" t="s">
         <v>115</v>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2841,7 +2867,7 @@
       <c r="C47" t="s">
         <v>119</v>
       </c>
-      <c r="H47" s="1">
+      <c r="H47" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2855,7 +2881,7 @@
       <c r="C48" t="s">
         <v>115</v>
       </c>
-      <c r="H48" s="1">
+      <c r="H48" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2872,13 +2898,13 @@
       <c r="D49" t="s">
         <v>139</v>
       </c>
-      <c r="E49" s="1">
+      <c r="E49" s="2">
         <v>46206</v>
       </c>
       <c r="G49" t="s">
         <v>192</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H49" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2901,7 +2927,7 @@
       <c r="G50" t="s">
         <v>175</v>
       </c>
-      <c r="H50" s="1">
+      <c r="H50" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2915,7 +2941,7 @@
       <c r="C51" t="s">
         <v>119</v>
       </c>
-      <c r="H51" s="1">
+      <c r="H51" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2929,7 +2955,7 @@
       <c r="C52" t="s">
         <v>115</v>
       </c>
-      <c r="H52" s="1">
+      <c r="H52" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2952,7 +2978,7 @@
       <c r="G53" t="s">
         <v>176</v>
       </c>
-      <c r="H53" s="1">
+      <c r="H53" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2969,7 +2995,7 @@
       <c r="D54" t="s">
         <v>132</v>
       </c>
-      <c r="H54" s="1">
+      <c r="H54" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -2992,7 +3018,7 @@
       <c r="G55" t="s">
         <v>177</v>
       </c>
-      <c r="H55" s="1">
+      <c r="H55" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3009,13 +3035,13 @@
       <c r="D56" t="s">
         <v>134</v>
       </c>
-      <c r="E56" s="1">
+      <c r="E56" s="2">
         <v>46209</v>
       </c>
       <c r="G56" t="s">
         <v>197</v>
       </c>
-      <c r="H56" s="1">
+      <c r="H56" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3038,7 +3064,7 @@
       <c r="G57" t="s">
         <v>178</v>
       </c>
-      <c r="H57" s="1">
+      <c r="H57" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3061,7 +3087,7 @@
       <c r="G58" t="s">
         <v>178</v>
       </c>
-      <c r="H58" s="1">
+      <c r="H58" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3084,7 +3110,7 @@
       <c r="G59" t="s">
         <v>179</v>
       </c>
-      <c r="H59" s="1">
+      <c r="H59" s="2">
         <v>46205</v>
       </c>
     </row>
@@ -3098,7 +3124,7 @@
       <c r="C60" t="s">
         <v>115</v>
       </c>
-      <c r="H60" s="1">
+      <c r="H60" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3112,7 +3138,7 @@
       <c r="C61" t="s">
         <v>115</v>
       </c>
-      <c r="H61" s="1">
+      <c r="H61" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3129,13 +3155,13 @@
       <c r="D62" t="s">
         <v>138</v>
       </c>
-      <c r="E62" s="1">
+      <c r="E62" s="2">
         <v>46210</v>
       </c>
       <c r="G62" t="s">
         <v>198</v>
       </c>
-      <c r="H62" s="1">
+      <c r="H62" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3149,7 +3175,7 @@
       <c r="C63" t="s">
         <v>115</v>
       </c>
-      <c r="H63" s="1">
+      <c r="H63" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3166,13 +3192,13 @@
       <c r="D64" t="s">
         <v>140</v>
       </c>
-      <c r="E64" s="1">
+      <c r="E64" s="2">
         <v>46217</v>
       </c>
       <c r="G64" t="s">
         <v>199</v>
       </c>
-      <c r="H64" s="1">
+      <c r="H64" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3186,7 +3212,7 @@
       <c r="C65" t="s">
         <v>115</v>
       </c>
-      <c r="H65" s="1">
+      <c r="H65" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3200,7 +3226,7 @@
       <c r="C66" t="s">
         <v>119</v>
       </c>
-      <c r="H66" s="1">
+      <c r="H66" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3217,13 +3243,13 @@
       <c r="D67" t="s">
         <v>125</v>
       </c>
-      <c r="E67" s="1">
+      <c r="E67" s="2">
         <v>46234</v>
       </c>
       <c r="G67" t="s">
         <v>193</v>
       </c>
-      <c r="H67" s="1">
+      <c r="H67" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3240,13 +3266,13 @@
       <c r="D68" t="s">
         <v>126</v>
       </c>
-      <c r="E68" s="1">
+      <c r="E68" s="2">
         <v>46213</v>
       </c>
       <c r="G68" t="s">
         <v>194</v>
       </c>
-      <c r="H68" s="1">
+      <c r="H68" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3260,7 +3286,7 @@
       <c r="C69" t="s">
         <v>115</v>
       </c>
-      <c r="H69" s="1">
+      <c r="H69" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3274,7 +3300,7 @@
       <c r="C70" t="s">
         <v>115</v>
       </c>
-      <c r="H70" s="1">
+      <c r="H70" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3291,13 +3317,13 @@
       <c r="D71" t="s">
         <v>127</v>
       </c>
-      <c r="E71" s="1">
+      <c r="E71" s="2">
         <v>46210</v>
       </c>
       <c r="G71" t="s">
         <v>198</v>
       </c>
-      <c r="H71" s="1">
+      <c r="H71" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3311,7 +3337,7 @@
       <c r="C72" t="s">
         <v>115</v>
       </c>
-      <c r="H72" s="1">
+      <c r="H72" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3328,13 +3354,13 @@
       <c r="D73" t="s">
         <v>128</v>
       </c>
-      <c r="E73" s="1">
+      <c r="E73" s="2">
         <v>46216</v>
       </c>
       <c r="G73" t="s">
         <v>195</v>
       </c>
-      <c r="H73" s="1">
+      <c r="H73" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3348,7 +3374,7 @@
       <c r="C74" t="s">
         <v>115</v>
       </c>
-      <c r="H74" s="1">
+      <c r="H74" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3362,7 +3388,7 @@
       <c r="C75" t="s">
         <v>115</v>
       </c>
-      <c r="H75" s="1">
+      <c r="H75" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3376,7 +3402,7 @@
       <c r="C76" t="s">
         <v>115</v>
       </c>
-      <c r="H76" s="1">
+      <c r="H76" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3390,7 +3416,7 @@
       <c r="C77" t="s">
         <v>115</v>
       </c>
-      <c r="H77" s="1">
+      <c r="H77" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3407,13 +3433,13 @@
       <c r="D78" t="s">
         <v>139</v>
       </c>
-      <c r="E78" s="1">
+      <c r="E78" s="2">
         <v>46210</v>
       </c>
       <c r="G78" t="s">
         <v>198</v>
       </c>
-      <c r="H78" s="1">
+      <c r="H78" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3436,7 +3462,7 @@
       <c r="G79" t="s">
         <v>181</v>
       </c>
-      <c r="H79" s="1">
+      <c r="H79" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3450,7 +3476,7 @@
       <c r="C80" t="s">
         <v>119</v>
       </c>
-      <c r="H80" s="1">
+      <c r="H80" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3464,7 +3490,7 @@
       <c r="C81" t="s">
         <v>115</v>
       </c>
-      <c r="H81" s="1">
+      <c r="H81" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3487,7 +3513,7 @@
       <c r="G82" t="s">
         <v>176</v>
       </c>
-      <c r="H82" s="1">
+      <c r="H82" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3504,7 +3530,7 @@
       <c r="D83" t="s">
         <v>132</v>
       </c>
-      <c r="H83" s="1">
+      <c r="H83" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3527,7 +3553,7 @@
       <c r="G84" t="s">
         <v>177</v>
       </c>
-      <c r="H84" s="1">
+      <c r="H84" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3544,13 +3570,13 @@
       <c r="D85" t="s">
         <v>134</v>
       </c>
-      <c r="E85" s="1">
+      <c r="E85" s="2">
         <v>46209</v>
       </c>
       <c r="G85" t="s">
         <v>197</v>
       </c>
-      <c r="H85" s="1">
+      <c r="H85" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3573,7 +3599,7 @@
       <c r="G86" t="s">
         <v>178</v>
       </c>
-      <c r="H86" s="1">
+      <c r="H86" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3596,7 +3622,7 @@
       <c r="G87" t="s">
         <v>178</v>
       </c>
-      <c r="H87" s="1">
+      <c r="H87" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3619,7 +3645,7 @@
       <c r="G88" t="s">
         <v>179</v>
       </c>
-      <c r="H88" s="1">
+      <c r="H88" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -3633,7 +3659,7 @@
       <c r="C89" t="s">
         <v>115</v>
       </c>
-      <c r="H89" s="1">
+      <c r="H89" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3650,13 +3676,13 @@
       <c r="D90" t="s">
         <v>142</v>
       </c>
-      <c r="E90" s="1">
+      <c r="E90" s="2">
         <v>46217</v>
       </c>
       <c r="G90" t="s">
         <v>199</v>
       </c>
-      <c r="H90" s="1">
+      <c r="H90" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3673,13 +3699,13 @@
       <c r="D91" t="s">
         <v>138</v>
       </c>
-      <c r="E91" s="1">
+      <c r="E91" s="2">
         <v>46210</v>
       </c>
       <c r="G91" t="s">
         <v>198</v>
       </c>
-      <c r="H91" s="1">
+      <c r="H91" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3693,7 +3719,7 @@
       <c r="C92" t="s">
         <v>115</v>
       </c>
-      <c r="H92" s="1">
+      <c r="H92" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3710,13 +3736,13 @@
       <c r="D93" t="s">
         <v>140</v>
       </c>
-      <c r="E93" s="1">
+      <c r="E93" s="2">
         <v>46217</v>
       </c>
       <c r="G93" t="s">
         <v>199</v>
       </c>
-      <c r="H93" s="1">
+      <c r="H93" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3730,7 +3756,7 @@
       <c r="C94" t="s">
         <v>115</v>
       </c>
-      <c r="H94" s="1">
+      <c r="H94" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3744,7 +3770,7 @@
       <c r="C95" t="s">
         <v>119</v>
       </c>
-      <c r="H95" s="1">
+      <c r="H95" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3761,13 +3787,13 @@
       <c r="D96" t="s">
         <v>125</v>
       </c>
-      <c r="E96" s="1">
+      <c r="E96" s="2">
         <v>46234</v>
       </c>
       <c r="G96" t="s">
         <v>193</v>
       </c>
-      <c r="H96" s="1">
+      <c r="H96" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3784,13 +3810,13 @@
       <c r="D97" t="s">
         <v>126</v>
       </c>
-      <c r="E97" s="1">
+      <c r="E97" s="2">
         <v>46213</v>
       </c>
       <c r="G97" t="s">
         <v>194</v>
       </c>
-      <c r="H97" s="1">
+      <c r="H97" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3804,7 +3830,7 @@
       <c r="C98" t="s">
         <v>115</v>
       </c>
-      <c r="H98" s="1">
+      <c r="H98" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3821,13 +3847,13 @@
       <c r="D99" t="s">
         <v>143</v>
       </c>
-      <c r="E99" s="1">
+      <c r="E99" s="2">
         <v>46213</v>
       </c>
       <c r="G99" t="s">
         <v>194</v>
       </c>
-      <c r="H99" s="1">
+      <c r="H99" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3844,13 +3870,13 @@
       <c r="D100" t="s">
         <v>127</v>
       </c>
-      <c r="E100" s="1">
+      <c r="E100" s="2">
         <v>46213</v>
       </c>
       <c r="G100" t="s">
         <v>194</v>
       </c>
-      <c r="H100" s="1">
+      <c r="H100" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3864,7 +3890,7 @@
       <c r="C101" t="s">
         <v>115</v>
       </c>
-      <c r="H101" s="1">
+      <c r="H101" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3881,13 +3907,13 @@
       <c r="D102" t="s">
         <v>128</v>
       </c>
-      <c r="E102" s="1">
+      <c r="E102" s="2">
         <v>46216</v>
       </c>
       <c r="G102" t="s">
         <v>195</v>
       </c>
-      <c r="H102" s="1">
+      <c r="H102" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3904,13 +3930,13 @@
       <c r="D103" t="s">
         <v>144</v>
       </c>
-      <c r="E103" s="1">
+      <c r="E103" s="2">
         <v>46213</v>
       </c>
       <c r="G103" t="s">
         <v>194</v>
       </c>
-      <c r="H103" s="1">
+      <c r="H103" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3924,7 +3950,7 @@
       <c r="C104" t="s">
         <v>115</v>
       </c>
-      <c r="H104" s="1">
+      <c r="H104" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3938,7 +3964,7 @@
       <c r="C105" t="s">
         <v>115</v>
       </c>
-      <c r="H105" s="1">
+      <c r="H105" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3952,7 +3978,7 @@
       <c r="C106" t="s">
         <v>115</v>
       </c>
-      <c r="H106" s="1">
+      <c r="H106" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3969,13 +3995,13 @@
       <c r="D107" t="s">
         <v>145</v>
       </c>
-      <c r="E107" s="1">
+      <c r="E107" s="2">
         <v>46213</v>
       </c>
       <c r="G107" t="s">
         <v>194</v>
       </c>
-      <c r="H107" s="1">
+      <c r="H107" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -3998,7 +4024,7 @@
       <c r="G108" t="s">
         <v>181</v>
       </c>
-      <c r="H108" s="1">
+      <c r="H108" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4012,7 +4038,7 @@
       <c r="C109" t="s">
         <v>119</v>
       </c>
-      <c r="H109" s="1">
+      <c r="H109" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4026,7 +4052,7 @@
       <c r="C110" t="s">
         <v>115</v>
       </c>
-      <c r="H110" s="1">
+      <c r="H110" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4049,7 +4075,7 @@
       <c r="G111" t="s">
         <v>176</v>
       </c>
-      <c r="H111" s="1">
+      <c r="H111" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4066,7 +4092,7 @@
       <c r="D112" t="s">
         <v>132</v>
       </c>
-      <c r="H112" s="1">
+      <c r="H112" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4089,7 +4115,7 @@
       <c r="G113" t="s">
         <v>177</v>
       </c>
-      <c r="H113" s="1">
+      <c r="H113" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4106,13 +4132,13 @@
       <c r="D114" t="s">
         <v>134</v>
       </c>
-      <c r="E114" s="1">
+      <c r="E114" s="2">
         <v>46209</v>
       </c>
       <c r="G114" t="s">
         <v>197</v>
       </c>
-      <c r="H114" s="1">
+      <c r="H114" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4135,7 +4161,7 @@
       <c r="G115" t="s">
         <v>178</v>
       </c>
-      <c r="H115" s="1">
+      <c r="H115" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4158,7 +4184,7 @@
       <c r="G116" t="s">
         <v>178</v>
       </c>
-      <c r="H116" s="1">
+      <c r="H116" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4181,7 +4207,7 @@
       <c r="G117" t="s">
         <v>179</v>
       </c>
-      <c r="H117" s="1">
+      <c r="H117" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -4195,7 +4221,7 @@
       <c r="C118" t="s">
         <v>115</v>
       </c>
-      <c r="H118" s="1">
+      <c r="H118" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4212,13 +4238,13 @@
       <c r="D119" t="s">
         <v>142</v>
       </c>
-      <c r="E119" s="1">
+      <c r="E119" s="2">
         <v>46217</v>
       </c>
       <c r="G119" t="s">
         <v>199</v>
       </c>
-      <c r="H119" s="1">
+      <c r="H119" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4232,7 +4258,7 @@
       <c r="C120" t="s">
         <v>119</v>
       </c>
-      <c r="H120" s="1">
+      <c r="H120" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4246,7 +4272,7 @@
       <c r="C121" t="s">
         <v>115</v>
       </c>
-      <c r="H121" s="1">
+      <c r="H121" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4260,7 +4286,7 @@
       <c r="C122" t="s">
         <v>119</v>
       </c>
-      <c r="H122" s="1">
+      <c r="H122" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4274,7 +4300,7 @@
       <c r="C123" t="s">
         <v>119</v>
       </c>
-      <c r="H123" s="1">
+      <c r="H123" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4288,7 +4314,7 @@
       <c r="C124" t="s">
         <v>119</v>
       </c>
-      <c r="H124" s="1">
+      <c r="H124" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4305,13 +4331,13 @@
       <c r="D125" t="s">
         <v>125</v>
       </c>
-      <c r="E125" s="1">
+      <c r="E125" s="2">
         <v>46234</v>
       </c>
       <c r="G125" t="s">
         <v>193</v>
       </c>
-      <c r="H125" s="1">
+      <c r="H125" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4328,13 +4354,13 @@
       <c r="D126" t="s">
         <v>126</v>
       </c>
-      <c r="E126" s="1">
+      <c r="E126" s="2">
         <v>46213</v>
       </c>
       <c r="G126" t="s">
         <v>194</v>
       </c>
-      <c r="H126" s="1">
+      <c r="H126" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4348,7 +4374,7 @@
       <c r="C127" t="s">
         <v>115</v>
       </c>
-      <c r="H127" s="1">
+      <c r="H127" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4365,13 +4391,13 @@
       <c r="D128" t="s">
         <v>143</v>
       </c>
-      <c r="E128" s="1">
+      <c r="E128" s="2">
         <v>46213</v>
       </c>
       <c r="G128" t="s">
         <v>194</v>
       </c>
-      <c r="H128" s="1">
+      <c r="H128" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4388,13 +4414,13 @@
       <c r="D129" t="s">
         <v>127</v>
       </c>
-      <c r="E129" s="1">
+      <c r="E129" s="2">
         <v>46213</v>
       </c>
       <c r="G129" t="s">
         <v>194</v>
       </c>
-      <c r="H129" s="1">
+      <c r="H129" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4408,7 +4434,7 @@
       <c r="C130" t="s">
         <v>115</v>
       </c>
-      <c r="H130" s="1">
+      <c r="H130" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4425,13 +4451,13 @@
       <c r="D131" t="s">
         <v>128</v>
       </c>
-      <c r="E131" s="1">
+      <c r="E131" s="2">
         <v>46216</v>
       </c>
       <c r="G131" t="s">
         <v>195</v>
       </c>
-      <c r="H131" s="1">
+      <c r="H131" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4448,13 +4474,13 @@
       <c r="D132" t="s">
         <v>144</v>
       </c>
-      <c r="E132" s="1">
+      <c r="E132" s="2">
         <v>46213</v>
       </c>
       <c r="G132" t="s">
         <v>194</v>
       </c>
-      <c r="H132" s="1">
+      <c r="H132" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4468,7 +4494,7 @@
       <c r="C133" t="s">
         <v>115</v>
       </c>
-      <c r="H133" s="1">
+      <c r="H133" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4482,7 +4508,7 @@
       <c r="C134" t="s">
         <v>115</v>
       </c>
-      <c r="H134" s="1">
+      <c r="H134" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4496,7 +4522,7 @@
       <c r="C135" t="s">
         <v>115</v>
       </c>
-      <c r="H135" s="1">
+      <c r="H135" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4513,13 +4539,13 @@
       <c r="D136" t="s">
         <v>146</v>
       </c>
-      <c r="E136" s="1">
+      <c r="E136" s="2">
         <v>46213</v>
       </c>
       <c r="G136" t="s">
         <v>194</v>
       </c>
-      <c r="H136" s="1">
+      <c r="H136" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4542,7 +4568,7 @@
       <c r="G137" t="s">
         <v>181</v>
       </c>
-      <c r="H137" s="1">
+      <c r="H137" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4556,7 +4582,7 @@
       <c r="C138" t="s">
         <v>119</v>
       </c>
-      <c r="H138" s="1">
+      <c r="H138" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4570,7 +4596,7 @@
       <c r="C139" t="s">
         <v>115</v>
       </c>
-      <c r="H139" s="1">
+      <c r="H139" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4593,7 +4619,7 @@
       <c r="G140" t="s">
         <v>176</v>
       </c>
-      <c r="H140" s="1">
+      <c r="H140" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4610,7 +4636,7 @@
       <c r="D141" t="s">
         <v>132</v>
       </c>
-      <c r="H141" s="1">
+      <c r="H141" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4633,7 +4659,7 @@
       <c r="G142" t="s">
         <v>177</v>
       </c>
-      <c r="H142" s="1">
+      <c r="H142" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4650,13 +4676,13 @@
       <c r="D143" t="s">
         <v>134</v>
       </c>
-      <c r="E143" s="1">
+      <c r="E143" s="2">
         <v>46209</v>
       </c>
       <c r="G143" t="s">
         <v>197</v>
       </c>
-      <c r="H143" s="1">
+      <c r="H143" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4679,7 +4705,7 @@
       <c r="G144" t="s">
         <v>178</v>
       </c>
-      <c r="H144" s="1">
+      <c r="H144" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4702,7 +4728,7 @@
       <c r="G145" t="s">
         <v>178</v>
       </c>
-      <c r="H145" s="1">
+      <c r="H145" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4725,7 +4751,7 @@
       <c r="G146" t="s">
         <v>179</v>
       </c>
-      <c r="H146" s="1">
+      <c r="H146" s="2">
         <v>46211</v>
       </c>
     </row>
@@ -4739,7 +4765,7 @@
       <c r="C147" t="s">
         <v>115</v>
       </c>
-      <c r="H147" s="1">
+      <c r="H147" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4756,13 +4782,13 @@
       <c r="D148" t="s">
         <v>142</v>
       </c>
-      <c r="E148" s="1">
+      <c r="E148" s="2">
         <v>46217</v>
       </c>
       <c r="G148" t="s">
         <v>199</v>
       </c>
-      <c r="H148" s="1">
+      <c r="H148" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4776,7 +4802,7 @@
       <c r="C149" t="s">
         <v>119</v>
       </c>
-      <c r="H149" s="1">
+      <c r="H149" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4790,7 +4816,7 @@
       <c r="C150" t="s">
         <v>115</v>
       </c>
-      <c r="H150" s="1">
+      <c r="H150" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4804,7 +4830,7 @@
       <c r="C151" t="s">
         <v>115</v>
       </c>
-      <c r="H151" s="1">
+      <c r="H151" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4818,7 +4844,7 @@
       <c r="C152" t="s">
         <v>119</v>
       </c>
-      <c r="H152" s="1">
+      <c r="H152" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4832,7 +4858,7 @@
       <c r="C153" t="s">
         <v>119</v>
       </c>
-      <c r="H153" s="1">
+      <c r="H153" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4849,13 +4875,13 @@
       <c r="D154" t="s">
         <v>125</v>
       </c>
-      <c r="E154" s="1">
+      <c r="E154" s="2">
         <v>46234</v>
       </c>
       <c r="G154" t="s">
         <v>193</v>
       </c>
-      <c r="H154" s="1">
+      <c r="H154" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4872,13 +4898,13 @@
       <c r="D155" t="s">
         <v>126</v>
       </c>
-      <c r="E155" s="1">
+      <c r="E155" s="2">
         <v>46213</v>
       </c>
       <c r="G155" t="s">
         <v>194</v>
       </c>
-      <c r="H155" s="1">
+      <c r="H155" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4892,7 +4918,7 @@
       <c r="C156" t="s">
         <v>115</v>
       </c>
-      <c r="H156" s="1">
+      <c r="H156" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4909,13 +4935,13 @@
       <c r="D157" t="s">
         <v>143</v>
       </c>
-      <c r="E157" s="1">
+      <c r="E157" s="2">
         <v>46213</v>
       </c>
       <c r="G157" t="s">
         <v>194</v>
       </c>
-      <c r="H157" s="1">
+      <c r="H157" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4932,13 +4958,13 @@
       <c r="D158" t="s">
         <v>127</v>
       </c>
-      <c r="E158" s="1">
+      <c r="E158" s="2">
         <v>46213</v>
       </c>
       <c r="G158" t="s">
         <v>194</v>
       </c>
-      <c r="H158" s="1">
+      <c r="H158" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4955,13 +4981,13 @@
       <c r="D159" t="s">
         <v>147</v>
       </c>
-      <c r="E159" s="1">
+      <c r="E159" s="2">
         <v>46212</v>
       </c>
       <c r="G159" t="s">
         <v>200</v>
       </c>
-      <c r="H159" s="1">
+      <c r="H159" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -4978,13 +5004,13 @@
       <c r="D160" t="s">
         <v>128</v>
       </c>
-      <c r="E160" s="1">
+      <c r="E160" s="2">
         <v>46216</v>
       </c>
       <c r="G160" t="s">
         <v>195</v>
       </c>
-      <c r="H160" s="1">
+      <c r="H160" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5001,13 +5027,13 @@
       <c r="D161" t="s">
         <v>144</v>
       </c>
-      <c r="E161" s="1">
+      <c r="E161" s="2">
         <v>46213</v>
       </c>
       <c r="G161" t="s">
         <v>194</v>
       </c>
-      <c r="H161" s="1">
+      <c r="H161" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5021,7 +5047,7 @@
       <c r="C162" t="s">
         <v>115</v>
       </c>
-      <c r="H162" s="1">
+      <c r="H162" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5035,7 +5061,7 @@
       <c r="C163" t="s">
         <v>115</v>
       </c>
-      <c r="H163" s="1">
+      <c r="H163" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5049,7 +5075,7 @@
       <c r="C164" t="s">
         <v>115</v>
       </c>
-      <c r="H164" s="1">
+      <c r="H164" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5066,13 +5092,13 @@
       <c r="D165" t="s">
         <v>146</v>
       </c>
-      <c r="E165" s="1">
+      <c r="E165" s="2">
         <v>46213</v>
       </c>
       <c r="G165" t="s">
         <v>194</v>
       </c>
-      <c r="H165" s="1">
+      <c r="H165" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5095,7 +5121,7 @@
       <c r="G166" t="s">
         <v>181</v>
       </c>
-      <c r="H166" s="1">
+      <c r="H166" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5109,7 +5135,7 @@
       <c r="C167" t="s">
         <v>119</v>
       </c>
-      <c r="H167" s="1">
+      <c r="H167" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5123,7 +5149,7 @@
       <c r="C168" t="s">
         <v>115</v>
       </c>
-      <c r="H168" s="1">
+      <c r="H168" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5146,7 +5172,7 @@
       <c r="G169" t="s">
         <v>176</v>
       </c>
-      <c r="H169" s="1">
+      <c r="H169" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5163,7 +5189,7 @@
       <c r="D170" t="s">
         <v>132</v>
       </c>
-      <c r="H170" s="1">
+      <c r="H170" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5186,7 +5212,7 @@
       <c r="G171" t="s">
         <v>177</v>
       </c>
-      <c r="H171" s="1">
+      <c r="H171" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5203,13 +5229,13 @@
       <c r="D172" t="s">
         <v>134</v>
       </c>
-      <c r="E172" s="1">
+      <c r="E172" s="2">
         <v>46209</v>
       </c>
       <c r="G172" t="s">
         <v>197</v>
       </c>
-      <c r="H172" s="1">
+      <c r="H172" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5232,7 +5258,7 @@
       <c r="G173" t="s">
         <v>178</v>
       </c>
-      <c r="H173" s="1">
+      <c r="H173" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5255,7 +5281,7 @@
       <c r="G174" t="s">
         <v>178</v>
       </c>
-      <c r="H174" s="1">
+      <c r="H174" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5278,7 +5304,7 @@
       <c r="G175" t="s">
         <v>179</v>
       </c>
-      <c r="H175" s="1">
+      <c r="H175" s="2">
         <v>46212</v>
       </c>
     </row>
@@ -5292,7 +5318,7 @@
       <c r="C176" t="s">
         <v>115</v>
       </c>
-      <c r="H176" s="1">
+      <c r="H176" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5309,13 +5335,13 @@
       <c r="D177" t="s">
         <v>148</v>
       </c>
-      <c r="E177" s="1">
+      <c r="E177" s="2">
         <v>46217</v>
       </c>
       <c r="G177" t="s">
         <v>199</v>
       </c>
-      <c r="H177" s="1">
+      <c r="H177" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5329,7 +5355,7 @@
       <c r="C178" t="s">
         <v>115</v>
       </c>
-      <c r="H178" s="1">
+      <c r="H178" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5346,13 +5372,13 @@
       <c r="D179" t="s">
         <v>149</v>
       </c>
-      <c r="E179" s="1">
+      <c r="E179" s="2">
         <v>46216</v>
       </c>
       <c r="G179" t="s">
         <v>195</v>
       </c>
-      <c r="H179" s="1">
+      <c r="H179" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5366,7 +5392,7 @@
       <c r="C180" t="s">
         <v>115</v>
       </c>
-      <c r="H180" s="1">
+      <c r="H180" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5380,7 +5406,7 @@
       <c r="C181" t="s">
         <v>119</v>
       </c>
-      <c r="H181" s="1">
+      <c r="H181" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5394,7 +5420,7 @@
       <c r="C182" t="s">
         <v>119</v>
       </c>
-      <c r="H182" s="1">
+      <c r="H182" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5411,13 +5437,13 @@
       <c r="D183" t="s">
         <v>125</v>
       </c>
-      <c r="E183" s="1">
+      <c r="E183" s="2">
         <v>46234</v>
       </c>
       <c r="G183" t="s">
         <v>193</v>
       </c>
-      <c r="H183" s="1">
+      <c r="H183" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5434,13 +5460,13 @@
       <c r="D184" t="s">
         <v>126</v>
       </c>
-      <c r="E184" s="1">
+      <c r="E184" s="2">
         <v>46213</v>
       </c>
       <c r="G184" t="s">
         <v>194</v>
       </c>
-      <c r="H184" s="1">
+      <c r="H184" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5454,7 +5480,7 @@
       <c r="C185" t="s">
         <v>115</v>
       </c>
-      <c r="H185" s="1">
+      <c r="H185" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5471,13 +5497,13 @@
       <c r="D186" t="s">
         <v>143</v>
       </c>
-      <c r="E186" s="1">
+      <c r="E186" s="2">
         <v>46213</v>
       </c>
       <c r="G186" t="s">
         <v>194</v>
       </c>
-      <c r="H186" s="1">
+      <c r="H186" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5494,13 +5520,13 @@
       <c r="D187" t="s">
         <v>150</v>
       </c>
-      <c r="E187" s="1">
+      <c r="E187" s="2">
         <v>46213</v>
       </c>
       <c r="G187" t="s">
         <v>194</v>
       </c>
-      <c r="H187" s="1">
+      <c r="H187" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5517,13 +5543,13 @@
       <c r="D188" t="s">
         <v>151</v>
       </c>
-      <c r="E188" s="1">
+      <c r="E188" s="2">
         <v>46213</v>
       </c>
       <c r="G188" t="s">
         <v>194</v>
       </c>
-      <c r="H188" s="1">
+      <c r="H188" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5540,13 +5566,13 @@
       <c r="D189" t="s">
         <v>128</v>
       </c>
-      <c r="E189" s="1">
+      <c r="E189" s="2">
         <v>46216</v>
       </c>
       <c r="G189" t="s">
         <v>195</v>
       </c>
-      <c r="H189" s="1">
+      <c r="H189" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5563,13 +5589,13 @@
       <c r="D190" t="s">
         <v>144</v>
       </c>
-      <c r="E190" s="1">
+      <c r="E190" s="2">
         <v>46213</v>
       </c>
       <c r="G190" t="s">
         <v>194</v>
       </c>
-      <c r="H190" s="1">
+      <c r="H190" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5583,7 +5609,7 @@
       <c r="C191" t="s">
         <v>115</v>
       </c>
-      <c r="H191" s="1">
+      <c r="H191" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5597,7 +5623,7 @@
       <c r="C192" t="s">
         <v>115</v>
       </c>
-      <c r="H192" s="1">
+      <c r="H192" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5611,7 +5637,7 @@
       <c r="C193" t="s">
         <v>115</v>
       </c>
-      <c r="H193" s="1">
+      <c r="H193" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5628,13 +5654,13 @@
       <c r="D194" t="s">
         <v>146</v>
       </c>
-      <c r="E194" s="1">
+      <c r="E194" s="2">
         <v>46218</v>
       </c>
       <c r="G194" t="s">
         <v>201</v>
       </c>
-      <c r="H194" s="1">
+      <c r="H194" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5657,7 +5683,7 @@
       <c r="G195" t="s">
         <v>181</v>
       </c>
-      <c r="H195" s="1">
+      <c r="H195" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5671,7 +5697,7 @@
       <c r="C196" t="s">
         <v>119</v>
       </c>
-      <c r="H196" s="1">
+      <c r="H196" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5685,7 +5711,7 @@
       <c r="C197" t="s">
         <v>115</v>
       </c>
-      <c r="H197" s="1">
+      <c r="H197" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5708,7 +5734,7 @@
       <c r="G198" t="s">
         <v>176</v>
       </c>
-      <c r="H198" s="1">
+      <c r="H198" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5725,7 +5751,7 @@
       <c r="D199" t="s">
         <v>132</v>
       </c>
-      <c r="H199" s="1">
+      <c r="H199" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5748,7 +5774,7 @@
       <c r="G200" t="s">
         <v>177</v>
       </c>
-      <c r="H200" s="1">
+      <c r="H200" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5765,13 +5791,13 @@
       <c r="D201" t="s">
         <v>134</v>
       </c>
-      <c r="E201" s="1">
+      <c r="E201" s="2">
         <v>46209</v>
       </c>
       <c r="G201" t="s">
         <v>197</v>
       </c>
-      <c r="H201" s="1">
+      <c r="H201" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5794,7 +5820,7 @@
       <c r="G202" t="s">
         <v>178</v>
       </c>
-      <c r="H202" s="1">
+      <c r="H202" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5817,7 +5843,7 @@
       <c r="G203" t="s">
         <v>178</v>
       </c>
-      <c r="H203" s="1">
+      <c r="H203" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5840,7 +5866,7 @@
       <c r="G204" t="s">
         <v>179</v>
       </c>
-      <c r="H204" s="1">
+      <c r="H204" s="2">
         <v>46213</v>
       </c>
     </row>
@@ -5854,7 +5880,7 @@
       <c r="C205" t="s">
         <v>115</v>
       </c>
-      <c r="H205" s="1">
+      <c r="H205" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5871,13 +5897,13 @@
       <c r="D206" t="s">
         <v>148</v>
       </c>
-      <c r="E206" s="1">
+      <c r="E206" s="2">
         <v>46217</v>
       </c>
       <c r="G206" t="s">
         <v>199</v>
       </c>
-      <c r="H206" s="1">
+      <c r="H206" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5891,7 +5917,7 @@
       <c r="C207" t="s">
         <v>115</v>
       </c>
-      <c r="H207" s="1">
+      <c r="H207" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5905,7 +5931,7 @@
       <c r="C208" t="s">
         <v>119</v>
       </c>
-      <c r="H208" s="1">
+      <c r="H208" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5919,7 +5945,7 @@
       <c r="C209" t="s">
         <v>115</v>
       </c>
-      <c r="H209" s="1">
+      <c r="H209" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5933,7 +5959,7 @@
       <c r="C210" t="s">
         <v>119</v>
       </c>
-      <c r="H210" s="1">
+      <c r="H210" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5947,7 +5973,7 @@
       <c r="C211" t="s">
         <v>119</v>
       </c>
-      <c r="H211" s="1">
+      <c r="H211" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5964,13 +5990,13 @@
       <c r="D212" t="s">
         <v>125</v>
       </c>
-      <c r="E212" s="1">
+      <c r="E212" s="2">
         <v>46234</v>
       </c>
       <c r="G212" t="s">
         <v>193</v>
       </c>
-      <c r="H212" s="1">
+      <c r="H212" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5984,7 +6010,7 @@
       <c r="C213" t="s">
         <v>119</v>
       </c>
-      <c r="H213" s="1">
+      <c r="H213" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -5998,7 +6024,7 @@
       <c r="C214" t="s">
         <v>115</v>
       </c>
-      <c r="H214" s="1">
+      <c r="H214" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6015,13 +6041,13 @@
       <c r="D215" t="s">
         <v>143</v>
       </c>
-      <c r="E215" s="1">
+      <c r="E215" s="2">
         <v>46220</v>
       </c>
       <c r="G215" t="s">
         <v>202</v>
       </c>
-      <c r="H215" s="1">
+      <c r="H215" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6038,13 +6064,13 @@
       <c r="D216" t="s">
         <v>150</v>
       </c>
-      <c r="E216" s="1">
+      <c r="E216" s="2">
         <v>46216</v>
       </c>
       <c r="G216" t="s">
         <v>195</v>
       </c>
-      <c r="H216" s="1">
+      <c r="H216" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6058,7 +6084,7 @@
       <c r="C217" t="s">
         <v>115</v>
       </c>
-      <c r="H217" s="1">
+      <c r="H217" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6075,13 +6101,13 @@
       <c r="D218" t="s">
         <v>128</v>
       </c>
-      <c r="E218" s="1">
+      <c r="E218" s="2">
         <v>46216</v>
       </c>
       <c r="G218" t="s">
         <v>195</v>
       </c>
-      <c r="H218" s="1">
+      <c r="H218" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6095,7 +6121,7 @@
       <c r="C219" t="s">
         <v>115</v>
       </c>
-      <c r="H219" s="1">
+      <c r="H219" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6109,7 +6135,7 @@
       <c r="C220" t="s">
         <v>115</v>
       </c>
-      <c r="H220" s="1">
+      <c r="H220" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6126,13 +6152,13 @@
       <c r="D221" t="s">
         <v>152</v>
       </c>
-      <c r="E221" s="1">
+      <c r="E221" s="2">
         <v>46217</v>
       </c>
       <c r="G221" t="s">
         <v>199</v>
       </c>
-      <c r="H221" s="1">
+      <c r="H221" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6146,7 +6172,7 @@
       <c r="C222" t="s">
         <v>115</v>
       </c>
-      <c r="H222" s="1">
+      <c r="H222" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6163,13 +6189,13 @@
       <c r="D223" t="s">
         <v>153</v>
       </c>
-      <c r="E223" s="1">
+      <c r="E223" s="2">
         <v>46241</v>
       </c>
       <c r="G223" t="s">
         <v>203</v>
       </c>
-      <c r="H223" s="1">
+      <c r="H223" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6192,7 +6218,7 @@
       <c r="G224" t="s">
         <v>181</v>
       </c>
-      <c r="H224" s="1">
+      <c r="H224" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6206,7 +6232,7 @@
       <c r="C225" t="s">
         <v>119</v>
       </c>
-      <c r="H225" s="1">
+      <c r="H225" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="C226" t="s">
         <v>115</v>
       </c>
-      <c r="H226" s="1">
+      <c r="H226" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6243,7 +6269,7 @@
       <c r="G227" t="s">
         <v>176</v>
       </c>
-      <c r="H227" s="1">
+      <c r="H227" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6260,7 +6286,7 @@
       <c r="D228" t="s">
         <v>132</v>
       </c>
-      <c r="H228" s="1">
+      <c r="H228" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6283,7 +6309,7 @@
       <c r="G229" t="s">
         <v>177</v>
       </c>
-      <c r="H229" s="1">
+      <c r="H229" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6300,13 +6326,13 @@
       <c r="D230" t="s">
         <v>154</v>
       </c>
-      <c r="E230" s="1">
+      <c r="E230" s="2">
         <v>46295</v>
       </c>
       <c r="G230" t="s">
         <v>204</v>
       </c>
-      <c r="H230" s="1">
+      <c r="H230" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6329,7 +6355,7 @@
       <c r="G231" t="s">
         <v>178</v>
       </c>
-      <c r="H231" s="1">
+      <c r="H231" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6352,7 +6378,7 @@
       <c r="G232" t="s">
         <v>178</v>
       </c>
-      <c r="H232" s="1">
+      <c r="H232" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6375,7 +6401,7 @@
       <c r="G233" t="s">
         <v>179</v>
       </c>
-      <c r="H233" s="1">
+      <c r="H233" s="2">
         <v>46216</v>
       </c>
     </row>
@@ -6389,7 +6415,7 @@
       <c r="C234" t="s">
         <v>115</v>
       </c>
-      <c r="H234" s="1">
+      <c r="H234" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6406,13 +6432,13 @@
       <c r="D235" t="s">
         <v>155</v>
       </c>
-      <c r="E235" s="1">
+      <c r="E235" s="2">
         <v>46217</v>
       </c>
       <c r="G235" t="s">
         <v>199</v>
       </c>
-      <c r="H235" s="1">
+      <c r="H235" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6426,7 +6452,7 @@
       <c r="C236" t="s">
         <v>115</v>
       </c>
-      <c r="H236" s="1">
+      <c r="H236" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6440,7 +6466,7 @@
       <c r="C237" t="s">
         <v>119</v>
       </c>
-      <c r="H237" s="1">
+      <c r="H237" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6454,7 +6480,7 @@
       <c r="C238" t="s">
         <v>115</v>
       </c>
-      <c r="H238" s="1">
+      <c r="H238" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6468,7 +6494,7 @@
       <c r="C239" t="s">
         <v>119</v>
       </c>
-      <c r="H239" s="1">
+      <c r="H239" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6482,7 +6508,7 @@
       <c r="C240" t="s">
         <v>119</v>
       </c>
-      <c r="H240" s="1">
+      <c r="H240" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6499,13 +6525,13 @@
       <c r="D241" t="s">
         <v>125</v>
       </c>
-      <c r="E241" s="1">
+      <c r="E241" s="2">
         <v>46234</v>
       </c>
       <c r="G241" t="s">
         <v>193</v>
       </c>
-      <c r="H241" s="1">
+      <c r="H241" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6519,7 +6545,7 @@
       <c r="C242" t="s">
         <v>119</v>
       </c>
-      <c r="H242" s="1">
+      <c r="H242" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6536,13 +6562,13 @@
       <c r="D243" t="s">
         <v>156</v>
       </c>
-      <c r="E243" s="1">
+      <c r="E243" s="2">
         <v>46224</v>
       </c>
       <c r="G243" t="s">
         <v>205</v>
       </c>
-      <c r="H243" s="1">
+      <c r="H243" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6559,13 +6585,13 @@
       <c r="D244" t="s">
         <v>157</v>
       </c>
-      <c r="E244" s="1">
+      <c r="E244" s="2">
         <v>46220</v>
       </c>
       <c r="G244" t="s">
         <v>202</v>
       </c>
-      <c r="H244" s="1">
+      <c r="H244" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6579,7 +6605,7 @@
       <c r="C245" t="s">
         <v>119</v>
       </c>
-      <c r="H245" s="1">
+      <c r="H245" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6593,7 +6619,7 @@
       <c r="C246" t="s">
         <v>115</v>
       </c>
-      <c r="H246" s="1">
+      <c r="H246" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6610,13 +6636,13 @@
       <c r="D247" t="s">
         <v>128</v>
       </c>
-      <c r="E247" s="1">
+      <c r="E247" s="2">
         <v>46237</v>
       </c>
       <c r="G247" t="s">
         <v>206</v>
       </c>
-      <c r="H247" s="1">
+      <c r="H247" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6630,7 +6656,7 @@
       <c r="C248" t="s">
         <v>115</v>
       </c>
-      <c r="H248" s="1">
+      <c r="H248" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6644,7 +6670,7 @@
       <c r="C249" t="s">
         <v>115</v>
       </c>
-      <c r="H249" s="1">
+      <c r="H249" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6661,13 +6687,13 @@
       <c r="D250" t="s">
         <v>158</v>
       </c>
-      <c r="E250" s="1">
+      <c r="E250" s="2">
         <v>46218</v>
       </c>
       <c r="G250" t="s">
         <v>201</v>
       </c>
-      <c r="H250" s="1">
+      <c r="H250" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6681,7 +6707,7 @@
       <c r="C251" t="s">
         <v>115</v>
       </c>
-      <c r="H251" s="1">
+      <c r="H251" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6698,13 +6724,13 @@
       <c r="D252" t="s">
         <v>159</v>
       </c>
-      <c r="E252" s="1">
+      <c r="E252" s="2">
         <v>46241</v>
       </c>
       <c r="G252" t="s">
         <v>203</v>
       </c>
-      <c r="H252" s="1">
+      <c r="H252" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6727,7 +6753,7 @@
       <c r="G253" t="s">
         <v>181</v>
       </c>
-      <c r="H253" s="1">
+      <c r="H253" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6741,7 +6767,7 @@
       <c r="C254" t="s">
         <v>119</v>
       </c>
-      <c r="H254" s="1">
+      <c r="H254" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6755,7 +6781,7 @@
       <c r="C255" t="s">
         <v>115</v>
       </c>
-      <c r="H255" s="1">
+      <c r="H255" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6778,7 +6804,7 @@
       <c r="G256" t="s">
         <v>176</v>
       </c>
-      <c r="H256" s="1">
+      <c r="H256" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6795,7 +6821,7 @@
       <c r="D257" t="s">
         <v>132</v>
       </c>
-      <c r="H257" s="1">
+      <c r="H257" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6818,7 +6844,7 @@
       <c r="G258" t="s">
         <v>177</v>
       </c>
-      <c r="H258" s="1">
+      <c r="H258" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6835,13 +6861,13 @@
       <c r="D259" t="s">
         <v>154</v>
       </c>
-      <c r="E259" s="1">
+      <c r="E259" s="2">
         <v>46295</v>
       </c>
       <c r="G259" t="s">
         <v>204</v>
       </c>
-      <c r="H259" s="1">
+      <c r="H259" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6864,7 +6890,7 @@
       <c r="G260" t="s">
         <v>178</v>
       </c>
-      <c r="H260" s="1">
+      <c r="H260" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6887,7 +6913,7 @@
       <c r="G261" t="s">
         <v>178</v>
       </c>
-      <c r="H261" s="1">
+      <c r="H261" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6910,7 +6936,7 @@
       <c r="G262" t="s">
         <v>179</v>
       </c>
-      <c r="H262" s="1">
+      <c r="H262" s="2">
         <v>46217</v>
       </c>
     </row>
@@ -6924,7 +6950,7 @@
       <c r="C263" t="s">
         <v>115</v>
       </c>
-      <c r="H263" s="1">
+      <c r="H263" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6941,13 +6967,13 @@
       <c r="D264" t="s">
         <v>155</v>
       </c>
-      <c r="E264" s="1">
+      <c r="E264" s="2">
         <v>46217</v>
       </c>
       <c r="G264" t="s">
         <v>199</v>
       </c>
-      <c r="H264" s="1">
+      <c r="H264" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6961,7 +6987,7 @@
       <c r="C265" t="s">
         <v>115</v>
       </c>
-      <c r="H265" s="1">
+      <c r="H265" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6975,7 +7001,7 @@
       <c r="C266" t="s">
         <v>119</v>
       </c>
-      <c r="H266" s="1">
+      <c r="H266" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -6989,7 +7015,7 @@
       <c r="C267" t="s">
         <v>115</v>
       </c>
-      <c r="H267" s="1">
+      <c r="H267" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7003,7 +7029,7 @@
       <c r="C268" t="s">
         <v>119</v>
       </c>
-      <c r="H268" s="1">
+      <c r="H268" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7017,7 +7043,7 @@
       <c r="C269" t="s">
         <v>119</v>
       </c>
-      <c r="H269" s="1">
+      <c r="H269" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7034,13 +7060,13 @@
       <c r="D270" t="s">
         <v>125</v>
       </c>
-      <c r="E270" s="1">
+      <c r="E270" s="2">
         <v>46234</v>
       </c>
       <c r="G270" t="s">
         <v>193</v>
       </c>
-      <c r="H270" s="1">
+      <c r="H270" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7054,7 +7080,7 @@
       <c r="C271" t="s">
         <v>119</v>
       </c>
-      <c r="H271" s="1">
+      <c r="H271" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7071,13 +7097,13 @@
       <c r="D272" t="s">
         <v>156</v>
       </c>
-      <c r="E272" s="1">
+      <c r="E272" s="2">
         <v>46224</v>
       </c>
       <c r="G272" t="s">
         <v>205</v>
       </c>
-      <c r="H272" s="1">
+      <c r="H272" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7094,13 +7120,13 @@
       <c r="D273" t="s">
         <v>157</v>
       </c>
-      <c r="E273" s="1">
+      <c r="E273" s="2">
         <v>46219</v>
       </c>
       <c r="G273" t="s">
         <v>207</v>
       </c>
-      <c r="H273" s="1">
+      <c r="H273" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7114,7 +7140,7 @@
       <c r="C274" t="s">
         <v>115</v>
       </c>
-      <c r="H274" s="1">
+      <c r="H274" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7128,7 +7154,7 @@
       <c r="C275" t="s">
         <v>115</v>
       </c>
-      <c r="H275" s="1">
+      <c r="H275" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7145,13 +7171,13 @@
       <c r="D276" t="s">
         <v>128</v>
       </c>
-      <c r="E276" s="1">
+      <c r="E276" s="2">
         <v>46237</v>
       </c>
       <c r="G276" t="s">
         <v>206</v>
       </c>
-      <c r="H276" s="1">
+      <c r="H276" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7165,7 +7191,7 @@
       <c r="C277" t="s">
         <v>115</v>
       </c>
-      <c r="H277" s="1">
+      <c r="H277" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7182,13 +7208,13 @@
       <c r="D278" t="s">
         <v>160</v>
       </c>
-      <c r="E278" s="1">
+      <c r="E278" s="2">
         <v>46227</v>
       </c>
       <c r="G278" t="s">
         <v>208</v>
       </c>
-      <c r="H278" s="1">
+      <c r="H278" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7205,13 +7231,13 @@
       <c r="D279" t="s">
         <v>158</v>
       </c>
-      <c r="E279" s="1">
+      <c r="E279" s="2">
         <v>46219</v>
       </c>
       <c r="G279" t="s">
         <v>207</v>
       </c>
-      <c r="H279" s="1">
+      <c r="H279" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7225,7 +7251,7 @@
       <c r="C280" t="s">
         <v>115</v>
       </c>
-      <c r="H280" s="1">
+      <c r="H280" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7242,13 +7268,13 @@
       <c r="D281" t="s">
         <v>161</v>
       </c>
-      <c r="E281" s="1">
+      <c r="E281" s="2">
         <v>46241</v>
       </c>
       <c r="G281" t="s">
         <v>203</v>
       </c>
-      <c r="H281" s="1">
+      <c r="H281" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7271,7 +7297,7 @@
       <c r="G282" t="s">
         <v>181</v>
       </c>
-      <c r="H282" s="1">
+      <c r="H282" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7285,7 +7311,7 @@
       <c r="C283" t="s">
         <v>119</v>
       </c>
-      <c r="H283" s="1">
+      <c r="H283" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7299,7 +7325,7 @@
       <c r="C284" t="s">
         <v>115</v>
       </c>
-      <c r="H284" s="1">
+      <c r="H284" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7322,7 +7348,7 @@
       <c r="G285" t="s">
         <v>176</v>
       </c>
-      <c r="H285" s="1">
+      <c r="H285" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7339,7 +7365,7 @@
       <c r="D286" t="s">
         <v>132</v>
       </c>
-      <c r="H286" s="1">
+      <c r="H286" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7362,7 +7388,7 @@
       <c r="G287" t="s">
         <v>177</v>
       </c>
-      <c r="H287" s="1">
+      <c r="H287" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7379,13 +7405,13 @@
       <c r="D288" t="s">
         <v>154</v>
       </c>
-      <c r="E288" s="1">
+      <c r="E288" s="2">
         <v>46295</v>
       </c>
       <c r="G288" t="s">
         <v>204</v>
       </c>
-      <c r="H288" s="1">
+      <c r="H288" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7408,7 +7434,7 @@
       <c r="G289" t="s">
         <v>178</v>
       </c>
-      <c r="H289" s="1">
+      <c r="H289" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7431,7 +7457,7 @@
       <c r="G290" t="s">
         <v>178</v>
       </c>
-      <c r="H290" s="1">
+      <c r="H290" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7454,7 +7480,7 @@
       <c r="G291" t="s">
         <v>179</v>
       </c>
-      <c r="H291" s="1">
+      <c r="H291" s="2">
         <v>46218</v>
       </c>
     </row>
@@ -7468,7 +7494,7 @@
       <c r="C292" t="s">
         <v>115</v>
       </c>
-      <c r="H292" s="1">
+      <c r="H292" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7491,7 +7517,7 @@
       <c r="G293" t="s">
         <v>182</v>
       </c>
-      <c r="H293" s="1">
+      <c r="H293" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7505,7 +7531,7 @@
       <c r="C294" t="s">
         <v>115</v>
       </c>
-      <c r="H294" s="1">
+      <c r="H294" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7528,7 +7554,7 @@
       <c r="G295" t="s">
         <v>183</v>
       </c>
-      <c r="H295" s="1">
+      <c r="H295" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7542,7 +7568,7 @@
       <c r="C296" t="s">
         <v>115</v>
       </c>
-      <c r="H296" s="1">
+      <c r="H296" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7556,7 +7582,7 @@
       <c r="C297" t="s">
         <v>119</v>
       </c>
-      <c r="H297" s="1">
+      <c r="H297" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7579,7 +7605,7 @@
       <c r="G298" t="s">
         <v>184</v>
       </c>
-      <c r="H298" s="1">
+      <c r="H298" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7596,13 +7622,13 @@
       <c r="D299" t="s">
         <v>125</v>
       </c>
-      <c r="E299" s="1">
+      <c r="E299" s="2">
         <v>46234</v>
       </c>
       <c r="G299" t="s">
         <v>193</v>
       </c>
-      <c r="H299" s="1">
+      <c r="H299" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7616,7 +7642,7 @@
       <c r="C300" t="s">
         <v>115</v>
       </c>
-      <c r="H300" s="1">
+      <c r="H300" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7633,13 +7659,13 @@
       <c r="D301" t="s">
         <v>156</v>
       </c>
-      <c r="E301" s="1">
+      <c r="E301" s="2">
         <v>46224</v>
       </c>
       <c r="G301" t="s">
         <v>205</v>
       </c>
-      <c r="H301" s="1">
+      <c r="H301" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7656,13 +7682,13 @@
       <c r="D302" t="s">
         <v>157</v>
       </c>
-      <c r="E302" s="1">
+      <c r="E302" s="2">
         <v>46220</v>
       </c>
       <c r="G302" t="s">
         <v>202</v>
       </c>
-      <c r="H302" s="1">
+      <c r="H302" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7676,7 +7702,7 @@
       <c r="C303" t="s">
         <v>115</v>
       </c>
-      <c r="H303" s="1">
+      <c r="H303" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7690,7 +7716,7 @@
       <c r="C304" t="s">
         <v>115</v>
       </c>
-      <c r="H304" s="1">
+      <c r="H304" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7707,13 +7733,13 @@
       <c r="D305" t="s">
         <v>128</v>
       </c>
-      <c r="E305" s="1">
+      <c r="E305" s="2">
         <v>46237</v>
       </c>
       <c r="G305" t="s">
         <v>206</v>
       </c>
-      <c r="H305" s="1">
+      <c r="H305" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7727,7 +7753,7 @@
       <c r="C306" t="s">
         <v>115</v>
       </c>
-      <c r="H306" s="1">
+      <c r="H306" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7744,13 +7770,13 @@
       <c r="D307" t="s">
         <v>160</v>
       </c>
-      <c r="E307" s="1">
+      <c r="E307" s="2">
         <v>46227</v>
       </c>
       <c r="G307" t="s">
         <v>208</v>
       </c>
-      <c r="H307" s="1">
+      <c r="H307" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7764,7 +7790,7 @@
       <c r="C308" t="s">
         <v>119</v>
       </c>
-      <c r="H308" s="1">
+      <c r="H308" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7787,7 +7813,7 @@
       <c r="G309" t="s">
         <v>182</v>
       </c>
-      <c r="H309" s="1">
+      <c r="H309" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7810,7 +7836,7 @@
       <c r="G310" t="s">
         <v>185</v>
       </c>
-      <c r="H310" s="1">
+      <c r="H310" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7827,7 +7853,7 @@
       <c r="D311" t="s">
         <v>166</v>
       </c>
-      <c r="H311" s="1">
+      <c r="H311" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7841,7 +7867,7 @@
       <c r="C312" t="s">
         <v>119</v>
       </c>
-      <c r="H312" s="1">
+      <c r="H312" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7855,7 +7881,7 @@
       <c r="C313" t="s">
         <v>115</v>
       </c>
-      <c r="H313" s="1">
+      <c r="H313" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7878,7 +7904,7 @@
       <c r="G314" t="s">
         <v>176</v>
       </c>
-      <c r="H314" s="1">
+      <c r="H314" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7895,7 +7921,7 @@
       <c r="D315" t="s">
         <v>132</v>
       </c>
-      <c r="H315" s="1">
+      <c r="H315" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7918,7 +7944,7 @@
       <c r="G316" t="s">
         <v>177</v>
       </c>
-      <c r="H316" s="1">
+      <c r="H316" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7941,7 +7967,7 @@
       <c r="G317" t="s">
         <v>186</v>
       </c>
-      <c r="H317" s="1">
+      <c r="H317" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7964,7 +7990,7 @@
       <c r="G318" t="s">
         <v>178</v>
       </c>
-      <c r="H318" s="1">
+      <c r="H318" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -7987,7 +8013,7 @@
       <c r="G319" t="s">
         <v>178</v>
       </c>
-      <c r="H319" s="1">
+      <c r="H319" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -8010,7 +8036,7 @@
       <c r="G320" t="s">
         <v>179</v>
       </c>
-      <c r="H320" s="1">
+      <c r="H320" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -8024,7 +8050,7 @@
       <c r="C321" t="s">
         <v>115</v>
       </c>
-      <c r="H321" s="1">
+      <c r="H321" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8047,7 +8073,7 @@
       <c r="G322" t="s">
         <v>187</v>
       </c>
-      <c r="H322" s="1">
+      <c r="H322" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8061,7 +8087,7 @@
       <c r="C323" t="s">
         <v>115</v>
       </c>
-      <c r="H323" s="1">
+      <c r="H323" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8084,7 +8110,7 @@
       <c r="G324" t="s">
         <v>188</v>
       </c>
-      <c r="H324" s="1">
+      <c r="H324" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8098,7 +8124,7 @@
       <c r="C325" t="s">
         <v>115</v>
       </c>
-      <c r="H325" s="1">
+      <c r="H325" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8112,7 +8138,7 @@
       <c r="C326" t="s">
         <v>119</v>
       </c>
-      <c r="H326" s="1">
+      <c r="H326" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8126,7 +8152,7 @@
       <c r="C327" t="s">
         <v>119</v>
       </c>
-      <c r="H327" s="1">
+      <c r="H327" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8143,13 +8169,13 @@
       <c r="D328" t="s">
         <v>125</v>
       </c>
-      <c r="E328" s="1">
+      <c r="E328" s="2">
         <v>46234</v>
       </c>
       <c r="G328" t="s">
         <v>193</v>
       </c>
-      <c r="H328" s="1">
+      <c r="H328" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8172,7 +8198,7 @@
       <c r="G329" t="s">
         <v>188</v>
       </c>
-      <c r="H329" s="1">
+      <c r="H329" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8195,7 +8221,7 @@
       <c r="G330" t="s">
         <v>188</v>
       </c>
-      <c r="H330" s="1">
+      <c r="H330" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8209,7 +8235,7 @@
       <c r="C331" t="s">
         <v>115</v>
       </c>
-      <c r="H331" s="1">
+      <c r="H331" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8232,7 +8258,7 @@
       <c r="G332" t="s">
         <v>188</v>
       </c>
-      <c r="H332" s="1">
+      <c r="H332" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8255,7 +8281,7 @@
       <c r="G333" t="s">
         <v>187</v>
       </c>
-      <c r="H333" s="1">
+      <c r="H333" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8272,13 +8298,13 @@
       <c r="D334" t="s">
         <v>128</v>
       </c>
-      <c r="E334" s="1">
+      <c r="E334" s="2">
         <v>46237</v>
       </c>
       <c r="G334" t="s">
         <v>206</v>
       </c>
-      <c r="H334" s="1">
+      <c r="H334" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8292,7 +8318,7 @@
       <c r="C335" t="s">
         <v>115</v>
       </c>
-      <c r="H335" s="1">
+      <c r="H335" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8309,13 +8335,13 @@
       <c r="D336" t="s">
         <v>160</v>
       </c>
-      <c r="E336" s="1">
+      <c r="E336" s="2">
         <v>46227</v>
       </c>
       <c r="G336" t="s">
         <v>208</v>
       </c>
-      <c r="H336" s="1">
+      <c r="H336" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8329,7 +8355,7 @@
       <c r="C337" t="s">
         <v>115</v>
       </c>
-      <c r="H337" s="1">
+      <c r="H337" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8343,7 +8369,7 @@
       <c r="C338" t="s">
         <v>115</v>
       </c>
-      <c r="H338" s="1">
+      <c r="H338" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8366,7 +8392,7 @@
       <c r="G339" t="s">
         <v>185</v>
       </c>
-      <c r="H339" s="1">
+      <c r="H339" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8383,7 +8409,7 @@
       <c r="D340" t="s">
         <v>171</v>
       </c>
-      <c r="H340" s="1">
+      <c r="H340" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8397,7 +8423,7 @@
       <c r="C341" t="s">
         <v>119</v>
       </c>
-      <c r="H341" s="1">
+      <c r="H341" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8411,7 +8437,7 @@
       <c r="C342" t="s">
         <v>115</v>
       </c>
-      <c r="H342" s="1">
+      <c r="H342" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8434,7 +8460,7 @@
       <c r="G343" t="s">
         <v>176</v>
       </c>
-      <c r="H343" s="1">
+      <c r="H343" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8451,7 +8477,7 @@
       <c r="D344" t="s">
         <v>132</v>
       </c>
-      <c r="H344" s="1">
+      <c r="H344" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8474,7 +8500,7 @@
       <c r="G345" t="s">
         <v>177</v>
       </c>
-      <c r="H345" s="1">
+      <c r="H345" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8497,7 +8523,7 @@
       <c r="G346" t="s">
         <v>186</v>
       </c>
-      <c r="H346" s="1">
+      <c r="H346" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8520,7 +8546,7 @@
       <c r="G347" t="s">
         <v>178</v>
       </c>
-      <c r="H347" s="1">
+      <c r="H347" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8543,7 +8569,7 @@
       <c r="G348" t="s">
         <v>178</v>
       </c>
-      <c r="H348" s="1">
+      <c r="H348" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8566,7 +8592,7 @@
       <c r="G349" t="s">
         <v>179</v>
       </c>
-      <c r="H349" s="1">
+      <c r="H349" s="2">
         <v>46224</v>
       </c>
     </row>
@@ -8580,7 +8606,7 @@
       <c r="C350" t="s">
         <v>115</v>
       </c>
-      <c r="H350" s="1">
+      <c r="H350" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8603,7 +8629,7 @@
       <c r="G351" t="s">
         <v>187</v>
       </c>
-      <c r="H351" s="1">
+      <c r="H351" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8617,7 +8643,7 @@
       <c r="C352" t="s">
         <v>115</v>
       </c>
-      <c r="H352" s="1">
+      <c r="H352" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8631,7 +8657,7 @@
       <c r="C353" t="s">
         <v>115</v>
       </c>
-      <c r="H353" s="1">
+      <c r="H353" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8645,7 +8671,7 @@
       <c r="C354" t="s">
         <v>115</v>
       </c>
-      <c r="H354" s="1">
+      <c r="H354" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8659,7 +8685,7 @@
       <c r="C355" t="s">
         <v>119</v>
       </c>
-      <c r="H355" s="1">
+      <c r="H355" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8673,7 +8699,7 @@
       <c r="C356" t="s">
         <v>119</v>
       </c>
-      <c r="H356" s="1">
+      <c r="H356" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8696,7 +8722,7 @@
       <c r="G357" t="s">
         <v>189</v>
       </c>
-      <c r="H357" s="1">
+      <c r="H357" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8710,7 +8736,7 @@
       <c r="C358" t="s">
         <v>115</v>
       </c>
-      <c r="H358" s="1">
+      <c r="H358" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8733,7 +8759,7 @@
       <c r="G359" t="s">
         <v>190</v>
       </c>
-      <c r="H359" s="1">
+      <c r="H359" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8747,7 +8773,7 @@
       <c r="C360" t="s">
         <v>115</v>
       </c>
-      <c r="H360" s="1">
+      <c r="H360" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8761,7 +8787,7 @@
       <c r="C361" t="s">
         <v>115</v>
       </c>
-      <c r="H361" s="1">
+      <c r="H361" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8784,7 +8810,7 @@
       <c r="G362" t="s">
         <v>187</v>
       </c>
-      <c r="H362" s="1">
+      <c r="H362" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8807,7 +8833,7 @@
       <c r="G363" t="s">
         <v>191</v>
       </c>
-      <c r="H363" s="1">
+      <c r="H363" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8821,7 +8847,7 @@
       <c r="C364" t="s">
         <v>115</v>
       </c>
-      <c r="H364" s="1">
+      <c r="H364" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8844,7 +8870,7 @@
       <c r="G365" t="s">
         <v>190</v>
       </c>
-      <c r="H365" s="1">
+      <c r="H365" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8858,7 +8884,7 @@
       <c r="C366" t="s">
         <v>115</v>
       </c>
-      <c r="H366" s="1">
+      <c r="H366" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8872,7 +8898,7 @@
       <c r="C367" t="s">
         <v>115</v>
       </c>
-      <c r="H367" s="1">
+      <c r="H367" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8895,7 +8921,7 @@
       <c r="G368" t="s">
         <v>189</v>
       </c>
-      <c r="H368" s="1">
+      <c r="H368" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8918,7 +8944,7 @@
       <c r="G369" t="s">
         <v>190</v>
       </c>
-      <c r="H369" s="1">
+      <c r="H369" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8935,7 +8961,7 @@
       <c r="D370" t="s">
         <v>171</v>
       </c>
-      <c r="H370" s="1">
+      <c r="H370" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8949,7 +8975,7 @@
       <c r="C371" t="s">
         <v>115</v>
       </c>
-      <c r="H371" s="1">
+      <c r="H371" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8972,7 +8998,7 @@
       <c r="G372" t="s">
         <v>176</v>
       </c>
-      <c r="H372" s="1">
+      <c r="H372" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -8989,7 +9015,7 @@
       <c r="D373" t="s">
         <v>132</v>
       </c>
-      <c r="H373" s="1">
+      <c r="H373" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9012,7 +9038,7 @@
       <c r="G374" t="s">
         <v>177</v>
       </c>
-      <c r="H374" s="1">
+      <c r="H374" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9035,7 +9061,7 @@
       <c r="G375" t="s">
         <v>186</v>
       </c>
-      <c r="H375" s="1">
+      <c r="H375" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9058,7 +9084,7 @@
       <c r="G376" t="s">
         <v>178</v>
       </c>
-      <c r="H376" s="1">
+      <c r="H376" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9081,7 +9107,7 @@
       <c r="G377" t="s">
         <v>178</v>
       </c>
-      <c r="H377" s="1">
+      <c r="H377" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9104,7 +9130,7 @@
       <c r="G378" t="s">
         <v>179</v>
       </c>
-      <c r="H378" s="1">
+      <c r="H378" s="2">
         <v>46225</v>
       </c>
     </row>
@@ -9118,7 +9144,7 @@
       <c r="C379" t="s">
         <v>115</v>
       </c>
-      <c r="H379" s="1">
+      <c r="H379" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9141,7 +9167,7 @@
       <c r="G380" t="s">
         <v>190</v>
       </c>
-      <c r="H380" s="1">
+      <c r="H380" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9155,7 +9181,7 @@
       <c r="C381" t="s">
         <v>115</v>
       </c>
-      <c r="H381" s="1">
+      <c r="H381" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9169,7 +9195,7 @@
       <c r="C382" t="s">
         <v>115</v>
       </c>
-      <c r="H382" s="1">
+      <c r="H382" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9183,7 +9209,7 @@
       <c r="C383" t="s">
         <v>115</v>
       </c>
-      <c r="H383" s="1">
+      <c r="H383" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9197,7 +9223,7 @@
       <c r="C384" t="s">
         <v>119</v>
       </c>
-      <c r="H384" s="1">
+      <c r="H384" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9211,7 +9237,7 @@
       <c r="C385" t="s">
         <v>119</v>
       </c>
-      <c r="H385" s="1">
+      <c r="H385" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9234,7 +9260,7 @@
       <c r="G386" t="s">
         <v>189</v>
       </c>
-      <c r="H386" s="1">
+      <c r="H386" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9248,7 +9274,7 @@
       <c r="C387" t="s">
         <v>115</v>
       </c>
-      <c r="H387" s="1">
+      <c r="H387" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9262,7 +9288,7 @@
       <c r="C388" t="s">
         <v>119</v>
       </c>
-      <c r="H388" s="1">
+      <c r="H388" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9276,7 +9302,7 @@
       <c r="C389" t="s">
         <v>115</v>
       </c>
-      <c r="H389" s="1">
+      <c r="H389" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9290,7 +9316,7 @@
       <c r="C390" t="s">
         <v>115</v>
       </c>
-      <c r="H390" s="1">
+      <c r="H390" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9313,7 +9339,7 @@
       <c r="G391" t="s">
         <v>190</v>
       </c>
-      <c r="H391" s="1">
+      <c r="H391" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9336,7 +9362,7 @@
       <c r="G392" t="s">
         <v>191</v>
       </c>
-      <c r="H392" s="1">
+      <c r="H392" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9350,7 +9376,7 @@
       <c r="C393" t="s">
         <v>115</v>
       </c>
-      <c r="H393" s="1">
+      <c r="H393" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9373,7 +9399,7 @@
       <c r="G394" t="s">
         <v>190</v>
       </c>
-      <c r="H394" s="1">
+      <c r="H394" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9387,7 +9413,7 @@
       <c r="C395" t="s">
         <v>115</v>
       </c>
-      <c r="H395" s="1">
+      <c r="H395" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9401,7 +9427,7 @@
       <c r="C396" t="s">
         <v>115</v>
       </c>
-      <c r="H396" s="1">
+      <c r="H396" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9424,7 +9450,7 @@
       <c r="G397" t="s">
         <v>189</v>
       </c>
-      <c r="H397" s="1">
+      <c r="H397" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9447,7 +9473,7 @@
       <c r="G398" t="s">
         <v>190</v>
       </c>
-      <c r="H398" s="1">
+      <c r="H398" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9464,7 +9490,7 @@
       <c r="D399" t="s">
         <v>171</v>
       </c>
-      <c r="H399" s="1">
+      <c r="H399" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9478,7 +9504,7 @@
       <c r="C400" t="s">
         <v>115</v>
       </c>
-      <c r="H400" s="1">
+      <c r="H400" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9501,7 +9527,7 @@
       <c r="G401" t="s">
         <v>176</v>
       </c>
-      <c r="H401" s="1">
+      <c r="H401" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9518,7 +9544,7 @@
       <c r="D402" t="s">
         <v>132</v>
       </c>
-      <c r="H402" s="1">
+      <c r="H402" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9541,7 +9567,7 @@
       <c r="G403" t="s">
         <v>177</v>
       </c>
-      <c r="H403" s="1">
+      <c r="H403" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9564,7 +9590,7 @@
       <c r="G404" t="s">
         <v>186</v>
       </c>
-      <c r="H404" s="1">
+      <c r="H404" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9587,7 +9613,7 @@
       <c r="G405" t="s">
         <v>178</v>
       </c>
-      <c r="H405" s="1">
+      <c r="H405" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9610,7 +9636,7 @@
       <c r="G406" t="s">
         <v>178</v>
       </c>
-      <c r="H406" s="1">
+      <c r="H406" s="2">
         <v>46226</v>
       </c>
     </row>
@@ -9633,7 +9659,7 @@
       <c r="G407" t="s">
         <v>179</v>
       </c>
-      <c r="H407" s="1">
+      <c r="H407" s="2">
         <v>46226</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige DPE nunca reconhecida — ponto final da linha quebrava o regex
RE_DATA_CURTA exigia fim de string logo após os dígitos, mas o relatório
sempre fecha a linha da aeronave com ponto ("DPE: 28/07."), então NENHUMA
DPE real era reconhecida — dpe_data ficava vazio pra quase toda aeronave
indisponível. Isso fazia a "Previsão de situação — próximos 7 dias" (Diagonal
de Manutenção) cair sempre no fallback de +14 dias em vez da DPE real,
parecendo travada a semana toda (Wallace: "previsao de disponibilidade ta
tudo igual 27 ate dia 02/08").

Corrigido tirando o ponto final antes de casar com os regex de data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_disponibilidade_diaria.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2090" uniqueCount="222">
   <si>
     <t>data_referencia</t>
   </si>
@@ -596,12 +596,63 @@
     <t>02 DIAS após chegada do item - Solicitado alteração de DPE e situação no SILOMS.</t>
   </si>
   <si>
+    <t>01 DIA APÓS CHEGADA DO MATERIAL.</t>
+  </si>
+  <si>
+    <t>03/07</t>
+  </si>
+  <si>
+    <t>31/07</t>
+  </si>
+  <si>
+    <t>10/07</t>
+  </si>
+  <si>
+    <t>13/07</t>
+  </si>
+  <si>
+    <t>01/07</t>
+  </si>
+  <si>
+    <t>06/07</t>
+  </si>
+  <si>
+    <t>07/07</t>
+  </si>
+  <si>
+    <t>14/07</t>
+  </si>
+  <si>
+    <t>09/07</t>
+  </si>
+  <si>
+    <t>15/07</t>
+  </si>
+  <si>
+    <t>17/07</t>
+  </si>
+  <si>
+    <t>07/08</t>
+  </si>
+  <si>
+    <t>30/09</t>
+  </si>
+  <si>
+    <t>21/07</t>
+  </si>
+  <si>
+    <t>03/08</t>
+  </si>
+  <si>
+    <t>16/07</t>
+  </si>
+  <si>
+    <t>24/07</t>
+  </si>
+  <si>
     <t>17/07.</t>
   </si>
   <si>
-    <t>01 DIA APÓS CHEGADA DO MATERIAL.</t>
-  </si>
-  <si>
     <t>20/07.</t>
   </si>
   <si>
@@ -630,57 +681,6 @@
   </si>
   <si>
     <t>27/07.</t>
-  </si>
-  <si>
-    <t>03/07</t>
-  </si>
-  <si>
-    <t>31/07</t>
-  </si>
-  <si>
-    <t>10/07</t>
-  </si>
-  <si>
-    <t>13/07</t>
-  </si>
-  <si>
-    <t>01/07</t>
-  </si>
-  <si>
-    <t>06/07</t>
-  </si>
-  <si>
-    <t>07/07</t>
-  </si>
-  <si>
-    <t>14/07</t>
-  </si>
-  <si>
-    <t>09/07</t>
-  </si>
-  <si>
-    <t>15/07</t>
-  </si>
-  <si>
-    <t>17/07</t>
-  </si>
-  <si>
-    <t>07/08</t>
-  </si>
-  <si>
-    <t>30/09</t>
-  </si>
-  <si>
-    <t>21/07</t>
-  </si>
-  <si>
-    <t>03/08</t>
-  </si>
-  <si>
-    <t>16/07</t>
-  </si>
-  <si>
-    <t>24/07</t>
   </si>
 </sst>
 </file>
@@ -2282,7 +2282,7 @@
         <v>46206</v>
       </c>
       <c r="G7" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H7" s="2">
         <v>46204</v>
@@ -2305,7 +2305,7 @@
         <v>46206</v>
       </c>
       <c r="G8" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H8" s="2">
         <v>46204</v>
@@ -2328,7 +2328,7 @@
         <v>46234</v>
       </c>
       <c r="G9" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H9" s="2">
         <v>46204</v>
@@ -2351,7 +2351,7 @@
         <v>46213</v>
       </c>
       <c r="G10" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H10" s="2">
         <v>46204</v>
@@ -2402,7 +2402,7 @@
         <v>46206</v>
       </c>
       <c r="G13" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H13" s="2">
         <v>46204</v>
@@ -2439,7 +2439,7 @@
         <v>46216</v>
       </c>
       <c r="G15" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H15" s="2">
         <v>46204</v>
@@ -2490,7 +2490,7 @@
         <v>46204</v>
       </c>
       <c r="G18" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="H18" s="2">
         <v>46204</v>
@@ -2527,7 +2527,7 @@
         <v>46206</v>
       </c>
       <c r="G20" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H20" s="2">
         <v>46204</v>
@@ -2664,7 +2664,7 @@
         <v>46209</v>
       </c>
       <c r="G27" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H27" s="2">
         <v>46204</v>
@@ -2835,7 +2835,7 @@
         <v>46206</v>
       </c>
       <c r="G36" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H36" s="2">
         <v>46205</v>
@@ -2858,7 +2858,7 @@
         <v>46206</v>
       </c>
       <c r="G37" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H37" s="2">
         <v>46205</v>
@@ -2881,7 +2881,7 @@
         <v>46234</v>
       </c>
       <c r="G38" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H38" s="2">
         <v>46205</v>
@@ -2904,7 +2904,7 @@
         <v>46213</v>
       </c>
       <c r="G39" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H39" s="2">
         <v>46205</v>
@@ -2955,7 +2955,7 @@
         <v>46206</v>
       </c>
       <c r="G42" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H42" s="2">
         <v>46205</v>
@@ -2992,7 +2992,7 @@
         <v>46216</v>
       </c>
       <c r="G44" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H44" s="2">
         <v>46205</v>
@@ -3071,7 +3071,7 @@
         <v>46206</v>
       </c>
       <c r="G49" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="H49" s="2">
         <v>46205</v>
@@ -3208,7 +3208,7 @@
         <v>46209</v>
       </c>
       <c r="G56" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H56" s="2">
         <v>46205</v>
@@ -3328,7 +3328,7 @@
         <v>46210</v>
       </c>
       <c r="G62" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="H62" s="2">
         <v>46209</v>
@@ -3365,7 +3365,7 @@
         <v>46217</v>
       </c>
       <c r="G64" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H64" s="2">
         <v>46209</v>
@@ -3416,7 +3416,7 @@
         <v>46234</v>
       </c>
       <c r="G67" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H67" s="2">
         <v>46209</v>
@@ -3439,7 +3439,7 @@
         <v>46213</v>
       </c>
       <c r="G68" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H68" s="2">
         <v>46209</v>
@@ -3490,7 +3490,7 @@
         <v>46210</v>
       </c>
       <c r="G71" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="H71" s="2">
         <v>46209</v>
@@ -3527,7 +3527,7 @@
         <v>46216</v>
       </c>
       <c r="G73" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H73" s="2">
         <v>46209</v>
@@ -3606,7 +3606,7 @@
         <v>46210</v>
       </c>
       <c r="G78" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="H78" s="2">
         <v>46209</v>
@@ -3743,7 +3743,7 @@
         <v>46209</v>
       </c>
       <c r="G85" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H85" s="2">
         <v>46209</v>
@@ -3849,7 +3849,7 @@
         <v>46217</v>
       </c>
       <c r="G90" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H90" s="2">
         <v>46210</v>
@@ -3872,7 +3872,7 @@
         <v>46210</v>
       </c>
       <c r="G91" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="H91" s="2">
         <v>46210</v>
@@ -3909,7 +3909,7 @@
         <v>46217</v>
       </c>
       <c r="G93" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H93" s="2">
         <v>46210</v>
@@ -3960,7 +3960,7 @@
         <v>46234</v>
       </c>
       <c r="G96" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H96" s="2">
         <v>46210</v>
@@ -3983,7 +3983,7 @@
         <v>46213</v>
       </c>
       <c r="G97" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H97" s="2">
         <v>46210</v>
@@ -4020,7 +4020,7 @@
         <v>46213</v>
       </c>
       <c r="G99" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H99" s="2">
         <v>46210</v>
@@ -4043,7 +4043,7 @@
         <v>46213</v>
       </c>
       <c r="G100" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H100" s="2">
         <v>46210</v>
@@ -4080,7 +4080,7 @@
         <v>46216</v>
       </c>
       <c r="G102" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H102" s="2">
         <v>46210</v>
@@ -4103,7 +4103,7 @@
         <v>46213</v>
       </c>
       <c r="G103" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H103" s="2">
         <v>46210</v>
@@ -4168,7 +4168,7 @@
         <v>46213</v>
       </c>
       <c r="G107" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H107" s="2">
         <v>46210</v>
@@ -4305,7 +4305,7 @@
         <v>46209</v>
       </c>
       <c r="G114" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H114" s="2">
         <v>46210</v>
@@ -4411,7 +4411,7 @@
         <v>46217</v>
       </c>
       <c r="G119" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H119" s="2">
         <v>46211</v>
@@ -4504,7 +4504,7 @@
         <v>46234</v>
       </c>
       <c r="G125" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H125" s="2">
         <v>46211</v>
@@ -4527,7 +4527,7 @@
         <v>46213</v>
       </c>
       <c r="G126" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H126" s="2">
         <v>46211</v>
@@ -4564,7 +4564,7 @@
         <v>46213</v>
       </c>
       <c r="G128" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H128" s="2">
         <v>46211</v>
@@ -4587,7 +4587,7 @@
         <v>46213</v>
       </c>
       <c r="G129" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H129" s="2">
         <v>46211</v>
@@ -4624,7 +4624,7 @@
         <v>46216</v>
       </c>
       <c r="G131" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H131" s="2">
         <v>46211</v>
@@ -4647,7 +4647,7 @@
         <v>46213</v>
       </c>
       <c r="G132" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H132" s="2">
         <v>46211</v>
@@ -4712,7 +4712,7 @@
         <v>46213</v>
       </c>
       <c r="G136" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H136" s="2">
         <v>46211</v>
@@ -4849,7 +4849,7 @@
         <v>46209</v>
       </c>
       <c r="G143" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H143" s="2">
         <v>46211</v>
@@ -4955,7 +4955,7 @@
         <v>46217</v>
       </c>
       <c r="G148" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H148" s="2">
         <v>46212</v>
@@ -5048,7 +5048,7 @@
         <v>46234</v>
       </c>
       <c r="G154" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H154" s="2">
         <v>46212</v>
@@ -5071,7 +5071,7 @@
         <v>46213</v>
       </c>
       <c r="G155" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H155" s="2">
         <v>46212</v>
@@ -5108,7 +5108,7 @@
         <v>46213</v>
       </c>
       <c r="G157" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H157" s="2">
         <v>46212</v>
@@ -5131,7 +5131,7 @@
         <v>46213</v>
       </c>
       <c r="G158" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H158" s="2">
         <v>46212</v>
@@ -5154,7 +5154,7 @@
         <v>46212</v>
       </c>
       <c r="G159" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="H159" s="2">
         <v>46212</v>
@@ -5177,7 +5177,7 @@
         <v>46216</v>
       </c>
       <c r="G160" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H160" s="2">
         <v>46212</v>
@@ -5200,7 +5200,7 @@
         <v>46213</v>
       </c>
       <c r="G161" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H161" s="2">
         <v>46212</v>
@@ -5265,7 +5265,7 @@
         <v>46213</v>
       </c>
       <c r="G165" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H165" s="2">
         <v>46212</v>
@@ -5402,7 +5402,7 @@
         <v>46209</v>
       </c>
       <c r="G172" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H172" s="2">
         <v>46212</v>
@@ -5508,7 +5508,7 @@
         <v>46217</v>
       </c>
       <c r="G177" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H177" s="2">
         <v>46213</v>
@@ -5545,7 +5545,7 @@
         <v>46216</v>
       </c>
       <c r="G179" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H179" s="2">
         <v>46213</v>
@@ -5610,7 +5610,7 @@
         <v>46234</v>
       </c>
       <c r="G183" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H183" s="2">
         <v>46213</v>
@@ -5633,7 +5633,7 @@
         <v>46213</v>
       </c>
       <c r="G184" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H184" s="2">
         <v>46213</v>
@@ -5670,7 +5670,7 @@
         <v>46213</v>
       </c>
       <c r="G186" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H186" s="2">
         <v>46213</v>
@@ -5693,7 +5693,7 @@
         <v>46213</v>
       </c>
       <c r="G187" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H187" s="2">
         <v>46213</v>
@@ -5716,7 +5716,7 @@
         <v>46213</v>
       </c>
       <c r="G188" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H188" s="2">
         <v>46213</v>
@@ -5739,7 +5739,7 @@
         <v>46216</v>
       </c>
       <c r="G189" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H189" s="2">
         <v>46213</v>
@@ -5762,7 +5762,7 @@
         <v>46213</v>
       </c>
       <c r="G190" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="H190" s="2">
         <v>46213</v>
@@ -5827,7 +5827,7 @@
         <v>46218</v>
       </c>
       <c r="G194" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="H194" s="2">
         <v>46213</v>
@@ -5964,7 +5964,7 @@
         <v>46209</v>
       </c>
       <c r="G201" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H201" s="2">
         <v>46213</v>
@@ -6070,7 +6070,7 @@
         <v>46217</v>
       </c>
       <c r="G206" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H206" s="2">
         <v>46216</v>
@@ -6163,7 +6163,7 @@
         <v>46234</v>
       </c>
       <c r="G212" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H212" s="2">
         <v>46216</v>
@@ -6214,7 +6214,7 @@
         <v>46220</v>
       </c>
       <c r="G215" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="H215" s="2">
         <v>46216</v>
@@ -6237,7 +6237,7 @@
         <v>46216</v>
       </c>
       <c r="G216" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H216" s="2">
         <v>46216</v>
@@ -6274,7 +6274,7 @@
         <v>46216</v>
       </c>
       <c r="G218" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H218" s="2">
         <v>46216</v>
@@ -6325,7 +6325,7 @@
         <v>46217</v>
       </c>
       <c r="G221" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H221" s="2">
         <v>46216</v>
@@ -6362,7 +6362,7 @@
         <v>46241</v>
       </c>
       <c r="G223" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="H223" s="2">
         <v>46216</v>
@@ -6499,7 +6499,7 @@
         <v>46295</v>
       </c>
       <c r="G230" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="H230" s="2">
         <v>46216</v>
@@ -6605,7 +6605,7 @@
         <v>46217</v>
       </c>
       <c r="G235" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H235" s="2">
         <v>46217</v>
@@ -6698,7 +6698,7 @@
         <v>46234</v>
       </c>
       <c r="G241" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H241" s="2">
         <v>46217</v>
@@ -6735,7 +6735,7 @@
         <v>46224</v>
       </c>
       <c r="G243" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="H243" s="2">
         <v>46217</v>
@@ -6758,7 +6758,7 @@
         <v>46220</v>
       </c>
       <c r="G244" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="H244" s="2">
         <v>46217</v>
@@ -6809,7 +6809,7 @@
         <v>46237</v>
       </c>
       <c r="G247" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="H247" s="2">
         <v>46217</v>
@@ -6860,7 +6860,7 @@
         <v>46218</v>
       </c>
       <c r="G250" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="H250" s="2">
         <v>46217</v>
@@ -6897,7 +6897,7 @@
         <v>46241</v>
       </c>
       <c r="G252" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="H252" s="2">
         <v>46217</v>
@@ -7034,7 +7034,7 @@
         <v>46295</v>
       </c>
       <c r="G259" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="H259" s="2">
         <v>46217</v>
@@ -7140,7 +7140,7 @@
         <v>46217</v>
       </c>
       <c r="G264" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="H264" s="2">
         <v>46218</v>
@@ -7233,7 +7233,7 @@
         <v>46234</v>
       </c>
       <c r="G270" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H270" s="2">
         <v>46218</v>
@@ -7270,7 +7270,7 @@
         <v>46224</v>
       </c>
       <c r="G272" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="H272" s="2">
         <v>46218</v>
@@ -7293,7 +7293,7 @@
         <v>46219</v>
       </c>
       <c r="G273" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="H273" s="2">
         <v>46218</v>
@@ -7344,7 +7344,7 @@
         <v>46237</v>
       </c>
       <c r="G276" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="H276" s="2">
         <v>46218</v>
@@ -7381,7 +7381,7 @@
         <v>46227</v>
       </c>
       <c r="G278" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="H278" s="2">
         <v>46218</v>
@@ -7404,7 +7404,7 @@
         <v>46219</v>
       </c>
       <c r="G279" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="H279" s="2">
         <v>46218</v>
@@ -7441,7 +7441,7 @@
         <v>46241</v>
       </c>
       <c r="G281" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="H281" s="2">
         <v>46218</v>
@@ -7578,7 +7578,7 @@
         <v>46295</v>
       </c>
       <c r="G288" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="H288" s="2">
         <v>46218</v>
@@ -7680,11 +7680,11 @@
       <c r="D293" t="s">
         <v>163</v>
       </c>
-      <c r="F293" t="s">
-        <v>193</v>
+      <c r="E293" s="2">
+        <v>46220</v>
       </c>
       <c r="G293" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="H293" s="2">
         <v>46220</v>
@@ -7718,10 +7718,10 @@
         <v>170</v>
       </c>
       <c r="F295" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G295" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H295" s="2">
         <v>46220</v>
@@ -7768,11 +7768,11 @@
       <c r="D298" t="s">
         <v>171</v>
       </c>
-      <c r="F298" t="s">
-        <v>195</v>
+      <c r="E298" s="2">
+        <v>46223</v>
       </c>
       <c r="G298" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="H298" s="2">
         <v>46220</v>
@@ -7795,7 +7795,7 @@
         <v>46234</v>
       </c>
       <c r="G299" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H299" s="2">
         <v>46220</v>
@@ -7832,7 +7832,7 @@
         <v>46224</v>
       </c>
       <c r="G301" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="H301" s="2">
         <v>46220</v>
@@ -7855,7 +7855,7 @@
         <v>46220</v>
       </c>
       <c r="G302" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="H302" s="2">
         <v>46220</v>
@@ -7906,7 +7906,7 @@
         <v>46237</v>
       </c>
       <c r="G305" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="H305" s="2">
         <v>46220</v>
@@ -7943,7 +7943,7 @@
         <v>46227</v>
       </c>
       <c r="G307" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="H307" s="2">
         <v>46220</v>
@@ -7976,11 +7976,11 @@
       <c r="D309" t="s">
         <v>172</v>
       </c>
-      <c r="F309" t="s">
-        <v>193</v>
+      <c r="E309" s="2">
+        <v>46220</v>
       </c>
       <c r="G309" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="H309" s="2">
         <v>46220</v>
@@ -7999,11 +7999,11 @@
       <c r="D310" t="s">
         <v>173</v>
       </c>
-      <c r="F310" t="s">
-        <v>196</v>
+      <c r="E310" s="2">
+        <v>46265</v>
       </c>
       <c r="G310" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="H310" s="2">
         <v>46220</v>
@@ -8130,11 +8130,11 @@
       <c r="D317" t="s">
         <v>162</v>
       </c>
-      <c r="F317" t="s">
-        <v>197</v>
+      <c r="E317" s="2">
+        <v>46295</v>
       </c>
       <c r="G317" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H317" s="2">
         <v>46220</v>
@@ -8236,11 +8236,11 @@
       <c r="D322" t="s">
         <v>163</v>
       </c>
-      <c r="F322" t="s">
-        <v>198</v>
+      <c r="E322" s="2">
+        <v>46225</v>
       </c>
       <c r="G322" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="H322" s="2">
         <v>46224</v>
@@ -8273,11 +8273,11 @@
       <c r="D324" t="s">
         <v>175</v>
       </c>
-      <c r="F324" t="s">
-        <v>199</v>
+      <c r="E324" s="2">
+        <v>46224</v>
       </c>
       <c r="G324" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="H324" s="2">
         <v>46224</v>
@@ -8342,7 +8342,7 @@
         <v>46234</v>
       </c>
       <c r="G328" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="H328" s="2">
         <v>46224</v>
@@ -8361,11 +8361,11 @@
       <c r="D329" t="s">
         <v>176</v>
       </c>
-      <c r="F329" t="s">
-        <v>199</v>
+      <c r="E329" s="2">
+        <v>46224</v>
       </c>
       <c r="G329" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="H329" s="2">
         <v>46224</v>
@@ -8384,11 +8384,11 @@
       <c r="D330" t="s">
         <v>164</v>
       </c>
-      <c r="F330" t="s">
-        <v>199</v>
+      <c r="E330" s="2">
+        <v>46224</v>
       </c>
       <c r="G330" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="H330" s="2">
         <v>46224</v>
@@ -8421,11 +8421,11 @@
       <c r="D332" t="s">
         <v>177</v>
       </c>
-      <c r="F332" t="s">
-        <v>199</v>
+      <c r="E332" s="2">
+        <v>46224</v>
       </c>
       <c r="G332" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="H332" s="2">
         <v>46224</v>
@@ -8444,11 +8444,11 @@
       <c r="D333" t="s">
         <v>178</v>
       </c>
-      <c r="F333" t="s">
-        <v>198</v>
+      <c r="E333" s="2">
+        <v>46225</v>
       </c>
       <c r="G333" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="H333" s="2">
         <v>46224</v>
@@ -8471,7 +8471,7 @@
         <v>46237</v>
       </c>
       <c r="G334" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="H334" s="2">
         <v>46224</v>
@@ -8508,7 +8508,7 @@
         <v>46227</v>
       </c>
       <c r="G336" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="H336" s="2">
         <v>46224</v>
@@ -8555,11 +8555,11 @@
       <c r="D339" t="s">
         <v>173</v>
       </c>
-      <c r="F339" t="s">
-        <v>196</v>
+      <c r="E339" s="2">
+        <v>46265</v>
       </c>
       <c r="G339" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="H339" s="2">
         <v>46224</v>
@@ -8686,11 +8686,11 @@
       <c r="D346" t="s">
         <v>162</v>
       </c>
-      <c r="F346" t="s">
-        <v>197</v>
+      <c r="E346" s="2">
+        <v>46295</v>
       </c>
       <c r="G346" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H346" s="2">
         <v>46224</v>
@@ -8792,11 +8792,11 @@
       <c r="D351" t="s">
         <v>163</v>
       </c>
-      <c r="F351" t="s">
-        <v>198</v>
+      <c r="E351" s="2">
+        <v>46225</v>
       </c>
       <c r="G351" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="H351" s="2">
         <v>46225</v>
@@ -8885,11 +8885,11 @@
       <c r="D357" t="s">
         <v>133</v>
       </c>
-      <c r="F357" t="s">
-        <v>200</v>
+      <c r="E357" s="2">
+        <v>46234</v>
       </c>
       <c r="G357" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H357" s="2">
         <v>46225</v>
@@ -8922,11 +8922,11 @@
       <c r="D359" t="s">
         <v>164</v>
       </c>
-      <c r="F359" t="s">
-        <v>201</v>
+      <c r="E359" s="2">
+        <v>46227</v>
       </c>
       <c r="G359" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H359" s="2">
         <v>46225</v>
@@ -8973,11 +8973,11 @@
       <c r="D362" t="s">
         <v>178</v>
       </c>
-      <c r="F362" t="s">
-        <v>198</v>
+      <c r="E362" s="2">
+        <v>46225</v>
       </c>
       <c r="G362" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="H362" s="2">
         <v>46225</v>
@@ -8996,11 +8996,11 @@
       <c r="D363" t="s">
         <v>136</v>
       </c>
-      <c r="F363" t="s">
-        <v>202</v>
+      <c r="E363" s="2">
+        <v>46237</v>
       </c>
       <c r="G363" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="H363" s="2">
         <v>46225</v>
@@ -9033,11 +9033,11 @@
       <c r="D365" t="s">
         <v>168</v>
       </c>
-      <c r="F365" t="s">
-        <v>201</v>
+      <c r="E365" s="2">
+        <v>46227</v>
       </c>
       <c r="G365" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H365" s="2">
         <v>46225</v>
@@ -9084,11 +9084,11 @@
       <c r="D368" t="s">
         <v>173</v>
       </c>
-      <c r="F368" t="s">
-        <v>200</v>
+      <c r="E368" s="2">
+        <v>46234</v>
       </c>
       <c r="G368" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H368" s="2">
         <v>46225</v>
@@ -9107,11 +9107,11 @@
       <c r="D369" t="s">
         <v>180</v>
       </c>
-      <c r="F369" t="s">
-        <v>201</v>
+      <c r="E369" s="2">
+        <v>46227</v>
       </c>
       <c r="G369" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H369" s="2">
         <v>46225</v>
@@ -9224,11 +9224,11 @@
       <c r="D375" t="s">
         <v>162</v>
       </c>
-      <c r="F375" t="s">
-        <v>197</v>
+      <c r="E375" s="2">
+        <v>46295</v>
       </c>
       <c r="G375" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H375" s="2">
         <v>46225</v>
@@ -9330,11 +9330,11 @@
       <c r="D380" t="s">
         <v>163</v>
       </c>
-      <c r="F380" t="s">
-        <v>201</v>
+      <c r="E380" s="2">
+        <v>46227</v>
       </c>
       <c r="G380" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H380" s="2">
         <v>46226</v>
@@ -9423,11 +9423,11 @@
       <c r="D386" t="s">
         <v>133</v>
       </c>
-      <c r="F386" t="s">
-        <v>200</v>
+      <c r="E386" s="2">
+        <v>46234</v>
       </c>
       <c r="G386" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H386" s="2">
         <v>46226</v>
@@ -9502,11 +9502,11 @@
       <c r="D391" t="s">
         <v>181</v>
       </c>
-      <c r="F391" t="s">
-        <v>201</v>
+      <c r="E391" s="2">
+        <v>46227</v>
       </c>
       <c r="G391" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H391" s="2">
         <v>46226</v>
@@ -9525,11 +9525,11 @@
       <c r="D392" t="s">
         <v>136</v>
       </c>
-      <c r="F392" t="s">
-        <v>202</v>
+      <c r="E392" s="2">
+        <v>46237</v>
       </c>
       <c r="G392" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="H392" s="2">
         <v>46226</v>
@@ -9562,11 +9562,11 @@
       <c r="D394" t="s">
         <v>168</v>
       </c>
-      <c r="F394" t="s">
-        <v>201</v>
+      <c r="E394" s="2">
+        <v>46227</v>
       </c>
       <c r="G394" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H394" s="2">
         <v>46226</v>
@@ -9613,11 +9613,11 @@
       <c r="D397" t="s">
         <v>173</v>
       </c>
-      <c r="F397" t="s">
-        <v>200</v>
+      <c r="E397" s="2">
+        <v>46234</v>
       </c>
       <c r="G397" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H397" s="2">
         <v>46226</v>
@@ -9636,11 +9636,11 @@
       <c r="D398" t="s">
         <v>180</v>
       </c>
-      <c r="F398" t="s">
-        <v>201</v>
+      <c r="E398" s="2">
+        <v>46227</v>
       </c>
       <c r="G398" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H398" s="2">
         <v>46226</v>
@@ -9753,11 +9753,11 @@
       <c r="D404" t="s">
         <v>162</v>
       </c>
-      <c r="F404" t="s">
-        <v>197</v>
+      <c r="E404" s="2">
+        <v>46295</v>
       </c>
       <c r="G404" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H404" s="2">
         <v>46226</v>
@@ -9859,11 +9859,11 @@
       <c r="D409" t="s">
         <v>150</v>
       </c>
-      <c r="F409" t="s">
-        <v>203</v>
+      <c r="E409" s="2">
+        <v>46231</v>
       </c>
       <c r="G409" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
       <c r="H409" s="2">
         <v>46227</v>
@@ -9952,11 +9952,11 @@
       <c r="D415" t="s">
         <v>182</v>
       </c>
-      <c r="F415" t="s">
-        <v>200</v>
+      <c r="E415" s="2">
+        <v>46234</v>
       </c>
       <c r="G415" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H415" s="2">
         <v>46227</v>
@@ -10031,11 +10031,11 @@
       <c r="D420" t="s">
         <v>136</v>
       </c>
-      <c r="F420" t="s">
-        <v>202</v>
+      <c r="E420" s="2">
+        <v>46237</v>
       </c>
       <c r="G420" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="H420" s="2">
         <v>46227</v>
@@ -10068,11 +10068,11 @@
       <c r="D422" t="s">
         <v>168</v>
       </c>
-      <c r="F422" t="s">
-        <v>201</v>
+      <c r="E422" s="2">
+        <v>46227</v>
       </c>
       <c r="G422" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H422" s="2">
         <v>46227</v>
@@ -10119,11 +10119,11 @@
       <c r="D425" t="s">
         <v>173</v>
       </c>
-      <c r="F425" t="s">
-        <v>200</v>
+      <c r="E425" s="2">
+        <v>46234</v>
       </c>
       <c r="G425" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H425" s="2">
         <v>46227</v>
@@ -10142,11 +10142,11 @@
       <c r="D426" t="s">
         <v>180</v>
       </c>
-      <c r="F426" t="s">
-        <v>201</v>
+      <c r="E426" s="2">
+        <v>46227</v>
       </c>
       <c r="G426" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="H426" s="2">
         <v>46227</v>
@@ -10259,11 +10259,11 @@
       <c r="D432" t="s">
         <v>162</v>
       </c>
-      <c r="F432" t="s">
-        <v>197</v>
+      <c r="E432" s="2">
+        <v>46295</v>
       </c>
       <c r="G432" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H432" s="2">
         <v>46227</v>
@@ -10351,11 +10351,11 @@
       <c r="D436" t="s">
         <v>183</v>
       </c>
-      <c r="F436" t="s">
-        <v>204</v>
+      <c r="E436" s="2">
+        <v>46230</v>
       </c>
       <c r="G436" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="H436" s="2">
         <v>46227</v>
@@ -10388,11 +10388,11 @@
       <c r="D438" t="s">
         <v>150</v>
       </c>
-      <c r="F438" t="s">
-        <v>203</v>
+      <c r="E438" s="2">
+        <v>46231</v>
       </c>
       <c r="G438" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
       <c r="H438" s="2">
         <v>46230</v>
@@ -10481,11 +10481,11 @@
       <c r="D444" t="s">
         <v>182</v>
       </c>
-      <c r="F444" t="s">
-        <v>200</v>
+      <c r="E444" s="2">
+        <v>46234</v>
       </c>
       <c r="G444" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H444" s="2">
         <v>46230</v>
@@ -10518,11 +10518,11 @@
       <c r="D446" t="s">
         <v>184</v>
       </c>
-      <c r="F446" t="s">
-        <v>204</v>
+      <c r="E446" s="2">
+        <v>46230</v>
       </c>
       <c r="G446" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="H446" s="2">
         <v>46230</v>
@@ -10569,11 +10569,11 @@
       <c r="D449" t="s">
         <v>136</v>
       </c>
-      <c r="F449" t="s">
-        <v>202</v>
+      <c r="E449" s="2">
+        <v>46237</v>
       </c>
       <c r="G449" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="H449" s="2">
         <v>46230</v>
@@ -10648,11 +10648,11 @@
       <c r="D454" t="s">
         <v>173</v>
       </c>
-      <c r="F454" t="s">
-        <v>200</v>
+      <c r="E454" s="2">
+        <v>46234</v>
       </c>
       <c r="G454" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="H454" s="2">
         <v>46230</v>
@@ -10779,11 +10779,11 @@
       <c r="D461" t="s">
         <v>162</v>
       </c>
-      <c r="F461" t="s">
-        <v>197</v>
+      <c r="E461" s="2">
+        <v>46295</v>
       </c>
       <c r="G461" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="H461" s="2">
         <v>46230</v>
@@ -10871,11 +10871,11 @@
       <c r="D465" t="s">
         <v>183</v>
       </c>
-      <c r="F465" t="s">
-        <v>204</v>
+      <c r="E465" s="2">
+        <v>46230</v>
       </c>
       <c r="G465" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="H465" s="2">
         <v>46230</v>

</xml_diff>